<commit_message>
House search data from run 8
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'For Sale'!$A$1:$W$212</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$169</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$174</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -16832,7 +16832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W169"/>
+  <dimension ref="A1:W174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -26888,7 +26888,7 @@
         </is>
       </c>
       <c r="C135" s="17" t="n">
-        <v>1100</v>
+        <v>1540</v>
       </c>
       <c r="D135" s="8" t="n">
         <v>1</v>
@@ -26903,21 +26903,23 @@
       </c>
       <c r="G135" s="9" t="inlineStr">
         <is>
-          <t>St Michaels Hill Ref 708</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H135" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I135" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I135" s="8" t="n">
+        <v>451</v>
+      </c>
       <c r="J135" s="8" t="n"/>
       <c r="K135" s="8" t="n"/>
       <c r="L135" s="8" t="n"/>
       <c r="M135" s="8" t="n"/>
       <c r="N135" s="8" t="n">
-        <v>19512</v>
+        <v>20820</v>
       </c>
       <c r="O135" s="8" t="n">
         <v>0</v>
@@ -26925,12 +26927,12 @@
       <c r="P135" s="8" t="n"/>
       <c r="Q135" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R135" s="8" t="inlineStr">
         <is>
-          <t>Jackson Property Management Ltd, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S135" s="9" t="inlineStr"/>
@@ -26947,7 +26949,7 @@
       <c r="V135" s="7" t="inlineStr"/>
       <c r="W135" s="8" t="inlineStr">
         <is>
-          <t>ad53fb9cd96ec72adbc7f3d6c8a52caba547cc20</t>
+          <t>824c36c2d3a0e83cbee4b39af6447bcd28387770</t>
         </is>
       </c>
     </row>
@@ -26961,13 +26963,13 @@
         </is>
       </c>
       <c r="C136" s="17" t="n">
-        <v>1095</v>
+        <v>2095</v>
       </c>
       <c r="D136" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E136" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F136" s="8" t="inlineStr">
         <is>
@@ -26976,21 +26978,23 @@
       </c>
       <c r="G136" s="9" t="inlineStr">
         <is>
-          <t>Manor House Lane, Whitchurch, Bristol, Bristol City</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H136" s="8" t="inlineStr">
         <is>
-          <t>BS14</t>
-        </is>
-      </c>
-      <c r="I136" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I136" s="8" t="n">
+        <v>705</v>
+      </c>
       <c r="J136" s="8" t="n"/>
       <c r="K136" s="8" t="n"/>
       <c r="L136" s="8" t="n"/>
       <c r="M136" s="8" t="n"/>
       <c r="N136" s="8" t="n">
-        <v>2652</v>
+        <v>20820</v>
       </c>
       <c r="O136" s="8" t="n">
         <v>0</v>
@@ -26998,12 +27002,12 @@
       <c r="P136" s="8" t="n"/>
       <c r="Q136" s="8" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R136" s="8" t="inlineStr">
         <is>
-          <t>Millennium Lettings &amp; Management, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S136" s="9" t="inlineStr"/>
@@ -27020,7 +27024,7 @@
       <c r="V136" s="7" t="inlineStr"/>
       <c r="W136" s="8" t="inlineStr">
         <is>
-          <t>ab692cb96ad18ebe26a6d19d737d0b539752370a</t>
+          <t>e2c2bae80b390d851516faec1c36e11343db8533</t>
         </is>
       </c>
     </row>
@@ -27034,7 +27038,7 @@
         </is>
       </c>
       <c r="C137" s="17" t="n">
-        <v>1200</v>
+        <v>1660</v>
       </c>
       <c r="D137" s="8" t="n">
         <v>1</v>
@@ -27049,23 +27053,23 @@
       </c>
       <c r="G137" s="9" t="inlineStr">
         <is>
-          <t>Old Market, Verdigris, BS2 0AF</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H137" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I137" s="8" t="n">
-        <v>388</v>
+        <v>486</v>
       </c>
       <c r="J137" s="8" t="n"/>
       <c r="K137" s="8" t="n"/>
       <c r="L137" s="8" t="n"/>
       <c r="M137" s="8" t="n"/>
       <c r="N137" s="8" t="n">
-        <v>21220</v>
+        <v>21504</v>
       </c>
       <c r="O137" s="8" t="n">
         <v>0</v>
@@ -27073,12 +27077,12 @@
       <c r="P137" s="8" t="n"/>
       <c r="Q137" s="8" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R137" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S137" s="9" t="inlineStr"/>
@@ -27095,314 +27099,383 @@
       <c r="V137" s="7" t="inlineStr"/>
       <c r="W137" s="8" t="inlineStr">
         <is>
+          <t>c2c660e4e8cefc047b4bc72bf19b48ce9ef7ec99</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B138" s="9" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C138" s="17" t="n">
+        <v>2175</v>
+      </c>
+      <c r="D138" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E138" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F138" s="8" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G138" s="9" t="inlineStr">
+        <is>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+        </is>
+      </c>
+      <c r="H138" s="8" t="inlineStr">
+        <is>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I138" s="8" t="n">
+        <v>814</v>
+      </c>
+      <c r="J138" s="8" t="n"/>
+      <c r="K138" s="8" t="n"/>
+      <c r="L138" s="8" t="n"/>
+      <c r="M138" s="8" t="n"/>
+      <c r="N138" s="8" t="n">
+        <v>21504</v>
+      </c>
+      <c r="O138" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P138" s="8" t="n"/>
+      <c r="Q138" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="R138" s="8" t="inlineStr">
+        <is>
+          <t>Grainger, Hawkins &amp; George</t>
+        </is>
+      </c>
+      <c r="S138" s="9" t="inlineStr"/>
+      <c r="T138" s="12" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U138" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V138" s="7" t="inlineStr"/>
+      <c r="W138" s="8" t="inlineStr">
+        <is>
+          <t>83406f05c9aded812a566cc6806036dda0d45fc0</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B139" s="9" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C139" s="17" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D139" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E139" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F139" s="8" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G139" s="9" t="inlineStr">
+        <is>
+          <t>Small Street - City Centre</t>
+        </is>
+      </c>
+      <c r="H139" s="8" t="inlineStr">
+        <is>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I139" s="8" t="n"/>
+      <c r="J139" s="8" t="n"/>
+      <c r="K139" s="8" t="n"/>
+      <c r="L139" s="8" t="n"/>
+      <c r="M139" s="8" t="n"/>
+      <c r="N139" s="8" t="n">
+        <v>21816</v>
+      </c>
+      <c r="O139" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P139" s="8" t="n"/>
+      <c r="Q139" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="R139" s="8" t="inlineStr">
+        <is>
+          <t>Ocean, Clifton</t>
+        </is>
+      </c>
+      <c r="S139" s="9" t="inlineStr"/>
+      <c r="T139" s="12" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U139" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V139" s="7" t="inlineStr"/>
+      <c r="W139" s="8" t="inlineStr">
+        <is>
+          <t>cb4b1af676ff54ae12ad7bf4fa94acd8ef94a533</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B140" s="9" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C140" s="17" t="n">
+        <v>1100</v>
+      </c>
+      <c r="D140" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E140" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F140" s="8" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G140" s="9" t="inlineStr">
+        <is>
+          <t>St Michaels Hill Ref 708</t>
+        </is>
+      </c>
+      <c r="H140" s="8" t="inlineStr">
+        <is>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I140" s="8" t="n"/>
+      <c r="J140" s="8" t="n"/>
+      <c r="K140" s="8" t="n"/>
+      <c r="L140" s="8" t="n"/>
+      <c r="M140" s="8" t="n"/>
+      <c r="N140" s="8" t="n">
+        <v>19512</v>
+      </c>
+      <c r="O140" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P140" s="8" t="n"/>
+      <c r="Q140" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="R140" s="8" t="inlineStr">
+        <is>
+          <t>Jackson Property Management Ltd, Bristol</t>
+        </is>
+      </c>
+      <c r="S140" s="9" t="inlineStr"/>
+      <c r="T140" s="12" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U140" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V140" s="7" t="inlineStr"/>
+      <c r="W140" s="8" t="inlineStr">
+        <is>
+          <t>ad53fb9cd96ec72adbc7f3d6c8a52caba547cc20</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B141" s="9" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C141" s="17" t="n">
+        <v>1095</v>
+      </c>
+      <c r="D141" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E141" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F141" s="8" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G141" s="9" t="inlineStr">
+        <is>
+          <t>Manor House Lane, Whitchurch, Bristol, Bristol City</t>
+        </is>
+      </c>
+      <c r="H141" s="8" t="inlineStr">
+        <is>
+          <t>BS14</t>
+        </is>
+      </c>
+      <c r="I141" s="8" t="n"/>
+      <c r="J141" s="8" t="n"/>
+      <c r="K141" s="8" t="n"/>
+      <c r="L141" s="8" t="n"/>
+      <c r="M141" s="8" t="n"/>
+      <c r="N141" s="8" t="n">
+        <v>2652</v>
+      </c>
+      <c r="O141" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P141" s="8" t="n"/>
+      <c r="Q141" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="R141" s="8" t="inlineStr">
+        <is>
+          <t>Millennium Lettings &amp; Management, Bristol</t>
+        </is>
+      </c>
+      <c r="S141" s="9" t="inlineStr"/>
+      <c r="T141" s="12" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U141" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V141" s="7" t="inlineStr"/>
+      <c r="W141" s="8" t="inlineStr">
+        <is>
+          <t>ab692cb96ad18ebe26a6d19d737d0b539752370a</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B142" s="9" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C142" s="17" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D142" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E142" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F142" s="8" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G142" s="9" t="inlineStr">
+        <is>
+          <t>Old Market, Verdigris, BS2 0AF</t>
+        </is>
+      </c>
+      <c r="H142" s="8" t="inlineStr">
+        <is>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I142" s="8" t="n">
+        <v>388</v>
+      </c>
+      <c r="J142" s="8" t="n"/>
+      <c r="K142" s="8" t="n"/>
+      <c r="L142" s="8" t="n"/>
+      <c r="M142" s="8" t="n"/>
+      <c r="N142" s="8" t="n">
+        <v>21220</v>
+      </c>
+      <c r="O142" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P142" s="8" t="n"/>
+      <c r="Q142" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="R142" s="8" t="inlineStr">
+        <is>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
+        </is>
+      </c>
+      <c r="S142" s="9" t="inlineStr"/>
+      <c r="T142" s="12" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U142" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V142" s="7" t="inlineStr"/>
+      <c r="W142" s="8" t="inlineStr">
+        <is>
           <t>4bd094575ff83a26d208b8ea7ce8140210cc94b9</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="B138" s="7" t="n"/>
-      <c r="C138" s="18" t="n">
-        <v>800</v>
-      </c>
-      <c r="D138" t="n">
-        <v>2</v>
-      </c>
-      <c r="E138" t="n">
-        <v>1</v>
-      </c>
-      <c r="F138" t="inlineStr">
-        <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="G138" s="7" t="inlineStr">
-        <is>
-          <t>Rehoboth Court, Coedpoeth, Wrexham, LL11</t>
-        </is>
-      </c>
-      <c r="H138" t="inlineStr">
-        <is>
-          <t>LL11</t>
-        </is>
-      </c>
-      <c r="N138" t="n">
-        <v>448</v>
-      </c>
-      <c r="O138" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q138" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="R138" t="inlineStr">
-        <is>
-          <t>OpenRent, London</t>
-        </is>
-      </c>
-      <c r="S138" s="7" t="inlineStr"/>
-      <c r="T138" s="14" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U138" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V138" s="7" t="inlineStr"/>
-      <c r="W138" t="inlineStr">
-        <is>
-          <t>c4ca3b08a858fe282766d1680bb80dd10c24ce32</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="B139" s="7" t="n"/>
-      <c r="C139" s="18" t="n">
-        <v>900</v>
-      </c>
-      <c r="D139" t="n">
-        <v>2</v>
-      </c>
-      <c r="E139" t="n">
-        <v>1</v>
-      </c>
-      <c r="F139" t="inlineStr">
-        <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="G139" s="7" t="inlineStr">
-        <is>
-          <t>Newmarket Road, Dyserth, LL18</t>
-        </is>
-      </c>
-      <c r="H139" t="inlineStr">
-        <is>
-          <t>LL18</t>
-        </is>
-      </c>
-      <c r="N139" t="n">
-        <v>328</v>
-      </c>
-      <c r="O139" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q139" t="inlineStr">
-        <is>
-          <t>2026-07-07</t>
-        </is>
-      </c>
-      <c r="R139" t="inlineStr">
-        <is>
-          <t>Fifty North West, Chester</t>
-        </is>
-      </c>
-      <c r="S139" s="7" t="inlineStr"/>
-      <c r="T139" s="14" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U139" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V139" s="7" t="inlineStr"/>
-      <c r="W139" t="inlineStr">
-        <is>
-          <t>19dde05bbe4ff1dc0306104719519db3f4baa597</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="B140" s="7" t="n"/>
-      <c r="C140" s="18" t="n">
-        <v>625</v>
-      </c>
-      <c r="D140" t="n">
-        <v>1</v>
-      </c>
-      <c r="E140" t="n">
-        <v>1</v>
-      </c>
-      <c r="F140" t="inlineStr">
-        <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="G140" s="7" t="inlineStr">
-        <is>
-          <t>Field View, Mancot, Deeside, CH5 2EY</t>
-        </is>
-      </c>
-      <c r="H140" t="inlineStr">
-        <is>
-          <t>CH5</t>
-        </is>
-      </c>
-      <c r="N140" t="n">
-        <v>824</v>
-      </c>
-      <c r="O140" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q140" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="R140" t="inlineStr">
-        <is>
-          <t>Habodel Property Services Ltd, Doncaster</t>
-        </is>
-      </c>
-      <c r="S140" s="7" t="inlineStr"/>
-      <c r="T140" s="14" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U140" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V140" s="7" t="inlineStr"/>
-      <c r="W140" t="inlineStr">
-        <is>
-          <t>c123bf34773b0afd208b42a23676d0de104b0aa4</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="B141" s="7" t="n"/>
-      <c r="C141" s="18" t="n">
-        <v>795</v>
-      </c>
-      <c r="D141" t="n">
-        <v>2</v>
-      </c>
-      <c r="E141" t="n">
-        <v>1</v>
-      </c>
-      <c r="F141" t="inlineStr">
-        <is>
-          <t>semi_detached</t>
-        </is>
-      </c>
-      <c r="G141" s="7" t="inlineStr">
-        <is>
-          <t>Cilcain, The Square, CH7</t>
-        </is>
-      </c>
-      <c r="H141" t="inlineStr">
-        <is>
-          <t>CH7</t>
-        </is>
-      </c>
-      <c r="N141" t="n">
-        <v>0</v>
-      </c>
-      <c r="O141" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q141" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="R141" t="inlineStr">
-        <is>
-          <t>Williams Estates, Rhuddlan</t>
-        </is>
-      </c>
-      <c r="S141" s="7" t="inlineStr"/>
-      <c r="T141" s="14" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U141" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V141" s="7" t="inlineStr"/>
-      <c r="W141" t="inlineStr">
-        <is>
-          <t>87b32c4489714d9b512693daad46cef94dcd76a1</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="B142" s="7" t="n"/>
-      <c r="C142" s="18" t="n">
-        <v>950</v>
-      </c>
-      <c r="D142" t="n">
-        <v>2</v>
-      </c>
-      <c r="E142" t="n">
-        <v>1</v>
-      </c>
-      <c r="F142" t="inlineStr">
-        <is>
-          <t>semi_detached</t>
-        </is>
-      </c>
-      <c r="G142" s="7" t="inlineStr">
-        <is>
-          <t>Cae Masarn, Pentre Halkyn, Holywell, Flintshire, CH8</t>
-        </is>
-      </c>
-      <c r="H142" t="inlineStr">
-        <is>
-          <t>CH8</t>
-        </is>
-      </c>
-      <c r="N142" t="n">
-        <v>56</v>
-      </c>
-      <c r="O142" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q142" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="R142" t="inlineStr">
-        <is>
-          <t>William Gleave, Deeside</t>
-        </is>
-      </c>
-      <c r="S142" s="7" t="inlineStr"/>
-      <c r="T142" s="14" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U142" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V142" s="7" t="inlineStr"/>
-      <c r="W142" t="inlineStr">
-        <is>
-          <t>21cedfdeff38e71da260f36d15fc7a90e3806efc</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="B143" s="7" t="n"/>
       <c r="C143" s="18" t="n">
-        <v>925</v>
+        <v>800</v>
       </c>
       <c r="D143" t="n">
         <v>2</v>
@@ -27412,36 +27485,33 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G143" s="7" t="inlineStr">
         <is>
-          <t>Hill Top Close, Ewloe, CH5</t>
+          <t>Rehoboth Court, Coedpoeth, Wrexham, LL11</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>CH5</t>
-        </is>
-      </c>
-      <c r="I143" t="n">
-        <v>721</v>
+          <t>LL11</t>
+        </is>
       </c>
       <c r="N143" t="n">
-        <v>472</v>
+        <v>448</v>
       </c>
       <c r="O143" t="n">
         <v>0</v>
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="R143" t="inlineStr">
         <is>
-          <t>Reades, Hawarden Lettings</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S143" s="7" t="inlineStr"/>
@@ -27458,17 +27528,17 @@
       <c r="V143" s="7" t="inlineStr"/>
       <c r="W143" t="inlineStr">
         <is>
-          <t>1b94ffba8e84bd8bda3a33b448f8f35102e29484</t>
+          <t>c4ca3b08a858fe282766d1680bb80dd10c24ce32</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="B144" s="7" t="n"/>
       <c r="C144" s="18" t="n">
-        <v>650</v>
+        <v>900</v>
       </c>
       <c r="D144" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E144" t="n">
         <v>1</v>
@@ -27480,31 +27550,28 @@
       </c>
       <c r="G144" s="7" t="inlineStr">
         <is>
-          <t>Chester Road East, Shotton, Deeside</t>
+          <t>Newmarket Road, Dyserth, LL18</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>CH5</t>
-        </is>
-      </c>
-      <c r="I144" t="n">
-        <v>474</v>
+          <t>LL18</t>
+        </is>
       </c>
       <c r="N144" t="n">
-        <v>2016</v>
+        <v>328</v>
       </c>
       <c r="O144" t="n">
         <v>0</v>
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="R144" t="inlineStr">
         <is>
-          <t>Thomas Property Group, Chester</t>
+          <t>Fifty North West, Chester</t>
         </is>
       </c>
       <c r="S144" s="7" t="inlineStr"/>
@@ -27521,50 +27588,50 @@
       <c r="V144" s="7" t="inlineStr"/>
       <c r="W144" t="inlineStr">
         <is>
-          <t>f80c03a584803371ab95595ae7a449a94715fbd1</t>
+          <t>19dde05bbe4ff1dc0306104719519db3f4baa597</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="B145" s="7" t="n"/>
       <c r="C145" s="18" t="n">
-        <v>750</v>
+        <v>625</v>
       </c>
       <c r="D145" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E145" t="n">
         <v>1</v>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G145" s="7" t="inlineStr">
         <is>
-          <t>Sycamore Terrace, Rhosrobin, Wrexham</t>
+          <t>Field View, Mancot, Deeside, CH5 2EY</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>LL11</t>
+          <t>CH5</t>
         </is>
       </c>
       <c r="N145" t="n">
-        <v>1300</v>
+        <v>824</v>
       </c>
       <c r="O145" t="n">
         <v>0</v>
       </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R145" t="inlineStr">
         <is>
-          <t>Bowen, Wrexham</t>
+          <t>Habodel Property Services Ltd, Doncaster</t>
         </is>
       </c>
       <c r="S145" s="7" t="inlineStr"/>
@@ -27581,14 +27648,14 @@
       <c r="V145" s="7" t="inlineStr"/>
       <c r="W145" t="inlineStr">
         <is>
-          <t>40274ada7dfa710e5054184216178477a704016c</t>
+          <t>c123bf34773b0afd208b42a23676d0de104b0aa4</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="B146" s="7" t="n"/>
       <c r="C146" s="18" t="n">
-        <v>900</v>
+        <v>795</v>
       </c>
       <c r="D146" t="n">
         <v>2</v>
@@ -27603,7 +27670,7 @@
       </c>
       <c r="G146" s="7" t="inlineStr">
         <is>
-          <t>Kiln Close, Buckley, Flintshire, CH7</t>
+          <t>Cilcain, The Square, CH7</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
@@ -27612,19 +27679,19 @@
         </is>
       </c>
       <c r="N146" t="n">
-        <v>936</v>
+        <v>0</v>
       </c>
       <c r="O146" t="n">
         <v>0</v>
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="R146" t="inlineStr">
         <is>
-          <t>William Gleave, Deeside</t>
+          <t>Williams Estates, Rhuddlan</t>
         </is>
       </c>
       <c r="S146" s="7" t="inlineStr"/>
@@ -27641,14 +27708,14 @@
       <c r="V146" s="7" t="inlineStr"/>
       <c r="W146" t="inlineStr">
         <is>
-          <t>780cbc2857d57b036f046702f312e0298790c096</t>
+          <t>87b32c4489714d9b512693daad46cef94dcd76a1</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="B147" s="7" t="n"/>
       <c r="C147" s="18" t="n">
-        <v>900</v>
+        <v>950</v>
       </c>
       <c r="D147" t="n">
         <v>2</v>
@@ -27658,33 +27725,33 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>semi_detached</t>
         </is>
       </c>
       <c r="G147" s="7" t="inlineStr">
         <is>
-          <t>9 Park Road, Ruthin</t>
+          <t>Cae Masarn, Pentre Halkyn, Holywell, Flintshire, CH8</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>LL15</t>
+          <t>CH8</t>
         </is>
       </c>
       <c r="N147" t="n">
-        <v>576</v>
+        <v>56</v>
       </c>
       <c r="O147" t="n">
         <v>0</v>
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="R147" t="inlineStr">
         <is>
-          <t>Cavendish Rentals Ltd, Ruthin</t>
+          <t>William Gleave, Deeside</t>
         </is>
       </c>
       <c r="S147" s="7" t="inlineStr"/>
@@ -27701,14 +27768,14 @@
       <c r="V147" s="7" t="inlineStr"/>
       <c r="W147" t="inlineStr">
         <is>
-          <t>c771916d30aebac19d1f346f767747d7b73a7d6c</t>
+          <t>21cedfdeff38e71da260f36d15fc7a90e3806efc</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="B148" s="7" t="n"/>
       <c r="C148" s="18" t="n">
-        <v>795</v>
+        <v>925</v>
       </c>
       <c r="D148" t="n">
         <v>2</v>
@@ -27723,31 +27790,31 @@
       </c>
       <c r="G148" s="7" t="inlineStr">
         <is>
-          <t>Gladstone Street, Mold</t>
+          <t>Hill Top Close, Ewloe, CH5</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>CH7</t>
+          <t>CH5</t>
         </is>
       </c>
       <c r="I148" t="n">
-        <v>905</v>
+        <v>721</v>
       </c>
       <c r="N148" t="n">
-        <v>1356</v>
+        <v>472</v>
       </c>
       <c r="O148" t="n">
         <v>0</v>
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R148" t="inlineStr">
         <is>
-          <t>Reid and Roberts, Mold</t>
+          <t>Reades, Hawarden Lettings</t>
         </is>
       </c>
       <c r="S148" s="7" t="inlineStr"/>
@@ -27764,48 +27831,48 @@
       <c r="V148" s="7" t="inlineStr"/>
       <c r="W148" t="inlineStr">
         <is>
-          <t>0fe090dd4efb58d6db540fc88a63048e9a1b679d</t>
+          <t>1b94ffba8e84bd8bda3a33b448f8f35102e29484</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="B149" s="7" t="n"/>
       <c r="C149" s="18" t="n">
-        <v>1200</v>
+        <v>650</v>
       </c>
       <c r="D149" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E149" t="n">
         <v>1</v>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>semi_detached</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G149" s="7" t="inlineStr">
         <is>
-          <t>Llwyn Dinas Fechan, St. Asaph</t>
+          <t>Chester Road East, Shotton, Deeside</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>LL17</t>
+          <t>CH5</t>
         </is>
       </c>
       <c r="I149" t="n">
-        <v>710</v>
+        <v>474</v>
       </c>
       <c r="N149" t="n">
-        <v>248</v>
+        <v>2016</v>
       </c>
       <c r="O149" t="n">
         <v>0</v>
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">
@@ -27827,14 +27894,14 @@
       <c r="V149" s="7" t="inlineStr"/>
       <c r="W149" t="inlineStr">
         <is>
-          <t>01f8dda2f09c16566df7d00ae192327104586ec6</t>
+          <t>f80c03a584803371ab95595ae7a449a94715fbd1</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="B150" s="7" t="n"/>
       <c r="C150" s="18" t="n">
-        <v>700</v>
+        <v>750</v>
       </c>
       <c r="D150" t="n">
         <v>2</v>
@@ -27844,36 +27911,33 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G150" s="7" t="inlineStr">
         <is>
-          <t>Central Drive, Shotton, Deeside</t>
+          <t>Sycamore Terrace, Rhosrobin, Wrexham</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>CH5</t>
-        </is>
-      </c>
-      <c r="I150" t="n">
-        <v>636</v>
+          <t>LL11</t>
+        </is>
       </c>
       <c r="N150" t="n">
-        <v>1924</v>
+        <v>1300</v>
       </c>
       <c r="O150" t="n">
         <v>0</v>
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R150" t="inlineStr">
         <is>
-          <t>Reid and Roberts, Mold</t>
+          <t>Bowen, Wrexham</t>
         </is>
       </c>
       <c r="S150" s="7" t="inlineStr"/>
@@ -27890,29 +27954,29 @@
       <c r="V150" s="7" t="inlineStr"/>
       <c r="W150" t="inlineStr">
         <is>
-          <t>a8679975fd318f064c6646b7ec603ef505c73b91</t>
+          <t>40274ada7dfa710e5054184216178477a704016c</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="B151" s="7" t="n"/>
       <c r="C151" s="18" t="n">
-        <v>850</v>
+        <v>900</v>
       </c>
       <c r="D151" t="n">
         <v>2</v>
       </c>
       <c r="E151" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>semi_detached</t>
         </is>
       </c>
       <c r="G151" s="7" t="inlineStr">
         <is>
-          <t>Llys Y Ddol, Mold</t>
+          <t>Kiln Close, Buckley, Flintshire, CH7</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
@@ -27921,19 +27985,19 @@
         </is>
       </c>
       <c r="N151" t="n">
-        <v>1368</v>
+        <v>936</v>
       </c>
       <c r="O151" t="n">
         <v>0</v>
       </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R151" t="inlineStr">
         <is>
-          <t>Cavendish Rentals Ltd, Mold</t>
+          <t>William Gleave, Deeside</t>
         </is>
       </c>
       <c r="S151" s="7" t="inlineStr"/>
@@ -27950,53 +28014,50 @@
       <c r="V151" s="7" t="inlineStr"/>
       <c r="W151" t="inlineStr">
         <is>
-          <t>454191bb7bc0e7fb7e64e3fd4f1802d398e2254c</t>
+          <t>780cbc2857d57b036f046702f312e0298790c096</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="B152" s="7" t="n"/>
       <c r="C152" s="18" t="n">
-        <v>1000</v>
+        <v>900</v>
       </c>
       <c r="D152" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E152" t="n">
         <v>1</v>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>semi_detached</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G152" s="7" t="inlineStr">
         <is>
-          <t>Mill View Road, Shotton, CH5</t>
+          <t>9 Park Road, Ruthin</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>CH5</t>
-        </is>
-      </c>
-      <c r="I152" t="n">
-        <v>1087</v>
+          <t>LL15</t>
+        </is>
       </c>
       <c r="N152" t="n">
-        <v>2236</v>
+        <v>576</v>
       </c>
       <c r="O152" t="n">
         <v>0</v>
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R152" t="inlineStr">
         <is>
-          <t>Pinewood Estate Agency, Deeside</t>
+          <t>Cavendish Rentals Ltd, Ruthin</t>
         </is>
       </c>
       <c r="S152" s="7" t="inlineStr"/>
@@ -28013,48 +28074,48 @@
       <c r="V152" s="7" t="inlineStr"/>
       <c r="W152" t="inlineStr">
         <is>
-          <t>709d3dbb0469602a30f2232c43318e1004ee28e3</t>
+          <t>c771916d30aebac19d1f346f767747d7b73a7d6c</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="B153" s="7" t="n"/>
       <c r="C153" s="18" t="n">
-        <v>1100</v>
+        <v>795</v>
       </c>
       <c r="D153" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E153" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>semi_detached</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G153" s="7" t="inlineStr">
         <is>
-          <t>Chestnut Way, Penyffordd, Chester</t>
+          <t>Gladstone Street, Mold</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>CH4</t>
+          <t>CH7</t>
         </is>
       </c>
       <c r="I153" t="n">
-        <v>765</v>
+        <v>905</v>
       </c>
       <c r="N153" t="n">
-        <v>144</v>
+        <v>1356</v>
       </c>
       <c r="O153" t="n">
         <v>0</v>
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R153" t="inlineStr">
@@ -28076,17 +28137,17 @@
       <c r="V153" s="7" t="inlineStr"/>
       <c r="W153" t="inlineStr">
         <is>
-          <t>0c6f7f5dcf9483acf81dd96394cb138955cd345f</t>
+          <t>0fe090dd4efb58d6db540fc88a63048e9a1b679d</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="B154" s="7" t="n"/>
       <c r="C154" s="18" t="n">
-        <v>975</v>
+        <v>1200</v>
       </c>
       <c r="D154" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E154" t="n">
         <v>1</v>
@@ -28098,28 +28159,31 @@
       </c>
       <c r="G154" s="7" t="inlineStr">
         <is>
-          <t>Maes Offa, Trelawynd, Rhyl, Flintshire, LL18</t>
+          <t>Llwyn Dinas Fechan, St. Asaph</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>LL18</t>
-        </is>
+          <t>LL17</t>
+        </is>
+      </c>
+      <c r="I154" t="n">
+        <v>710</v>
       </c>
       <c r="N154" t="n">
-        <v>32</v>
+        <v>248</v>
       </c>
       <c r="O154" t="n">
         <v>0</v>
       </c>
       <c r="Q154" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R154" t="inlineStr">
         <is>
-          <t>Monopoly, Denbigh</t>
+          <t>Thomas Property Group, Chester</t>
         </is>
       </c>
       <c r="S154" s="7" t="inlineStr"/>
@@ -28136,50 +28200,53 @@
       <c r="V154" s="7" t="inlineStr"/>
       <c r="W154" t="inlineStr">
         <is>
-          <t>7010522a251f536737688e6768df8c1ca7b26c26</t>
+          <t>01f8dda2f09c16566df7d00ae192327104586ec6</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="B155" s="7" t="n"/>
       <c r="C155" s="18" t="n">
-        <v>875</v>
+        <v>700</v>
       </c>
       <c r="D155" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E155" t="n">
         <v>1</v>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>semi_detached</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G155" s="7" t="inlineStr">
         <is>
-          <t>Glan Y Don, Greenfield, Holywell, CH8 7HG</t>
+          <t>Central Drive, Shotton, Deeside</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>CH8</t>
-        </is>
+          <t>CH5</t>
+        </is>
+      </c>
+      <c r="I155" t="n">
+        <v>636</v>
       </c>
       <c r="N155" t="n">
-        <v>540</v>
+        <v>1924</v>
       </c>
       <c r="O155" t="n">
         <v>0</v>
       </c>
       <c r="Q155" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="R155" t="inlineStr">
         <is>
-          <t>Visum, Nationwide</t>
+          <t>Reid and Roberts, Mold</t>
         </is>
       </c>
       <c r="S155" s="7" t="inlineStr"/>
@@ -28196,17 +28263,20 @@
       <c r="V155" s="7" t="inlineStr"/>
       <c r="W155" t="inlineStr">
         <is>
-          <t>2de321765047d8487aaad5d86e92b523486e594c</t>
+          <t>a8679975fd318f064c6646b7ec603ef505c73b91</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="B156" s="7" t="n"/>
       <c r="C156" s="18" t="n">
-        <v>725</v>
+        <v>850</v>
       </c>
       <c r="D156" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="E156" t="n">
+        <v>2</v>
       </c>
       <c r="F156" t="inlineStr">
         <is>
@@ -28215,28 +28285,28 @@
       </c>
       <c r="G156" s="7" t="inlineStr">
         <is>
-          <t>High Street, Connah's Quay, CH5</t>
+          <t>Llys Y Ddol, Mold</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>CH5</t>
+          <t>CH7</t>
         </is>
       </c>
       <c r="N156" t="n">
-        <v>1904</v>
+        <v>1368</v>
       </c>
       <c r="O156" t="n">
         <v>0</v>
       </c>
       <c r="Q156" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="R156" t="inlineStr">
         <is>
-          <t>Pinewood Estate Agency, Deeside</t>
+          <t>Cavendish Rentals Ltd, Mold</t>
         </is>
       </c>
       <c r="S156" s="7" t="inlineStr"/>
@@ -28253,50 +28323,53 @@
       <c r="V156" s="7" t="inlineStr"/>
       <c r="W156" t="inlineStr">
         <is>
-          <t>db6095b2965d70713395b1458e1bc20535687531</t>
+          <t>454191bb7bc0e7fb7e64e3fd4f1802d398e2254c</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="B157" s="7" t="n"/>
       <c r="C157" s="18" t="n">
-        <v>625</v>
+        <v>1000</v>
       </c>
       <c r="D157" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E157" t="n">
         <v>1</v>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>semi_detached</t>
         </is>
       </c>
       <c r="G157" s="7" t="inlineStr">
         <is>
-          <t>Well Street, Holywell</t>
+          <t>Mill View Road, Shotton, CH5</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>CH8</t>
-        </is>
+          <t>CH5</t>
+        </is>
+      </c>
+      <c r="I157" t="n">
+        <v>1087</v>
       </c>
       <c r="N157" t="n">
-        <v>904</v>
+        <v>2236</v>
       </c>
       <c r="O157" t="n">
         <v>0</v>
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="R157" t="inlineStr">
         <is>
-          <t>Cavendish Rentals Ltd, Mold</t>
+          <t>Pinewood Estate Agency, Deeside</t>
         </is>
       </c>
       <c r="S157" s="7" t="inlineStr"/>
@@ -28313,50 +28386,53 @@
       <c r="V157" s="7" t="inlineStr"/>
       <c r="W157" t="inlineStr">
         <is>
-          <t>2723b2ee048a058cfba581ae81cc808012ed35c5</t>
+          <t>709d3dbb0469602a30f2232c43318e1004ee28e3</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="B158" s="7" t="n"/>
       <c r="C158" s="18" t="n">
-        <v>900</v>
+        <v>1100</v>
       </c>
       <c r="D158" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E158" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>semi_detached</t>
         </is>
       </c>
       <c r="G158" s="7" t="inlineStr">
         <is>
-          <t>Bryntirion Road, Bagillt, Flintshire, CH6</t>
+          <t>Chestnut Way, Penyffordd, Chester</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>CH6</t>
-        </is>
+          <t>CH4</t>
+        </is>
+      </c>
+      <c r="I158" t="n">
+        <v>765</v>
       </c>
       <c r="N158" t="n">
-        <v>200</v>
+        <v>144</v>
       </c>
       <c r="O158" t="n">
         <v>0</v>
       </c>
       <c r="Q158" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="R158" t="inlineStr">
         <is>
-          <t>William Gleave, Deeside</t>
+          <t>Reid and Roberts, Mold</t>
         </is>
       </c>
       <c r="S158" s="7" t="inlineStr"/>
@@ -28373,20 +28449,20 @@
       <c r="V158" s="7" t="inlineStr"/>
       <c r="W158" t="inlineStr">
         <is>
-          <t>0c1595e8a037ae10970a3d68c03447fcb7c78d28</t>
+          <t>0c6f7f5dcf9483acf81dd96394cb138955cd345f</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="B159" s="7" t="n"/>
       <c r="C159" s="18" t="n">
-        <v>950</v>
+        <v>975</v>
       </c>
       <c r="D159" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E159" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F159" t="inlineStr">
         <is>
@@ -28395,31 +28471,28 @@
       </c>
       <c r="G159" s="7" t="inlineStr">
         <is>
-          <t>Rue St. Gregoire, Holywell, CH8</t>
+          <t>Maes Offa, Trelawynd, Rhyl, Flintshire, LL18</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>CH8</t>
-        </is>
-      </c>
-      <c r="I159" t="n">
-        <v>657</v>
+          <t>LL18</t>
+        </is>
       </c>
       <c r="N159" t="n">
-        <v>876</v>
+        <v>32</v>
       </c>
       <c r="O159" t="n">
         <v>0</v>
       </c>
       <c r="Q159" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="R159" t="inlineStr">
         <is>
-          <t>Currans, North Wales</t>
+          <t>Monopoly, Denbigh</t>
         </is>
       </c>
       <c r="S159" s="7" t="inlineStr"/>
@@ -28436,50 +28509,50 @@
       <c r="V159" s="7" t="inlineStr"/>
       <c r="W159" t="inlineStr">
         <is>
-          <t>dc3b6e39f27fc3549e5a88505b34a5efb8d772c4</t>
+          <t>7010522a251f536737688e6768df8c1ca7b26c26</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="B160" s="7" t="n"/>
       <c r="C160" s="18" t="n">
-        <v>750</v>
+        <v>875</v>
       </c>
       <c r="D160" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E160" t="n">
         <v>1</v>
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>semi_detached</t>
         </is>
       </c>
       <c r="G160" s="7" t="inlineStr">
         <is>
-          <t>29 Tai Maes, Mold</t>
+          <t>Glan Y Don, Greenfield, Holywell, CH8 7HG</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>CH7</t>
+          <t>CH8</t>
         </is>
       </c>
       <c r="N160" t="n">
-        <v>1356</v>
+        <v>540</v>
       </c>
       <c r="O160" t="n">
         <v>0</v>
       </c>
       <c r="Q160" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="R160" t="inlineStr">
         <is>
-          <t>Cavendish Rentals Ltd, Mold</t>
+          <t>Visum, Nationwide</t>
         </is>
       </c>
       <c r="S160" s="7" t="inlineStr"/>
@@ -28496,21 +28569,18 @@
       <c r="V160" s="7" t="inlineStr"/>
       <c r="W160" t="inlineStr">
         <is>
-          <t>e07eb711fdcf6d56ea28189fffc8e0176a5a3a88</t>
+          <t>2de321765047d8487aaad5d86e92b523486e594c</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="B161" s="7" t="n"/>
       <c r="C161" s="18" t="n">
-        <v>600</v>
+        <v>725</v>
       </c>
       <c r="D161" t="n">
         <v>1</v>
       </c>
-      <c r="E161" t="n">
-        <v>1</v>
-      </c>
       <c r="F161" t="inlineStr">
         <is>
           <t>flat</t>
@@ -28518,28 +28588,28 @@
       </c>
       <c r="G161" s="7" t="inlineStr">
         <is>
-          <t>St Marys Mews, Mold</t>
+          <t>High Street, Connah's Quay, CH5</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>CH7</t>
+          <t>CH5</t>
         </is>
       </c>
       <c r="N161" t="n">
-        <v>1372</v>
+        <v>1904</v>
       </c>
       <c r="O161" t="n">
         <v>0</v>
       </c>
       <c r="Q161" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="R161" t="inlineStr">
         <is>
-          <t>Cavendish Rentals Ltd, Mold</t>
+          <t>Pinewood Estate Agency, Deeside</t>
         </is>
       </c>
       <c r="S161" s="7" t="inlineStr"/>
@@ -28556,50 +28626,50 @@
       <c r="V161" s="7" t="inlineStr"/>
       <c r="W161" t="inlineStr">
         <is>
-          <t>af36d8744de8391ae981eb3d46fe462a829b50fc</t>
+          <t>db6095b2965d70713395b1458e1bc20535687531</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="B162" s="7" t="n"/>
       <c r="C162" s="18" t="n">
-        <v>875</v>
+        <v>625</v>
       </c>
       <c r="D162" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E162" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G162" s="7" t="inlineStr">
         <is>
-          <t>Castle Street, Caergwrle</t>
+          <t>Well Street, Holywell</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>LL12</t>
+          <t>CH8</t>
         </is>
       </c>
       <c r="N162" t="n">
-        <v>264</v>
+        <v>904</v>
       </c>
       <c r="O162" t="n">
         <v>0</v>
       </c>
       <c r="Q162" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="R162" t="inlineStr">
         <is>
-          <t>Town &amp; Country Estate Agents, Wrexham</t>
+          <t>Cavendish Rentals Ltd, Mold</t>
         </is>
       </c>
       <c r="S162" s="7" t="inlineStr"/>
@@ -28616,14 +28686,14 @@
       <c r="V162" s="7" t="inlineStr"/>
       <c r="W162" t="inlineStr">
         <is>
-          <t>64420bc3a588da08d4b7e360992c14bddef406b0</t>
+          <t>2723b2ee048a058cfba581ae81cc808012ed35c5</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="B163" s="7" t="n"/>
       <c r="C163" s="18" t="n">
-        <v>800</v>
+        <v>900</v>
       </c>
       <c r="D163" t="n">
         <v>2</v>
@@ -28633,33 +28703,33 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G163" s="7" t="inlineStr">
         <is>
-          <t>Fagl Lane, Hope, LL12</t>
+          <t>Bryntirion Road, Bagillt, Flintshire, CH6</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>LL12</t>
+          <t>CH6</t>
         </is>
       </c>
       <c r="N163" t="n">
-        <v>244</v>
+        <v>200</v>
       </c>
       <c r="O163" t="n">
         <v>0</v>
       </c>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="R163" t="inlineStr">
         <is>
-          <t>Belvoir, Wrexham</t>
+          <t>William Gleave, Deeside</t>
         </is>
       </c>
       <c r="S163" s="7" t="inlineStr"/>
@@ -28676,50 +28746,53 @@
       <c r="V163" s="7" t="inlineStr"/>
       <c r="W163" t="inlineStr">
         <is>
-          <t>2e367fcb5325f10c32c7f8598ffffb977d48bccf</t>
+          <t>0c1595e8a037ae10970a3d68c03447fcb7c78d28</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="B164" s="7" t="n"/>
       <c r="C164" s="18" t="n">
-        <v>595</v>
+        <v>950</v>
       </c>
       <c r="D164" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E164" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>semi_detached</t>
         </is>
       </c>
       <c r="G164" s="7" t="inlineStr">
         <is>
-          <t>Ryeland Street, Deeside</t>
+          <t>Rue St. Gregoire, Holywell, CH8</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>CH5</t>
-        </is>
+          <t>CH8</t>
+        </is>
+      </c>
+      <c r="I164" t="n">
+        <v>657</v>
       </c>
       <c r="N164" t="n">
-        <v>2152</v>
+        <v>876</v>
       </c>
       <c r="O164" t="n">
         <v>0</v>
       </c>
       <c r="Q164" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="R164" t="inlineStr">
         <is>
-          <t>Bowen, Wrexham</t>
+          <t>Currans, North Wales</t>
         </is>
       </c>
       <c r="S164" s="7" t="inlineStr"/>
@@ -28736,7 +28809,7 @@
       <c r="V164" s="7" t="inlineStr"/>
       <c r="W164" t="inlineStr">
         <is>
-          <t>3502024b9ccf3c5846dbd8b2f4e5148495660759</t>
+          <t>dc3b6e39f27fc3549e5a88505b34a5efb8d772c4</t>
         </is>
       </c>
     </row>
@@ -28758,28 +28831,28 @@
       </c>
       <c r="G165" s="7" t="inlineStr">
         <is>
-          <t>High Street, Dyserth, LL18</t>
+          <t>29 Tai Maes, Mold</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>LL18</t>
+          <t>CH7</t>
         </is>
       </c>
       <c r="N165" t="n">
-        <v>232</v>
+        <v>1356</v>
       </c>
       <c r="O165" t="n">
         <v>0</v>
       </c>
       <c r="Q165" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="R165" t="inlineStr">
         <is>
-          <t>Fifty North West, Chester</t>
+          <t>Cavendish Rentals Ltd, Mold</t>
         </is>
       </c>
       <c r="S165" s="7" t="inlineStr"/>
@@ -28796,17 +28869,17 @@
       <c r="V165" s="7" t="inlineStr"/>
       <c r="W165" t="inlineStr">
         <is>
-          <t>c2d205c9da5502fe82c6529faa7073858d43318b</t>
+          <t>e07eb711fdcf6d56ea28189fffc8e0176a5a3a88</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="B166" s="7" t="n"/>
       <c r="C166" s="18" t="n">
-        <v>900</v>
+        <v>600</v>
       </c>
       <c r="D166" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E166" t="n">
         <v>1</v>
@@ -28818,28 +28891,28 @@
       </c>
       <c r="G166" s="7" t="inlineStr">
         <is>
-          <t>Newmarket Road, Dyserth, LL18</t>
+          <t>St Marys Mews, Mold</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>LL18</t>
+          <t>CH7</t>
         </is>
       </c>
       <c r="N166" t="n">
-        <v>328</v>
+        <v>1372</v>
       </c>
       <c r="O166" t="n">
         <v>0</v>
       </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="R166" t="inlineStr">
         <is>
-          <t>Fifty North West, Chester</t>
+          <t>Cavendish Rentals Ltd, Mold</t>
         </is>
       </c>
       <c r="S166" s="7" t="inlineStr"/>
@@ -28856,20 +28929,20 @@
       <c r="V166" s="7" t="inlineStr"/>
       <c r="W166" t="inlineStr">
         <is>
-          <t>8e3b047de4dea7640f383c9c16a3741e55ca202e</t>
+          <t>af36d8744de8391ae981eb3d46fe462a829b50fc</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="B167" s="7" t="n"/>
       <c r="C167" s="18" t="n">
-        <v>795</v>
+        <v>875</v>
       </c>
       <c r="D167" t="n">
         <v>2</v>
       </c>
       <c r="E167" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F167" t="inlineStr">
         <is>
@@ -28878,28 +28951,28 @@
       </c>
       <c r="G167" s="7" t="inlineStr">
         <is>
-          <t>Tower Terrace, Denbigh, Denbighshire, LL16</t>
+          <t>Castle Street, Caergwrle</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>LL16</t>
+          <t>LL12</t>
         </is>
       </c>
       <c r="N167" t="n">
-        <v>940</v>
+        <v>264</v>
       </c>
       <c r="O167" t="n">
         <v>0</v>
       </c>
       <c r="Q167" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="R167" t="inlineStr">
         <is>
-          <t>Monopoly, Denbigh</t>
+          <t>Town &amp; Country Estate Agents, Wrexham</t>
         </is>
       </c>
       <c r="S167" s="7" t="inlineStr"/>
@@ -28916,29 +28989,29 @@
       <c r="V167" s="7" t="inlineStr"/>
       <c r="W167" t="inlineStr">
         <is>
-          <t>a759cdaa8d9f724f2ecce2ccbf99e547c19fde5a</t>
+          <t>64420bc3a588da08d4b7e360992c14bddef406b0</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="B168" s="7" t="n"/>
       <c r="C168" s="18" t="n">
-        <v>975</v>
+        <v>800</v>
       </c>
       <c r="D168" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E168" t="n">
         <v>1</v>
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G168" s="7" t="inlineStr">
         <is>
-          <t>Derby Road, Caergwrle, Wrexham</t>
+          <t>Fagl Lane, Hope, LL12</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
@@ -28947,19 +29020,19 @@
         </is>
       </c>
       <c r="N168" t="n">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="O168" t="n">
         <v>0</v>
       </c>
       <c r="Q168" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="R168" t="inlineStr">
         <is>
-          <t>Bowen, Wrexham</t>
+          <t>Belvoir, Wrexham</t>
         </is>
       </c>
       <c r="S168" s="7" t="inlineStr"/>
@@ -28976,20 +29049,20 @@
       <c r="V168" s="7" t="inlineStr"/>
       <c r="W168" t="inlineStr">
         <is>
-          <t>9c715b658948566fb2a4a4b90c3c6b2f1f91a752</t>
+          <t>2e367fcb5325f10c32c7f8598ffffb977d48bccf</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="B169" s="7" t="n"/>
       <c r="C169" s="18" t="n">
-        <v>985</v>
+        <v>595</v>
       </c>
       <c r="D169" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E169" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F169" t="inlineStr">
         <is>
@@ -28998,28 +29071,28 @@
       </c>
       <c r="G169" s="7" t="inlineStr">
         <is>
-          <t>Livingstone Place, St. Asaph, LL17</t>
+          <t>Ryeland Street, Deeside</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>LL17</t>
+          <t>CH5</t>
         </is>
       </c>
       <c r="N169" t="n">
-        <v>268</v>
+        <v>2152</v>
       </c>
       <c r="O169" t="n">
         <v>0</v>
       </c>
       <c r="Q169" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="R169" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Bowen, Wrexham</t>
         </is>
       </c>
       <c r="S169" s="7" t="inlineStr"/>
@@ -29036,12 +29109,312 @@
       <c r="V169" s="7" t="inlineStr"/>
       <c r="W169" t="inlineStr">
         <is>
+          <t>3502024b9ccf3c5846dbd8b2f4e5148495660759</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="B170" s="7" t="n"/>
+      <c r="C170" s="18" t="n">
+        <v>750</v>
+      </c>
+      <c r="D170" t="n">
+        <v>2</v>
+      </c>
+      <c r="E170" t="n">
+        <v>1</v>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G170" s="7" t="inlineStr">
+        <is>
+          <t>High Street, Dyserth, LL18</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>LL18</t>
+        </is>
+      </c>
+      <c r="N170" t="n">
+        <v>232</v>
+      </c>
+      <c r="O170" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q170" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="R170" t="inlineStr">
+        <is>
+          <t>Fifty North West, Chester</t>
+        </is>
+      </c>
+      <c r="S170" s="7" t="inlineStr"/>
+      <c r="T170" s="14" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U170" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V170" s="7" t="inlineStr"/>
+      <c r="W170" t="inlineStr">
+        <is>
+          <t>c2d205c9da5502fe82c6529faa7073858d43318b</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="B171" s="7" t="n"/>
+      <c r="C171" s="18" t="n">
+        <v>900</v>
+      </c>
+      <c r="D171" t="n">
+        <v>2</v>
+      </c>
+      <c r="E171" t="n">
+        <v>1</v>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G171" s="7" t="inlineStr">
+        <is>
+          <t>Newmarket Road, Dyserth, LL18</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>LL18</t>
+        </is>
+      </c>
+      <c r="N171" t="n">
+        <v>328</v>
+      </c>
+      <c r="O171" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q171" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="R171" t="inlineStr">
+        <is>
+          <t>Fifty North West, Chester</t>
+        </is>
+      </c>
+      <c r="S171" s="7" t="inlineStr"/>
+      <c r="T171" s="14" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U171" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V171" s="7" t="inlineStr"/>
+      <c r="W171" t="inlineStr">
+        <is>
+          <t>8e3b047de4dea7640f383c9c16a3741e55ca202e</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="B172" s="7" t="n"/>
+      <c r="C172" s="18" t="n">
+        <v>795</v>
+      </c>
+      <c r="D172" t="n">
+        <v>2</v>
+      </c>
+      <c r="E172" t="n">
+        <v>1</v>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>terraced</t>
+        </is>
+      </c>
+      <c r="G172" s="7" t="inlineStr">
+        <is>
+          <t>Tower Terrace, Denbigh, Denbighshire, LL16</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>LL16</t>
+        </is>
+      </c>
+      <c r="N172" t="n">
+        <v>940</v>
+      </c>
+      <c r="O172" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q172" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="R172" t="inlineStr">
+        <is>
+          <t>Monopoly, Denbigh</t>
+        </is>
+      </c>
+      <c r="S172" s="7" t="inlineStr"/>
+      <c r="T172" s="14" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U172" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V172" s="7" t="inlineStr"/>
+      <c r="W172" t="inlineStr">
+        <is>
+          <t>a759cdaa8d9f724f2ecce2ccbf99e547c19fde5a</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="B173" s="7" t="n"/>
+      <c r="C173" s="18" t="n">
+        <v>975</v>
+      </c>
+      <c r="D173" t="n">
+        <v>3</v>
+      </c>
+      <c r="E173" t="n">
+        <v>1</v>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>terraced</t>
+        </is>
+      </c>
+      <c r="G173" s="7" t="inlineStr">
+        <is>
+          <t>Derby Road, Caergwrle, Wrexham</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>LL12</t>
+        </is>
+      </c>
+      <c r="N173" t="n">
+        <v>252</v>
+      </c>
+      <c r="O173" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q173" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="R173" t="inlineStr">
+        <is>
+          <t>Bowen, Wrexham</t>
+        </is>
+      </c>
+      <c r="S173" s="7" t="inlineStr"/>
+      <c r="T173" s="14" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U173" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V173" s="7" t="inlineStr"/>
+      <c r="W173" t="inlineStr">
+        <is>
+          <t>9c715b658948566fb2a4a4b90c3c6b2f1f91a752</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="B174" s="7" t="n"/>
+      <c r="C174" s="18" t="n">
+        <v>985</v>
+      </c>
+      <c r="D174" t="n">
+        <v>2</v>
+      </c>
+      <c r="E174" t="n">
+        <v>2</v>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G174" s="7" t="inlineStr">
+        <is>
+          <t>Livingstone Place, St. Asaph, LL17</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>LL17</t>
+        </is>
+      </c>
+      <c r="N174" t="n">
+        <v>268</v>
+      </c>
+      <c r="O174" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q174" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="R174" t="inlineStr">
+        <is>
+          <t>OpenRent, London</t>
+        </is>
+      </c>
+      <c r="S174" s="7" t="inlineStr"/>
+      <c r="T174" s="14" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U174" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V174" s="7" t="inlineStr"/>
+      <c r="W174" t="inlineStr">
+        <is>
           <t>b0ba112a09e1577fca8332db332a7e1693926a4e</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W169"/>
+  <autoFilter ref="A1:W174"/>
   <dataValidations count="1">
     <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199 U200 U201 U202 U203 U204 U205 U206 U207 U208 U209 U210 U211 U212" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
@@ -29216,6 +29589,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T167" r:id="rId166"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T168" r:id="rId167"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T169" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T170" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T171" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T172" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T173" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T174" r:id="rId173"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
House search data from run 10
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'For Sale'!$A$1:$W$212</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$175</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$179</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -16832,7 +16832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W175"/>
+  <dimension ref="A1:W179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -17326,7 +17326,7 @@
       <c r="L6" s="8" t="n"/>
       <c r="M6" s="8" t="n"/>
       <c r="N6" s="8" t="n">
-        <v>21660</v>
+        <v>21616</v>
       </c>
       <c r="O6" s="8" t="n">
         <v>0</v>
@@ -25272,7 +25272,7 @@
         </is>
       </c>
       <c r="C113" s="17" t="n">
-        <v>1200</v>
+        <v>1630</v>
       </c>
       <c r="D113" s="8" t="n">
         <v>1</v>
@@ -25287,21 +25287,23 @@
       </c>
       <c r="G113" s="9" t="inlineStr">
         <is>
-          <t>Alma Road, Flat 6, Clifton, Bristol, BS8</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H113" s="8" t="inlineStr">
         <is>
-          <t>BS8</t>
-        </is>
-      </c>
-      <c r="I113" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I113" s="8" t="n">
+        <v>560</v>
+      </c>
       <c r="J113" s="8" t="n"/>
       <c r="K113" s="8" t="n"/>
       <c r="L113" s="8" t="n"/>
       <c r="M113" s="8" t="n"/>
       <c r="N113" s="8" t="n">
-        <v>8636</v>
+        <v>20820</v>
       </c>
       <c r="O113" s="8" t="n">
         <v>0</v>
@@ -25309,12 +25311,12 @@
       <c r="P113" s="8" t="n"/>
       <c r="Q113" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="R113" s="8" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S113" s="9" t="inlineStr"/>
@@ -25331,7 +25333,7 @@
       <c r="V113" s="7" t="inlineStr"/>
       <c r="W113" s="8" t="inlineStr">
         <is>
-          <t>de364d91e6b651d1cfef840c60f9266ca9665382</t>
+          <t>0afbcf3acfc8707595a116822a42ea844dc8ad7e</t>
         </is>
       </c>
     </row>
@@ -25345,13 +25347,13 @@
         </is>
       </c>
       <c r="C114" s="17" t="n">
-        <v>1100</v>
+        <v>2115</v>
       </c>
       <c r="D114" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E114" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F114" s="8" t="inlineStr">
         <is>
@@ -25360,21 +25362,23 @@
       </c>
       <c r="G114" s="9" t="inlineStr">
         <is>
-          <t>St Peter's Rise, Headley Park, Bristol, BS13</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H114" s="8" t="inlineStr">
         <is>
-          <t>BS13</t>
-        </is>
-      </c>
-      <c r="I114" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I114" s="8" t="n">
+        <v>823</v>
+      </c>
       <c r="J114" s="8" t="n"/>
       <c r="K114" s="8" t="n"/>
       <c r="L114" s="8" t="n"/>
       <c r="M114" s="8" t="n"/>
       <c r="N114" s="8" t="n">
-        <v>4936</v>
+        <v>20820</v>
       </c>
       <c r="O114" s="8" t="n">
         <v>0</v>
@@ -25382,12 +25386,12 @@
       <c r="P114" s="8" t="n"/>
       <c r="Q114" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="R114" s="8" t="inlineStr">
         <is>
-          <t>CJ Hole, Southville</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S114" s="9" t="inlineStr"/>
@@ -25404,7 +25408,7 @@
       <c r="V114" s="7" t="inlineStr"/>
       <c r="W114" s="8" t="inlineStr">
         <is>
-          <t>d84ed54d6320edc245d61712b43d63702c789d06</t>
+          <t>0b78c6e29d96ae73c643d0d50d50949797b02893</t>
         </is>
       </c>
     </row>
@@ -25418,7 +25422,7 @@
         </is>
       </c>
       <c r="C115" s="17" t="n">
-        <v>1100</v>
+        <v>1660</v>
       </c>
       <c r="D115" s="8" t="n">
         <v>1</v>
@@ -25433,21 +25437,23 @@
       </c>
       <c r="G115" s="9" t="inlineStr">
         <is>
-          <t>Flat B, City Road, Bristol</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H115" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I115" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I115" s="8" t="n">
+        <v>486</v>
+      </c>
       <c r="J115" s="8" t="n"/>
       <c r="K115" s="8" t="n"/>
       <c r="L115" s="8" t="n"/>
       <c r="M115" s="8" t="n"/>
       <c r="N115" s="8" t="n">
-        <v>20108</v>
+        <v>21504</v>
       </c>
       <c r="O115" s="8" t="n">
         <v>0</v>
@@ -25455,12 +25461,12 @@
       <c r="P115" s="8" t="n"/>
       <c r="Q115" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="R115" s="8" t="inlineStr">
         <is>
-          <t>Holbrook Moran, Redfield</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S115" s="9" t="inlineStr"/>
@@ -25477,7 +25483,7 @@
       <c r="V115" s="7" t="inlineStr"/>
       <c r="W115" s="8" t="inlineStr">
         <is>
-          <t>144b3ddc5d76a111148e107efa0e01de8a7835b3</t>
+          <t>c798c669d03fa2e42fd418ff0916de022d3380ad</t>
         </is>
       </c>
     </row>
@@ -25491,13 +25497,13 @@
         </is>
       </c>
       <c r="C116" s="17" t="n">
-        <v>1200</v>
+        <v>1915</v>
       </c>
       <c r="D116" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E116" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F116" s="8" t="inlineStr">
         <is>
@@ -25506,7 +25512,7 @@
       </c>
       <c r="G116" s="9" t="inlineStr">
         <is>
-          <t>City Centre, Unity Street, BS1 5HH</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H116" s="8" t="inlineStr">
@@ -25515,14 +25521,14 @@
         </is>
       </c>
       <c r="I116" s="8" t="n">
-        <v>452</v>
+        <v>746</v>
       </c>
       <c r="J116" s="8" t="n"/>
       <c r="K116" s="8" t="n"/>
       <c r="L116" s="8" t="n"/>
       <c r="M116" s="8" t="n"/>
       <c r="N116" s="8" t="n">
-        <v>20772</v>
+        <v>21680</v>
       </c>
       <c r="O116" s="8" t="n">
         <v>0</v>
@@ -25530,12 +25536,12 @@
       <c r="P116" s="8" t="n"/>
       <c r="Q116" s="8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="R116" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Clifton</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S116" s="9" t="inlineStr"/>
@@ -25552,7 +25558,7 @@
       <c r="V116" s="7" t="inlineStr"/>
       <c r="W116" s="8" t="inlineStr">
         <is>
-          <t>bc1549c52c7b716065fff0163d60cc723a0ab301</t>
+          <t>36797023cff0095f1bf764fa2f176d5595124854</t>
         </is>
       </c>
     </row>
@@ -25569,7 +25575,7 @@
         <v>1200</v>
       </c>
       <c r="D117" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E117" s="8" t="n">
         <v>1</v>
@@ -25581,12 +25587,12 @@
       </c>
       <c r="G117" s="9" t="inlineStr">
         <is>
-          <t>Bull Lane, Crews Hole, Bristol, BS5</t>
+          <t>Alma Road, Flat 6, Clifton, Bristol, BS8</t>
         </is>
       </c>
       <c r="H117" s="8" t="inlineStr">
         <is>
-          <t>BS5</t>
+          <t>BS8</t>
         </is>
       </c>
       <c r="I117" s="8" t="n"/>
@@ -25595,7 +25601,7 @@
       <c r="L117" s="8" t="n"/>
       <c r="M117" s="8" t="n"/>
       <c r="N117" s="8" t="n">
-        <v>4160</v>
+        <v>8636</v>
       </c>
       <c r="O117" s="8" t="n">
         <v>0</v>
@@ -25603,12 +25609,12 @@
       <c r="P117" s="8" t="n"/>
       <c r="Q117" s="8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="R117" s="8" t="inlineStr">
         <is>
-          <t>Morgan &amp; Sons, Bristol</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S117" s="9" t="inlineStr"/>
@@ -25625,7 +25631,7 @@
       <c r="V117" s="7" t="inlineStr"/>
       <c r="W117" s="8" t="inlineStr">
         <is>
-          <t>297b43bd732a4c243907fc8bc1c888a888e057d1</t>
+          <t>de364d91e6b651d1cfef840c60f9266ca9665382</t>
         </is>
       </c>
     </row>
@@ -25639,7 +25645,7 @@
         </is>
       </c>
       <c r="C118" s="17" t="n">
-        <v>965</v>
+        <v>1100</v>
       </c>
       <c r="D118" s="8" t="n">
         <v>1</v>
@@ -25654,12 +25660,12 @@
       </c>
       <c r="G118" s="9" t="inlineStr">
         <is>
-          <t>Boulevard View, Whitchurch Lane</t>
+          <t>St Peter's Rise, Headley Park, Bristol, BS13</t>
         </is>
       </c>
       <c r="H118" s="8" t="inlineStr">
         <is>
-          <t>BS14</t>
+          <t>BS13</t>
         </is>
       </c>
       <c r="I118" s="8" t="n"/>
@@ -25668,7 +25674,7 @@
       <c r="L118" s="8" t="n"/>
       <c r="M118" s="8" t="n"/>
       <c r="N118" s="8" t="n">
-        <v>5764</v>
+        <v>4936</v>
       </c>
       <c r="O118" s="8" t="n">
         <v>0</v>
@@ -25676,12 +25682,12 @@
       <c r="P118" s="8" t="n"/>
       <c r="Q118" s="8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="R118" s="8" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>CJ Hole, Southville</t>
         </is>
       </c>
       <c r="S118" s="9" t="inlineStr"/>
@@ -25698,7 +25704,7 @@
       <c r="V118" s="7" t="inlineStr"/>
       <c r="W118" s="8" t="inlineStr">
         <is>
-          <t>ecef3f674f68cbf8b8e0c35c0fe5f8b0099a6a5b</t>
+          <t>d84ed54d6320edc245d61712b43d63702c789d06</t>
         </is>
       </c>
     </row>
@@ -25712,7 +25718,7 @@
         </is>
       </c>
       <c r="C119" s="17" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="D119" s="8" t="n">
         <v>1</v>
@@ -25727,7 +25733,7 @@
       </c>
       <c r="G119" s="9" t="inlineStr">
         <is>
-          <t>Braggs Lane, Bristol</t>
+          <t>Flat B, City Road, Bristol</t>
         </is>
       </c>
       <c r="H119" s="8" t="inlineStr">
@@ -25735,15 +25741,13 @@
           <t>BS2</t>
         </is>
       </c>
-      <c r="I119" s="8" t="n">
-        <v>409</v>
-      </c>
+      <c r="I119" s="8" t="n"/>
       <c r="J119" s="8" t="n"/>
       <c r="K119" s="8" t="n"/>
       <c r="L119" s="8" t="n"/>
       <c r="M119" s="8" t="n"/>
       <c r="N119" s="8" t="n">
-        <v>20360</v>
+        <v>20108</v>
       </c>
       <c r="O119" s="8" t="n">
         <v>0</v>
@@ -25751,12 +25755,12 @@
       <c r="P119" s="8" t="n"/>
       <c r="Q119" s="8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="R119" s="8" t="inlineStr">
         <is>
-          <t>House + Co Property, Bristol</t>
+          <t>Holbrook Moran, Redfield</t>
         </is>
       </c>
       <c r="S119" s="9" t="inlineStr"/>
@@ -25773,7 +25777,7 @@
       <c r="V119" s="7" t="inlineStr"/>
       <c r="W119" s="8" t="inlineStr">
         <is>
-          <t>b7418b86260a082ce0b767afb48615e82b4efe93</t>
+          <t>144b3ddc5d76a111148e107efa0e01de8a7835b3</t>
         </is>
       </c>
     </row>
@@ -25802,21 +25806,23 @@
       </c>
       <c r="G120" s="9" t="inlineStr">
         <is>
-          <t>Montague Court, Bristol</t>
+          <t>City Centre, Unity Street, BS1 5HH</t>
         </is>
       </c>
       <c r="H120" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I120" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I120" s="8" t="n">
+        <v>452</v>
+      </c>
       <c r="J120" s="8" t="n"/>
       <c r="K120" s="8" t="n"/>
       <c r="L120" s="8" t="n"/>
       <c r="M120" s="8" t="n"/>
       <c r="N120" s="8" t="n">
-        <v>21632</v>
+        <v>20772</v>
       </c>
       <c r="O120" s="8" t="n">
         <v>0</v>
@@ -25829,7 +25835,7 @@
       </c>
       <c r="R120" s="8" t="inlineStr">
         <is>
-          <t>Connells Lettings, Southville</t>
+          <t>The Bristol Residential Letting Co, Clifton</t>
         </is>
       </c>
       <c r="S120" s="9" t="inlineStr"/>
@@ -25846,7 +25852,7 @@
       <c r="V120" s="7" t="inlineStr"/>
       <c r="W120" s="8" t="inlineStr">
         <is>
-          <t>99885bbff0ab6c180a4c8ba4e0379c6f0ab42f06</t>
+          <t>bc1549c52c7b716065fff0163d60cc723a0ab301</t>
         </is>
       </c>
     </row>
@@ -25860,10 +25866,10 @@
         </is>
       </c>
       <c r="C121" s="17" t="n">
-        <v>1150</v>
+        <v>1200</v>
       </c>
       <c r="D121" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E121" s="8" t="n">
         <v>1</v>
@@ -25875,23 +25881,21 @@
       </c>
       <c r="G121" s="9" t="inlineStr">
         <is>
-          <t>Bedminster Parade, Bedminster, Bristol, BS3</t>
+          <t>Bull Lane, Crews Hole, Bristol, BS5</t>
         </is>
       </c>
       <c r="H121" s="8" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I121" s="8" t="n">
-        <v>397</v>
-      </c>
+          <t>BS5</t>
+        </is>
+      </c>
+      <c r="I121" s="8" t="n"/>
       <c r="J121" s="8" t="n"/>
       <c r="K121" s="8" t="n"/>
       <c r="L121" s="8" t="n"/>
       <c r="M121" s="8" t="n"/>
       <c r="N121" s="8" t="n">
-        <v>15212</v>
+        <v>4160</v>
       </c>
       <c r="O121" s="8" t="n">
         <v>0</v>
@@ -25899,12 +25903,12 @@
       <c r="P121" s="8" t="n"/>
       <c r="Q121" s="8" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R121" s="8" t="inlineStr">
         <is>
-          <t>West Coast Properties, Bishopston</t>
+          <t>Morgan &amp; Sons, Bristol</t>
         </is>
       </c>
       <c r="S121" s="9" t="inlineStr"/>
@@ -25921,7 +25925,7 @@
       <c r="V121" s="7" t="inlineStr"/>
       <c r="W121" s="8" t="inlineStr">
         <is>
-          <t>c5ac268b24abaa99234fcf1c93fefdbb7e77813a</t>
+          <t>297b43bd732a4c243907fc8bc1c888a888e057d1</t>
         </is>
       </c>
     </row>
@@ -25935,7 +25939,7 @@
         </is>
       </c>
       <c r="C122" s="17" t="n">
-        <v>1100</v>
+        <v>965</v>
       </c>
       <c r="D122" s="8" t="n">
         <v>1</v>
@@ -25950,23 +25954,21 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>Barton Close, St. Annes Park, BS4</t>
+          <t>Boulevard View, Whitchurch Lane</t>
         </is>
       </c>
       <c r="H122" s="8" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I122" s="8" t="n">
-        <v>441</v>
-      </c>
+          <t>BS14</t>
+        </is>
+      </c>
+      <c r="I122" s="8" t="n"/>
       <c r="J122" s="8" t="n"/>
       <c r="K122" s="8" t="n"/>
       <c r="L122" s="8" t="n"/>
       <c r="M122" s="8" t="n"/>
       <c r="N122" s="8" t="n">
-        <v>5212</v>
+        <v>5764</v>
       </c>
       <c r="O122" s="8" t="n">
         <v>0</v>
@@ -25974,12 +25976,12 @@
       <c r="P122" s="8" t="n"/>
       <c r="Q122" s="8" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R122" s="8" t="inlineStr">
         <is>
-          <t>Nook Lettings, Bristol</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S122" s="9" t="inlineStr"/>
@@ -25996,7 +25998,7 @@
       <c r="V122" s="7" t="inlineStr"/>
       <c r="W122" s="8" t="inlineStr">
         <is>
-          <t>f5910166d7abf794c3d121c920cea7bb7aaab2d9</t>
+          <t>ecef3f674f68cbf8b8e0c35c0fe5f8b0099a6a5b</t>
         </is>
       </c>
     </row>
@@ -26010,7 +26012,7 @@
         </is>
       </c>
       <c r="C123" s="17" t="n">
-        <v>1100</v>
+        <v>1200</v>
       </c>
       <c r="D123" s="8" t="n">
         <v>1</v>
@@ -26025,21 +26027,23 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>Netham Road, St George, Bristol, Bristol City</t>
+          <t>Braggs Lane, Bristol</t>
         </is>
       </c>
       <c r="H123" s="8" t="inlineStr">
         <is>
-          <t>BS5</t>
-        </is>
-      </c>
-      <c r="I123" s="8" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I123" s="8" t="n">
+        <v>409</v>
+      </c>
       <c r="J123" s="8" t="n"/>
       <c r="K123" s="8" t="n"/>
       <c r="L123" s="8" t="n"/>
       <c r="M123" s="8" t="n"/>
       <c r="N123" s="8" t="n">
-        <v>7112</v>
+        <v>20360</v>
       </c>
       <c r="O123" s="8" t="n">
         <v>0</v>
@@ -26047,12 +26051,12 @@
       <c r="P123" s="8" t="n"/>
       <c r="Q123" s="8" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R123" s="8" t="inlineStr">
         <is>
-          <t>Just Lets, Bristol</t>
+          <t>House + Co Property, Bristol</t>
         </is>
       </c>
       <c r="S123" s="9" t="inlineStr"/>
@@ -26069,7 +26073,7 @@
       <c r="V123" s="7" t="inlineStr"/>
       <c r="W123" s="8" t="inlineStr">
         <is>
-          <t>8a0efeef760593a517251fb9f7aa92b7e20ff405</t>
+          <t>b7418b86260a082ce0b767afb48615e82b4efe93</t>
         </is>
       </c>
     </row>
@@ -26083,7 +26087,7 @@
         </is>
       </c>
       <c r="C124" s="17" t="n">
-        <v>1100</v>
+        <v>1200</v>
       </c>
       <c r="D124" s="8" t="n">
         <v>1</v>
@@ -26098,7 +26102,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>Chapel Street, St Philips, Bristol, BS2</t>
+          <t>Montague Court, Bristol</t>
         </is>
       </c>
       <c r="H124" s="8" t="inlineStr">
@@ -26106,15 +26110,13 @@
           <t>BS2</t>
         </is>
       </c>
-      <c r="I124" s="8" t="n">
-        <v>549</v>
-      </c>
+      <c r="I124" s="8" t="n"/>
       <c r="J124" s="8" t="n"/>
       <c r="K124" s="8" t="n"/>
       <c r="L124" s="8" t="n"/>
       <c r="M124" s="8" t="n"/>
       <c r="N124" s="8" t="n">
-        <v>11732</v>
+        <v>21632</v>
       </c>
       <c r="O124" s="8" t="n">
         <v>0</v>
@@ -26122,12 +26124,12 @@
       <c r="P124" s="8" t="n"/>
       <c r="Q124" s="8" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R124" s="8" t="inlineStr">
         <is>
-          <t>Morgan &amp; Sons, Bristol</t>
+          <t>Connells Lettings, Southville</t>
         </is>
       </c>
       <c r="S124" s="9" t="inlineStr"/>
@@ -26144,7 +26146,7 @@
       <c r="V124" s="7" t="inlineStr"/>
       <c r="W124" s="8" t="inlineStr">
         <is>
-          <t>ef55f6374006e7f3e9b91e752a031c654a098e1f</t>
+          <t>99885bbff0ab6c180a4c8ba4e0379c6f0ab42f06</t>
         </is>
       </c>
     </row>
@@ -26173,23 +26175,23 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>Harbourside Apartments, 32-34 Hotwell Road, Bristol, BS8</t>
+          <t>Bedminster Parade, Bedminster, Bristol, BS3</t>
         </is>
       </c>
       <c r="H125" s="8" t="inlineStr">
         <is>
-          <t>BS8</t>
+          <t>BS3</t>
         </is>
       </c>
       <c r="I125" s="8" t="n">
-        <v>211</v>
+        <v>397</v>
       </c>
       <c r="J125" s="8" t="n"/>
       <c r="K125" s="8" t="n"/>
       <c r="L125" s="8" t="n"/>
       <c r="M125" s="8" t="n"/>
       <c r="N125" s="8" t="n">
-        <v>14596</v>
+        <v>15212</v>
       </c>
       <c r="O125" s="8" t="n">
         <v>0</v>
@@ -26197,12 +26199,12 @@
       <c r="P125" s="8" t="n"/>
       <c r="Q125" s="8" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="R125" s="8" t="inlineStr">
         <is>
-          <t>Savills Lettings, Clifton</t>
+          <t>West Coast Properties, Bishopston</t>
         </is>
       </c>
       <c r="S125" s="9" t="inlineStr"/>
@@ -26219,7 +26221,7 @@
       <c r="V125" s="7" t="inlineStr"/>
       <c r="W125" s="8" t="inlineStr">
         <is>
-          <t>cbabe39dc6d60b35752a40f29ab9452202acb80f</t>
+          <t>c5ac268b24abaa99234fcf1c93fefdbb7e77813a</t>
         </is>
       </c>
     </row>
@@ -26248,21 +26250,23 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>Tortworth Court, Tortworth Road, Horfield, Bristol</t>
+          <t>Barton Close, St. Annes Park, BS4</t>
         </is>
       </c>
       <c r="H126" s="8" t="inlineStr">
         <is>
-          <t>BS7</t>
-        </is>
-      </c>
-      <c r="I126" s="8" t="n"/>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I126" s="8" t="n">
+        <v>441</v>
+      </c>
       <c r="J126" s="8" t="n"/>
       <c r="K126" s="8" t="n"/>
       <c r="L126" s="8" t="n"/>
       <c r="M126" s="8" t="n"/>
       <c r="N126" s="8" t="n">
-        <v>5316</v>
+        <v>5212</v>
       </c>
       <c r="O126" s="8" t="n">
         <v>0</v>
@@ -26270,12 +26274,12 @@
       <c r="P126" s="8" t="n"/>
       <c r="Q126" s="8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="R126" s="8" t="inlineStr">
         <is>
-          <t>Holbrook Moran, Redfield</t>
+          <t>Nook Lettings, Bristol</t>
         </is>
       </c>
       <c r="S126" s="9" t="inlineStr"/>
@@ -26292,7 +26296,7 @@
       <c r="V126" s="7" t="inlineStr"/>
       <c r="W126" s="8" t="inlineStr">
         <is>
-          <t>a84a17170db7124059e6b156a1ae2181a8dd775e</t>
+          <t>f5910166d7abf794c3d121c920cea7bb7aaab2d9</t>
         </is>
       </c>
     </row>
@@ -26343,7 +26347,7 @@
       <c r="P127" s="8" t="n"/>
       <c r="Q127" s="8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="R127" s="8" t="inlineStr">
@@ -26365,7 +26369,7 @@
       <c r="V127" s="7" t="inlineStr"/>
       <c r="W127" s="8" t="inlineStr">
         <is>
-          <t>db2a5e02a3c10590c5cff5921a380c56b0683cc6</t>
+          <t>8a0efeef760593a517251fb9f7aa92b7e20ff405</t>
         </is>
       </c>
     </row>
@@ -26379,7 +26383,7 @@
         </is>
       </c>
       <c r="C128" s="17" t="n">
-        <v>1150</v>
+        <v>1100</v>
       </c>
       <c r="D128" s="8" t="n">
         <v>1</v>
@@ -26394,23 +26398,23 @@
       </c>
       <c r="G128" s="9" t="inlineStr">
         <is>
-          <t>Seymour Road, Bristol, BS5</t>
+          <t>Chapel Street, St Philips, Bristol, BS2</t>
         </is>
       </c>
       <c r="H128" s="8" t="inlineStr">
         <is>
-          <t>BS5</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I128" s="8" t="n">
-        <v>484</v>
+        <v>549</v>
       </c>
       <c r="J128" s="8" t="n"/>
       <c r="K128" s="8" t="n"/>
       <c r="L128" s="8" t="n"/>
       <c r="M128" s="8" t="n"/>
       <c r="N128" s="8" t="n">
-        <v>17164</v>
+        <v>11732</v>
       </c>
       <c r="O128" s="8" t="n">
         <v>0</v>
@@ -26418,12 +26422,12 @@
       <c r="P128" s="8" t="n"/>
       <c r="Q128" s="8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="R128" s="8" t="inlineStr">
         <is>
-          <t>Bristol Property Centre, Bristol</t>
+          <t>Morgan &amp; Sons, Bristol</t>
         </is>
       </c>
       <c r="S128" s="9" t="inlineStr"/>
@@ -26440,7 +26444,7 @@
       <c r="V128" s="7" t="inlineStr"/>
       <c r="W128" s="8" t="inlineStr">
         <is>
-          <t>1677ebd43e26e44c6ed83a5fdce71b66bc0f7dad</t>
+          <t>ef55f6374006e7f3e9b91e752a031c654a098e1f</t>
         </is>
       </c>
     </row>
@@ -26469,21 +26473,23 @@
       </c>
       <c r="G129" s="9" t="inlineStr">
         <is>
-          <t>Pinkhams Twist, Bristol</t>
+          <t>Harbourside Apartments, 32-34 Hotwell Road, Bristol, BS8</t>
         </is>
       </c>
       <c r="H129" s="8" t="inlineStr">
         <is>
-          <t>BS14</t>
-        </is>
-      </c>
-      <c r="I129" s="8" t="n"/>
+          <t>BS8</t>
+        </is>
+      </c>
+      <c r="I129" s="8" t="n">
+        <v>211</v>
+      </c>
       <c r="J129" s="8" t="n"/>
       <c r="K129" s="8" t="n"/>
       <c r="L129" s="8" t="n"/>
       <c r="M129" s="8" t="n"/>
       <c r="N129" s="8" t="n">
-        <v>4276</v>
+        <v>14596</v>
       </c>
       <c r="O129" s="8" t="n">
         <v>0</v>
@@ -26491,12 +26497,12 @@
       <c r="P129" s="8" t="n"/>
       <c r="Q129" s="8" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R129" s="8" t="inlineStr">
         <is>
-          <t>Hunters, Whitchurch</t>
+          <t>Savills Lettings, Clifton</t>
         </is>
       </c>
       <c r="S129" s="9" t="inlineStr"/>
@@ -26513,7 +26519,7 @@
       <c r="V129" s="7" t="inlineStr"/>
       <c r="W129" s="8" t="inlineStr">
         <is>
-          <t>a4ad0b3e107526f57126e848274507d4a2d88310</t>
+          <t>cbabe39dc6d60b35752a40f29ab9452202acb80f</t>
         </is>
       </c>
     </row>
@@ -26527,7 +26533,7 @@
         </is>
       </c>
       <c r="C130" s="17" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="D130" s="8" t="n">
         <v>1</v>
@@ -26537,17 +26543,17 @@
       </c>
       <c r="F130" s="8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G130" s="9" t="inlineStr">
         <is>
-          <t>Alexandra Park, Redland, Bristol, BS6</t>
+          <t>Tortworth Court, Tortworth Road, Horfield, Bristol</t>
         </is>
       </c>
       <c r="H130" s="8" t="inlineStr">
         <is>
-          <t>BS6</t>
+          <t>BS7</t>
         </is>
       </c>
       <c r="I130" s="8" t="n"/>
@@ -26556,7 +26562,7 @@
       <c r="L130" s="8" t="n"/>
       <c r="M130" s="8" t="n"/>
       <c r="N130" s="8" t="n">
-        <v>12812</v>
+        <v>5316</v>
       </c>
       <c r="O130" s="8" t="n">
         <v>0</v>
@@ -26564,12 +26570,12 @@
       <c r="P130" s="8" t="n"/>
       <c r="Q130" s="8" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="R130" s="8" t="inlineStr">
         <is>
-          <t>Romans, Clifton</t>
+          <t>Holbrook Moran, Redfield</t>
         </is>
       </c>
       <c r="S130" s="9" t="inlineStr"/>
@@ -26586,7 +26592,7 @@
       <c r="V130" s="7" t="inlineStr"/>
       <c r="W130" s="8" t="inlineStr">
         <is>
-          <t>4bffe5bcc3b220c2e55881771c8cb06946a8f773</t>
+          <t>a84a17170db7124059e6b156a1ae2181a8dd775e</t>
         </is>
       </c>
     </row>
@@ -26615,12 +26621,12 @@
       </c>
       <c r="G131" s="9" t="inlineStr">
         <is>
-          <t>Lower College Street, Bristol City Centre, Bristol, BS1</t>
+          <t>Netham Road, St George, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H131" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS5</t>
         </is>
       </c>
       <c r="I131" s="8" t="n"/>
@@ -26629,7 +26635,7 @@
       <c r="L131" s="8" t="n"/>
       <c r="M131" s="8" t="n"/>
       <c r="N131" s="8" t="n">
-        <v>18020</v>
+        <v>7112</v>
       </c>
       <c r="O131" s="8" t="n">
         <v>0</v>
@@ -26637,12 +26643,12 @@
       <c r="P131" s="8" t="n"/>
       <c r="Q131" s="8" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="R131" s="8" t="inlineStr">
         <is>
-          <t>West Coast Properties, Bishopston</t>
+          <t>Just Lets, Bristol</t>
         </is>
       </c>
       <c r="S131" s="9" t="inlineStr"/>
@@ -26659,7 +26665,7 @@
       <c r="V131" s="7" t="inlineStr"/>
       <c r="W131" s="8" t="inlineStr">
         <is>
-          <t>b6b3d8e95529c1ffc6a7e396f88cd883930e9d79</t>
+          <t>db2a5e02a3c10590c5cff5921a380c56b0683cc6</t>
         </is>
       </c>
     </row>
@@ -26676,7 +26682,7 @@
         <v>1150</v>
       </c>
       <c r="D132" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E132" s="8" t="n">
         <v>1</v>
@@ -26688,7 +26694,7 @@
       </c>
       <c r="G132" s="9" t="inlineStr">
         <is>
-          <t>Church Road, Bristol, BS5</t>
+          <t>Seymour Road, Bristol, BS5</t>
         </is>
       </c>
       <c r="H132" s="8" t="inlineStr">
@@ -26697,14 +26703,14 @@
         </is>
       </c>
       <c r="I132" s="8" t="n">
-        <v>3057</v>
+        <v>484</v>
       </c>
       <c r="J132" s="8" t="n"/>
       <c r="K132" s="8" t="n"/>
       <c r="L132" s="8" t="n"/>
       <c r="M132" s="8" t="n"/>
       <c r="N132" s="8" t="n">
-        <v>11864</v>
+        <v>17164</v>
       </c>
       <c r="O132" s="8" t="n">
         <v>0</v>
@@ -26712,12 +26718,12 @@
       <c r="P132" s="8" t="n"/>
       <c r="Q132" s="8" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="R132" s="8" t="inlineStr">
         <is>
-          <t>Lets Rent Bristol, Bristol</t>
+          <t>Bristol Property Centre, Bristol</t>
         </is>
       </c>
       <c r="S132" s="9" t="inlineStr"/>
@@ -26734,7 +26740,7 @@
       <c r="V132" s="7" t="inlineStr"/>
       <c r="W132" s="8" t="inlineStr">
         <is>
-          <t>765c51adc42a96d23086446a7ab5c6c6fb234cca</t>
+          <t>1677ebd43e26e44c6ed83a5fdce71b66bc0f7dad</t>
         </is>
       </c>
     </row>
@@ -26748,7 +26754,7 @@
         </is>
       </c>
       <c r="C133" s="17" t="n">
-        <v>995</v>
+        <v>1150</v>
       </c>
       <c r="D133" s="8" t="n">
         <v>1</v>
@@ -26763,12 +26769,12 @@
       </c>
       <c r="G133" s="9" t="inlineStr">
         <is>
-          <t>Two Mile Hill Road, Kingswood, Bristol</t>
+          <t>Pinkhams Twist, Bristol</t>
         </is>
       </c>
       <c r="H133" s="8" t="inlineStr">
         <is>
-          <t>BS15</t>
+          <t>BS14</t>
         </is>
       </c>
       <c r="I133" s="8" t="n"/>
@@ -26777,7 +26783,7 @@
       <c r="L133" s="8" t="n"/>
       <c r="M133" s="8" t="n"/>
       <c r="N133" s="8" t="n">
-        <v>5116</v>
+        <v>4276</v>
       </c>
       <c r="O133" s="8" t="n">
         <v>0</v>
@@ -26785,12 +26791,12 @@
       <c r="P133" s="8" t="n"/>
       <c r="Q133" s="8" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="R133" s="8" t="inlineStr">
         <is>
-          <t>TLS Estate Agents, Bristol</t>
+          <t>Hunters, Whitchurch</t>
         </is>
       </c>
       <c r="S133" s="9" t="inlineStr"/>
@@ -26807,7 +26813,7 @@
       <c r="V133" s="7" t="inlineStr"/>
       <c r="W133" s="8" t="inlineStr">
         <is>
-          <t>4127db1eec9e5102c45835506c359c90057d0332</t>
+          <t>a4ad0b3e107526f57126e848274507d4a2d88310</t>
         </is>
       </c>
     </row>
@@ -26821,7 +26827,7 @@
         </is>
       </c>
       <c r="C134" s="17" t="n">
-        <v>1100</v>
+        <v>1200</v>
       </c>
       <c r="D134" s="8" t="n">
         <v>1</v>
@@ -26831,17 +26837,17 @@
       </c>
       <c r="F134" s="8" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G134" s="9" t="inlineStr">
         <is>
-          <t>Robertson Drive, St Annes Park</t>
+          <t>Alexandra Park, Redland, Bristol, BS6</t>
         </is>
       </c>
       <c r="H134" s="8" t="inlineStr">
         <is>
-          <t>BS4</t>
+          <t>BS6</t>
         </is>
       </c>
       <c r="I134" s="8" t="n"/>
@@ -26850,7 +26856,7 @@
       <c r="L134" s="8" t="n"/>
       <c r="M134" s="8" t="n"/>
       <c r="N134" s="8" t="n">
-        <v>4252</v>
+        <v>12812</v>
       </c>
       <c r="O134" s="8" t="n">
         <v>0</v>
@@ -26858,12 +26864,12 @@
       <c r="P134" s="8" t="n"/>
       <c r="Q134" s="8" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="R134" s="8" t="inlineStr">
         <is>
-          <t>D W Smith &amp; Company, Hanham</t>
+          <t>Romans, Clifton</t>
         </is>
       </c>
       <c r="S134" s="9" t="inlineStr"/>
@@ -26880,7 +26886,7 @@
       <c r="V134" s="7" t="inlineStr"/>
       <c r="W134" s="8" t="inlineStr">
         <is>
-          <t>da7b12e8670a61ba0296492df23cc29a51d7d8e0</t>
+          <t>4bffe5bcc3b220c2e55881771c8cb06946a8f773</t>
         </is>
       </c>
     </row>
@@ -26894,7 +26900,7 @@
         </is>
       </c>
       <c r="C135" s="17" t="n">
-        <v>1150</v>
+        <v>1100</v>
       </c>
       <c r="D135" s="8" t="n">
         <v>1</v>
@@ -26909,23 +26915,21 @@
       </c>
       <c r="G135" s="9" t="inlineStr">
         <is>
-          <t>Flat, Newquay Road, Knowle, Bristol, Bristol City</t>
+          <t>Lower College Street, Bristol City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H135" s="8" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I135" s="8" t="n">
-        <v>527</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I135" s="8" t="n"/>
       <c r="J135" s="8" t="n"/>
       <c r="K135" s="8" t="n"/>
       <c r="L135" s="8" t="n"/>
       <c r="M135" s="8" t="n"/>
       <c r="N135" s="8" t="n">
-        <v>5548</v>
+        <v>18020</v>
       </c>
       <c r="O135" s="8" t="n">
         <v>0</v>
@@ -26933,12 +26937,12 @@
       <c r="P135" s="8" t="n"/>
       <c r="Q135" s="8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="R135" s="8" t="inlineStr">
         <is>
-          <t>Sheedy &amp; Co, Covering Bristol</t>
+          <t>West Coast Properties, Bishopston</t>
         </is>
       </c>
       <c r="S135" s="9" t="inlineStr"/>
@@ -26955,7 +26959,7 @@
       <c r="V135" s="7" t="inlineStr"/>
       <c r="W135" s="8" t="inlineStr">
         <is>
-          <t>d6e7992bdb7662462ebba6fc8f5a0a065f5c0c34</t>
+          <t>b6b3d8e95529c1ffc6a7e396f88cd883930e9d79</t>
         </is>
       </c>
     </row>
@@ -26969,10 +26973,10 @@
         </is>
       </c>
       <c r="C136" s="17" t="n">
-        <v>1195</v>
+        <v>1150</v>
       </c>
       <c r="D136" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E136" s="8" t="n">
         <v>1</v>
@@ -26984,7 +26988,7 @@
       </c>
       <c r="G136" s="9" t="inlineStr">
         <is>
-          <t>Whitehall Road, Bristol, BS5</t>
+          <t>Church Road, Bristol, BS5</t>
         </is>
       </c>
       <c r="H136" s="8" t="inlineStr">
@@ -26993,14 +26997,14 @@
         </is>
       </c>
       <c r="I136" s="8" t="n">
-        <v>409</v>
+        <v>3057</v>
       </c>
       <c r="J136" s="8" t="n"/>
       <c r="K136" s="8" t="n"/>
       <c r="L136" s="8" t="n"/>
       <c r="M136" s="8" t="n"/>
       <c r="N136" s="8" t="n">
-        <v>10420</v>
+        <v>11864</v>
       </c>
       <c r="O136" s="8" t="n">
         <v>0</v>
@@ -27008,12 +27012,12 @@
       <c r="P136" s="8" t="n"/>
       <c r="Q136" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="R136" s="8" t="inlineStr">
         <is>
-          <t>Parks Estate Agents, Bristol</t>
+          <t>Lets Rent Bristol, Bristol</t>
         </is>
       </c>
       <c r="S136" s="9" t="inlineStr"/>
@@ -27030,7 +27034,7 @@
       <c r="V136" s="7" t="inlineStr"/>
       <c r="W136" s="8" t="inlineStr">
         <is>
-          <t>98d53bc43440611cb699e6844ca898806a2f4b28</t>
+          <t>765c51adc42a96d23086446a7ab5c6c6fb234cca</t>
         </is>
       </c>
     </row>
@@ -27044,7 +27048,7 @@
         </is>
       </c>
       <c r="C137" s="17" t="n">
-        <v>1200</v>
+        <v>995</v>
       </c>
       <c r="D137" s="8" t="n">
         <v>1</v>
@@ -27059,12 +27063,12 @@
       </c>
       <c r="G137" s="9" t="inlineStr">
         <is>
-          <t>Knowle Road, Bristol, BS4</t>
+          <t>Two Mile Hill Road, Kingswood, Bristol</t>
         </is>
       </c>
       <c r="H137" s="8" t="inlineStr">
         <is>
-          <t>BS4</t>
+          <t>BS15</t>
         </is>
       </c>
       <c r="I137" s="8" t="n"/>
@@ -27073,7 +27077,7 @@
       <c r="L137" s="8" t="n"/>
       <c r="M137" s="8" t="n"/>
       <c r="N137" s="8" t="n">
-        <v>6852</v>
+        <v>5116</v>
       </c>
       <c r="O137" s="8" t="n">
         <v>0</v>
@@ -27081,12 +27085,12 @@
       <c r="P137" s="8" t="n"/>
       <c r="Q137" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="R137" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>TLS Estate Agents, Bristol</t>
         </is>
       </c>
       <c r="S137" s="9" t="inlineStr"/>
@@ -27103,7 +27107,7 @@
       <c r="V137" s="7" t="inlineStr"/>
       <c r="W137" s="8" t="inlineStr">
         <is>
-          <t>bbb9b81c216b0de31ba8859ef50a78ed36377871</t>
+          <t>4127db1eec9e5102c45835506c359c90057d0332</t>
         </is>
       </c>
     </row>
@@ -27117,7 +27121,7 @@
         </is>
       </c>
       <c r="C138" s="17" t="n">
-        <v>850</v>
+        <v>1100</v>
       </c>
       <c r="D138" s="8" t="n">
         <v>1</v>
@@ -27127,28 +27131,26 @@
       </c>
       <c r="F138" s="8" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G138" s="9" t="inlineStr">
         <is>
-          <t>Whitehall Road, Bristol, BS5</t>
+          <t>Robertson Drive, St Annes Park</t>
         </is>
       </c>
       <c r="H138" s="8" t="inlineStr">
         <is>
-          <t>BS5</t>
-        </is>
-      </c>
-      <c r="I138" s="8" t="n">
-        <v>248</v>
-      </c>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I138" s="8" t="n"/>
       <c r="J138" s="8" t="n"/>
       <c r="K138" s="8" t="n"/>
       <c r="L138" s="8" t="n"/>
       <c r="M138" s="8" t="n"/>
       <c r="N138" s="8" t="n">
-        <v>10420</v>
+        <v>4252</v>
       </c>
       <c r="O138" s="8" t="n">
         <v>0</v>
@@ -27156,12 +27158,12 @@
       <c r="P138" s="8" t="n"/>
       <c r="Q138" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="R138" s="8" t="inlineStr">
         <is>
-          <t>Parks Estate Agents, Bristol</t>
+          <t>D W Smith &amp; Company, Hanham</t>
         </is>
       </c>
       <c r="S138" s="9" t="inlineStr"/>
@@ -27178,7 +27180,7 @@
       <c r="V138" s="7" t="inlineStr"/>
       <c r="W138" s="8" t="inlineStr">
         <is>
-          <t>17396b2e44a31a6428a3598c1935528dc4d5bd81</t>
+          <t>da7b12e8670a61ba0296492df23cc29a51d7d8e0</t>
         </is>
       </c>
     </row>
@@ -27192,13 +27194,13 @@
         </is>
       </c>
       <c r="C139" s="17" t="n">
-        <v>1600</v>
+        <v>1150</v>
       </c>
       <c r="D139" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E139" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F139" s="8" t="inlineStr">
         <is>
@@ -27207,21 +27209,23 @@
       </c>
       <c r="G139" s="9" t="inlineStr">
         <is>
-          <t>Central Quay North</t>
+          <t>Flat, Newquay Road, Knowle, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H139" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I139" s="8" t="n"/>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I139" s="8" t="n">
+        <v>527</v>
+      </c>
       <c r="J139" s="8" t="n"/>
       <c r="K139" s="8" t="n"/>
       <c r="L139" s="8" t="n"/>
       <c r="M139" s="8" t="n"/>
       <c r="N139" s="8" t="n">
-        <v>20792</v>
+        <v>5548</v>
       </c>
       <c r="O139" s="8" t="n">
         <v>0</v>
@@ -27229,12 +27233,12 @@
       <c r="P139" s="8" t="n"/>
       <c r="Q139" s="8" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="R139" s="8" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>Sheedy &amp; Co, Covering Bristol</t>
         </is>
       </c>
       <c r="S139" s="9" t="inlineStr"/>
@@ -27251,7 +27255,7 @@
       <c r="V139" s="7" t="inlineStr"/>
       <c r="W139" s="8" t="inlineStr">
         <is>
-          <t>8419d14a9ba13a5a7785694e74cc8e87937eb3c1</t>
+          <t>d6e7992bdb7662462ebba6fc8f5a0a065f5c0c34</t>
         </is>
       </c>
     </row>
@@ -27265,13 +27269,13 @@
         </is>
       </c>
       <c r="C140" s="17" t="n">
-        <v>1600</v>
+        <v>1195</v>
       </c>
       <c r="D140" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E140" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F140" s="8" t="inlineStr">
         <is>
@@ -27280,32 +27284,36 @@
       </c>
       <c r="G140" s="9" t="inlineStr">
         <is>
-          <t>Marsh Street, Bristol</t>
+          <t>Whitehall Road, Bristol, BS5</t>
         </is>
       </c>
       <c r="H140" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I140" s="8" t="n"/>
+          <t>BS5</t>
+        </is>
+      </c>
+      <c r="I140" s="8" t="n">
+        <v>409</v>
+      </c>
       <c r="J140" s="8" t="n"/>
       <c r="K140" s="8" t="n"/>
       <c r="L140" s="8" t="n"/>
       <c r="M140" s="8" t="n"/>
-      <c r="N140" s="8" t="n"/>
+      <c r="N140" s="8" t="n">
+        <v>10420</v>
+      </c>
       <c r="O140" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P140" s="8" t="n"/>
       <c r="Q140" s="8" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R140" s="8" t="inlineStr">
         <is>
-          <t>Stonebridge Shaw, Portishead</t>
+          <t>Parks Estate Agents, Bristol</t>
         </is>
       </c>
       <c r="S140" s="9" t="inlineStr"/>
@@ -27322,7 +27330,7 @@
       <c r="V140" s="7" t="inlineStr"/>
       <c r="W140" s="8" t="inlineStr">
         <is>
-          <t>7a1b3f42641b30502df555b92790f9c12b03583c</t>
+          <t>98d53bc43440611cb699e6844ca898806a2f4b28</t>
         </is>
       </c>
     </row>
@@ -27336,7 +27344,7 @@
         </is>
       </c>
       <c r="C141" s="17" t="n">
-        <v>1100</v>
+        <v>1200</v>
       </c>
       <c r="D141" s="8" t="n">
         <v>1</v>
@@ -27351,12 +27359,12 @@
       </c>
       <c r="G141" s="9" t="inlineStr">
         <is>
-          <t>St Michaels Hill Ref 708</t>
+          <t>Knowle Road, Bristol, BS4</t>
         </is>
       </c>
       <c r="H141" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS4</t>
         </is>
       </c>
       <c r="I141" s="8" t="n"/>
@@ -27365,7 +27373,7 @@
       <c r="L141" s="8" t="n"/>
       <c r="M141" s="8" t="n"/>
       <c r="N141" s="8" t="n">
-        <v>19512</v>
+        <v>6852</v>
       </c>
       <c r="O141" s="8" t="n">
         <v>0</v>
@@ -27373,12 +27381,12 @@
       <c r="P141" s="8" t="n"/>
       <c r="Q141" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R141" s="8" t="inlineStr">
         <is>
-          <t>Jackson Property Management Ltd, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S141" s="9" t="inlineStr"/>
@@ -27395,7 +27403,7 @@
       <c r="V141" s="7" t="inlineStr"/>
       <c r="W141" s="8" t="inlineStr">
         <is>
-          <t>ad53fb9cd96ec72adbc7f3d6c8a52caba547cc20</t>
+          <t>bbb9b81c216b0de31ba8859ef50a78ed36377871</t>
         </is>
       </c>
     </row>
@@ -27409,7 +27417,7 @@
         </is>
       </c>
       <c r="C142" s="17" t="n">
-        <v>1095</v>
+        <v>850</v>
       </c>
       <c r="D142" s="8" t="n">
         <v>1</v>
@@ -27424,21 +27432,23 @@
       </c>
       <c r="G142" s="9" t="inlineStr">
         <is>
-          <t>Manor House Lane, Whitchurch, Bristol, Bristol City</t>
+          <t>Whitehall Road, Bristol, BS5</t>
         </is>
       </c>
       <c r="H142" s="8" t="inlineStr">
         <is>
-          <t>BS14</t>
-        </is>
-      </c>
-      <c r="I142" s="8" t="n"/>
+          <t>BS5</t>
+        </is>
+      </c>
+      <c r="I142" s="8" t="n">
+        <v>248</v>
+      </c>
       <c r="J142" s="8" t="n"/>
       <c r="K142" s="8" t="n"/>
       <c r="L142" s="8" t="n"/>
       <c r="M142" s="8" t="n"/>
       <c r="N142" s="8" t="n">
-        <v>2652</v>
+        <v>10420</v>
       </c>
       <c r="O142" s="8" t="n">
         <v>0</v>
@@ -27446,12 +27456,12 @@
       <c r="P142" s="8" t="n"/>
       <c r="Q142" s="8" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R142" s="8" t="inlineStr">
         <is>
-          <t>Millennium Lettings &amp; Management, Bristol</t>
+          <t>Parks Estate Agents, Bristol</t>
         </is>
       </c>
       <c r="S142" s="9" t="inlineStr"/>
@@ -27468,7 +27478,7 @@
       <c r="V142" s="7" t="inlineStr"/>
       <c r="W142" s="8" t="inlineStr">
         <is>
-          <t>ab692cb96ad18ebe26a6d19d737d0b539752370a</t>
+          <t>17396b2e44a31a6428a3598c1935528dc4d5bd81</t>
         </is>
       </c>
     </row>
@@ -27482,13 +27492,13 @@
         </is>
       </c>
       <c r="C143" s="17" t="n">
-        <v>1200</v>
+        <v>1600</v>
       </c>
       <c r="D143" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E143" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F143" s="8" t="inlineStr">
         <is>
@@ -27497,23 +27507,21 @@
       </c>
       <c r="G143" s="9" t="inlineStr">
         <is>
-          <t>Old Market, Verdigris, BS2 0AF</t>
+          <t>Central Quay North</t>
         </is>
       </c>
       <c r="H143" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I143" s="8" t="n">
-        <v>388</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I143" s="8" t="n"/>
       <c r="J143" s="8" t="n"/>
       <c r="K143" s="8" t="n"/>
       <c r="L143" s="8" t="n"/>
       <c r="M143" s="8" t="n"/>
       <c r="N143" s="8" t="n">
-        <v>21220</v>
+        <v>20792</v>
       </c>
       <c r="O143" s="8" t="n">
         <v>0</v>
@@ -27521,12 +27529,12 @@
       <c r="P143" s="8" t="n"/>
       <c r="Q143" s="8" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R143" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S143" s="9" t="inlineStr"/>
@@ -27543,254 +27551,306 @@
       <c r="V143" s="7" t="inlineStr"/>
       <c r="W143" s="8" t="inlineStr">
         <is>
+          <t>8419d14a9ba13a5a7785694e74cc8e87937eb3c1</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B144" s="9" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C144" s="17" t="n">
+        <v>1600</v>
+      </c>
+      <c r="D144" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E144" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F144" s="8" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G144" s="9" t="inlineStr">
+        <is>
+          <t>Marsh Street, Bristol</t>
+        </is>
+      </c>
+      <c r="H144" s="8" t="inlineStr">
+        <is>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I144" s="8" t="n"/>
+      <c r="J144" s="8" t="n"/>
+      <c r="K144" s="8" t="n"/>
+      <c r="L144" s="8" t="n"/>
+      <c r="M144" s="8" t="n"/>
+      <c r="N144" s="8" t="n"/>
+      <c r="O144" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P144" s="8" t="n"/>
+      <c r="Q144" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="R144" s="8" t="inlineStr">
+        <is>
+          <t>Stonebridge Shaw, Portishead</t>
+        </is>
+      </c>
+      <c r="S144" s="9" t="inlineStr"/>
+      <c r="T144" s="12" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U144" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V144" s="7" t="inlineStr"/>
+      <c r="W144" s="8" t="inlineStr">
+        <is>
+          <t>7a1b3f42641b30502df555b92790f9c12b03583c</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B145" s="9" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C145" s="17" t="n">
+        <v>1100</v>
+      </c>
+      <c r="D145" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E145" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F145" s="8" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G145" s="9" t="inlineStr">
+        <is>
+          <t>St Michaels Hill Ref 708</t>
+        </is>
+      </c>
+      <c r="H145" s="8" t="inlineStr">
+        <is>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I145" s="8" t="n"/>
+      <c r="J145" s="8" t="n"/>
+      <c r="K145" s="8" t="n"/>
+      <c r="L145" s="8" t="n"/>
+      <c r="M145" s="8" t="n"/>
+      <c r="N145" s="8" t="n">
+        <v>19512</v>
+      </c>
+      <c r="O145" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P145" s="8" t="n"/>
+      <c r="Q145" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="R145" s="8" t="inlineStr">
+        <is>
+          <t>Jackson Property Management Ltd, Bristol</t>
+        </is>
+      </c>
+      <c r="S145" s="9" t="inlineStr"/>
+      <c r="T145" s="12" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U145" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V145" s="7" t="inlineStr"/>
+      <c r="W145" s="8" t="inlineStr">
+        <is>
+          <t>ad53fb9cd96ec72adbc7f3d6c8a52caba547cc20</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B146" s="9" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C146" s="17" t="n">
+        <v>1095</v>
+      </c>
+      <c r="D146" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E146" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F146" s="8" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G146" s="9" t="inlineStr">
+        <is>
+          <t>Manor House Lane, Whitchurch, Bristol, Bristol City</t>
+        </is>
+      </c>
+      <c r="H146" s="8" t="inlineStr">
+        <is>
+          <t>BS14</t>
+        </is>
+      </c>
+      <c r="I146" s="8" t="n"/>
+      <c r="J146" s="8" t="n"/>
+      <c r="K146" s="8" t="n"/>
+      <c r="L146" s="8" t="n"/>
+      <c r="M146" s="8" t="n"/>
+      <c r="N146" s="8" t="n">
+        <v>2652</v>
+      </c>
+      <c r="O146" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P146" s="8" t="n"/>
+      <c r="Q146" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="R146" s="8" t="inlineStr">
+        <is>
+          <t>Millennium Lettings &amp; Management, Bristol</t>
+        </is>
+      </c>
+      <c r="S146" s="9" t="inlineStr"/>
+      <c r="T146" s="12" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U146" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V146" s="7" t="inlineStr"/>
+      <c r="W146" s="8" t="inlineStr">
+        <is>
+          <t>ab692cb96ad18ebe26a6d19d737d0b539752370a</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B147" s="9" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C147" s="17" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D147" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E147" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F147" s="8" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G147" s="9" t="inlineStr">
+        <is>
+          <t>Old Market, Verdigris, BS2 0AF</t>
+        </is>
+      </c>
+      <c r="H147" s="8" t="inlineStr">
+        <is>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I147" s="8" t="n">
+        <v>388</v>
+      </c>
+      <c r="J147" s="8" t="n"/>
+      <c r="K147" s="8" t="n"/>
+      <c r="L147" s="8" t="n"/>
+      <c r="M147" s="8" t="n"/>
+      <c r="N147" s="8" t="n">
+        <v>21220</v>
+      </c>
+      <c r="O147" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P147" s="8" t="n"/>
+      <c r="Q147" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="R147" s="8" t="inlineStr">
+        <is>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
+        </is>
+      </c>
+      <c r="S147" s="9" t="inlineStr"/>
+      <c r="T147" s="12" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U147" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V147" s="7" t="inlineStr"/>
+      <c r="W147" s="8" t="inlineStr">
+        <is>
           <t>4bd094575ff83a26d208b8ea7ce8140210cc94b9</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="B144" s="7" t="n"/>
-      <c r="C144" s="18" t="n">
-        <v>800</v>
-      </c>
-      <c r="D144" t="n">
-        <v>2</v>
-      </c>
-      <c r="E144" t="n">
-        <v>1</v>
-      </c>
-      <c r="F144" t="inlineStr">
-        <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="G144" s="7" t="inlineStr">
-        <is>
-          <t>Rehoboth Court, Coedpoeth, Wrexham, LL11</t>
-        </is>
-      </c>
-      <c r="H144" t="inlineStr">
-        <is>
-          <t>LL11</t>
-        </is>
-      </c>
-      <c r="N144" t="n">
-        <v>448</v>
-      </c>
-      <c r="O144" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q144" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="R144" t="inlineStr">
-        <is>
-          <t>OpenRent, London</t>
-        </is>
-      </c>
-      <c r="S144" s="7" t="inlineStr"/>
-      <c r="T144" s="14" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U144" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V144" s="7" t="inlineStr"/>
-      <c r="W144" t="inlineStr">
-        <is>
-          <t>c4ca3b08a858fe282766d1680bb80dd10c24ce32</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="B145" s="7" t="n"/>
-      <c r="C145" s="18" t="n">
-        <v>900</v>
-      </c>
-      <c r="D145" t="n">
-        <v>2</v>
-      </c>
-      <c r="E145" t="n">
-        <v>1</v>
-      </c>
-      <c r="F145" t="inlineStr">
-        <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="G145" s="7" t="inlineStr">
-        <is>
-          <t>Newmarket Road, Dyserth, LL18</t>
-        </is>
-      </c>
-      <c r="H145" t="inlineStr">
-        <is>
-          <t>LL18</t>
-        </is>
-      </c>
-      <c r="N145" t="n">
-        <v>328</v>
-      </c>
-      <c r="O145" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q145" t="inlineStr">
-        <is>
-          <t>2026-07-07</t>
-        </is>
-      </c>
-      <c r="R145" t="inlineStr">
-        <is>
-          <t>Fifty North West, Chester</t>
-        </is>
-      </c>
-      <c r="S145" s="7" t="inlineStr"/>
-      <c r="T145" s="14" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U145" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V145" s="7" t="inlineStr"/>
-      <c r="W145" t="inlineStr">
-        <is>
-          <t>19dde05bbe4ff1dc0306104719519db3f4baa597</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="B146" s="7" t="n"/>
-      <c r="C146" s="18" t="n">
-        <v>625</v>
-      </c>
-      <c r="D146" t="n">
-        <v>1</v>
-      </c>
-      <c r="E146" t="n">
-        <v>1</v>
-      </c>
-      <c r="F146" t="inlineStr">
-        <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="G146" s="7" t="inlineStr">
-        <is>
-          <t>Field View, Mancot, Deeside, CH5 2EY</t>
-        </is>
-      </c>
-      <c r="H146" t="inlineStr">
-        <is>
-          <t>CH5</t>
-        </is>
-      </c>
-      <c r="N146" t="n">
-        <v>824</v>
-      </c>
-      <c r="O146" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q146" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="R146" t="inlineStr">
-        <is>
-          <t>Habodel Property Services Ltd, Doncaster</t>
-        </is>
-      </c>
-      <c r="S146" s="7" t="inlineStr"/>
-      <c r="T146" s="14" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U146" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V146" s="7" t="inlineStr"/>
-      <c r="W146" t="inlineStr">
-        <is>
-          <t>c123bf34773b0afd208b42a23676d0de104b0aa4</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="B147" s="7" t="n"/>
-      <c r="C147" s="18" t="n">
-        <v>795</v>
-      </c>
-      <c r="D147" t="n">
-        <v>2</v>
-      </c>
-      <c r="E147" t="n">
-        <v>1</v>
-      </c>
-      <c r="F147" t="inlineStr">
-        <is>
-          <t>semi_detached</t>
-        </is>
-      </c>
-      <c r="G147" s="7" t="inlineStr">
-        <is>
-          <t>Cilcain, The Square, CH7</t>
-        </is>
-      </c>
-      <c r="H147" t="inlineStr">
-        <is>
-          <t>CH7</t>
-        </is>
-      </c>
-      <c r="N147" t="n">
-        <v>0</v>
-      </c>
-      <c r="O147" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q147" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="R147" t="inlineStr">
-        <is>
-          <t>Williams Estates, Rhuddlan</t>
-        </is>
-      </c>
-      <c r="S147" s="7" t="inlineStr"/>
-      <c r="T147" s="14" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U147" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V147" s="7" t="inlineStr"/>
-      <c r="W147" t="inlineStr">
-        <is>
-          <t>87b32c4489714d9b512693daad46cef94dcd76a1</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="B148" s="7" t="n"/>
       <c r="C148" s="18" t="n">
-        <v>950</v>
+        <v>800</v>
       </c>
       <c r="D148" t="n">
         <v>2</v>
@@ -27800,33 +27860,33 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>semi_detached</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G148" s="7" t="inlineStr">
         <is>
-          <t>Cae Masarn, Pentre Halkyn, Holywell, Flintshire, CH8</t>
+          <t>Rehoboth Court, Coedpoeth, Wrexham, LL11</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>CH8</t>
+          <t>LL11</t>
         </is>
       </c>
       <c r="N148" t="n">
-        <v>56</v>
+        <v>448</v>
       </c>
       <c r="O148" t="n">
         <v>0</v>
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="R148" t="inlineStr">
         <is>
-          <t>William Gleave, Deeside</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S148" s="7" t="inlineStr"/>
@@ -27843,14 +27903,14 @@
       <c r="V148" s="7" t="inlineStr"/>
       <c r="W148" t="inlineStr">
         <is>
-          <t>21cedfdeff38e71da260f36d15fc7a90e3806efc</t>
+          <t>c4ca3b08a858fe282766d1680bb80dd10c24ce32</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="B149" s="7" t="n"/>
       <c r="C149" s="18" t="n">
-        <v>925</v>
+        <v>900</v>
       </c>
       <c r="D149" t="n">
         <v>2</v>
@@ -27860,36 +27920,33 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G149" s="7" t="inlineStr">
         <is>
-          <t>Hill Top Close, Ewloe, CH5</t>
+          <t>Newmarket Road, Dyserth, LL18</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>CH5</t>
-        </is>
-      </c>
-      <c r="I149" t="n">
-        <v>721</v>
+          <t>LL18</t>
+        </is>
       </c>
       <c r="N149" t="n">
-        <v>472</v>
+        <v>328</v>
       </c>
       <c r="O149" t="n">
         <v>0</v>
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">
         <is>
-          <t>Reades, Hawarden Lettings</t>
+          <t>Fifty North West, Chester</t>
         </is>
       </c>
       <c r="S149" s="7" t="inlineStr"/>
@@ -27906,14 +27963,14 @@
       <c r="V149" s="7" t="inlineStr"/>
       <c r="W149" t="inlineStr">
         <is>
-          <t>1b94ffba8e84bd8bda3a33b448f8f35102e29484</t>
+          <t>19dde05bbe4ff1dc0306104719519db3f4baa597</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="B150" s="7" t="n"/>
       <c r="C150" s="18" t="n">
-        <v>650</v>
+        <v>625</v>
       </c>
       <c r="D150" t="n">
         <v>1</v>
@@ -27928,7 +27985,7 @@
       </c>
       <c r="G150" s="7" t="inlineStr">
         <is>
-          <t>Chester Road East, Shotton, Deeside</t>
+          <t>Field View, Mancot, Deeside, CH5 2EY</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
@@ -27936,23 +27993,20 @@
           <t>CH5</t>
         </is>
       </c>
-      <c r="I150" t="n">
-        <v>474</v>
-      </c>
       <c r="N150" t="n">
-        <v>2016</v>
+        <v>824</v>
       </c>
       <c r="O150" t="n">
         <v>0</v>
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R150" t="inlineStr">
         <is>
-          <t>Thomas Property Group, Chester</t>
+          <t>Habodel Property Services Ltd, Doncaster</t>
         </is>
       </c>
       <c r="S150" s="7" t="inlineStr"/>
@@ -27969,14 +28023,14 @@
       <c r="V150" s="7" t="inlineStr"/>
       <c r="W150" t="inlineStr">
         <is>
-          <t>f80c03a584803371ab95595ae7a449a94715fbd1</t>
+          <t>c123bf34773b0afd208b42a23676d0de104b0aa4</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="B151" s="7" t="n"/>
       <c r="C151" s="18" t="n">
-        <v>750</v>
+        <v>795</v>
       </c>
       <c r="D151" t="n">
         <v>2</v>
@@ -27986,33 +28040,33 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>semi_detached</t>
         </is>
       </c>
       <c r="G151" s="7" t="inlineStr">
         <is>
-          <t>Sycamore Terrace, Rhosrobin, Wrexham</t>
+          <t>Cilcain, The Square, CH7</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>LL11</t>
+          <t>CH7</t>
         </is>
       </c>
       <c r="N151" t="n">
-        <v>1300</v>
+        <v>0</v>
       </c>
       <c r="O151" t="n">
         <v>0</v>
       </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="R151" t="inlineStr">
         <is>
-          <t>Bowen, Wrexham</t>
+          <t>Williams Estates, Rhuddlan</t>
         </is>
       </c>
       <c r="S151" s="7" t="inlineStr"/>
@@ -28029,14 +28083,14 @@
       <c r="V151" s="7" t="inlineStr"/>
       <c r="W151" t="inlineStr">
         <is>
-          <t>40274ada7dfa710e5054184216178477a704016c</t>
+          <t>87b32c4489714d9b512693daad46cef94dcd76a1</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="B152" s="7" t="n"/>
       <c r="C152" s="18" t="n">
-        <v>900</v>
+        <v>950</v>
       </c>
       <c r="D152" t="n">
         <v>2</v>
@@ -28051,23 +28105,23 @@
       </c>
       <c r="G152" s="7" t="inlineStr">
         <is>
-          <t>Kiln Close, Buckley, Flintshire, CH7</t>
+          <t>Cae Masarn, Pentre Halkyn, Holywell, Flintshire, CH8</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>CH7</t>
+          <t>CH8</t>
         </is>
       </c>
       <c r="N152" t="n">
-        <v>936</v>
+        <v>56</v>
       </c>
       <c r="O152" t="n">
         <v>0</v>
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="R152" t="inlineStr">
@@ -28089,14 +28143,14 @@
       <c r="V152" s="7" t="inlineStr"/>
       <c r="W152" t="inlineStr">
         <is>
-          <t>780cbc2857d57b036f046702f312e0298790c096</t>
+          <t>21cedfdeff38e71da260f36d15fc7a90e3806efc</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="B153" s="7" t="n"/>
       <c r="C153" s="18" t="n">
-        <v>900</v>
+        <v>925</v>
       </c>
       <c r="D153" t="n">
         <v>2</v>
@@ -28111,28 +28165,31 @@
       </c>
       <c r="G153" s="7" t="inlineStr">
         <is>
-          <t>9 Park Road, Ruthin</t>
+          <t>Hill Top Close, Ewloe, CH5</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>LL15</t>
-        </is>
+          <t>CH5</t>
+        </is>
+      </c>
+      <c r="I153" t="n">
+        <v>721</v>
       </c>
       <c r="N153" t="n">
-        <v>576</v>
+        <v>472</v>
       </c>
       <c r="O153" t="n">
         <v>0</v>
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R153" t="inlineStr">
         <is>
-          <t>Cavendish Rentals Ltd, Ruthin</t>
+          <t>Reades, Hawarden Lettings</t>
         </is>
       </c>
       <c r="S153" s="7" t="inlineStr"/>
@@ -28149,53 +28206,53 @@
       <c r="V153" s="7" t="inlineStr"/>
       <c r="W153" t="inlineStr">
         <is>
-          <t>c771916d30aebac19d1f346f767747d7b73a7d6c</t>
+          <t>1b94ffba8e84bd8bda3a33b448f8f35102e29484</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="B154" s="7" t="n"/>
       <c r="C154" s="18" t="n">
-        <v>795</v>
+        <v>650</v>
       </c>
       <c r="D154" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E154" t="n">
         <v>1</v>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G154" s="7" t="inlineStr">
         <is>
-          <t>Gladstone Street, Mold</t>
+          <t>Chester Road East, Shotton, Deeside</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>CH7</t>
+          <t>CH5</t>
         </is>
       </c>
       <c r="I154" t="n">
-        <v>905</v>
+        <v>474</v>
       </c>
       <c r="N154" t="n">
-        <v>1356</v>
+        <v>2016</v>
       </c>
       <c r="O154" t="n">
         <v>0</v>
       </c>
       <c r="Q154" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R154" t="inlineStr">
         <is>
-          <t>Reid and Roberts, Mold</t>
+          <t>Thomas Property Group, Chester</t>
         </is>
       </c>
       <c r="S154" s="7" t="inlineStr"/>
@@ -28212,14 +28269,14 @@
       <c r="V154" s="7" t="inlineStr"/>
       <c r="W154" t="inlineStr">
         <is>
-          <t>0fe090dd4efb58d6db540fc88a63048e9a1b679d</t>
+          <t>f80c03a584803371ab95595ae7a449a94715fbd1</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="B155" s="7" t="n"/>
       <c r="C155" s="18" t="n">
-        <v>1200</v>
+        <v>750</v>
       </c>
       <c r="D155" t="n">
         <v>2</v>
@@ -28229,36 +28286,33 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>semi_detached</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G155" s="7" t="inlineStr">
         <is>
-          <t>Llwyn Dinas Fechan, St. Asaph</t>
+          <t>Sycamore Terrace, Rhosrobin, Wrexham</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>LL17</t>
-        </is>
-      </c>
-      <c r="I155" t="n">
-        <v>710</v>
+          <t>LL11</t>
+        </is>
       </c>
       <c r="N155" t="n">
-        <v>248</v>
+        <v>1300</v>
       </c>
       <c r="O155" t="n">
         <v>0</v>
       </c>
       <c r="Q155" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R155" t="inlineStr">
         <is>
-          <t>Thomas Property Group, Chester</t>
+          <t>Bowen, Wrexham</t>
         </is>
       </c>
       <c r="S155" s="7" t="inlineStr"/>
@@ -28275,14 +28329,14 @@
       <c r="V155" s="7" t="inlineStr"/>
       <c r="W155" t="inlineStr">
         <is>
-          <t>01f8dda2f09c16566df7d00ae192327104586ec6</t>
+          <t>40274ada7dfa710e5054184216178477a704016c</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="B156" s="7" t="n"/>
       <c r="C156" s="18" t="n">
-        <v>700</v>
+        <v>900</v>
       </c>
       <c r="D156" t="n">
         <v>2</v>
@@ -28292,36 +28346,33 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>semi_detached</t>
         </is>
       </c>
       <c r="G156" s="7" t="inlineStr">
         <is>
-          <t>Central Drive, Shotton, Deeside</t>
+          <t>Kiln Close, Buckley, Flintshire, CH7</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>CH5</t>
-        </is>
-      </c>
-      <c r="I156" t="n">
-        <v>636</v>
+          <t>CH7</t>
+        </is>
       </c>
       <c r="N156" t="n">
-        <v>1924</v>
+        <v>936</v>
       </c>
       <c r="O156" t="n">
         <v>0</v>
       </c>
       <c r="Q156" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R156" t="inlineStr">
         <is>
-          <t>Reid and Roberts, Mold</t>
+          <t>William Gleave, Deeside</t>
         </is>
       </c>
       <c r="S156" s="7" t="inlineStr"/>
@@ -28338,50 +28389,50 @@
       <c r="V156" s="7" t="inlineStr"/>
       <c r="W156" t="inlineStr">
         <is>
-          <t>a8679975fd318f064c6646b7ec603ef505c73b91</t>
+          <t>780cbc2857d57b036f046702f312e0298790c096</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="B157" s="7" t="n"/>
       <c r="C157" s="18" t="n">
-        <v>850</v>
+        <v>900</v>
       </c>
       <c r="D157" t="n">
         <v>2</v>
       </c>
       <c r="E157" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G157" s="7" t="inlineStr">
         <is>
-          <t>Llys Y Ddol, Mold</t>
+          <t>9 Park Road, Ruthin</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>CH7</t>
+          <t>LL15</t>
         </is>
       </c>
       <c r="N157" t="n">
-        <v>1368</v>
+        <v>576</v>
       </c>
       <c r="O157" t="n">
         <v>0</v>
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R157" t="inlineStr">
         <is>
-          <t>Cavendish Rentals Ltd, Mold</t>
+          <t>Cavendish Rentals Ltd, Ruthin</t>
         </is>
       </c>
       <c r="S157" s="7" t="inlineStr"/>
@@ -28398,53 +28449,53 @@
       <c r="V157" s="7" t="inlineStr"/>
       <c r="W157" t="inlineStr">
         <is>
-          <t>454191bb7bc0e7fb7e64e3fd4f1802d398e2254c</t>
+          <t>c771916d30aebac19d1f346f767747d7b73a7d6c</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="B158" s="7" t="n"/>
       <c r="C158" s="18" t="n">
-        <v>1000</v>
+        <v>795</v>
       </c>
       <c r="D158" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E158" t="n">
         <v>1</v>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>semi_detached</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G158" s="7" t="inlineStr">
         <is>
-          <t>Mill View Road, Shotton, CH5</t>
+          <t>Gladstone Street, Mold</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>CH5</t>
+          <t>CH7</t>
         </is>
       </c>
       <c r="I158" t="n">
-        <v>1087</v>
+        <v>905</v>
       </c>
       <c r="N158" t="n">
-        <v>2236</v>
+        <v>1356</v>
       </c>
       <c r="O158" t="n">
         <v>0</v>
       </c>
       <c r="Q158" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R158" t="inlineStr">
         <is>
-          <t>Pinewood Estate Agency, Deeside</t>
+          <t>Reid and Roberts, Mold</t>
         </is>
       </c>
       <c r="S158" s="7" t="inlineStr"/>
@@ -28461,20 +28512,20 @@
       <c r="V158" s="7" t="inlineStr"/>
       <c r="W158" t="inlineStr">
         <is>
-          <t>709d3dbb0469602a30f2232c43318e1004ee28e3</t>
+          <t>0fe090dd4efb58d6db540fc88a63048e9a1b679d</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="B159" s="7" t="n"/>
       <c r="C159" s="18" t="n">
-        <v>1100</v>
+        <v>1200</v>
       </c>
       <c r="D159" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E159" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F159" t="inlineStr">
         <is>
@@ -28483,31 +28534,31 @@
       </c>
       <c r="G159" s="7" t="inlineStr">
         <is>
-          <t>Chestnut Way, Penyffordd, Chester</t>
+          <t>Llwyn Dinas Fechan, St. Asaph</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>CH4</t>
+          <t>LL17</t>
         </is>
       </c>
       <c r="I159" t="n">
-        <v>765</v>
+        <v>710</v>
       </c>
       <c r="N159" t="n">
-        <v>144</v>
+        <v>248</v>
       </c>
       <c r="O159" t="n">
         <v>0</v>
       </c>
       <c r="Q159" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R159" t="inlineStr">
         <is>
-          <t>Reid and Roberts, Mold</t>
+          <t>Thomas Property Group, Chester</t>
         </is>
       </c>
       <c r="S159" s="7" t="inlineStr"/>
@@ -28524,50 +28575,53 @@
       <c r="V159" s="7" t="inlineStr"/>
       <c r="W159" t="inlineStr">
         <is>
-          <t>0c6f7f5dcf9483acf81dd96394cb138955cd345f</t>
+          <t>01f8dda2f09c16566df7d00ae192327104586ec6</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="B160" s="7" t="n"/>
       <c r="C160" s="18" t="n">
-        <v>975</v>
+        <v>700</v>
       </c>
       <c r="D160" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E160" t="n">
         <v>1</v>
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>semi_detached</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G160" s="7" t="inlineStr">
         <is>
-          <t>Maes Offa, Trelawynd, Rhyl, Flintshire, LL18</t>
+          <t>Central Drive, Shotton, Deeside</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>LL18</t>
-        </is>
+          <t>CH5</t>
+        </is>
+      </c>
+      <c r="I160" t="n">
+        <v>636</v>
       </c>
       <c r="N160" t="n">
-        <v>32</v>
+        <v>1924</v>
       </c>
       <c r="O160" t="n">
         <v>0</v>
       </c>
       <c r="Q160" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="R160" t="inlineStr">
         <is>
-          <t>Monopoly, Denbigh</t>
+          <t>Reid and Roberts, Mold</t>
         </is>
       </c>
       <c r="S160" s="7" t="inlineStr"/>
@@ -28584,50 +28638,50 @@
       <c r="V160" s="7" t="inlineStr"/>
       <c r="W160" t="inlineStr">
         <is>
-          <t>7010522a251f536737688e6768df8c1ca7b26c26</t>
+          <t>a8679975fd318f064c6646b7ec603ef505c73b91</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="B161" s="7" t="n"/>
       <c r="C161" s="18" t="n">
-        <v>875</v>
+        <v>850</v>
       </c>
       <c r="D161" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E161" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>semi_detached</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G161" s="7" t="inlineStr">
         <is>
-          <t>Glan Y Don, Greenfield, Holywell, CH8 7HG</t>
+          <t>Llys Y Ddol, Mold</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>CH8</t>
+          <t>CH7</t>
         </is>
       </c>
       <c r="N161" t="n">
-        <v>540</v>
+        <v>1368</v>
       </c>
       <c r="O161" t="n">
         <v>0</v>
       </c>
       <c r="Q161" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="R161" t="inlineStr">
         <is>
-          <t>Visum, Nationwide</t>
+          <t>Cavendish Rentals Ltd, Mold</t>
         </is>
       </c>
       <c r="S161" s="7" t="inlineStr"/>
@@ -28644,26 +28698,29 @@
       <c r="V161" s="7" t="inlineStr"/>
       <c r="W161" t="inlineStr">
         <is>
-          <t>2de321765047d8487aaad5d86e92b523486e594c</t>
+          <t>454191bb7bc0e7fb7e64e3fd4f1802d398e2254c</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="B162" s="7" t="n"/>
       <c r="C162" s="18" t="n">
-        <v>725</v>
+        <v>1000</v>
       </c>
       <c r="D162" t="n">
+        <v>3</v>
+      </c>
+      <c r="E162" t="n">
         <v>1</v>
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>semi_detached</t>
         </is>
       </c>
       <c r="G162" s="7" t="inlineStr">
         <is>
-          <t>High Street, Connah's Quay, CH5</t>
+          <t>Mill View Road, Shotton, CH5</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
@@ -28671,15 +28728,18 @@
           <t>CH5</t>
         </is>
       </c>
+      <c r="I162" t="n">
+        <v>1087</v>
+      </c>
       <c r="N162" t="n">
-        <v>1904</v>
+        <v>2236</v>
       </c>
       <c r="O162" t="n">
         <v>0</v>
       </c>
       <c r="Q162" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="R162" t="inlineStr">
@@ -28701,50 +28761,53 @@
       <c r="V162" s="7" t="inlineStr"/>
       <c r="W162" t="inlineStr">
         <is>
-          <t>db6095b2965d70713395b1458e1bc20535687531</t>
+          <t>709d3dbb0469602a30f2232c43318e1004ee28e3</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="B163" s="7" t="n"/>
       <c r="C163" s="18" t="n">
-        <v>625</v>
+        <v>1100</v>
       </c>
       <c r="D163" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E163" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>semi_detached</t>
         </is>
       </c>
       <c r="G163" s="7" t="inlineStr">
         <is>
-          <t>Well Street, Holywell</t>
+          <t>Chestnut Way, Penyffordd, Chester</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>CH8</t>
-        </is>
+          <t>CH4</t>
+        </is>
+      </c>
+      <c r="I163" t="n">
+        <v>765</v>
       </c>
       <c r="N163" t="n">
-        <v>904</v>
+        <v>144</v>
       </c>
       <c r="O163" t="n">
         <v>0</v>
       </c>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="R163" t="inlineStr">
         <is>
-          <t>Cavendish Rentals Ltd, Mold</t>
+          <t>Reid and Roberts, Mold</t>
         </is>
       </c>
       <c r="S163" s="7" t="inlineStr"/>
@@ -28761,50 +28824,50 @@
       <c r="V163" s="7" t="inlineStr"/>
       <c r="W163" t="inlineStr">
         <is>
-          <t>2723b2ee048a058cfba581ae81cc808012ed35c5</t>
+          <t>0c6f7f5dcf9483acf81dd96394cb138955cd345f</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="B164" s="7" t="n"/>
       <c r="C164" s="18" t="n">
-        <v>900</v>
+        <v>975</v>
       </c>
       <c r="D164" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E164" t="n">
         <v>1</v>
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>semi_detached</t>
         </is>
       </c>
       <c r="G164" s="7" t="inlineStr">
         <is>
-          <t>Bryntirion Road, Bagillt, Flintshire, CH6</t>
+          <t>Maes Offa, Trelawynd, Rhyl, Flintshire, LL18</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>CH6</t>
+          <t>LL18</t>
         </is>
       </c>
       <c r="N164" t="n">
-        <v>200</v>
+        <v>32</v>
       </c>
       <c r="O164" t="n">
         <v>0</v>
       </c>
       <c r="Q164" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="R164" t="inlineStr">
         <is>
-          <t>William Gleave, Deeside</t>
+          <t>Monopoly, Denbigh</t>
         </is>
       </c>
       <c r="S164" s="7" t="inlineStr"/>
@@ -28821,20 +28884,20 @@
       <c r="V164" s="7" t="inlineStr"/>
       <c r="W164" t="inlineStr">
         <is>
-          <t>0c1595e8a037ae10970a3d68c03447fcb7c78d28</t>
+          <t>7010522a251f536737688e6768df8c1ca7b26c26</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="B165" s="7" t="n"/>
       <c r="C165" s="18" t="n">
-        <v>950</v>
+        <v>875</v>
       </c>
       <c r="D165" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E165" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F165" t="inlineStr">
         <is>
@@ -28843,7 +28906,7 @@
       </c>
       <c r="G165" s="7" t="inlineStr">
         <is>
-          <t>Rue St. Gregoire, Holywell, CH8</t>
+          <t>Glan Y Don, Greenfield, Holywell, CH8 7HG</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
@@ -28851,23 +28914,20 @@
           <t>CH8</t>
         </is>
       </c>
-      <c r="I165" t="n">
-        <v>657</v>
-      </c>
       <c r="N165" t="n">
-        <v>876</v>
+        <v>540</v>
       </c>
       <c r="O165" t="n">
         <v>0</v>
       </c>
       <c r="Q165" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="R165" t="inlineStr">
         <is>
-          <t>Currans, North Wales</t>
+          <t>Visum, Nationwide</t>
         </is>
       </c>
       <c r="S165" s="7" t="inlineStr"/>
@@ -28884,19 +28944,16 @@
       <c r="V165" s="7" t="inlineStr"/>
       <c r="W165" t="inlineStr">
         <is>
-          <t>dc3b6e39f27fc3549e5a88505b34a5efb8d772c4</t>
+          <t>2de321765047d8487aaad5d86e92b523486e594c</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="B166" s="7" t="n"/>
       <c r="C166" s="18" t="n">
-        <v>750</v>
+        <v>725</v>
       </c>
       <c r="D166" t="n">
-        <v>2</v>
-      </c>
-      <c r="E166" t="n">
         <v>1</v>
       </c>
       <c r="F166" t="inlineStr">
@@ -28906,28 +28963,28 @@
       </c>
       <c r="G166" s="7" t="inlineStr">
         <is>
-          <t>29 Tai Maes, Mold</t>
+          <t>High Street, Connah's Quay, CH5</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>CH7</t>
+          <t>CH5</t>
         </is>
       </c>
       <c r="N166" t="n">
-        <v>1356</v>
+        <v>1904</v>
       </c>
       <c r="O166" t="n">
         <v>0</v>
       </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="R166" t="inlineStr">
         <is>
-          <t>Cavendish Rentals Ltd, Mold</t>
+          <t>Pinewood Estate Agency, Deeside</t>
         </is>
       </c>
       <c r="S166" s="7" t="inlineStr"/>
@@ -28944,14 +29001,14 @@
       <c r="V166" s="7" t="inlineStr"/>
       <c r="W166" t="inlineStr">
         <is>
-          <t>e07eb711fdcf6d56ea28189fffc8e0176a5a3a88</t>
+          <t>db6095b2965d70713395b1458e1bc20535687531</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="B167" s="7" t="n"/>
       <c r="C167" s="18" t="n">
-        <v>600</v>
+        <v>625</v>
       </c>
       <c r="D167" t="n">
         <v>1</v>
@@ -28966,23 +29023,23 @@
       </c>
       <c r="G167" s="7" t="inlineStr">
         <is>
-          <t>St Marys Mews, Mold</t>
+          <t>Well Street, Holywell</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>CH7</t>
+          <t>CH8</t>
         </is>
       </c>
       <c r="N167" t="n">
-        <v>1372</v>
+        <v>904</v>
       </c>
       <c r="O167" t="n">
         <v>0</v>
       </c>
       <c r="Q167" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="R167" t="inlineStr">
@@ -29004,20 +29061,20 @@
       <c r="V167" s="7" t="inlineStr"/>
       <c r="W167" t="inlineStr">
         <is>
-          <t>af36d8744de8391ae981eb3d46fe462a829b50fc</t>
+          <t>2723b2ee048a058cfba581ae81cc808012ed35c5</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="B168" s="7" t="n"/>
       <c r="C168" s="18" t="n">
-        <v>875</v>
+        <v>900</v>
       </c>
       <c r="D168" t="n">
         <v>2</v>
       </c>
       <c r="E168" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F168" t="inlineStr">
         <is>
@@ -29026,28 +29083,28 @@
       </c>
       <c r="G168" s="7" t="inlineStr">
         <is>
-          <t>Castle Street, Caergwrle</t>
+          <t>Bryntirion Road, Bagillt, Flintshire, CH6</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>LL12</t>
+          <t>CH6</t>
         </is>
       </c>
       <c r="N168" t="n">
-        <v>264</v>
+        <v>200</v>
       </c>
       <c r="O168" t="n">
         <v>0</v>
       </c>
       <c r="Q168" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="R168" t="inlineStr">
         <is>
-          <t>Town &amp; Country Estate Agents, Wrexham</t>
+          <t>William Gleave, Deeside</t>
         </is>
       </c>
       <c r="S168" s="7" t="inlineStr"/>
@@ -29064,50 +29121,53 @@
       <c r="V168" s="7" t="inlineStr"/>
       <c r="W168" t="inlineStr">
         <is>
-          <t>64420bc3a588da08d4b7e360992c14bddef406b0</t>
+          <t>0c1595e8a037ae10970a3d68c03447fcb7c78d28</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="B169" s="7" t="n"/>
       <c r="C169" s="18" t="n">
-        <v>800</v>
+        <v>950</v>
       </c>
       <c r="D169" t="n">
         <v>2</v>
       </c>
       <c r="E169" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>semi_detached</t>
         </is>
       </c>
       <c r="G169" s="7" t="inlineStr">
         <is>
-          <t>Fagl Lane, Hope, LL12</t>
+          <t>Rue St. Gregoire, Holywell, CH8</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>LL12</t>
-        </is>
+          <t>CH8</t>
+        </is>
+      </c>
+      <c r="I169" t="n">
+        <v>657</v>
       </c>
       <c r="N169" t="n">
-        <v>244</v>
+        <v>876</v>
       </c>
       <c r="O169" t="n">
         <v>0</v>
       </c>
       <c r="Q169" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="R169" t="inlineStr">
         <is>
-          <t>Belvoir, Wrexham</t>
+          <t>Currans, North Wales</t>
         </is>
       </c>
       <c r="S169" s="7" t="inlineStr"/>
@@ -29124,17 +29184,17 @@
       <c r="V169" s="7" t="inlineStr"/>
       <c r="W169" t="inlineStr">
         <is>
-          <t>2e367fcb5325f10c32c7f8598ffffb977d48bccf</t>
+          <t>dc3b6e39f27fc3549e5a88505b34a5efb8d772c4</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="B170" s="7" t="n"/>
       <c r="C170" s="18" t="n">
-        <v>595</v>
+        <v>750</v>
       </c>
       <c r="D170" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E170" t="n">
         <v>1</v>
@@ -29146,28 +29206,28 @@
       </c>
       <c r="G170" s="7" t="inlineStr">
         <is>
-          <t>Ryeland Street, Deeside</t>
+          <t>29 Tai Maes, Mold</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>CH5</t>
+          <t>CH7</t>
         </is>
       </c>
       <c r="N170" t="n">
-        <v>2152</v>
+        <v>1356</v>
       </c>
       <c r="O170" t="n">
         <v>0</v>
       </c>
       <c r="Q170" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="R170" t="inlineStr">
         <is>
-          <t>Bowen, Wrexham</t>
+          <t>Cavendish Rentals Ltd, Mold</t>
         </is>
       </c>
       <c r="S170" s="7" t="inlineStr"/>
@@ -29184,17 +29244,17 @@
       <c r="V170" s="7" t="inlineStr"/>
       <c r="W170" t="inlineStr">
         <is>
-          <t>3502024b9ccf3c5846dbd8b2f4e5148495660759</t>
+          <t>e07eb711fdcf6d56ea28189fffc8e0176a5a3a88</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="B171" s="7" t="n"/>
       <c r="C171" s="18" t="n">
-        <v>750</v>
+        <v>600</v>
       </c>
       <c r="D171" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E171" t="n">
         <v>1</v>
@@ -29206,28 +29266,28 @@
       </c>
       <c r="G171" s="7" t="inlineStr">
         <is>
-          <t>High Street, Dyserth, LL18</t>
+          <t>St Marys Mews, Mold</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>LL18</t>
+          <t>CH7</t>
         </is>
       </c>
       <c r="N171" t="n">
-        <v>232</v>
+        <v>1372</v>
       </c>
       <c r="O171" t="n">
         <v>0</v>
       </c>
       <c r="Q171" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="R171" t="inlineStr">
         <is>
-          <t>Fifty North West, Chester</t>
+          <t>Cavendish Rentals Ltd, Mold</t>
         </is>
       </c>
       <c r="S171" s="7" t="inlineStr"/>
@@ -29244,50 +29304,50 @@
       <c r="V171" s="7" t="inlineStr"/>
       <c r="W171" t="inlineStr">
         <is>
-          <t>c2d205c9da5502fe82c6529faa7073858d43318b</t>
+          <t>af36d8744de8391ae981eb3d46fe462a829b50fc</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="B172" s="7" t="n"/>
       <c r="C172" s="18" t="n">
-        <v>900</v>
+        <v>875</v>
       </c>
       <c r="D172" t="n">
         <v>2</v>
       </c>
       <c r="E172" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G172" s="7" t="inlineStr">
         <is>
-          <t>Newmarket Road, Dyserth, LL18</t>
+          <t>Castle Street, Caergwrle</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>LL18</t>
+          <t>LL12</t>
         </is>
       </c>
       <c r="N172" t="n">
-        <v>328</v>
+        <v>264</v>
       </c>
       <c r="O172" t="n">
         <v>0</v>
       </c>
       <c r="Q172" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="R172" t="inlineStr">
         <is>
-          <t>Fifty North West, Chester</t>
+          <t>Town &amp; Country Estate Agents, Wrexham</t>
         </is>
       </c>
       <c r="S172" s="7" t="inlineStr"/>
@@ -29304,14 +29364,14 @@
       <c r="V172" s="7" t="inlineStr"/>
       <c r="W172" t="inlineStr">
         <is>
-          <t>8e3b047de4dea7640f383c9c16a3741e55ca202e</t>
+          <t>64420bc3a588da08d4b7e360992c14bddef406b0</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="B173" s="7" t="n"/>
       <c r="C173" s="18" t="n">
-        <v>795</v>
+        <v>800</v>
       </c>
       <c r="D173" t="n">
         <v>2</v>
@@ -29321,33 +29381,33 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G173" s="7" t="inlineStr">
         <is>
-          <t>Tower Terrace, Denbigh, Denbighshire, LL16</t>
+          <t>Fagl Lane, Hope, LL12</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>LL16</t>
+          <t>LL12</t>
         </is>
       </c>
       <c r="N173" t="n">
-        <v>940</v>
+        <v>244</v>
       </c>
       <c r="O173" t="n">
         <v>0</v>
       </c>
       <c r="Q173" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="R173" t="inlineStr">
         <is>
-          <t>Monopoly, Denbigh</t>
+          <t>Belvoir, Wrexham</t>
         </is>
       </c>
       <c r="S173" s="7" t="inlineStr"/>
@@ -29364,45 +29424,45 @@
       <c r="V173" s="7" t="inlineStr"/>
       <c r="W173" t="inlineStr">
         <is>
-          <t>a759cdaa8d9f724f2ecce2ccbf99e547c19fde5a</t>
+          <t>2e367fcb5325f10c32c7f8598ffffb977d48bccf</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="B174" s="7" t="n"/>
       <c r="C174" s="18" t="n">
-        <v>975</v>
+        <v>595</v>
       </c>
       <c r="D174" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E174" t="n">
         <v>1</v>
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G174" s="7" t="inlineStr">
         <is>
-          <t>Derby Road, Caergwrle, Wrexham</t>
+          <t>Ryeland Street, Deeside</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>LL12</t>
+          <t>CH5</t>
         </is>
       </c>
       <c r="N174" t="n">
-        <v>252</v>
+        <v>2152</v>
       </c>
       <c r="O174" t="n">
         <v>0</v>
       </c>
       <c r="Q174" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="R174" t="inlineStr">
@@ -29424,20 +29484,20 @@
       <c r="V174" s="7" t="inlineStr"/>
       <c r="W174" t="inlineStr">
         <is>
-          <t>9c715b658948566fb2a4a4b90c3c6b2f1f91a752</t>
+          <t>3502024b9ccf3c5846dbd8b2f4e5148495660759</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="B175" s="7" t="n"/>
       <c r="C175" s="18" t="n">
-        <v>985</v>
+        <v>750</v>
       </c>
       <c r="D175" t="n">
         <v>2</v>
       </c>
       <c r="E175" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F175" t="inlineStr">
         <is>
@@ -29446,28 +29506,28 @@
       </c>
       <c r="G175" s="7" t="inlineStr">
         <is>
-          <t>Livingstone Place, St. Asaph, LL17</t>
+          <t>High Street, Dyserth, LL18</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>LL17</t>
+          <t>LL18</t>
         </is>
       </c>
       <c r="N175" t="n">
-        <v>268</v>
+        <v>232</v>
       </c>
       <c r="O175" t="n">
         <v>0</v>
       </c>
       <c r="Q175" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="R175" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Fifty North West, Chester</t>
         </is>
       </c>
       <c r="S175" s="7" t="inlineStr"/>
@@ -29484,12 +29544,252 @@
       <c r="V175" s="7" t="inlineStr"/>
       <c r="W175" t="inlineStr">
         <is>
+          <t>c2d205c9da5502fe82c6529faa7073858d43318b</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="B176" s="7" t="n"/>
+      <c r="C176" s="18" t="n">
+        <v>900</v>
+      </c>
+      <c r="D176" t="n">
+        <v>2</v>
+      </c>
+      <c r="E176" t="n">
+        <v>1</v>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G176" s="7" t="inlineStr">
+        <is>
+          <t>Newmarket Road, Dyserth, LL18</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>LL18</t>
+        </is>
+      </c>
+      <c r="N176" t="n">
+        <v>328</v>
+      </c>
+      <c r="O176" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q176" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="R176" t="inlineStr">
+        <is>
+          <t>Fifty North West, Chester</t>
+        </is>
+      </c>
+      <c r="S176" s="7" t="inlineStr"/>
+      <c r="T176" s="14" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U176" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V176" s="7" t="inlineStr"/>
+      <c r="W176" t="inlineStr">
+        <is>
+          <t>8e3b047de4dea7640f383c9c16a3741e55ca202e</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="B177" s="7" t="n"/>
+      <c r="C177" s="18" t="n">
+        <v>795</v>
+      </c>
+      <c r="D177" t="n">
+        <v>2</v>
+      </c>
+      <c r="E177" t="n">
+        <v>1</v>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>terraced</t>
+        </is>
+      </c>
+      <c r="G177" s="7" t="inlineStr">
+        <is>
+          <t>Tower Terrace, Denbigh, Denbighshire, LL16</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>LL16</t>
+        </is>
+      </c>
+      <c r="N177" t="n">
+        <v>940</v>
+      </c>
+      <c r="O177" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="R177" t="inlineStr">
+        <is>
+          <t>Monopoly, Denbigh</t>
+        </is>
+      </c>
+      <c r="S177" s="7" t="inlineStr"/>
+      <c r="T177" s="14" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U177" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V177" s="7" t="inlineStr"/>
+      <c r="W177" t="inlineStr">
+        <is>
+          <t>a759cdaa8d9f724f2ecce2ccbf99e547c19fde5a</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="B178" s="7" t="n"/>
+      <c r="C178" s="18" t="n">
+        <v>975</v>
+      </c>
+      <c r="D178" t="n">
+        <v>3</v>
+      </c>
+      <c r="E178" t="n">
+        <v>1</v>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>terraced</t>
+        </is>
+      </c>
+      <c r="G178" s="7" t="inlineStr">
+        <is>
+          <t>Derby Road, Caergwrle, Wrexham</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>LL12</t>
+        </is>
+      </c>
+      <c r="N178" t="n">
+        <v>252</v>
+      </c>
+      <c r="O178" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q178" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="R178" t="inlineStr">
+        <is>
+          <t>Bowen, Wrexham</t>
+        </is>
+      </c>
+      <c r="S178" s="7" t="inlineStr"/>
+      <c r="T178" s="14" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U178" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V178" s="7" t="inlineStr"/>
+      <c r="W178" t="inlineStr">
+        <is>
+          <t>9c715b658948566fb2a4a4b90c3c6b2f1f91a752</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="B179" s="7" t="n"/>
+      <c r="C179" s="18" t="n">
+        <v>985</v>
+      </c>
+      <c r="D179" t="n">
+        <v>2</v>
+      </c>
+      <c r="E179" t="n">
+        <v>2</v>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G179" s="7" t="inlineStr">
+        <is>
+          <t>Livingstone Place, St. Asaph, LL17</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>LL17</t>
+        </is>
+      </c>
+      <c r="N179" t="n">
+        <v>268</v>
+      </c>
+      <c r="O179" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q179" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="R179" t="inlineStr">
+        <is>
+          <t>OpenRent, London</t>
+        </is>
+      </c>
+      <c r="S179" s="7" t="inlineStr"/>
+      <c r="T179" s="14" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U179" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V179" s="7" t="inlineStr"/>
+      <c r="W179" t="inlineStr">
+        <is>
           <t>b0ba112a09e1577fca8332db332a7e1693926a4e</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W175"/>
+  <autoFilter ref="A1:W179"/>
   <dataValidations count="1">
     <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199 U200 U201 U202 U203 U204 U205 U206 U207 U208 U209 U210 U211 U212" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
@@ -29670,6 +29970,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T173" r:id="rId172"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T174" r:id="rId173"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T175" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T176" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T177" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T178" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T179" r:id="rId178"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
House search data from run 17
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -17326,7 +17326,7 @@
       <c r="L6" s="8" t="n"/>
       <c r="M6" s="8" t="n"/>
       <c r="N6" s="8" t="n">
-        <v>21616</v>
+        <v>21660</v>
       </c>
       <c r="O6" s="8" t="n">
         <v>0</v>
@@ -20772,10 +20772,10 @@
         </is>
       </c>
       <c r="C51" s="17" t="n">
-        <v>1600</v>
+        <v>1300</v>
       </c>
       <c r="D51" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E51" s="8" t="n">
         <v>1</v>
@@ -20787,12 +20787,12 @@
       </c>
       <c r="G51" s="9" t="inlineStr">
         <is>
-          <t>Stapleton Road, Bristol, BS5</t>
+          <t>Hamilton Court - City Centre</t>
         </is>
       </c>
       <c r="H51" s="8" t="inlineStr">
         <is>
-          <t>BS5</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I51" s="8" t="n"/>
@@ -20801,7 +20801,7 @@
       <c r="L51" s="8" t="n"/>
       <c r="M51" s="8" t="n"/>
       <c r="N51" s="8" t="n">
-        <v>19576</v>
+        <v>21616</v>
       </c>
       <c r="O51" s="8" t="n">
         <v>0</v>
@@ -20809,12 +20809,12 @@
       <c r="P51" s="8" t="n"/>
       <c r="Q51" s="8" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R51" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Ocean, Clifton</t>
         </is>
       </c>
       <c r="S51" s="9" t="inlineStr"/>
@@ -20831,7 +20831,7 @@
       <c r="V51" s="7" t="inlineStr"/>
       <c r="W51" s="8" t="inlineStr">
         <is>
-          <t>2c4d3b36f040dfa0e294ad99ce0d43b5fa15d6c8</t>
+          <t>8bd3f395f80d9e75d404d499c9b227ed567374e3</t>
         </is>
       </c>
     </row>
@@ -20845,10 +20845,10 @@
         </is>
       </c>
       <c r="C52" s="17" t="n">
-        <v>1300</v>
+        <v>2200</v>
       </c>
       <c r="D52" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E52" s="8" t="n">
         <v>1</v>
@@ -20860,7 +20860,7 @@
       </c>
       <c r="G52" s="9" t="inlineStr">
         <is>
-          <t>Hamilton Court - City Centre</t>
+          <t>Castle Park View, Castle Street, Bristol</t>
         </is>
       </c>
       <c r="H52" s="8" t="inlineStr">
@@ -20874,7 +20874,7 @@
       <c r="L52" s="8" t="n"/>
       <c r="M52" s="8" t="n"/>
       <c r="N52" s="8" t="n">
-        <v>21616</v>
+        <v>21984</v>
       </c>
       <c r="O52" s="8" t="n">
         <v>0</v>
@@ -20882,12 +20882,12 @@
       <c r="P52" s="8" t="n"/>
       <c r="Q52" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="R52" s="8" t="inlineStr">
         <is>
-          <t>Ocean, Clifton</t>
+          <t>Savills Lettings, CPV</t>
         </is>
       </c>
       <c r="S52" s="9" t="inlineStr"/>
@@ -20904,7 +20904,7 @@
       <c r="V52" s="7" t="inlineStr"/>
       <c r="W52" s="8" t="inlineStr">
         <is>
-          <t>8bd3f395f80d9e75d404d499c9b227ed567374e3</t>
+          <t>406fab2577557efdd9382cee302acdc7a788c3d8</t>
         </is>
       </c>
     </row>
@@ -20918,13 +20918,13 @@
         </is>
       </c>
       <c r="C53" s="17" t="n">
-        <v>2200</v>
+        <v>2300</v>
       </c>
       <c r="D53" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E53" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F53" s="8" t="inlineStr">
         <is>
@@ -20941,7 +20941,9 @@
           <t>BS2</t>
         </is>
       </c>
-      <c r="I53" s="8" t="n"/>
+      <c r="I53" s="8" t="n">
+        <v>757</v>
+      </c>
       <c r="J53" s="8" t="n"/>
       <c r="K53" s="8" t="n"/>
       <c r="L53" s="8" t="n"/>
@@ -20977,7 +20979,7 @@
       <c r="V53" s="7" t="inlineStr"/>
       <c r="W53" s="8" t="inlineStr">
         <is>
-          <t>406fab2577557efdd9382cee302acdc7a788c3d8</t>
+          <t>82dded0955660a8ec4af3acb8db470436bdc522b</t>
         </is>
       </c>
     </row>
@@ -21006,7 +21008,7 @@
       </c>
       <c r="G54" s="9" t="inlineStr">
         <is>
-          <t>Castle Park View, Castle Street, Bristol</t>
+          <t>Castle Park View, Castle Street, Bristol, BS2 0ND</t>
         </is>
       </c>
       <c r="H54" s="8" t="inlineStr">
@@ -21050,7 +21052,7 @@
       <c r="V54" s="7" t="inlineStr"/>
       <c r="W54" s="8" t="inlineStr">
         <is>
-          <t>82dded0955660a8ec4af3acb8db470436bdc522b</t>
+          <t>fc4abec405a6b435cb290523f6e7784fc2de1099</t>
         </is>
       </c>
     </row>
@@ -21064,13 +21066,13 @@
         </is>
       </c>
       <c r="C55" s="17" t="n">
-        <v>2300</v>
+        <v>2095</v>
       </c>
       <c r="D55" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E55" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F55" s="8" t="inlineStr">
         <is>
@@ -21079,7 +21081,7 @@
       </c>
       <c r="G55" s="9" t="inlineStr">
         <is>
-          <t>Castle Park View, Castle Street, Bristol, BS2 0ND</t>
+          <t>Castle Park View, Castle Street, BS2 0ND, Bristol</t>
         </is>
       </c>
       <c r="H55" s="8" t="inlineStr">
@@ -21123,7 +21125,7 @@
       <c r="V55" s="7" t="inlineStr"/>
       <c r="W55" s="8" t="inlineStr">
         <is>
-          <t>fc4abec405a6b435cb290523f6e7784fc2de1099</t>
+          <t>7a4bff96a8fb36d99cc3d7825e84bee85f8c5ba7</t>
         </is>
       </c>
     </row>
@@ -21137,10 +21139,10 @@
         </is>
       </c>
       <c r="C56" s="17" t="n">
-        <v>2095</v>
+        <v>1400</v>
       </c>
       <c r="D56" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E56" s="8" t="n">
         <v>1</v>
@@ -21152,12 +21154,12 @@
       </c>
       <c r="G56" s="9" t="inlineStr">
         <is>
-          <t>Castle Park View, Castle Street, BS2 0ND, Bristol</t>
+          <t>Jessop Court Ferry Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H56" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I56" s="8" t="n"/>
@@ -21166,7 +21168,7 @@
       <c r="L56" s="8" t="n"/>
       <c r="M56" s="8" t="n"/>
       <c r="N56" s="8" t="n">
-        <v>21984</v>
+        <v>20908</v>
       </c>
       <c r="O56" s="8" t="n">
         <v>0</v>
@@ -21174,12 +21176,12 @@
       <c r="P56" s="8" t="n"/>
       <c r="Q56" s="8" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="R56" s="8" t="inlineStr">
         <is>
-          <t>Savills Lettings, CPV</t>
+          <t>Accommodation Unlimited, Bristol</t>
         </is>
       </c>
       <c r="S56" s="9" t="inlineStr"/>
@@ -21196,7 +21198,7 @@
       <c r="V56" s="7" t="inlineStr"/>
       <c r="W56" s="8" t="inlineStr">
         <is>
-          <t>7a4bff96a8fb36d99cc3d7825e84bee85f8c5ba7</t>
+          <t>45f17f505657c6333c92b921a50f7641e02f2c2f</t>
         </is>
       </c>
     </row>
@@ -21210,10 +21212,10 @@
         </is>
       </c>
       <c r="C57" s="17" t="n">
-        <v>1400</v>
+        <v>1500</v>
       </c>
       <c r="D57" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E57" s="8" t="n">
         <v>1</v>
@@ -21225,12 +21227,12 @@
       </c>
       <c r="G57" s="9" t="inlineStr">
         <is>
-          <t>Jessop Court Ferry Street, Bristol, BS1</t>
+          <t>St Clements Court, Wilson Street, Bristol</t>
         </is>
       </c>
       <c r="H57" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I57" s="8" t="n"/>
@@ -21239,7 +21241,7 @@
       <c r="L57" s="8" t="n"/>
       <c r="M57" s="8" t="n"/>
       <c r="N57" s="8" t="n">
-        <v>20908</v>
+        <v>21600</v>
       </c>
       <c r="O57" s="8" t="n">
         <v>0</v>
@@ -21247,12 +21249,12 @@
       <c r="P57" s="8" t="n"/>
       <c r="Q57" s="8" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="R57" s="8" t="inlineStr">
         <is>
-          <t>Accommodation Unlimited, Bristol</t>
+          <t>Kendall Harper, Bishopston</t>
         </is>
       </c>
       <c r="S57" s="9" t="inlineStr"/>
@@ -21269,7 +21271,7 @@
       <c r="V57" s="7" t="inlineStr"/>
       <c r="W57" s="8" t="inlineStr">
         <is>
-          <t>45f17f505657c6333c92b921a50f7641e02f2c2f</t>
+          <t>b3bf3a18fe9e3595ef643379d979e59ee826fcbc</t>
         </is>
       </c>
     </row>
@@ -21283,7 +21285,7 @@
         </is>
       </c>
       <c r="C58" s="17" t="n">
-        <v>1500</v>
+        <v>1600</v>
       </c>
       <c r="D58" s="8" t="n">
         <v>2</v>
@@ -21298,7 +21300,7 @@
       </c>
       <c r="G58" s="9" t="inlineStr">
         <is>
-          <t>St Clements Court, Wilson Street, Bristol</t>
+          <t>Waterloo Road, Midland Mews, BS2</t>
         </is>
       </c>
       <c r="H58" s="8" t="inlineStr">
@@ -21306,13 +21308,15 @@
           <t>BS2</t>
         </is>
       </c>
-      <c r="I58" s="8" t="n"/>
+      <c r="I58" s="8" t="n">
+        <v>721</v>
+      </c>
       <c r="J58" s="8" t="n"/>
       <c r="K58" s="8" t="n"/>
       <c r="L58" s="8" t="n"/>
       <c r="M58" s="8" t="n"/>
       <c r="N58" s="8" t="n">
-        <v>21600</v>
+        <v>20856</v>
       </c>
       <c r="O58" s="8" t="n">
         <v>0</v>
@@ -21320,12 +21324,12 @@
       <c r="P58" s="8" t="n"/>
       <c r="Q58" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R58" s="8" t="inlineStr">
         <is>
-          <t>Kendall Harper, Bishopston</t>
+          <t>Acen Properties, Bristol</t>
         </is>
       </c>
       <c r="S58" s="9" t="inlineStr"/>
@@ -21342,7 +21346,7 @@
       <c r="V58" s="7" t="inlineStr"/>
       <c r="W58" s="8" t="inlineStr">
         <is>
-          <t>b3bf3a18fe9e3595ef643379d979e59ee826fcbc</t>
+          <t>cf8a979c7c13e868d74a6828d64c93a46d2e7209</t>
         </is>
       </c>
     </row>
@@ -21356,13 +21360,13 @@
         </is>
       </c>
       <c r="C59" s="17" t="n">
-        <v>1600</v>
+        <v>2085</v>
       </c>
       <c r="D59" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E59" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F59" s="8" t="inlineStr">
         <is>
@@ -21371,23 +21375,23 @@
       </c>
       <c r="G59" s="9" t="inlineStr">
         <is>
-          <t>Waterloo Road, Midland Mews, BS2</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H59" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I59" s="8" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="J59" s="8" t="n"/>
       <c r="K59" s="8" t="n"/>
       <c r="L59" s="8" t="n"/>
       <c r="M59" s="8" t="n"/>
       <c r="N59" s="8" t="n">
-        <v>20856</v>
+        <v>21504</v>
       </c>
       <c r="O59" s="8" t="n">
         <v>0</v>
@@ -21395,12 +21399,12 @@
       <c r="P59" s="8" t="n"/>
       <c r="Q59" s="8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="R59" s="8" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S59" s="9" t="inlineStr"/>
@@ -21417,7 +21421,7 @@
       <c r="V59" s="7" t="inlineStr"/>
       <c r="W59" s="8" t="inlineStr">
         <is>
-          <t>cf8a979c7c13e868d74a6828d64c93a46d2e7209</t>
+          <t>12a5f2c4f1be2a8f1a9b2c6cbe66191abf1d7975</t>
         </is>
       </c>
     </row>
@@ -21431,13 +21435,13 @@
         </is>
       </c>
       <c r="C60" s="17" t="n">
-        <v>2085</v>
+        <v>1640</v>
       </c>
       <c r="D60" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E60" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
@@ -21446,7 +21450,7 @@
       </c>
       <c r="G60" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H60" s="8" t="inlineStr">
@@ -21455,14 +21459,14 @@
         </is>
       </c>
       <c r="I60" s="8" t="n">
-        <v>722</v>
+        <v>570</v>
       </c>
       <c r="J60" s="8" t="n"/>
       <c r="K60" s="8" t="n"/>
       <c r="L60" s="8" t="n"/>
       <c r="M60" s="8" t="n"/>
       <c r="N60" s="8" t="n">
-        <v>21504</v>
+        <v>20820</v>
       </c>
       <c r="O60" s="8" t="n">
         <v>0</v>
@@ -21475,7 +21479,7 @@
       </c>
       <c r="R60" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S60" s="9" t="inlineStr"/>
@@ -21492,7 +21496,7 @@
       <c r="V60" s="7" t="inlineStr"/>
       <c r="W60" s="8" t="inlineStr">
         <is>
-          <t>12a5f2c4f1be2a8f1a9b2c6cbe66191abf1d7975</t>
+          <t>f7afd1bbb106a22d180a78614dde509c1dbfa8c1</t>
         </is>
       </c>
     </row>
@@ -21506,10 +21510,10 @@
         </is>
       </c>
       <c r="C61" s="17" t="n">
-        <v>1640</v>
+        <v>1500</v>
       </c>
       <c r="D61" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E61" s="8" t="n">
         <v>1</v>
@@ -21521,23 +21525,21 @@
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Midland Mews Waterloo Road Old Market, Bristol, BS2</t>
         </is>
       </c>
       <c r="H61" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I61" s="8" t="n">
-        <v>570</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I61" s="8" t="n"/>
       <c r="J61" s="8" t="n"/>
       <c r="K61" s="8" t="n"/>
       <c r="L61" s="8" t="n"/>
       <c r="M61" s="8" t="n"/>
       <c r="N61" s="8" t="n">
-        <v>20820</v>
+        <v>20856</v>
       </c>
       <c r="O61" s="8" t="n">
         <v>0</v>
@@ -21550,7 +21552,7 @@
       </c>
       <c r="R61" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Accommodation Unlimited, Bristol</t>
         </is>
       </c>
       <c r="S61" s="9" t="inlineStr"/>
@@ -21567,7 +21569,7 @@
       <c r="V61" s="7" t="inlineStr"/>
       <c r="W61" s="8" t="inlineStr">
         <is>
-          <t>f7afd1bbb106a22d180a78614dde509c1dbfa8c1</t>
+          <t>f83555c1dc6f03087d999787a76db9b49794ddb4</t>
         </is>
       </c>
     </row>
@@ -21581,10 +21583,10 @@
         </is>
       </c>
       <c r="C62" s="17" t="n">
-        <v>1500</v>
+        <v>1300</v>
       </c>
       <c r="D62" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E62" s="8" t="n">
         <v>1</v>
@@ -21596,21 +21598,23 @@
       </c>
       <c r="G62" s="9" t="inlineStr">
         <is>
-          <t>Midland Mews Waterloo Road Old Market, Bristol, BS2</t>
+          <t>City Centre, Queen Square Apartments, BS1</t>
         </is>
       </c>
       <c r="H62" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I62" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I62" s="8" t="n">
+        <v>405</v>
+      </c>
       <c r="J62" s="8" t="n"/>
       <c r="K62" s="8" t="n"/>
       <c r="L62" s="8" t="n"/>
       <c r="M62" s="8" t="n"/>
       <c r="N62" s="8" t="n">
-        <v>20856</v>
+        <v>20316</v>
       </c>
       <c r="O62" s="8" t="n">
         <v>0</v>
@@ -21623,7 +21627,7 @@
       </c>
       <c r="R62" s="8" t="inlineStr">
         <is>
-          <t>Accommodation Unlimited, Bristol</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S62" s="9" t="inlineStr"/>
@@ -21640,7 +21644,7 @@
       <c r="V62" s="7" t="inlineStr"/>
       <c r="W62" s="8" t="inlineStr">
         <is>
-          <t>f83555c1dc6f03087d999787a76db9b49794ddb4</t>
+          <t>9ad2c7bc90885b9a9e65b462b952842a964f1d35</t>
         </is>
       </c>
     </row>
@@ -21654,13 +21658,13 @@
         </is>
       </c>
       <c r="C63" s="17" t="n">
-        <v>1300</v>
+        <v>2020</v>
       </c>
       <c r="D63" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E63" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F63" s="8" t="inlineStr">
         <is>
@@ -21669,7 +21673,7 @@
       </c>
       <c r="G63" s="9" t="inlineStr">
         <is>
-          <t>City Centre, Queen Square Apartments, BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H63" s="8" t="inlineStr">
@@ -21678,14 +21682,14 @@
         </is>
       </c>
       <c r="I63" s="8" t="n">
-        <v>405</v>
+        <v>764</v>
       </c>
       <c r="J63" s="8" t="n"/>
       <c r="K63" s="8" t="n"/>
       <c r="L63" s="8" t="n"/>
       <c r="M63" s="8" t="n"/>
       <c r="N63" s="8" t="n">
-        <v>20316</v>
+        <v>20856</v>
       </c>
       <c r="O63" s="8" t="n">
         <v>0</v>
@@ -21693,12 +21697,12 @@
       <c r="P63" s="8" t="n"/>
       <c r="Q63" s="8" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="R63" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S63" s="9" t="inlineStr"/>
@@ -21715,7 +21719,7 @@
       <c r="V63" s="7" t="inlineStr"/>
       <c r="W63" s="8" t="inlineStr">
         <is>
-          <t>9ad2c7bc90885b9a9e65b462b952842a964f1d35</t>
+          <t>6140b74b7d83ae5918fdabb6f9371e2f4b63a9c2</t>
         </is>
       </c>
     </row>
@@ -21729,7 +21733,7 @@
         </is>
       </c>
       <c r="C64" s="17" t="n">
-        <v>2020</v>
+        <v>2145</v>
       </c>
       <c r="D64" s="8" t="n">
         <v>2</v>
@@ -21744,7 +21748,7 @@
       </c>
       <c r="G64" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H64" s="8" t="inlineStr">
@@ -21753,14 +21757,14 @@
         </is>
       </c>
       <c r="I64" s="8" t="n">
-        <v>764</v>
+        <v>815</v>
       </c>
       <c r="J64" s="8" t="n"/>
       <c r="K64" s="8" t="n"/>
       <c r="L64" s="8" t="n"/>
       <c r="M64" s="8" t="n"/>
       <c r="N64" s="8" t="n">
-        <v>20856</v>
+        <v>21504</v>
       </c>
       <c r="O64" s="8" t="n">
         <v>0</v>
@@ -21773,7 +21777,7 @@
       </c>
       <c r="R64" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S64" s="9" t="inlineStr"/>
@@ -21790,7 +21794,7 @@
       <c r="V64" s="7" t="inlineStr"/>
       <c r="W64" s="8" t="inlineStr">
         <is>
-          <t>6140b74b7d83ae5918fdabb6f9371e2f4b63a9c2</t>
+          <t>24009eb3414633bf24b3b69631ba405866a1e5c9</t>
         </is>
       </c>
     </row>
@@ -21804,13 +21808,13 @@
         </is>
       </c>
       <c r="C65" s="17" t="n">
-        <v>2145</v>
+        <v>1635</v>
       </c>
       <c r="D65" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E65" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F65" s="8" t="inlineStr">
         <is>
@@ -21819,7 +21823,7 @@
       </c>
       <c r="G65" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H65" s="8" t="inlineStr">
@@ -21828,7 +21832,7 @@
         </is>
       </c>
       <c r="I65" s="8" t="n">
-        <v>815</v>
+        <v>486</v>
       </c>
       <c r="J65" s="8" t="n"/>
       <c r="K65" s="8" t="n"/>
@@ -21848,7 +21852,7 @@
       </c>
       <c r="R65" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S65" s="9" t="inlineStr"/>
@@ -21865,7 +21869,7 @@
       <c r="V65" s="7" t="inlineStr"/>
       <c r="W65" s="8" t="inlineStr">
         <is>
-          <t>24009eb3414633bf24b3b69631ba405866a1e5c9</t>
+          <t>bbf6e42784b6e4b7dae8d6bef9900115d0f3056e</t>
         </is>
       </c>
     </row>
@@ -21879,13 +21883,13 @@
         </is>
       </c>
       <c r="C66" s="17" t="n">
-        <v>1635</v>
+        <v>1750</v>
       </c>
       <c r="D66" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E66" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F66" s="8" t="inlineStr">
         <is>
@@ -21894,23 +21898,23 @@
       </c>
       <c r="G66" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Arnos Vale, Paintworks, BS4</t>
         </is>
       </c>
       <c r="H66" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS4</t>
         </is>
       </c>
       <c r="I66" s="8" t="n">
-        <v>486</v>
+        <v>731</v>
       </c>
       <c r="J66" s="8" t="n"/>
       <c r="K66" s="8" t="n"/>
       <c r="L66" s="8" t="n"/>
       <c r="M66" s="8" t="n"/>
       <c r="N66" s="8" t="n">
-        <v>21504</v>
+        <v>4680</v>
       </c>
       <c r="O66" s="8" t="n">
         <v>0</v>
@@ -21923,7 +21927,7 @@
       </c>
       <c r="R66" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S66" s="9" t="inlineStr"/>
@@ -21940,7 +21944,7 @@
       <c r="V66" s="7" t="inlineStr"/>
       <c r="W66" s="8" t="inlineStr">
         <is>
-          <t>bbf6e42784b6e4b7dae8d6bef9900115d0f3056e</t>
+          <t>1c0acc4cbbc0f239d4843e9eb56c0d04ca3a6278</t>
         </is>
       </c>
     </row>
@@ -21954,13 +21958,13 @@
         </is>
       </c>
       <c r="C67" s="17" t="n">
-        <v>1750</v>
+        <v>2100</v>
       </c>
       <c r="D67" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E67" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F67" s="8" t="inlineStr">
         <is>
@@ -21969,23 +21973,21 @@
       </c>
       <c r="G67" s="9" t="inlineStr">
         <is>
-          <t>Arnos Vale, Paintworks, BS4</t>
+          <t>Baldwin St, Bristol, BS1</t>
         </is>
       </c>
       <c r="H67" s="8" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I67" s="8" t="n">
-        <v>731</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I67" s="8" t="n"/>
       <c r="J67" s="8" t="n"/>
       <c r="K67" s="8" t="n"/>
       <c r="L67" s="8" t="n"/>
       <c r="M67" s="8" t="n"/>
       <c r="N67" s="8" t="n">
-        <v>4680</v>
+        <v>21148</v>
       </c>
       <c r="O67" s="8" t="n">
         <v>0</v>
@@ -21993,12 +21995,12 @@
       <c r="P67" s="8" t="n"/>
       <c r="Q67" s="8" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R67" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S67" s="9" t="inlineStr"/>
@@ -22015,7 +22017,7 @@
       <c r="V67" s="7" t="inlineStr"/>
       <c r="W67" s="8" t="inlineStr">
         <is>
-          <t>1c0acc4cbbc0f239d4843e9eb56c0d04ca3a6278</t>
+          <t>ba1c1abaa5dbfd6e19c20fa9df1e66799d9c2462</t>
         </is>
       </c>
     </row>
@@ -22029,13 +22031,13 @@
         </is>
       </c>
       <c r="C68" s="17" t="n">
-        <v>2100</v>
+        <v>2220</v>
       </c>
       <c r="D68" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E68" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
@@ -22044,7 +22046,7 @@
       </c>
       <c r="G68" s="9" t="inlineStr">
         <is>
-          <t>Baldwin St, Bristol, BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H68" s="8" t="inlineStr">
@@ -22052,13 +22054,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I68" s="8" t="n"/>
+      <c r="I68" s="8" t="n">
+        <v>697</v>
+      </c>
       <c r="J68" s="8" t="n"/>
       <c r="K68" s="8" t="n"/>
       <c r="L68" s="8" t="n"/>
       <c r="M68" s="8" t="n"/>
       <c r="N68" s="8" t="n">
-        <v>21148</v>
+        <v>20820</v>
       </c>
       <c r="O68" s="8" t="n">
         <v>0</v>
@@ -22071,7 +22075,7 @@
       </c>
       <c r="R68" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S68" s="9" t="inlineStr"/>
@@ -22088,7 +22092,7 @@
       <c r="V68" s="7" t="inlineStr"/>
       <c r="W68" s="8" t="inlineStr">
         <is>
-          <t>ba1c1abaa5dbfd6e19c20fa9df1e66799d9c2462</t>
+          <t>5870266ee1b15bf20f0a085f56358c762e522fa8</t>
         </is>
       </c>
     </row>
@@ -22102,13 +22106,13 @@
         </is>
       </c>
       <c r="C69" s="17" t="n">
-        <v>2220</v>
+        <v>1300</v>
       </c>
       <c r="D69" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E69" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F69" s="8" t="inlineStr">
         <is>
@@ -22117,7 +22121,7 @@
       </c>
       <c r="G69" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Bristol City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H69" s="8" t="inlineStr">
@@ -22125,15 +22129,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I69" s="8" t="n">
-        <v>697</v>
-      </c>
+      <c r="I69" s="8" t="n"/>
       <c r="J69" s="8" t="n"/>
       <c r="K69" s="8" t="n"/>
       <c r="L69" s="8" t="n"/>
       <c r="M69" s="8" t="n"/>
       <c r="N69" s="8" t="n">
-        <v>20820</v>
+        <v>21428</v>
       </c>
       <c r="O69" s="8" t="n">
         <v>0</v>
@@ -22141,12 +22143,12 @@
       <c r="P69" s="8" t="n"/>
       <c r="Q69" s="8" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="R69" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S69" s="9" t="inlineStr"/>
@@ -22163,7 +22165,7 @@
       <c r="V69" s="7" t="inlineStr"/>
       <c r="W69" s="8" t="inlineStr">
         <is>
-          <t>5870266ee1b15bf20f0a085f56358c762e522fa8</t>
+          <t>317e9ab29cad2381c41672743d877feba2c14e45</t>
         </is>
       </c>
     </row>
@@ -22177,7 +22179,7 @@
         </is>
       </c>
       <c r="C70" s="17" t="n">
-        <v>1300</v>
+        <v>1500</v>
       </c>
       <c r="D70" s="8" t="n">
         <v>1</v>
@@ -22192,7 +22194,7 @@
       </c>
       <c r="G70" s="9" t="inlineStr">
         <is>
-          <t>Bristol City Centre, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H70" s="8" t="inlineStr">
@@ -22200,13 +22202,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I70" s="8" t="n"/>
+      <c r="I70" s="8" t="n">
+        <v>548</v>
+      </c>
       <c r="J70" s="8" t="n"/>
       <c r="K70" s="8" t="n"/>
       <c r="L70" s="8" t="n"/>
       <c r="M70" s="8" t="n"/>
       <c r="N70" s="8" t="n">
-        <v>21428</v>
+        <v>21504</v>
       </c>
       <c r="O70" s="8" t="n">
         <v>0</v>
@@ -22214,12 +22218,12 @@
       <c r="P70" s="8" t="n"/>
       <c r="Q70" s="8" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R70" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S70" s="9" t="inlineStr"/>
@@ -22236,7 +22240,7 @@
       <c r="V70" s="7" t="inlineStr"/>
       <c r="W70" s="8" t="inlineStr">
         <is>
-          <t>317e9ab29cad2381c41672743d877feba2c14e45</t>
+          <t>bad1e4584285201ef9995d2b437343fca870009c</t>
         </is>
       </c>
     </row>
@@ -22250,7 +22254,7 @@
         </is>
       </c>
       <c r="C71" s="17" t="n">
-        <v>1500</v>
+        <v>1615</v>
       </c>
       <c r="D71" s="8" t="n">
         <v>1</v>
@@ -22265,7 +22269,7 @@
       </c>
       <c r="G71" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H71" s="8" t="inlineStr">
@@ -22274,7 +22278,7 @@
         </is>
       </c>
       <c r="I71" s="8" t="n">
-        <v>548</v>
+        <v>486</v>
       </c>
       <c r="J71" s="8" t="n"/>
       <c r="K71" s="8" t="n"/>
@@ -22294,7 +22298,7 @@
       </c>
       <c r="R71" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S71" s="9" t="inlineStr"/>
@@ -22311,7 +22315,7 @@
       <c r="V71" s="7" t="inlineStr"/>
       <c r="W71" s="8" t="inlineStr">
         <is>
-          <t>bad1e4584285201ef9995d2b437343fca870009c</t>
+          <t>67ff71428df47b0eb7f7da47600378ffdad1f97c</t>
         </is>
       </c>
     </row>
@@ -22325,10 +22329,10 @@
         </is>
       </c>
       <c r="C72" s="17" t="n">
-        <v>1615</v>
+        <v>1965</v>
       </c>
       <c r="D72" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E72" s="8" t="n">
         <v>1</v>
@@ -22340,7 +22344,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
@@ -22349,7 +22353,7 @@
         </is>
       </c>
       <c r="I72" s="8" t="n">
-        <v>486</v>
+        <v>655</v>
       </c>
       <c r="J72" s="8" t="n"/>
       <c r="K72" s="8" t="n"/>
@@ -22364,12 +22368,12 @@
       <c r="P72" s="8" t="n"/>
       <c r="Q72" s="8" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="R72" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S72" s="9" t="inlineStr"/>
@@ -22386,7 +22390,7 @@
       <c r="V72" s="7" t="inlineStr"/>
       <c r="W72" s="8" t="inlineStr">
         <is>
-          <t>67ff71428df47b0eb7f7da47600378ffdad1f97c</t>
+          <t>1a5b509e1606992acea1736489630b2bc57cc717</t>
         </is>
       </c>
     </row>
@@ -22400,13 +22404,13 @@
         </is>
       </c>
       <c r="C73" s="17" t="n">
-        <v>1965</v>
+        <v>2080</v>
       </c>
       <c r="D73" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E73" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F73" s="8" t="inlineStr">
         <is>
@@ -22415,7 +22419,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H73" s="8" t="inlineStr">
@@ -22424,14 +22428,14 @@
         </is>
       </c>
       <c r="I73" s="8" t="n">
-        <v>655</v>
+        <v>705</v>
       </c>
       <c r="J73" s="8" t="n"/>
       <c r="K73" s="8" t="n"/>
       <c r="L73" s="8" t="n"/>
       <c r="M73" s="8" t="n"/>
       <c r="N73" s="8" t="n">
-        <v>21504</v>
+        <v>20820</v>
       </c>
       <c r="O73" s="8" t="n">
         <v>0</v>
@@ -22444,7 +22448,7 @@
       </c>
       <c r="R73" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S73" s="9" t="inlineStr"/>
@@ -22461,7 +22465,7 @@
       <c r="V73" s="7" t="inlineStr"/>
       <c r="W73" s="8" t="inlineStr">
         <is>
-          <t>1a5b509e1606992acea1736489630b2bc57cc717</t>
+          <t>0453e07b653a16ada93327f26a41e0b204d289a4</t>
         </is>
       </c>
     </row>
@@ -22475,13 +22479,13 @@
         </is>
       </c>
       <c r="C74" s="17" t="n">
-        <v>2080</v>
+        <v>1400</v>
       </c>
       <c r="D74" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E74" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F74" s="8" t="inlineStr">
         <is>
@@ -22490,7 +22494,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Redcliffe Parade West, Flat 3, City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr">
@@ -22498,15 +22502,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I74" s="8" t="n">
-        <v>705</v>
-      </c>
+      <c r="I74" s="8" t="n"/>
       <c r="J74" s="8" t="n"/>
       <c r="K74" s="8" t="n"/>
       <c r="L74" s="8" t="n"/>
       <c r="M74" s="8" t="n"/>
       <c r="N74" s="8" t="n">
-        <v>20820</v>
+        <v>19484</v>
       </c>
       <c r="O74" s="8" t="n">
         <v>0</v>
@@ -22519,7 +22521,7 @@
       </c>
       <c r="R74" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S74" s="9" t="inlineStr"/>
@@ -22536,7 +22538,7 @@
       <c r="V74" s="7" t="inlineStr"/>
       <c r="W74" s="8" t="inlineStr">
         <is>
-          <t>0453e07b653a16ada93327f26a41e0b204d289a4</t>
+          <t>9b65e5a0fb0bc8fc27d566eae912cddf76828cc9</t>
         </is>
       </c>
     </row>
@@ -22550,13 +22552,13 @@
         </is>
       </c>
       <c r="C75" s="17" t="n">
-        <v>1400</v>
+        <v>2000</v>
       </c>
       <c r="D75" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E75" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F75" s="8" t="inlineStr">
         <is>
@@ -22565,7 +22567,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>Redcliffe Parade West, Flat 3, City Centre, Bristol, BS1</t>
+          <t>Welsh Back, Bristol, BS1</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr">
@@ -22573,14 +22575,14 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I75" s="8" t="n"/>
+      <c r="I75" s="8" t="n">
+        <v>908</v>
+      </c>
       <c r="J75" s="8" t="n"/>
       <c r="K75" s="8" t="n"/>
       <c r="L75" s="8" t="n"/>
       <c r="M75" s="8" t="n"/>
-      <c r="N75" s="8" t="n">
-        <v>19484</v>
-      </c>
+      <c r="N75" s="8" t="n"/>
       <c r="O75" s="8" t="n">
         <v>0</v>
       </c>
@@ -22592,7 +22594,7 @@
       </c>
       <c r="R75" s="8" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>Hello Neighbour, London</t>
         </is>
       </c>
       <c r="S75" s="9" t="inlineStr"/>
@@ -22609,7 +22611,7 @@
       <c r="V75" s="7" t="inlineStr"/>
       <c r="W75" s="8" t="inlineStr">
         <is>
-          <t>9b65e5a0fb0bc8fc27d566eae912cddf76828cc9</t>
+          <t>65ed2520fdf37e6dde4abe0097cc3edbbbeff957</t>
         </is>
       </c>
     </row>
@@ -22623,13 +22625,13 @@
         </is>
       </c>
       <c r="C76" s="17" t="n">
-        <v>2000</v>
+        <v>2020</v>
       </c>
       <c r="D76" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E76" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
@@ -22638,7 +22640,7 @@
       </c>
       <c r="G76" s="9" t="inlineStr">
         <is>
-          <t>Welsh Back, Bristol, BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H76" s="8" t="inlineStr">
@@ -22647,7 +22649,7 @@
         </is>
       </c>
       <c r="I76" s="8" t="n">
-        <v>908</v>
+        <v>705</v>
       </c>
       <c r="J76" s="8" t="n"/>
       <c r="K76" s="8" t="n"/>
@@ -22660,12 +22662,12 @@
       <c r="P76" s="8" t="n"/>
       <c r="Q76" s="8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="R76" s="8" t="inlineStr">
         <is>
-          <t>Hello Neighbour, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S76" s="9" t="inlineStr"/>
@@ -22682,7 +22684,7 @@
       <c r="V76" s="7" t="inlineStr"/>
       <c r="W76" s="8" t="inlineStr">
         <is>
-          <t>65ed2520fdf37e6dde4abe0097cc3edbbbeff957</t>
+          <t>75b3ee81b8ecb4015a80108f6d509e4156f4e8e4</t>
         </is>
       </c>
     </row>
@@ -22696,7 +22698,7 @@
         </is>
       </c>
       <c r="C77" s="17" t="n">
-        <v>2020</v>
+        <v>2000</v>
       </c>
       <c r="D77" s="8" t="n">
         <v>2</v>
@@ -22711,7 +22713,7 @@
       </c>
       <c r="G77" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Eclipse - City Centre</t>
         </is>
       </c>
       <c r="H77" s="8" t="inlineStr">
@@ -22719,9 +22721,7 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I77" s="8" t="n">
-        <v>705</v>
-      </c>
+      <c r="I77" s="8" t="n"/>
       <c r="J77" s="8" t="n"/>
       <c r="K77" s="8" t="n"/>
       <c r="L77" s="8" t="n"/>
@@ -22733,12 +22733,12 @@
       <c r="P77" s="8" t="n"/>
       <c r="Q77" s="8" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="R77" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Ocean, Clifton</t>
         </is>
       </c>
       <c r="S77" s="9" t="inlineStr"/>
@@ -22755,7 +22755,7 @@
       <c r="V77" s="7" t="inlineStr"/>
       <c r="W77" s="8" t="inlineStr">
         <is>
-          <t>75b3ee81b8ecb4015a80108f6d509e4156f4e8e4</t>
+          <t>638ecbe81729048ffda61524ca9b06c4a208ce7b</t>
         </is>
       </c>
     </row>
@@ -22769,10 +22769,10 @@
         </is>
       </c>
       <c r="C78" s="17" t="n">
-        <v>2175</v>
+        <v>1595</v>
       </c>
       <c r="D78" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E78" s="8" t="n">
         <v>1</v>
@@ -22784,7 +22784,7 @@
       </c>
       <c r="G78" s="9" t="inlineStr">
         <is>
-          <t>Park St, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H78" s="8" t="inlineStr">
@@ -22792,7 +22792,9 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I78" s="8" t="n"/>
+      <c r="I78" s="8" t="n">
+        <v>499</v>
+      </c>
       <c r="J78" s="8" t="n"/>
       <c r="K78" s="8" t="n"/>
       <c r="L78" s="8" t="n"/>
@@ -22804,12 +22806,12 @@
       <c r="P78" s="8" t="n"/>
       <c r="Q78" s="8" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="R78" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S78" s="9" t="inlineStr"/>
@@ -22826,7 +22828,7 @@
       <c r="V78" s="7" t="inlineStr"/>
       <c r="W78" s="8" t="inlineStr">
         <is>
-          <t>6a00f91534112c4504453102597619449da3a2c1</t>
+          <t>f2f3afa9f34b35c1d7d84b8e8f6c80b9a91340b1</t>
         </is>
       </c>
     </row>
@@ -22840,7 +22842,7 @@
         </is>
       </c>
       <c r="C79" s="17" t="n">
-        <v>2000</v>
+        <v>2085</v>
       </c>
       <c r="D79" s="8" t="n">
         <v>2</v>
@@ -22855,7 +22857,7 @@
       </c>
       <c r="G79" s="9" t="inlineStr">
         <is>
-          <t>Eclipse - City Centre</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H79" s="8" t="inlineStr">
@@ -22863,7 +22865,9 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I79" s="8" t="n"/>
+      <c r="I79" s="8" t="n">
+        <v>705</v>
+      </c>
       <c r="J79" s="8" t="n"/>
       <c r="K79" s="8" t="n"/>
       <c r="L79" s="8" t="n"/>
@@ -22875,12 +22879,12 @@
       <c r="P79" s="8" t="n"/>
       <c r="Q79" s="8" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="R79" s="8" t="inlineStr">
         <is>
-          <t>Ocean, Clifton</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S79" s="9" t="inlineStr"/>
@@ -22897,7 +22901,7 @@
       <c r="V79" s="7" t="inlineStr"/>
       <c r="W79" s="8" t="inlineStr">
         <is>
-          <t>638ecbe81729048ffda61524ca9b06c4a208ce7b</t>
+          <t>16c89eb9a4cdeb57ddb3fd1201b7084ea2f3c007</t>
         </is>
       </c>
     </row>
@@ -22911,7 +22915,7 @@
         </is>
       </c>
       <c r="C80" s="17" t="n">
-        <v>1595</v>
+        <v>1615</v>
       </c>
       <c r="D80" s="8" t="n">
         <v>1</v>
@@ -22926,7 +22930,7 @@
       </c>
       <c r="G80" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H80" s="8" t="inlineStr">
@@ -22935,7 +22939,7 @@
         </is>
       </c>
       <c r="I80" s="8" t="n">
-        <v>499</v>
+        <v>487</v>
       </c>
       <c r="J80" s="8" t="n"/>
       <c r="K80" s="8" t="n"/>
@@ -22948,12 +22952,12 @@
       <c r="P80" s="8" t="n"/>
       <c r="Q80" s="8" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="R80" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S80" s="9" t="inlineStr"/>
@@ -22970,7 +22974,7 @@
       <c r="V80" s="7" t="inlineStr"/>
       <c r="W80" s="8" t="inlineStr">
         <is>
-          <t>f2f3afa9f34b35c1d7d84b8e8f6c80b9a91340b1</t>
+          <t>cd57661c8d996d20c5c1c7c34b12787f40073ec9</t>
         </is>
       </c>
     </row>
@@ -22984,7 +22988,7 @@
         </is>
       </c>
       <c r="C81" s="17" t="n">
-        <v>2085</v>
+        <v>2065</v>
       </c>
       <c r="D81" s="8" t="n">
         <v>2</v>
@@ -22999,7 +23003,7 @@
       </c>
       <c r="G81" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H81" s="8" t="inlineStr">
@@ -23008,7 +23012,7 @@
         </is>
       </c>
       <c r="I81" s="8" t="n">
-        <v>705</v>
+        <v>641</v>
       </c>
       <c r="J81" s="8" t="n"/>
       <c r="K81" s="8" t="n"/>
@@ -23021,12 +23025,12 @@
       <c r="P81" s="8" t="n"/>
       <c r="Q81" s="8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="R81" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S81" s="9" t="inlineStr"/>
@@ -23043,7 +23047,7 @@
       <c r="V81" s="7" t="inlineStr"/>
       <c r="W81" s="8" t="inlineStr">
         <is>
-          <t>16c89eb9a4cdeb57ddb3fd1201b7084ea2f3c007</t>
+          <t>d23eb397c84a723416c257acf4e25973ede40bc5</t>
         </is>
       </c>
     </row>
@@ -23057,13 +23061,13 @@
         </is>
       </c>
       <c r="C82" s="17" t="n">
-        <v>1615</v>
+        <v>2185</v>
       </c>
       <c r="D82" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E82" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F82" s="8" t="inlineStr">
         <is>
@@ -23081,7 +23085,7 @@
         </is>
       </c>
       <c r="I82" s="8" t="n">
-        <v>487</v>
+        <v>721</v>
       </c>
       <c r="J82" s="8" t="n"/>
       <c r="K82" s="8" t="n"/>
@@ -23094,7 +23098,7 @@
       <c r="P82" s="8" t="n"/>
       <c r="Q82" s="8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="R82" s="8" t="inlineStr">
@@ -23116,7 +23120,7 @@
       <c r="V82" s="7" t="inlineStr"/>
       <c r="W82" s="8" t="inlineStr">
         <is>
-          <t>cd57661c8d996d20c5c1c7c34b12787f40073ec9</t>
+          <t>6446e0c7d9c4f21f9eb6239caeeeee0599a68101</t>
         </is>
       </c>
     </row>
@@ -23130,13 +23134,13 @@
         </is>
       </c>
       <c r="C83" s="17" t="n">
-        <v>2065</v>
+        <v>1565</v>
       </c>
       <c r="D83" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E83" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F83" s="8" t="inlineStr">
         <is>
@@ -23145,7 +23149,7 @@
       </c>
       <c r="G83" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H83" s="8" t="inlineStr">
@@ -23154,7 +23158,7 @@
         </is>
       </c>
       <c r="I83" s="8" t="n">
-        <v>641</v>
+        <v>484</v>
       </c>
       <c r="J83" s="8" t="n"/>
       <c r="K83" s="8" t="n"/>
@@ -23172,7 +23176,7 @@
       </c>
       <c r="R83" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S83" s="9" t="inlineStr"/>
@@ -23189,7 +23193,7 @@
       <c r="V83" s="7" t="inlineStr"/>
       <c r="W83" s="8" t="inlineStr">
         <is>
-          <t>d23eb397c84a723416c257acf4e25973ede40bc5</t>
+          <t>34d9877a23c82be120784d9dd55c23c17584c91a</t>
         </is>
       </c>
     </row>
@@ -23203,13 +23207,13 @@
         </is>
       </c>
       <c r="C84" s="17" t="n">
-        <v>2185</v>
+        <v>1650</v>
       </c>
       <c r="D84" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E84" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F84" s="8" t="inlineStr">
         <is>
@@ -23218,7 +23222,7 @@
       </c>
       <c r="G84" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Horizon, Broad Weir, Bristol, BS1</t>
         </is>
       </c>
       <c r="H84" s="8" t="inlineStr">
@@ -23226,9 +23230,7 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I84" s="8" t="n">
-        <v>721</v>
-      </c>
+      <c r="I84" s="8" t="n"/>
       <c r="J84" s="8" t="n"/>
       <c r="K84" s="8" t="n"/>
       <c r="L84" s="8" t="n"/>
@@ -23240,12 +23242,12 @@
       <c r="P84" s="8" t="n"/>
       <c r="Q84" s="8" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="R84" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>CJ Hole, Bishopston</t>
         </is>
       </c>
       <c r="S84" s="9" t="inlineStr"/>
@@ -23262,7 +23264,7 @@
       <c r="V84" s="7" t="inlineStr"/>
       <c r="W84" s="8" t="inlineStr">
         <is>
-          <t>6446e0c7d9c4f21f9eb6239caeeeee0599a68101</t>
+          <t>aa3cf620ad25601a026424157bd8c0abb746373f</t>
         </is>
       </c>
     </row>
@@ -23276,7 +23278,7 @@
         </is>
       </c>
       <c r="C85" s="17" t="n">
-        <v>1565</v>
+        <v>1625</v>
       </c>
       <c r="D85" s="8" t="n">
         <v>1</v>
@@ -23300,7 +23302,7 @@
         </is>
       </c>
       <c r="I85" s="8" t="n">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="J85" s="8" t="n"/>
       <c r="K85" s="8" t="n"/>
@@ -23313,7 +23315,7 @@
       <c r="P85" s="8" t="n"/>
       <c r="Q85" s="8" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="R85" s="8" t="inlineStr">
@@ -23335,7 +23337,7 @@
       <c r="V85" s="7" t="inlineStr"/>
       <c r="W85" s="8" t="inlineStr">
         <is>
-          <t>34d9877a23c82be120784d9dd55c23c17584c91a</t>
+          <t>ea3758a9fd1b4190b4e5ae17519645f00d2e6a8f</t>
         </is>
       </c>
     </row>
@@ -23349,13 +23351,13 @@
         </is>
       </c>
       <c r="C86" s="17" t="n">
-        <v>1650</v>
+        <v>2175</v>
       </c>
       <c r="D86" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E86" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F86" s="8" t="inlineStr">
         <is>
@@ -23364,7 +23366,7 @@
       </c>
       <c r="G86" s="9" t="inlineStr">
         <is>
-          <t>Horizon, Broad Weir, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H86" s="8" t="inlineStr">
@@ -23372,7 +23374,9 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I86" s="8" t="n"/>
+      <c r="I86" s="8" t="n">
+        <v>722</v>
+      </c>
       <c r="J86" s="8" t="n"/>
       <c r="K86" s="8" t="n"/>
       <c r="L86" s="8" t="n"/>
@@ -23384,12 +23388,12 @@
       <c r="P86" s="8" t="n"/>
       <c r="Q86" s="8" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="R86" s="8" t="inlineStr">
         <is>
-          <t>CJ Hole, Bishopston</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S86" s="9" t="inlineStr"/>
@@ -23406,7 +23410,7 @@
       <c r="V86" s="7" t="inlineStr"/>
       <c r="W86" s="8" t="inlineStr">
         <is>
-          <t>aa3cf620ad25601a026424157bd8c0abb746373f</t>
+          <t>ab566c9b065047cd166a2ad3ae56e88704bc1358</t>
         </is>
       </c>
     </row>
@@ -23420,10 +23424,10 @@
         </is>
       </c>
       <c r="C87" s="17" t="n">
-        <v>1625</v>
+        <v>2100</v>
       </c>
       <c r="D87" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E87" s="8" t="n">
         <v>1</v>
@@ -23435,7 +23439,7 @@
       </c>
       <c r="G87" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>The Three Kings Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H87" s="8" t="inlineStr">
@@ -23443,9 +23447,7 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I87" s="8" t="n">
-        <v>485</v>
-      </c>
+      <c r="I87" s="8" t="n"/>
       <c r="J87" s="8" t="n"/>
       <c r="K87" s="8" t="n"/>
       <c r="L87" s="8" t="n"/>
@@ -23457,12 +23459,12 @@
       <c r="P87" s="8" t="n"/>
       <c r="Q87" s="8" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="R87" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S87" s="9" t="inlineStr"/>
@@ -23479,7 +23481,7 @@
       <c r="V87" s="7" t="inlineStr"/>
       <c r="W87" s="8" t="inlineStr">
         <is>
-          <t>ea3758a9fd1b4190b4e5ae17519645f00d2e6a8f</t>
+          <t>954007c82f6f3a495c465b72c9a1c44c0c84713e</t>
         </is>
       </c>
     </row>
@@ -23493,7 +23495,7 @@
         </is>
       </c>
       <c r="C88" s="17" t="n">
-        <v>2175</v>
+        <v>1900</v>
       </c>
       <c r="D88" s="8" t="n">
         <v>2</v>
@@ -23508,7 +23510,7 @@
       </c>
       <c r="G88" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>The Granary, Queen Charlotte Street, BRISTOL, BS1</t>
         </is>
       </c>
       <c r="H88" s="8" t="inlineStr">
@@ -23516,9 +23518,7 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I88" s="8" t="n">
-        <v>722</v>
-      </c>
+      <c r="I88" s="8" t="n"/>
       <c r="J88" s="8" t="n"/>
       <c r="K88" s="8" t="n"/>
       <c r="L88" s="8" t="n"/>
@@ -23530,12 +23530,12 @@
       <c r="P88" s="8" t="n"/>
       <c r="Q88" s="8" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="R88" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Andrews Letting and Management, Clifton</t>
         </is>
       </c>
       <c r="S88" s="9" t="inlineStr"/>
@@ -23552,7 +23552,7 @@
       <c r="V88" s="7" t="inlineStr"/>
       <c r="W88" s="8" t="inlineStr">
         <is>
-          <t>ab566c9b065047cd166a2ad3ae56e88704bc1358</t>
+          <t>b19bc62dddbc90526344a15be65fbc2e74a96d22</t>
         </is>
       </c>
     </row>
@@ -23566,7 +23566,7 @@
         </is>
       </c>
       <c r="C89" s="17" t="n">
-        <v>1500</v>
+        <v>1660</v>
       </c>
       <c r="D89" s="8" t="n">
         <v>1</v>
@@ -23581,7 +23581,7 @@
       </c>
       <c r="G89" s="9" t="inlineStr">
         <is>
-          <t>Baldwin Street, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H89" s="8" t="inlineStr">
@@ -23590,25 +23590,27 @@
         </is>
       </c>
       <c r="I89" s="8" t="n">
-        <v>721</v>
+        <v>486</v>
       </c>
       <c r="J89" s="8" t="n"/>
       <c r="K89" s="8" t="n"/>
       <c r="L89" s="8" t="n"/>
       <c r="M89" s="8" t="n"/>
-      <c r="N89" s="8" t="n"/>
+      <c r="N89" s="8" t="n">
+        <v>21504</v>
+      </c>
       <c r="O89" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P89" s="8" t="n"/>
       <c r="Q89" s="8" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R89" s="8" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S89" s="9" t="inlineStr"/>
@@ -23625,7 +23627,7 @@
       <c r="V89" s="7" t="inlineStr"/>
       <c r="W89" s="8" t="inlineStr">
         <is>
-          <t>02aa80149673ef91597cd6a5dd8c1688c9e61b9f</t>
+          <t>c2c660e4e8cefc047b4bc72bf19b48ce9ef7ec99</t>
         </is>
       </c>
     </row>
@@ -23639,13 +23641,13 @@
         </is>
       </c>
       <c r="C90" s="17" t="n">
-        <v>2100</v>
+        <v>2175</v>
       </c>
       <c r="D90" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E90" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F90" s="8" t="inlineStr">
         <is>
@@ -23654,7 +23656,7 @@
       </c>
       <c r="G90" s="9" t="inlineStr">
         <is>
-          <t>The Three Kings Court, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H90" s="8" t="inlineStr">
@@ -23662,24 +23664,28 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I90" s="8" t="n"/>
+      <c r="I90" s="8" t="n">
+        <v>814</v>
+      </c>
       <c r="J90" s="8" t="n"/>
       <c r="K90" s="8" t="n"/>
       <c r="L90" s="8" t="n"/>
       <c r="M90" s="8" t="n"/>
-      <c r="N90" s="8" t="n"/>
+      <c r="N90" s="8" t="n">
+        <v>21504</v>
+      </c>
       <c r="O90" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P90" s="8" t="n"/>
       <c r="Q90" s="8" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R90" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S90" s="9" t="inlineStr"/>
@@ -23696,7 +23702,7 @@
       <c r="V90" s="7" t="inlineStr"/>
       <c r="W90" s="8" t="inlineStr">
         <is>
-          <t>954007c82f6f3a495c465b72c9a1c44c0c84713e</t>
+          <t>83406f05c9aded812a566cc6806036dda0d45fc0</t>
         </is>
       </c>
     </row>
@@ -23710,7 +23716,7 @@
         </is>
       </c>
       <c r="C91" s="17" t="n">
-        <v>1900</v>
+        <v>1500</v>
       </c>
       <c r="D91" s="8" t="n">
         <v>2</v>
@@ -23725,7 +23731,7 @@
       </c>
       <c r="G91" s="9" t="inlineStr">
         <is>
-          <t>The Granary, Queen Charlotte Street, BRISTOL, BS1</t>
+          <t>Small Street - City Centre</t>
         </is>
       </c>
       <c r="H91" s="8" t="inlineStr">
@@ -23738,19 +23744,21 @@
       <c r="K91" s="8" t="n"/>
       <c r="L91" s="8" t="n"/>
       <c r="M91" s="8" t="n"/>
-      <c r="N91" s="8" t="n"/>
+      <c r="N91" s="8" t="n">
+        <v>21816</v>
+      </c>
       <c r="O91" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P91" s="8" t="n"/>
       <c r="Q91" s="8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R91" s="8" t="inlineStr">
         <is>
-          <t>Andrews Letting and Management, Clifton</t>
+          <t>Ocean, Clifton</t>
         </is>
       </c>
       <c r="S91" s="9" t="inlineStr"/>
@@ -23767,7 +23775,7 @@
       <c r="V91" s="7" t="inlineStr"/>
       <c r="W91" s="8" t="inlineStr">
         <is>
-          <t>b19bc62dddbc90526344a15be65fbc2e74a96d22</t>
+          <t>cb4b1af676ff54ae12ad7bf4fa94acd8ef94a533</t>
         </is>
       </c>
     </row>
@@ -23781,7 +23789,7 @@
         </is>
       </c>
       <c r="C92" s="17" t="n">
-        <v>2500</v>
+        <v>2115</v>
       </c>
       <c r="D92" s="8" t="n">
         <v>2</v>
@@ -23796,7 +23804,7 @@
       </c>
       <c r="G92" s="9" t="inlineStr">
         <is>
-          <t>Liberty Gardens, Caledonian Road, BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H92" s="8" t="inlineStr">
@@ -23805,25 +23813,27 @@
         </is>
       </c>
       <c r="I92" s="8" t="n">
-        <v>1238</v>
+        <v>823</v>
       </c>
       <c r="J92" s="8" t="n"/>
       <c r="K92" s="8" t="n"/>
       <c r="L92" s="8" t="n"/>
       <c r="M92" s="8" t="n"/>
-      <c r="N92" s="8" t="n"/>
+      <c r="N92" s="8" t="n">
+        <v>20820</v>
+      </c>
       <c r="O92" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P92" s="8" t="n"/>
       <c r="Q92" s="8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="R92" s="8" t="inlineStr">
         <is>
-          <t>Sarah Kenny Residential Lettings, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S92" s="9" t="inlineStr"/>
@@ -23840,7 +23850,7 @@
       <c r="V92" s="7" t="inlineStr"/>
       <c r="W92" s="8" t="inlineStr">
         <is>
-          <t>5190fc249258ef945384f72c42f49bfb1154cc31</t>
+          <t>0b78c6e29d96ae73c643d0d50d50949797b02893</t>
         </is>
       </c>
     </row>
@@ -23893,7 +23903,7 @@
       <c r="P93" s="8" t="n"/>
       <c r="Q93" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="R93" s="8" t="inlineStr">
@@ -23915,7 +23925,7 @@
       <c r="V93" s="7" t="inlineStr"/>
       <c r="W93" s="8" t="inlineStr">
         <is>
-          <t>c2c660e4e8cefc047b4bc72bf19b48ce9ef7ec99</t>
+          <t>c798c669d03fa2e42fd418ff0916de022d3380ad</t>
         </is>
       </c>
     </row>
@@ -23929,7 +23939,7 @@
         </is>
       </c>
       <c r="C94" s="17" t="n">
-        <v>2175</v>
+        <v>1915</v>
       </c>
       <c r="D94" s="8" t="n">
         <v>2</v>
@@ -23953,14 +23963,14 @@
         </is>
       </c>
       <c r="I94" s="8" t="n">
-        <v>814</v>
+        <v>746</v>
       </c>
       <c r="J94" s="8" t="n"/>
       <c r="K94" s="8" t="n"/>
       <c r="L94" s="8" t="n"/>
       <c r="M94" s="8" t="n"/>
       <c r="N94" s="8" t="n">
-        <v>21504</v>
+        <v>21680</v>
       </c>
       <c r="O94" s="8" t="n">
         <v>0</v>
@@ -23968,7 +23978,7 @@
       <c r="P94" s="8" t="n"/>
       <c r="Q94" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="R94" s="8" t="inlineStr">
@@ -23990,7 +24000,7 @@
       <c r="V94" s="7" t="inlineStr"/>
       <c r="W94" s="8" t="inlineStr">
         <is>
-          <t>83406f05c9aded812a566cc6806036dda0d45fc0</t>
+          <t>36797023cff0095f1bf764fa2f176d5595124854</t>
         </is>
       </c>
     </row>
@@ -24004,13 +24014,13 @@
         </is>
       </c>
       <c r="C95" s="17" t="n">
-        <v>1500</v>
+        <v>1150</v>
       </c>
       <c r="D95" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E95" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F95" s="8" t="inlineStr">
         <is>
@@ -24019,12 +24029,12 @@
       </c>
       <c r="G95" s="9" t="inlineStr">
         <is>
-          <t>Small Street - City Centre</t>
+          <t>Knowle Road, Bristol</t>
         </is>
       </c>
       <c r="H95" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS4</t>
         </is>
       </c>
       <c r="I95" s="8" t="n"/>
@@ -24033,7 +24043,7 @@
       <c r="L95" s="8" t="n"/>
       <c r="M95" s="8" t="n"/>
       <c r="N95" s="8" t="n">
-        <v>21816</v>
+        <v>6872</v>
       </c>
       <c r="O95" s="8" t="n">
         <v>0</v>
@@ -24041,12 +24051,12 @@
       <c r="P95" s="8" t="n"/>
       <c r="Q95" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R95" s="8" t="inlineStr">
         <is>
-          <t>Ocean, Clifton</t>
+          <t>Hopewell, Bristol</t>
         </is>
       </c>
       <c r="S95" s="9" t="inlineStr"/>
@@ -24063,7 +24073,7 @@
       <c r="V95" s="7" t="inlineStr"/>
       <c r="W95" s="8" t="inlineStr">
         <is>
-          <t>cb4b1af676ff54ae12ad7bf4fa94acd8ef94a533</t>
+          <t>edac1b499f84e07ce85894b488f82dc5cd104202</t>
         </is>
       </c>
     </row>
@@ -24077,13 +24087,13 @@
         </is>
       </c>
       <c r="C96" s="17" t="n">
-        <v>1450</v>
+        <v>2450</v>
       </c>
       <c r="D96" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E96" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F96" s="8" t="inlineStr">
         <is>
@@ -24092,12 +24102,12 @@
       </c>
       <c r="G96" s="9" t="inlineStr">
         <is>
-          <t>The Old Drill Hall, Bristol, BS2</t>
+          <t>The Herbert Ashman Building, Bristol, BS1</t>
         </is>
       </c>
       <c r="H96" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I96" s="8" t="n"/>
@@ -24105,14 +24115,16 @@
       <c r="K96" s="8" t="n"/>
       <c r="L96" s="8" t="n"/>
       <c r="M96" s="8" t="n"/>
-      <c r="N96" s="8" t="n"/>
+      <c r="N96" s="8" t="n">
+        <v>21788</v>
+      </c>
       <c r="O96" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P96" s="8" t="n"/>
       <c r="Q96" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R96" s="8" t="inlineStr">
@@ -24134,7 +24146,7 @@
       <c r="V96" s="7" t="inlineStr"/>
       <c r="W96" s="8" t="inlineStr">
         <is>
-          <t>c847859d6a4555381482a51e75495800df35917d</t>
+          <t>4cd4fdc09f26b6316c31aa22f38853db44d1ea9a</t>
         </is>
       </c>
     </row>
@@ -24148,7 +24160,7 @@
         </is>
       </c>
       <c r="C97" s="17" t="n">
-        <v>2115</v>
+        <v>1700</v>
       </c>
       <c r="D97" s="8" t="n">
         <v>2</v>
@@ -24163,7 +24175,7 @@
       </c>
       <c r="G97" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>The Crescent</t>
         </is>
       </c>
       <c r="H97" s="8" t="inlineStr">
@@ -24171,15 +24183,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I97" s="8" t="n">
-        <v>823</v>
-      </c>
+      <c r="I97" s="8" t="n"/>
       <c r="J97" s="8" t="n"/>
       <c r="K97" s="8" t="n"/>
       <c r="L97" s="8" t="n"/>
       <c r="M97" s="8" t="n"/>
       <c r="N97" s="8" t="n">
-        <v>20820</v>
+        <v>16368</v>
       </c>
       <c r="O97" s="8" t="n">
         <v>0</v>
@@ -24187,12 +24197,12 @@
       <c r="P97" s="8" t="n"/>
       <c r="Q97" s="8" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R97" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S97" s="9" t="inlineStr"/>
@@ -24209,7 +24219,7 @@
       <c r="V97" s="7" t="inlineStr"/>
       <c r="W97" s="8" t="inlineStr">
         <is>
-          <t>0b78c6e29d96ae73c643d0d50d50949797b02893</t>
+          <t>8a8446c119238f7a042580aed1922ef6cfd79ae2</t>
         </is>
       </c>
     </row>
@@ -24223,7 +24233,7 @@
         </is>
       </c>
       <c r="C98" s="17" t="n">
-        <v>1660</v>
+        <v>1250</v>
       </c>
       <c r="D98" s="8" t="n">
         <v>1</v>
@@ -24238,7 +24248,7 @@
       </c>
       <c r="G98" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Victoria Street, Bristol, BS1 6DR</t>
         </is>
       </c>
       <c r="H98" s="8" t="inlineStr">
@@ -24246,15 +24256,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I98" s="8" t="n">
-        <v>486</v>
-      </c>
+      <c r="I98" s="8" t="n"/>
       <c r="J98" s="8" t="n"/>
       <c r="K98" s="8" t="n"/>
       <c r="L98" s="8" t="n"/>
       <c r="M98" s="8" t="n"/>
       <c r="N98" s="8" t="n">
-        <v>21504</v>
+        <v>21160</v>
       </c>
       <c r="O98" s="8" t="n">
         <v>0</v>
@@ -24262,12 +24270,12 @@
       <c r="P98" s="8" t="n"/>
       <c r="Q98" s="8" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R98" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Visum, Nationwide</t>
         </is>
       </c>
       <c r="S98" s="9" t="inlineStr"/>
@@ -24284,7 +24292,7 @@
       <c r="V98" s="7" t="inlineStr"/>
       <c r="W98" s="8" t="inlineStr">
         <is>
-          <t>c798c669d03fa2e42fd418ff0916de022d3380ad</t>
+          <t>78fe8e0511ccc37f104368075238c845f57d7864</t>
         </is>
       </c>
     </row>
@@ -24298,7 +24306,7 @@
         </is>
       </c>
       <c r="C99" s="17" t="n">
-        <v>1915</v>
+        <v>1600</v>
       </c>
       <c r="D99" s="8" t="n">
         <v>2</v>
@@ -24313,23 +24321,21 @@
       </c>
       <c r="G99" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Ratcliffe Court, Bristol, BS2</t>
         </is>
       </c>
       <c r="H99" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I99" s="8" t="n">
-        <v>746</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I99" s="8" t="n"/>
       <c r="J99" s="8" t="n"/>
       <c r="K99" s="8" t="n"/>
       <c r="L99" s="8" t="n"/>
       <c r="M99" s="8" t="n"/>
       <c r="N99" s="8" t="n">
-        <v>21680</v>
+        <v>20124</v>
       </c>
       <c r="O99" s="8" t="n">
         <v>0</v>
@@ -24337,12 +24343,12 @@
       <c r="P99" s="8" t="n"/>
       <c r="Q99" s="8" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R99" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S99" s="9" t="inlineStr"/>
@@ -24359,7 +24365,7 @@
       <c r="V99" s="7" t="inlineStr"/>
       <c r="W99" s="8" t="inlineStr">
         <is>
-          <t>36797023cff0095f1bf764fa2f176d5595124854</t>
+          <t>e9219c4f68722ad3bdeee0c4c4cb31134f26af57</t>
         </is>
       </c>
     </row>
@@ -24373,13 +24379,13 @@
         </is>
       </c>
       <c r="C100" s="17" t="n">
-        <v>1150</v>
+        <v>2145</v>
       </c>
       <c r="D100" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E100" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F100" s="8" t="inlineStr">
         <is>
@@ -24388,21 +24394,23 @@
       </c>
       <c r="G100" s="9" t="inlineStr">
         <is>
-          <t>Knowle Road, Bristol</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H100" s="8" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I100" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I100" s="8" t="n">
+        <v>796</v>
+      </c>
       <c r="J100" s="8" t="n"/>
       <c r="K100" s="8" t="n"/>
       <c r="L100" s="8" t="n"/>
       <c r="M100" s="8" t="n"/>
       <c r="N100" s="8" t="n">
-        <v>6872</v>
+        <v>20820</v>
       </c>
       <c r="O100" s="8" t="n">
         <v>0</v>
@@ -24410,12 +24418,12 @@
       <c r="P100" s="8" t="n"/>
       <c r="Q100" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R100" s="8" t="inlineStr">
         <is>
-          <t>Hopewell, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S100" s="9" t="inlineStr"/>
@@ -24432,7 +24440,7 @@
       <c r="V100" s="7" t="inlineStr"/>
       <c r="W100" s="8" t="inlineStr">
         <is>
-          <t>edac1b499f84e07ce85894b488f82dc5cd104202</t>
+          <t>898ba227d5b949e4e7f18b49536b3c908560d145</t>
         </is>
       </c>
     </row>
@@ -24446,13 +24454,13 @@
         </is>
       </c>
       <c r="C101" s="17" t="n">
-        <v>2450</v>
+        <v>1999</v>
       </c>
       <c r="D101" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E101" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F101" s="8" t="inlineStr">
         <is>
@@ -24461,7 +24469,7 @@
       </c>
       <c r="G101" s="9" t="inlineStr">
         <is>
-          <t>The Herbert Ashman Building, Bristol, BS1</t>
+          <t>Swann House, Bristol, BS1</t>
         </is>
       </c>
       <c r="H101" s="8" t="inlineStr">
@@ -24475,7 +24483,7 @@
       <c r="L101" s="8" t="n"/>
       <c r="M101" s="8" t="n"/>
       <c r="N101" s="8" t="n">
-        <v>21788</v>
+        <v>20800</v>
       </c>
       <c r="O101" s="8" t="n">
         <v>0</v>
@@ -24483,7 +24491,7 @@
       <c r="P101" s="8" t="n"/>
       <c r="Q101" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R101" s="8" t="inlineStr">
@@ -24505,7 +24513,7 @@
       <c r="V101" s="7" t="inlineStr"/>
       <c r="W101" s="8" t="inlineStr">
         <is>
-          <t>4cd4fdc09f26b6316c31aa22f38853db44d1ea9a</t>
+          <t>5cec67aa8ba885c4c8f85e47d3354d187da9d897</t>
         </is>
       </c>
     </row>
@@ -24519,13 +24527,13 @@
         </is>
       </c>
       <c r="C102" s="17" t="n">
-        <v>1700</v>
+        <v>1670</v>
       </c>
       <c r="D102" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E102" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F102" s="8" t="inlineStr">
         <is>
@@ -24534,7 +24542,7 @@
       </c>
       <c r="G102" s="9" t="inlineStr">
         <is>
-          <t>The Crescent</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H102" s="8" t="inlineStr">
@@ -24542,13 +24550,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I102" s="8" t="n"/>
+      <c r="I102" s="8" t="n">
+        <v>485</v>
+      </c>
       <c r="J102" s="8" t="n"/>
       <c r="K102" s="8" t="n"/>
       <c r="L102" s="8" t="n"/>
       <c r="M102" s="8" t="n"/>
       <c r="N102" s="8" t="n">
-        <v>16368</v>
+        <v>21504</v>
       </c>
       <c r="O102" s="8" t="n">
         <v>0</v>
@@ -24556,12 +24566,12 @@
       <c r="P102" s="8" t="n"/>
       <c r="Q102" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R102" s="8" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S102" s="9" t="inlineStr"/>
@@ -24578,7 +24588,7 @@
       <c r="V102" s="7" t="inlineStr"/>
       <c r="W102" s="8" t="inlineStr">
         <is>
-          <t>8a8446c119238f7a042580aed1922ef6cfd79ae2</t>
+          <t>73f3509a6c69eef7af4c6b9ff0dc69b97478c20a</t>
         </is>
       </c>
     </row>
@@ -24592,7 +24602,7 @@
         </is>
       </c>
       <c r="C103" s="17" t="n">
-        <v>1250</v>
+        <v>1645</v>
       </c>
       <c r="D103" s="8" t="n">
         <v>1</v>
@@ -24607,7 +24617,7 @@
       </c>
       <c r="G103" s="9" t="inlineStr">
         <is>
-          <t>Victoria Street, Bristol, BS1 6DR</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H103" s="8" t="inlineStr">
@@ -24615,13 +24625,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I103" s="8" t="n"/>
+      <c r="I103" s="8" t="n">
+        <v>517</v>
+      </c>
       <c r="J103" s="8" t="n"/>
       <c r="K103" s="8" t="n"/>
       <c r="L103" s="8" t="n"/>
       <c r="M103" s="8" t="n"/>
       <c r="N103" s="8" t="n">
-        <v>21160</v>
+        <v>20820</v>
       </c>
       <c r="O103" s="8" t="n">
         <v>0</v>
@@ -24629,12 +24641,12 @@
       <c r="P103" s="8" t="n"/>
       <c r="Q103" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R103" s="8" t="inlineStr">
         <is>
-          <t>Visum, Nationwide</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S103" s="9" t="inlineStr"/>
@@ -24651,7 +24663,7 @@
       <c r="V103" s="7" t="inlineStr"/>
       <c r="W103" s="8" t="inlineStr">
         <is>
-          <t>78fe8e0511ccc37f104368075238c845f57d7864</t>
+          <t>4efcb79ae710a68f5f272a2f9030937499117f9d</t>
         </is>
       </c>
     </row>
@@ -24665,7 +24677,7 @@
         </is>
       </c>
       <c r="C104" s="17" t="n">
-        <v>1600</v>
+        <v>2120</v>
       </c>
       <c r="D104" s="8" t="n">
         <v>2</v>
@@ -24680,21 +24692,23 @@
       </c>
       <c r="G104" s="9" t="inlineStr">
         <is>
-          <t>Ratcliffe Court, Bristol, BS2</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H104" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I104" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I104" s="8" t="n">
+        <v>705</v>
+      </c>
       <c r="J104" s="8" t="n"/>
       <c r="K104" s="8" t="n"/>
       <c r="L104" s="8" t="n"/>
       <c r="M104" s="8" t="n"/>
       <c r="N104" s="8" t="n">
-        <v>20124</v>
+        <v>20820</v>
       </c>
       <c r="O104" s="8" t="n">
         <v>0</v>
@@ -24702,12 +24716,12 @@
       <c r="P104" s="8" t="n"/>
       <c r="Q104" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="R104" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S104" s="9" t="inlineStr"/>
@@ -24724,7 +24738,7 @@
       <c r="V104" s="7" t="inlineStr"/>
       <c r="W104" s="8" t="inlineStr">
         <is>
-          <t>e9219c4f68722ad3bdeee0c4c4cb31134f26af57</t>
+          <t>c5c1741357dfce3547bdab7d4d5a0e7602846192</t>
         </is>
       </c>
     </row>
@@ -24738,13 +24752,13 @@
         </is>
       </c>
       <c r="C105" s="17" t="n">
-        <v>2145</v>
+        <v>1645</v>
       </c>
       <c r="D105" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E105" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F105" s="8" t="inlineStr">
         <is>
@@ -24762,7 +24776,7 @@
         </is>
       </c>
       <c r="I105" s="8" t="n">
-        <v>796</v>
+        <v>571</v>
       </c>
       <c r="J105" s="8" t="n"/>
       <c r="K105" s="8" t="n"/>
@@ -24777,7 +24791,7 @@
       <c r="P105" s="8" t="n"/>
       <c r="Q105" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="R105" s="8" t="inlineStr">
@@ -24799,7 +24813,7 @@
       <c r="V105" s="7" t="inlineStr"/>
       <c r="W105" s="8" t="inlineStr">
         <is>
-          <t>898ba227d5b949e4e7f18b49536b3c908560d145</t>
+          <t>487e67b2d6680ebaabfcc49d4d33e21cb65cca6d</t>
         </is>
       </c>
     </row>
@@ -24813,7 +24827,7 @@
         </is>
       </c>
       <c r="C106" s="17" t="n">
-        <v>1999</v>
+        <v>2250</v>
       </c>
       <c r="D106" s="8" t="n">
         <v>2</v>
@@ -24828,7 +24842,7 @@
       </c>
       <c r="G106" s="9" t="inlineStr">
         <is>
-          <t>Swann House, Bristol, BS1</t>
+          <t>Apartments, Bristol, BS1</t>
         </is>
       </c>
       <c r="H106" s="8" t="inlineStr">
@@ -24842,7 +24856,7 @@
       <c r="L106" s="8" t="n"/>
       <c r="M106" s="8" t="n"/>
       <c r="N106" s="8" t="n">
-        <v>20800</v>
+        <v>22132</v>
       </c>
       <c r="O106" s="8" t="n">
         <v>0</v>
@@ -24850,7 +24864,7 @@
       <c r="P106" s="8" t="n"/>
       <c r="Q106" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="R106" s="8" t="inlineStr">
@@ -24872,7 +24886,7 @@
       <c r="V106" s="7" t="inlineStr"/>
       <c r="W106" s="8" t="inlineStr">
         <is>
-          <t>5cec67aa8ba885c4c8f85e47d3354d187da9d897</t>
+          <t>b3bc6f44f28301ca7ff059723f3c836424cd082f</t>
         </is>
       </c>
     </row>
@@ -24886,10 +24900,10 @@
         </is>
       </c>
       <c r="C107" s="17" t="n">
-        <v>1670</v>
+        <v>1600</v>
       </c>
       <c r="D107" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E107" s="8" t="n">
         <v>1</v>
@@ -24901,23 +24915,21 @@
       </c>
       <c r="G107" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Stapleton Road, Bristol, BS5</t>
         </is>
       </c>
       <c r="H107" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I107" s="8" t="n">
-        <v>485</v>
-      </c>
+          <t>BS5</t>
+        </is>
+      </c>
+      <c r="I107" s="8" t="n"/>
       <c r="J107" s="8" t="n"/>
       <c r="K107" s="8" t="n"/>
       <c r="L107" s="8" t="n"/>
       <c r="M107" s="8" t="n"/>
       <c r="N107" s="8" t="n">
-        <v>21504</v>
+        <v>19576</v>
       </c>
       <c r="O107" s="8" t="n">
         <v>0</v>
@@ -24925,12 +24937,12 @@
       <c r="P107" s="8" t="n"/>
       <c r="Q107" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="R107" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S107" s="9" t="inlineStr"/>
@@ -24947,7 +24959,7 @@
       <c r="V107" s="7" t="inlineStr"/>
       <c r="W107" s="8" t="inlineStr">
         <is>
-          <t>73f3509a6c69eef7af4c6b9ff0dc69b97478c20a</t>
+          <t>2c4d3b36f040dfa0e294ad99ce0d43b5fa15d6c8</t>
         </is>
       </c>
     </row>
@@ -24961,10 +24973,10 @@
         </is>
       </c>
       <c r="C108" s="17" t="n">
-        <v>1645</v>
+        <v>2175</v>
       </c>
       <c r="D108" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E108" s="8" t="n">
         <v>1</v>
@@ -24976,7 +24988,7 @@
       </c>
       <c r="G108" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Park St, Bristol, BS1</t>
         </is>
       </c>
       <c r="H108" s="8" t="inlineStr">
@@ -24984,28 +24996,24 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I108" s="8" t="n">
-        <v>517</v>
-      </c>
+      <c r="I108" s="8" t="n"/>
       <c r="J108" s="8" t="n"/>
       <c r="K108" s="8" t="n"/>
       <c r="L108" s="8" t="n"/>
       <c r="M108" s="8" t="n"/>
-      <c r="N108" s="8" t="n">
-        <v>20820</v>
-      </c>
+      <c r="N108" s="8" t="n"/>
       <c r="O108" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P108" s="8" t="n"/>
       <c r="Q108" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="R108" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S108" s="9" t="inlineStr"/>
@@ -25022,7 +25030,7 @@
       <c r="V108" s="7" t="inlineStr"/>
       <c r="W108" s="8" t="inlineStr">
         <is>
-          <t>4efcb79ae710a68f5f272a2f9030937499117f9d</t>
+          <t>6a00f91534112c4504453102597619449da3a2c1</t>
         </is>
       </c>
     </row>
@@ -25036,13 +25044,13 @@
         </is>
       </c>
       <c r="C109" s="17" t="n">
-        <v>2120</v>
+        <v>1500</v>
       </c>
       <c r="D109" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E109" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F109" s="8" t="inlineStr">
         <is>
@@ -25051,7 +25059,7 @@
       </c>
       <c r="G109" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Baldwin Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H109" s="8" t="inlineStr">
@@ -25060,27 +25068,25 @@
         </is>
       </c>
       <c r="I109" s="8" t="n">
-        <v>705</v>
+        <v>721</v>
       </c>
       <c r="J109" s="8" t="n"/>
       <c r="K109" s="8" t="n"/>
       <c r="L109" s="8" t="n"/>
       <c r="M109" s="8" t="n"/>
-      <c r="N109" s="8" t="n">
-        <v>20820</v>
-      </c>
+      <c r="N109" s="8" t="n"/>
       <c r="O109" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P109" s="8" t="n"/>
       <c r="Q109" s="8" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="R109" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Acen Properties, Bristol</t>
         </is>
       </c>
       <c r="S109" s="9" t="inlineStr"/>
@@ -25097,7 +25103,7 @@
       <c r="V109" s="7" t="inlineStr"/>
       <c r="W109" s="8" t="inlineStr">
         <is>
-          <t>c5c1741357dfce3547bdab7d4d5a0e7602846192</t>
+          <t>02aa80149673ef91597cd6a5dd8c1688c9e61b9f</t>
         </is>
       </c>
     </row>
@@ -25111,13 +25117,13 @@
         </is>
       </c>
       <c r="C110" s="17" t="n">
-        <v>1645</v>
+        <v>2500</v>
       </c>
       <c r="D110" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E110" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F110" s="8" t="inlineStr">
         <is>
@@ -25126,7 +25132,7 @@
       </c>
       <c r="G110" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Liberty Gardens, Caledonian Road, BS1</t>
         </is>
       </c>
       <c r="H110" s="8" t="inlineStr">
@@ -25135,27 +25141,25 @@
         </is>
       </c>
       <c r="I110" s="8" t="n">
-        <v>571</v>
+        <v>1238</v>
       </c>
       <c r="J110" s="8" t="n"/>
       <c r="K110" s="8" t="n"/>
       <c r="L110" s="8" t="n"/>
       <c r="M110" s="8" t="n"/>
-      <c r="N110" s="8" t="n">
-        <v>20820</v>
-      </c>
+      <c r="N110" s="8" t="n"/>
       <c r="O110" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P110" s="8" t="n"/>
       <c r="Q110" s="8" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="R110" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Sarah Kenny Residential Lettings, Bristol</t>
         </is>
       </c>
       <c r="S110" s="9" t="inlineStr"/>
@@ -25172,7 +25176,7 @@
       <c r="V110" s="7" t="inlineStr"/>
       <c r="W110" s="8" t="inlineStr">
         <is>
-          <t>487e67b2d6680ebaabfcc49d4d33e21cb65cca6d</t>
+          <t>5190fc249258ef945384f72c42f49bfb1154cc31</t>
         </is>
       </c>
     </row>
@@ -25186,10 +25190,10 @@
         </is>
       </c>
       <c r="C111" s="17" t="n">
-        <v>2250</v>
+        <v>1450</v>
       </c>
       <c r="D111" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E111" s="8" t="n">
         <v>1</v>
@@ -25201,12 +25205,12 @@
       </c>
       <c r="G111" s="9" t="inlineStr">
         <is>
-          <t>Apartments, Bristol, BS1</t>
+          <t>The Old Drill Hall, Bristol, BS2</t>
         </is>
       </c>
       <c r="H111" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I111" s="8" t="n"/>
@@ -25214,16 +25218,14 @@
       <c r="K111" s="8" t="n"/>
       <c r="L111" s="8" t="n"/>
       <c r="M111" s="8" t="n"/>
-      <c r="N111" s="8" t="n">
-        <v>22132</v>
-      </c>
+      <c r="N111" s="8" t="n"/>
       <c r="O111" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P111" s="8" t="n"/>
       <c r="Q111" s="8" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R111" s="8" t="inlineStr">
@@ -25245,7 +25247,7 @@
       <c r="V111" s="7" t="inlineStr"/>
       <c r="W111" s="8" t="inlineStr">
         <is>
-          <t>b3bc6f44f28301ca7ff059723f3c836424cd082f</t>
+          <t>c847859d6a4555381482a51e75495800df35917d</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
House search data from run 19
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -17141,10 +17141,10 @@
         </is>
       </c>
       <c r="C4" s="17" t="n">
-        <v>1300</v>
+        <v>1900</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" s="8" t="n">
         <v>1</v>
@@ -17156,21 +17156,23 @@
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>St. Johns Lane, Bedminster, BS3</t>
+          <t>Redcliff Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H4" s="8" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I4" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>731</v>
+      </c>
       <c r="J4" s="8" t="n"/>
       <c r="K4" s="8" t="n"/>
       <c r="L4" s="8" t="n"/>
       <c r="M4" s="8" t="n"/>
       <c r="N4" s="8" t="n">
-        <v>7112</v>
+        <v>20892</v>
       </c>
       <c r="O4" s="8" t="n">
         <v>0</v>
@@ -17178,17 +17180,17 @@
       <c r="P4" s="8" t="n"/>
       <c r="Q4" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="R4" s="8" t="inlineStr">
         <is>
-          <t>Taylors Lettings, Bedminster</t>
+          <t>A2Dominion Group, A2Dominion Lettings</t>
         </is>
       </c>
       <c r="S4" s="9" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T4" s="12" t="inlineStr">
@@ -17204,7 +17206,7 @@
       <c r="V4" s="7" t="inlineStr"/>
       <c r="W4" s="8" t="inlineStr">
         <is>
-          <t>91339ed58a9e4347ac017823b498695129a40922</t>
+          <t>c11b7a868ede7c3b0a3d524aa4d4e8f661494706</t>
         </is>
       </c>
     </row>
@@ -17218,10 +17220,10 @@
         </is>
       </c>
       <c r="C5" s="17" t="n">
-        <v>1900</v>
+        <v>1395</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" s="8" t="n">
         <v>1</v>
@@ -17233,23 +17235,21 @@
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>Redcliff Street, Bristol, BS1</t>
+          <t>Hamilton Court, Bristol, BS2</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I5" s="8" t="n">
-        <v>731</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="n"/>
       <c r="J5" s="8" t="n"/>
       <c r="K5" s="8" t="n"/>
       <c r="L5" s="8" t="n"/>
       <c r="M5" s="8" t="n"/>
       <c r="N5" s="8" t="n">
-        <v>20892</v>
+        <v>21660</v>
       </c>
       <c r="O5" s="8" t="n">
         <v>0</v>
@@ -17257,17 +17257,17 @@
       <c r="P5" s="8" t="n"/>
       <c r="Q5" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R5" s="8" t="inlineStr">
         <is>
-          <t>A2Dominion Group, A2Dominion Lettings</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S5" s="9" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T5" s="12" t="inlineStr">
@@ -17283,7 +17283,7 @@
       <c r="V5" s="7" t="inlineStr"/>
       <c r="W5" s="8" t="inlineStr">
         <is>
-          <t>c11b7a868ede7c3b0a3d524aa4d4e8f661494706</t>
+          <t>55512167c7894bf9991618275f495f9b5aa0a1af</t>
         </is>
       </c>
     </row>
@@ -17297,13 +17297,13 @@
         </is>
       </c>
       <c r="C6" s="17" t="n">
-        <v>1395</v>
+        <v>2000</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
@@ -17312,12 +17312,12 @@
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>Hamilton Court, Bristol, BS2</t>
+          <t>Deanery Road, Bristol, BS1</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I6" s="8" t="n"/>
@@ -17326,7 +17326,7 @@
       <c r="L6" s="8" t="n"/>
       <c r="M6" s="8" t="n"/>
       <c r="N6" s="8" t="n">
-        <v>21660</v>
+        <v>18292</v>
       </c>
       <c r="O6" s="8" t="n">
         <v>0</v>
@@ -17339,12 +17339,12 @@
       </c>
       <c r="R6" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Howard, Bristol</t>
         </is>
       </c>
       <c r="S6" s="9" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T6" s="12" t="inlineStr">
@@ -17360,7 +17360,7 @@
       <c r="V6" s="7" t="inlineStr"/>
       <c r="W6" s="8" t="inlineStr">
         <is>
-          <t>55512167c7894bf9991618275f495f9b5aa0a1af</t>
+          <t>591cc261a1f5973aaa4a7b3adbcbe4699bcc6440</t>
         </is>
       </c>
     </row>
@@ -17374,13 +17374,13 @@
         </is>
       </c>
       <c r="C7" s="17" t="n">
-        <v>2000</v>
+        <v>1550</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
@@ -17389,12 +17389,12 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>Deanery Road, Bristol, BS1</t>
+          <t>Beaufort Street, Stapleton, Bristol</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS5</t>
         </is>
       </c>
       <c r="I7" s="8" t="n"/>
@@ -17403,7 +17403,7 @@
       <c r="L7" s="8" t="n"/>
       <c r="M7" s="8" t="n"/>
       <c r="N7" s="8" t="n">
-        <v>18292</v>
+        <v>19400</v>
       </c>
       <c r="O7" s="8" t="n">
         <v>0</v>
@@ -17416,7 +17416,7 @@
       </c>
       <c r="R7" s="8" t="inlineStr">
         <is>
-          <t>Howard, Bristol</t>
+          <t>Taylors Lettings, Bradley Stoke</t>
         </is>
       </c>
       <c r="S7" s="9" t="inlineStr">
@@ -17437,7 +17437,7 @@
       <c r="V7" s="7" t="inlineStr"/>
       <c r="W7" s="8" t="inlineStr">
         <is>
-          <t>591cc261a1f5973aaa4a7b3adbcbe4699bcc6440</t>
+          <t>81712a02a3a8827c0a71232c3b582e0d2b990a2a</t>
         </is>
       </c>
     </row>
@@ -17451,13 +17451,13 @@
         </is>
       </c>
       <c r="C8" s="17" t="n">
-        <v>1550</v>
+        <v>1900</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
@@ -17466,21 +17466,23 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>Beaufort Street, Stapleton, Bristol</t>
+          <t>Arnos Vale, Paintworks, BS4</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>BS5</t>
-        </is>
-      </c>
-      <c r="I8" s="8" t="n"/>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="n">
+        <v>783</v>
+      </c>
       <c r="J8" s="8" t="n"/>
       <c r="K8" s="8" t="n"/>
       <c r="L8" s="8" t="n"/>
       <c r="M8" s="8" t="n"/>
       <c r="N8" s="8" t="n">
-        <v>19400</v>
+        <v>4680</v>
       </c>
       <c r="O8" s="8" t="n">
         <v>0</v>
@@ -17488,12 +17490,12 @@
       <c r="P8" s="8" t="n"/>
       <c r="Q8" s="8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="R8" s="8" t="inlineStr">
         <is>
-          <t>Taylors Lettings, Bradley Stoke</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S8" s="9" t="inlineStr">
@@ -17514,7 +17516,7 @@
       <c r="V8" s="7" t="inlineStr"/>
       <c r="W8" s="8" t="inlineStr">
         <is>
-          <t>81712a02a3a8827c0a71232c3b582e0d2b990a2a</t>
+          <t>ec80bfb810dff72d9cbd21b8e12b70951ce557a7</t>
         </is>
       </c>
     </row>
@@ -17528,7 +17530,7 @@
         </is>
       </c>
       <c r="C9" s="17" t="n">
-        <v>1900</v>
+        <v>2170</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>2</v>
@@ -17543,23 +17545,23 @@
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>Arnos Vale, Paintworks, BS4</t>
+          <t>522 Rosewood, Box Makers Yard, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>BS4</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I9" s="8" t="n">
-        <v>783</v>
+        <v>799</v>
       </c>
       <c r="J9" s="8" t="n"/>
       <c r="K9" s="8" t="n"/>
       <c r="L9" s="8" t="n"/>
       <c r="M9" s="8" t="n"/>
       <c r="N9" s="8" t="n">
-        <v>4680</v>
+        <v>20800</v>
       </c>
       <c r="O9" s="8" t="n">
         <v>0</v>
@@ -17567,12 +17569,12 @@
       <c r="P9" s="8" t="n"/>
       <c r="Q9" s="8" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R9" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S9" s="9" t="inlineStr">
@@ -17593,7 +17595,7 @@
       <c r="V9" s="7" t="inlineStr"/>
       <c r="W9" s="8" t="inlineStr">
         <is>
-          <t>ec80bfb810dff72d9cbd21b8e12b70951ce557a7</t>
+          <t>c0573087585d4e3e5716cf3f127e0ed418364345</t>
         </is>
       </c>
     </row>
@@ -17607,7 +17609,7 @@
         </is>
       </c>
       <c r="C10" s="17" t="n">
-        <v>2170</v>
+        <v>2195</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>2</v>
@@ -17622,7 +17624,7 @@
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>522 Rosewood, Box Makers Yard, New Kingsley Road, Bristol, BS2</t>
+          <t>802 Rosewood, Box Makers Yard, New Kingsley Road, Bristol, BS2 0GJ</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
@@ -17631,7 +17633,7 @@
         </is>
       </c>
       <c r="I10" s="8" t="n">
-        <v>799</v>
+        <v>809</v>
       </c>
       <c r="J10" s="8" t="n"/>
       <c r="K10" s="8" t="n"/>
@@ -17672,7 +17674,7 @@
       <c r="V10" s="7" t="inlineStr"/>
       <c r="W10" s="8" t="inlineStr">
         <is>
-          <t>c0573087585d4e3e5716cf3f127e0ed418364345</t>
+          <t>ad6f591658988c13d13881686e197fa878817439</t>
         </is>
       </c>
     </row>
@@ -17686,7 +17688,7 @@
         </is>
       </c>
       <c r="C11" s="17" t="n">
-        <v>2195</v>
+        <v>1995</v>
       </c>
       <c r="D11" s="8" t="n">
         <v>2</v>
@@ -17701,23 +17703,21 @@
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>802 Rosewood, Box Makers Yard, New Kingsley Road, Bristol, BS2 0GJ</t>
+          <t>Sugar House, French Yard, City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I11" s="8" t="n">
-        <v>809</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="n"/>
       <c r="J11" s="8" t="n"/>
       <c r="K11" s="8" t="n"/>
       <c r="L11" s="8" t="n"/>
       <c r="M11" s="8" t="n"/>
       <c r="N11" s="8" t="n">
-        <v>20800</v>
+        <v>18544</v>
       </c>
       <c r="O11" s="8" t="n">
         <v>0</v>
@@ -17730,7 +17730,7 @@
       </c>
       <c r="R11" s="8" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S11" s="9" t="inlineStr">
@@ -17751,7 +17751,7 @@
       <c r="V11" s="7" t="inlineStr"/>
       <c r="W11" s="8" t="inlineStr">
         <is>
-          <t>ad6f591658988c13d13881686e197fa878817439</t>
+          <t>f829bfa651ebc050b5c2fa24aea7bca4147d62c3</t>
         </is>
       </c>
     </row>
@@ -17765,13 +17765,13 @@
         </is>
       </c>
       <c r="C12" s="17" t="n">
-        <v>1995</v>
+        <v>1450</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
@@ -17780,21 +17780,23 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>Sugar House, French Yard, City Centre, Bristol, BS1</t>
+          <t>Bedminster, Berkeley Place, BS3</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I12" s="8" t="n"/>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>7685</v>
+      </c>
       <c r="J12" s="8" t="n"/>
       <c r="K12" s="8" t="n"/>
       <c r="L12" s="8" t="n"/>
       <c r="M12" s="8" t="n"/>
       <c r="N12" s="8" t="n">
-        <v>18544</v>
+        <v>7648</v>
       </c>
       <c r="O12" s="8" t="n">
         <v>0</v>
@@ -17807,7 +17809,7 @@
       </c>
       <c r="R12" s="8" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S12" s="9" t="inlineStr">
@@ -17828,7 +17830,7 @@
       <c r="V12" s="7" t="inlineStr"/>
       <c r="W12" s="8" t="inlineStr">
         <is>
-          <t>f829bfa651ebc050b5c2fa24aea7bca4147d62c3</t>
+          <t>4855da62cb452e8973968307d05f937e5ab76b6c</t>
         </is>
       </c>
     </row>
@@ -17842,10 +17844,10 @@
         </is>
       </c>
       <c r="C13" s="17" t="n">
-        <v>1450</v>
+        <v>1655</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" s="8" t="n">
         <v>1</v>
@@ -17857,23 +17859,23 @@
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>Bedminster, Berkeley Place, BS3</t>
+          <t>New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>BS3</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I13" s="8" t="n">
-        <v>7685</v>
+        <v>547</v>
       </c>
       <c r="J13" s="8" t="n"/>
       <c r="K13" s="8" t="n"/>
       <c r="L13" s="8" t="n"/>
       <c r="M13" s="8" t="n"/>
       <c r="N13" s="8" t="n">
-        <v>7648</v>
+        <v>20800</v>
       </c>
       <c r="O13" s="8" t="n">
         <v>0</v>
@@ -17881,12 +17883,12 @@
       <c r="P13" s="8" t="n"/>
       <c r="Q13" s="8" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R13" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S13" s="9" t="inlineStr">
@@ -17907,7 +17909,7 @@
       <c r="V13" s="7" t="inlineStr"/>
       <c r="W13" s="8" t="inlineStr">
         <is>
-          <t>4855da62cb452e8973968307d05f937e5ab76b6c</t>
+          <t>1f8489d296d842011bdf7a2ca1f952e6b948c3d3</t>
         </is>
       </c>
     </row>
@@ -17921,13 +17923,13 @@
         </is>
       </c>
       <c r="C14" s="17" t="n">
-        <v>1655</v>
+        <v>2500</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
@@ -17936,23 +17938,21 @@
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>New Kingsley Road, Bristol, BS2</t>
+          <t>Electricity House, Colston Avenue, BS1</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I14" s="8" t="n">
-        <v>547</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="n"/>
       <c r="J14" s="8" t="n"/>
       <c r="K14" s="8" t="n"/>
       <c r="L14" s="8" t="n"/>
       <c r="M14" s="8" t="n"/>
       <c r="N14" s="8" t="n">
-        <v>20800</v>
+        <v>21876</v>
       </c>
       <c r="O14" s="8" t="n">
         <v>0</v>
@@ -17965,7 +17965,7 @@
       </c>
       <c r="R14" s="8" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S14" s="9" t="inlineStr">
@@ -17986,7 +17986,7 @@
       <c r="V14" s="7" t="inlineStr"/>
       <c r="W14" s="8" t="inlineStr">
         <is>
-          <t>1f8489d296d842011bdf7a2ca1f952e6b948c3d3</t>
+          <t>b2e83643f78121776465be4134c64aa64f0141c3</t>
         </is>
       </c>
     </row>
@@ -18000,13 +18000,13 @@
         </is>
       </c>
       <c r="C15" s="17" t="n">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
@@ -18015,7 +18015,7 @@
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>Electricity House, Colston Avenue, BS1</t>
+          <t>The Crescent, Hannover Quay, BS1</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
@@ -18029,7 +18029,7 @@
       <c r="L15" s="8" t="n"/>
       <c r="M15" s="8" t="n"/>
       <c r="N15" s="8" t="n">
-        <v>21876</v>
+        <v>16232</v>
       </c>
       <c r="O15" s="8" t="n">
         <v>0</v>
@@ -18063,7 +18063,7 @@
       <c r="V15" s="7" t="inlineStr"/>
       <c r="W15" s="8" t="inlineStr">
         <is>
-          <t>b2e83643f78121776465be4134c64aa64f0141c3</t>
+          <t>6bb8673e1999d1e987f72fb4720f3d7b072fa45e</t>
         </is>
       </c>
     </row>
@@ -18077,13 +18077,13 @@
         </is>
       </c>
       <c r="C16" s="17" t="n">
-        <v>1500</v>
+        <v>1850</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
@@ -18092,7 +18092,7 @@
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>The Crescent, Hannover Quay, BS1</t>
+          <t>Park Row, Bristol, BS1</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
@@ -18100,26 +18100,26 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I16" s="8" t="n"/>
+      <c r="I16" s="8" t="n">
+        <v>797</v>
+      </c>
       <c r="J16" s="8" t="n"/>
       <c r="K16" s="8" t="n"/>
       <c r="L16" s="8" t="n"/>
       <c r="M16" s="8" t="n"/>
-      <c r="N16" s="8" t="n">
-        <v>16232</v>
-      </c>
+      <c r="N16" s="8" t="n"/>
       <c r="O16" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P16" s="8" t="n"/>
       <c r="Q16" s="8" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="R16" s="8" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>CJ Hole, Bishopston</t>
         </is>
       </c>
       <c r="S16" s="9" t="inlineStr">
@@ -18140,7 +18140,7 @@
       <c r="V16" s="7" t="inlineStr"/>
       <c r="W16" s="8" t="inlineStr">
         <is>
-          <t>6bb8673e1999d1e987f72fb4720f3d7b072fa45e</t>
+          <t>50b953f0114e0c02556c27be640db0024cba0be6</t>
         </is>
       </c>
     </row>
@@ -18154,13 +18154,13 @@
         </is>
       </c>
       <c r="C17" s="17" t="n">
-        <v>1495</v>
+        <v>2975</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
@@ -18169,21 +18169,23 @@
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>Baldwin Street, Bristol, Somerset, BS1</t>
+          <t>Capricorn Place, Hotwells</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I17" s="8" t="n"/>
+          <t>BS8</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="n">
+        <v>1615</v>
+      </c>
       <c r="J17" s="8" t="n"/>
       <c r="K17" s="8" t="n"/>
       <c r="L17" s="8" t="n"/>
       <c r="M17" s="8" t="n"/>
       <c r="N17" s="8" t="n">
-        <v>20848</v>
+        <v>15104</v>
       </c>
       <c r="O17" s="8" t="n">
         <v>0</v>
@@ -18191,12 +18193,12 @@
       <c r="P17" s="8" t="n"/>
       <c r="Q17" s="8" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="R17" s="8" t="inlineStr">
         <is>
-          <t>Romans, Clifton</t>
+          <t>Sarah Kenny Residential Lettings, Bristol</t>
         </is>
       </c>
       <c r="S17" s="9" t="inlineStr">
@@ -18217,7 +18219,7 @@
       <c r="V17" s="7" t="inlineStr"/>
       <c r="W17" s="8" t="inlineStr">
         <is>
-          <t>21a50ee847cce4668d3bf6b9117fdfe0f1917533</t>
+          <t>24fea285cbc5f197ed72b50a372f175ddb5fa732</t>
         </is>
       </c>
     </row>
@@ -18231,7 +18233,7 @@
         </is>
       </c>
       <c r="C18" s="17" t="n">
-        <v>1850</v>
+        <v>2000</v>
       </c>
       <c r="D18" s="8" t="n">
         <v>2</v>
@@ -18246,7 +18248,7 @@
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>Park Row, Bristol, BS1</t>
+          <t>Horizon - City Centre</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
@@ -18254,31 +18256,31 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I18" s="8" t="n">
-        <v>797</v>
-      </c>
+      <c r="I18" s="8" t="n"/>
       <c r="J18" s="8" t="n"/>
       <c r="K18" s="8" t="n"/>
       <c r="L18" s="8" t="n"/>
       <c r="M18" s="8" t="n"/>
-      <c r="N18" s="8" t="n"/>
+      <c r="N18" s="8" t="n">
+        <v>22020</v>
+      </c>
       <c r="O18" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P18" s="8" t="n"/>
       <c r="Q18" s="8" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R18" s="8" t="inlineStr">
         <is>
-          <t>CJ Hole, Bishopston</t>
+          <t>Ocean, Clifton</t>
         </is>
       </c>
       <c r="S18" s="9" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T18" s="12" t="inlineStr">
@@ -18294,7 +18296,7 @@
       <c r="V18" s="7" t="inlineStr"/>
       <c r="W18" s="8" t="inlineStr">
         <is>
-          <t>50b953f0114e0c02556c27be640db0024cba0be6</t>
+          <t>8988913a4580793e64d3ae8351174e2d71317d16</t>
         </is>
       </c>
     </row>
@@ -18308,13 +18310,13 @@
         </is>
       </c>
       <c r="C19" s="17" t="n">
-        <v>2975</v>
+        <v>1400</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
@@ -18323,23 +18325,21 @@
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>Capricorn Place, Hotwells</t>
+          <t>The Crescent, Harbourside, Bristol</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>BS8</t>
-        </is>
-      </c>
-      <c r="I19" s="8" t="n">
-        <v>1615</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="n"/>
       <c r="J19" s="8" t="n"/>
       <c r="K19" s="8" t="n"/>
       <c r="L19" s="8" t="n"/>
       <c r="M19" s="8" t="n"/>
       <c r="N19" s="8" t="n">
-        <v>15104</v>
+        <v>16368</v>
       </c>
       <c r="O19" s="8" t="n">
         <v>0</v>
@@ -18347,12 +18347,12 @@
       <c r="P19" s="8" t="n"/>
       <c r="Q19" s="8" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R19" s="8" t="inlineStr">
         <is>
-          <t>Sarah Kenny Residential Lettings, Bristol</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S19" s="9" t="inlineStr">
@@ -18373,7 +18373,7 @@
       <c r="V19" s="7" t="inlineStr"/>
       <c r="W19" s="8" t="inlineStr">
         <is>
-          <t>24fea285cbc5f197ed72b50a372f175ddb5fa732</t>
+          <t>59af10441dff618517a35c62d6a67a8485c2f2fa</t>
         </is>
       </c>
     </row>
@@ -18387,7 +18387,7 @@
         </is>
       </c>
       <c r="C20" s="17" t="n">
-        <v>2000</v>
+        <v>1900</v>
       </c>
       <c r="D20" s="8" t="n">
         <v>2</v>
@@ -18402,7 +18402,7 @@
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>Horizon - City Centre</t>
+          <t>51.02 - St James Barton</t>
         </is>
       </c>
       <c r="H20" s="8" t="inlineStr">
@@ -18416,7 +18416,7 @@
       <c r="L20" s="8" t="n"/>
       <c r="M20" s="8" t="n"/>
       <c r="N20" s="8" t="n">
-        <v>22020</v>
+        <v>22132</v>
       </c>
       <c r="O20" s="8" t="n">
         <v>0</v>
@@ -18434,7 +18434,7 @@
       </c>
       <c r="S20" s="9" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T20" s="12" t="inlineStr">
@@ -18450,7 +18450,7 @@
       <c r="V20" s="7" t="inlineStr"/>
       <c r="W20" s="8" t="inlineStr">
         <is>
-          <t>8988913a4580793e64d3ae8351174e2d71317d16</t>
+          <t>1d421f07eb2d142471d3e293f8cb751813656c56</t>
         </is>
       </c>
     </row>
@@ -18464,13 +18464,13 @@
         </is>
       </c>
       <c r="C21" s="17" t="n">
-        <v>1400</v>
+        <v>1700</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
@@ -18479,7 +18479,7 @@
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>The Crescent, Harbourside, Bristol</t>
+          <t>Steamship House, Gas Ferry Road, BS1</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
@@ -18493,7 +18493,7 @@
       <c r="L21" s="8" t="n"/>
       <c r="M21" s="8" t="n"/>
       <c r="N21" s="8" t="n">
-        <v>16368</v>
+        <v>14420</v>
       </c>
       <c r="O21" s="8" t="n">
         <v>0</v>
@@ -18501,7 +18501,7 @@
       <c r="P21" s="8" t="n"/>
       <c r="Q21" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R21" s="8" t="inlineStr">
@@ -18527,7 +18527,7 @@
       <c r="V21" s="7" t="inlineStr"/>
       <c r="W21" s="8" t="inlineStr">
         <is>
-          <t>59af10441dff618517a35c62d6a67a8485c2f2fa</t>
+          <t>f7b6312c22af08d7f7e765adf92d9a3fb0f82781</t>
         </is>
       </c>
     </row>
@@ -18541,7 +18541,7 @@
         </is>
       </c>
       <c r="C22" s="17" t="n">
-        <v>1900</v>
+        <v>1950</v>
       </c>
       <c r="D22" s="8" t="n">
         <v>2</v>
@@ -18556,7 +18556,7 @@
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>51.02 - St James Barton</t>
+          <t>Harbourside, The Crescent, BS1 5JP</t>
         </is>
       </c>
       <c r="H22" s="8" t="inlineStr">
@@ -18564,13 +18564,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I22" s="8" t="n"/>
+      <c r="I22" s="8" t="n">
+        <v>969</v>
+      </c>
       <c r="J22" s="8" t="n"/>
       <c r="K22" s="8" t="n"/>
       <c r="L22" s="8" t="n"/>
       <c r="M22" s="8" t="n"/>
       <c r="N22" s="8" t="n">
-        <v>22132</v>
+        <v>16368</v>
       </c>
       <c r="O22" s="8" t="n">
         <v>0</v>
@@ -18578,12 +18580,12 @@
       <c r="P22" s="8" t="n"/>
       <c r="Q22" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R22" s="8" t="inlineStr">
         <is>
-          <t>Ocean, Clifton</t>
+          <t>The Bristol Residential Letting Co, Clifton</t>
         </is>
       </c>
       <c r="S22" s="9" t="inlineStr">
@@ -18604,7 +18606,7 @@
       <c r="V22" s="7" t="inlineStr"/>
       <c r="W22" s="8" t="inlineStr">
         <is>
-          <t>1d421f07eb2d142471d3e293f8cb751813656c56</t>
+          <t>384c19ad899eb10f0c99305f716bbf9cc2030cb0</t>
         </is>
       </c>
     </row>
@@ -18618,13 +18620,13 @@
         </is>
       </c>
       <c r="C23" s="17" t="n">
-        <v>1700</v>
+        <v>1350</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
@@ -18633,7 +18635,7 @@
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>Steamship House, Gas Ferry Road, BS1</t>
+          <t>Millennium Promenade, Bristol, BS1</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
@@ -18641,13 +18643,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I23" s="8" t="n"/>
+      <c r="I23" s="8" t="n">
+        <v>491</v>
+      </c>
       <c r="J23" s="8" t="n"/>
       <c r="K23" s="8" t="n"/>
       <c r="L23" s="8" t="n"/>
       <c r="M23" s="8" t="n"/>
       <c r="N23" s="8" t="n">
-        <v>14420</v>
+        <v>17096</v>
       </c>
       <c r="O23" s="8" t="n">
         <v>0</v>
@@ -18660,7 +18664,7 @@
       </c>
       <c r="R23" s="8" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>A2Dominion Group, A2Dominion Lettings</t>
         </is>
       </c>
       <c r="S23" s="9" t="inlineStr">
@@ -18681,7 +18685,7 @@
       <c r="V23" s="7" t="inlineStr"/>
       <c r="W23" s="8" t="inlineStr">
         <is>
-          <t>f7b6312c22af08d7f7e765adf92d9a3fb0f82781</t>
+          <t>3ab86f4fbffd37f02afac44cadd6ec8a27da6f0a</t>
         </is>
       </c>
     </row>
@@ -18695,7 +18699,7 @@
         </is>
       </c>
       <c r="C24" s="17" t="n">
-        <v>1950</v>
+        <v>2000</v>
       </c>
       <c r="D24" s="8" t="n">
         <v>2</v>
@@ -18710,7 +18714,7 @@
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>Harbourside, The Crescent, BS1 5JP</t>
+          <t>Caledonian Road, Bristol, BS1</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr">
@@ -18718,15 +18722,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I24" s="8" t="n">
-        <v>969</v>
-      </c>
+      <c r="I24" s="8" t="n"/>
       <c r="J24" s="8" t="n"/>
       <c r="K24" s="8" t="n"/>
       <c r="L24" s="8" t="n"/>
       <c r="M24" s="8" t="n"/>
       <c r="N24" s="8" t="n">
-        <v>16368</v>
+        <v>14632</v>
       </c>
       <c r="O24" s="8" t="n">
         <v>0</v>
@@ -18739,7 +18741,7 @@
       </c>
       <c r="R24" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Clifton</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S24" s="9" t="inlineStr">
@@ -18760,7 +18762,7 @@
       <c r="V24" s="7" t="inlineStr"/>
       <c r="W24" s="8" t="inlineStr">
         <is>
-          <t>384c19ad899eb10f0c99305f716bbf9cc2030cb0</t>
+          <t>9a270cf54e31627246aef21daa26a60bb5f977ad</t>
         </is>
       </c>
     </row>
@@ -18774,13 +18776,13 @@
         </is>
       </c>
       <c r="C25" s="17" t="n">
-        <v>1350</v>
+        <v>1650</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
@@ -18789,23 +18791,21 @@
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>Millennium Promenade, Bristol, BS1</t>
+          <t>Sweetman Place, Bristol, BS2</t>
         </is>
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I25" s="8" t="n">
-        <v>491</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="n"/>
       <c r="J25" s="8" t="n"/>
       <c r="K25" s="8" t="n"/>
       <c r="L25" s="8" t="n"/>
       <c r="M25" s="8" t="n"/>
       <c r="N25" s="8" t="n">
-        <v>17096</v>
+        <v>20416</v>
       </c>
       <c r="O25" s="8" t="n">
         <v>0</v>
@@ -18818,7 +18818,7 @@
       </c>
       <c r="R25" s="8" t="inlineStr">
         <is>
-          <t>A2Dominion Group, A2Dominion Lettings</t>
+          <t>Andrews Letting and Management, Clifton</t>
         </is>
       </c>
       <c r="S25" s="9" t="inlineStr">
@@ -18839,7 +18839,7 @@
       <c r="V25" s="7" t="inlineStr"/>
       <c r="W25" s="8" t="inlineStr">
         <is>
-          <t>3ab86f4fbffd37f02afac44cadd6ec8a27da6f0a</t>
+          <t>54fa42ef8d0349a295f45392644c43dec3321c5b</t>
         </is>
       </c>
     </row>
@@ -18853,13 +18853,13 @@
         </is>
       </c>
       <c r="C26" s="17" t="n">
-        <v>2000</v>
+        <v>1200</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
@@ -18868,7 +18868,7 @@
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>Caledonian Road, Bristol, BS1</t>
+          <t>City Centre, Corinthian Court, BS1</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">
@@ -18876,13 +18876,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I26" s="8" t="n"/>
+      <c r="I26" s="8" t="n">
+        <v>389</v>
+      </c>
       <c r="J26" s="8" t="n"/>
       <c r="K26" s="8" t="n"/>
       <c r="L26" s="8" t="n"/>
       <c r="M26" s="8" t="n"/>
       <c r="N26" s="8" t="n">
-        <v>14632</v>
+        <v>18820</v>
       </c>
       <c r="O26" s="8" t="n">
         <v>0</v>
@@ -18890,12 +18892,12 @@
       <c r="P26" s="8" t="n"/>
       <c r="Q26" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="R26" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S26" s="9" t="inlineStr">
@@ -18916,7 +18918,7 @@
       <c r="V26" s="7" t="inlineStr"/>
       <c r="W26" s="8" t="inlineStr">
         <is>
-          <t>9a270cf54e31627246aef21daa26a60bb5f977ad</t>
+          <t>5aed40eba285a7fa0266bfe8eb49613bb2f96c97</t>
         </is>
       </c>
     </row>
@@ -18930,13 +18932,13 @@
         </is>
       </c>
       <c r="C27" s="17" t="n">
-        <v>1650</v>
+        <v>1500</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
@@ -18945,21 +18947,23 @@
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>Sweetman Place, Bristol, BS2</t>
+          <t>Harbourside, Steamship House, BS1 6GL</t>
         </is>
       </c>
       <c r="H27" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I27" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="n">
+        <v>506</v>
+      </c>
       <c r="J27" s="8" t="n"/>
       <c r="K27" s="8" t="n"/>
       <c r="L27" s="8" t="n"/>
       <c r="M27" s="8" t="n"/>
       <c r="N27" s="8" t="n">
-        <v>20416</v>
+        <v>14420</v>
       </c>
       <c r="O27" s="8" t="n">
         <v>0</v>
@@ -18967,12 +18971,12 @@
       <c r="P27" s="8" t="n"/>
       <c r="Q27" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="R27" s="8" t="inlineStr">
         <is>
-          <t>Andrews Letting and Management, Clifton</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S27" s="9" t="inlineStr">
@@ -18993,7 +18997,7 @@
       <c r="V27" s="7" t="inlineStr"/>
       <c r="W27" s="8" t="inlineStr">
         <is>
-          <t>54fa42ef8d0349a295f45392644c43dec3321c5b</t>
+          <t>bf329b73db0d1de077d78cddc284f1017fcfc43a</t>
         </is>
       </c>
     </row>
@@ -19007,7 +19011,7 @@
         </is>
       </c>
       <c r="C28" s="17" t="n">
-        <v>1200</v>
+        <v>1400</v>
       </c>
       <c r="D28" s="8" t="n">
         <v>1</v>
@@ -19022,7 +19026,7 @@
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>City Centre, Corinthian Court, BS1</t>
+          <t>St. James Barton, Bristol, Somerset, BS1</t>
         </is>
       </c>
       <c r="H28" s="8" t="inlineStr">
@@ -19030,15 +19034,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I28" s="8" t="n">
-        <v>389</v>
-      </c>
+      <c r="I28" s="8" t="n"/>
       <c r="J28" s="8" t="n"/>
       <c r="K28" s="8" t="n"/>
       <c r="L28" s="8" t="n"/>
       <c r="M28" s="8" t="n"/>
       <c r="N28" s="8" t="n">
-        <v>18820</v>
+        <v>22132</v>
       </c>
       <c r="O28" s="8" t="n">
         <v>0</v>
@@ -19051,7 +19053,7 @@
       </c>
       <c r="R28" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Balloon Letting Company, Bristol</t>
         </is>
       </c>
       <c r="S28" s="9" t="inlineStr">
@@ -19072,7 +19074,7 @@
       <c r="V28" s="7" t="inlineStr"/>
       <c r="W28" s="8" t="inlineStr">
         <is>
-          <t>5aed40eba285a7fa0266bfe8eb49613bb2f96c97</t>
+          <t>f2c75a0f99c7c358be96a67019a6c639e60845fb</t>
         </is>
       </c>
     </row>
@@ -19086,38 +19088,36 @@
         </is>
       </c>
       <c r="C29" s="17" t="n">
-        <v>1500</v>
+        <v>3750</v>
       </c>
       <c r="D29" s="8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E29" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>Harbourside, Steamship House, BS1 6GL</t>
+          <t>Dove Street, Bristol, BS2</t>
         </is>
       </c>
       <c r="H29" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I29" s="8" t="n">
-        <v>506</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="n"/>
       <c r="J29" s="8" t="n"/>
       <c r="K29" s="8" t="n"/>
       <c r="L29" s="8" t="n"/>
       <c r="M29" s="8" t="n"/>
       <c r="N29" s="8" t="n">
-        <v>14420</v>
+        <v>21288</v>
       </c>
       <c r="O29" s="8" t="n">
         <v>0</v>
@@ -19130,12 +19130,12 @@
       </c>
       <c r="R29" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Phoenix Property Company, Bristol</t>
         </is>
       </c>
       <c r="S29" s="9" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T29" s="12" t="inlineStr">
@@ -19151,7 +19151,7 @@
       <c r="V29" s="7" t="inlineStr"/>
       <c r="W29" s="8" t="inlineStr">
         <is>
-          <t>bf329b73db0d1de077d78cddc284f1017fcfc43a</t>
+          <t>1bcb0667c3a3efe864816ea971273f0e1ff48f01</t>
         </is>
       </c>
     </row>
@@ -19165,7 +19165,7 @@
         </is>
       </c>
       <c r="C30" s="17" t="n">
-        <v>1400</v>
+        <v>1300</v>
       </c>
       <c r="D30" s="8" t="n">
         <v>1</v>
@@ -19180,7 +19180,7 @@
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>St. James Barton, Bristol, Somerset, BS1</t>
+          <t>Three Queens Lane, Bristol, BS1</t>
         </is>
       </c>
       <c r="H30" s="8" t="inlineStr">
@@ -19194,7 +19194,7 @@
       <c r="L30" s="8" t="n"/>
       <c r="M30" s="8" t="n"/>
       <c r="N30" s="8" t="n">
-        <v>22132</v>
+        <v>20608</v>
       </c>
       <c r="O30" s="8" t="n">
         <v>0</v>
@@ -19202,12 +19202,12 @@
       <c r="P30" s="8" t="n"/>
       <c r="Q30" s="8" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
-          <t>Balloon Letting Company, Bristol</t>
+          <t>Romans, Clifton</t>
         </is>
       </c>
       <c r="S30" s="9" t="inlineStr">
@@ -19228,7 +19228,7 @@
       <c r="V30" s="7" t="inlineStr"/>
       <c r="W30" s="8" t="inlineStr">
         <is>
-          <t>f2c75a0f99c7c358be96a67019a6c639e60845fb</t>
+          <t>7c9f52e17d949cd3dc79f3eb8c1020a81c729d66</t>
         </is>
       </c>
     </row>
@@ -19242,27 +19242,27 @@
         </is>
       </c>
       <c r="C31" s="17" t="n">
-        <v>3750</v>
+        <v>1300</v>
       </c>
       <c r="D31" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>Dove Street, Bristol, BS2</t>
+          <t>St. Johns Lane, Bedminster, BS3</t>
         </is>
       </c>
       <c r="H31" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS3</t>
         </is>
       </c>
       <c r="I31" s="8" t="n"/>
@@ -19271,7 +19271,7 @@
       <c r="L31" s="8" t="n"/>
       <c r="M31" s="8" t="n"/>
       <c r="N31" s="8" t="n">
-        <v>21288</v>
+        <v>7112</v>
       </c>
       <c r="O31" s="8" t="n">
         <v>0</v>
@@ -19279,12 +19279,12 @@
       <c r="P31" s="8" t="n"/>
       <c r="Q31" s="8" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
-          <t>Phoenix Property Company, Bristol</t>
+          <t>Taylors Lettings, Bedminster</t>
         </is>
       </c>
       <c r="S31" s="9" t="inlineStr">
@@ -19305,7 +19305,7 @@
       <c r="V31" s="7" t="inlineStr"/>
       <c r="W31" s="8" t="inlineStr">
         <is>
-          <t>1bcb0667c3a3efe864816ea971273f0e1ff48f01</t>
+          <t>91339ed58a9e4347ac017823b498695129a40922</t>
         </is>
       </c>
     </row>
@@ -19319,7 +19319,7 @@
         </is>
       </c>
       <c r="C32" s="17" t="n">
-        <v>1300</v>
+        <v>1495</v>
       </c>
       <c r="D32" s="8" t="n">
         <v>1</v>
@@ -19334,7 +19334,7 @@
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>Three Queens Lane, Bristol, BS1</t>
+          <t>Baldwin Street, Bristol, Somerset, BS1</t>
         </is>
       </c>
       <c r="H32" s="8" t="inlineStr">
@@ -19348,7 +19348,7 @@
       <c r="L32" s="8" t="n"/>
       <c r="M32" s="8" t="n"/>
       <c r="N32" s="8" t="n">
-        <v>20608</v>
+        <v>20848</v>
       </c>
       <c r="O32" s="8" t="n">
         <v>0</v>
@@ -19356,7 +19356,7 @@
       <c r="P32" s="8" t="n"/>
       <c r="Q32" s="8" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="R32" s="8" t="inlineStr">
@@ -19382,7 +19382,7 @@
       <c r="V32" s="7" t="inlineStr"/>
       <c r="W32" s="8" t="inlineStr">
         <is>
-          <t>7c9f52e17d949cd3dc79f3eb8c1020a81c729d66</t>
+          <t>21a50ee847cce4668d3bf6b9117fdfe0f1917533</t>
         </is>
       </c>
     </row>
@@ -24383,7 +24383,7 @@
         </is>
       </c>
       <c r="C100" s="17" t="n">
-        <v>1600</v>
+        <v>2145</v>
       </c>
       <c r="D100" s="8" t="n">
         <v>2</v>
@@ -24398,21 +24398,23 @@
       </c>
       <c r="G100" s="9" t="inlineStr">
         <is>
-          <t>Ratcliffe Court, Bristol, BS2</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H100" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I100" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I100" s="8" t="n">
+        <v>796</v>
+      </c>
       <c r="J100" s="8" t="n"/>
       <c r="K100" s="8" t="n"/>
       <c r="L100" s="8" t="n"/>
       <c r="M100" s="8" t="n"/>
       <c r="N100" s="8" t="n">
-        <v>20124</v>
+        <v>20820</v>
       </c>
       <c r="O100" s="8" t="n">
         <v>0</v>
@@ -24420,12 +24422,12 @@
       <c r="P100" s="8" t="n"/>
       <c r="Q100" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R100" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S100" s="9" t="inlineStr"/>
@@ -24442,7 +24444,7 @@
       <c r="V100" s="7" t="inlineStr"/>
       <c r="W100" s="8" t="inlineStr">
         <is>
-          <t>e9219c4f68722ad3bdeee0c4c4cb31134f26af57</t>
+          <t>898ba227d5b949e4e7f18b49536b3c908560d145</t>
         </is>
       </c>
     </row>
@@ -24456,13 +24458,13 @@
         </is>
       </c>
       <c r="C101" s="17" t="n">
-        <v>2145</v>
+        <v>1999</v>
       </c>
       <c r="D101" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E101" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F101" s="8" t="inlineStr">
         <is>
@@ -24471,7 +24473,7 @@
       </c>
       <c r="G101" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Swann House, Bristol, BS1</t>
         </is>
       </c>
       <c r="H101" s="8" t="inlineStr">
@@ -24479,15 +24481,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I101" s="8" t="n">
-        <v>796</v>
-      </c>
+      <c r="I101" s="8" t="n"/>
       <c r="J101" s="8" t="n"/>
       <c r="K101" s="8" t="n"/>
       <c r="L101" s="8" t="n"/>
       <c r="M101" s="8" t="n"/>
       <c r="N101" s="8" t="n">
-        <v>20820</v>
+        <v>20800</v>
       </c>
       <c r="O101" s="8" t="n">
         <v>0</v>
@@ -24500,7 +24500,7 @@
       </c>
       <c r="R101" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S101" s="9" t="inlineStr"/>
@@ -24517,7 +24517,7 @@
       <c r="V101" s="7" t="inlineStr"/>
       <c r="W101" s="8" t="inlineStr">
         <is>
-          <t>898ba227d5b949e4e7f18b49536b3c908560d145</t>
+          <t>5cec67aa8ba885c4c8f85e47d3354d187da9d897</t>
         </is>
       </c>
     </row>
@@ -24531,10 +24531,10 @@
         </is>
       </c>
       <c r="C102" s="17" t="n">
-        <v>1999</v>
+        <v>1670</v>
       </c>
       <c r="D102" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E102" s="8" t="n">
         <v>1</v>
@@ -24546,7 +24546,7 @@
       </c>
       <c r="G102" s="9" t="inlineStr">
         <is>
-          <t>Swann House, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H102" s="8" t="inlineStr">
@@ -24554,13 +24554,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I102" s="8" t="n"/>
+      <c r="I102" s="8" t="n">
+        <v>485</v>
+      </c>
       <c r="J102" s="8" t="n"/>
       <c r="K102" s="8" t="n"/>
       <c r="L102" s="8" t="n"/>
       <c r="M102" s="8" t="n"/>
       <c r="N102" s="8" t="n">
-        <v>20800</v>
+        <v>21504</v>
       </c>
       <c r="O102" s="8" t="n">
         <v>0</v>
@@ -24573,7 +24575,7 @@
       </c>
       <c r="R102" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S102" s="9" t="inlineStr"/>
@@ -24590,7 +24592,7 @@
       <c r="V102" s="7" t="inlineStr"/>
       <c r="W102" s="8" t="inlineStr">
         <is>
-          <t>5cec67aa8ba885c4c8f85e47d3354d187da9d897</t>
+          <t>73f3509a6c69eef7af4c6b9ff0dc69b97478c20a</t>
         </is>
       </c>
     </row>
@@ -24604,7 +24606,7 @@
         </is>
       </c>
       <c r="C103" s="17" t="n">
-        <v>1670</v>
+        <v>1645</v>
       </c>
       <c r="D103" s="8" t="n">
         <v>1</v>
@@ -24619,7 +24621,7 @@
       </c>
       <c r="G103" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H103" s="8" t="inlineStr">
@@ -24628,14 +24630,14 @@
         </is>
       </c>
       <c r="I103" s="8" t="n">
-        <v>485</v>
+        <v>517</v>
       </c>
       <c r="J103" s="8" t="n"/>
       <c r="K103" s="8" t="n"/>
       <c r="L103" s="8" t="n"/>
       <c r="M103" s="8" t="n"/>
       <c r="N103" s="8" t="n">
-        <v>21504</v>
+        <v>20820</v>
       </c>
       <c r="O103" s="8" t="n">
         <v>0</v>
@@ -24648,7 +24650,7 @@
       </c>
       <c r="R103" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S103" s="9" t="inlineStr"/>
@@ -24665,7 +24667,7 @@
       <c r="V103" s="7" t="inlineStr"/>
       <c r="W103" s="8" t="inlineStr">
         <is>
-          <t>73f3509a6c69eef7af4c6b9ff0dc69b97478c20a</t>
+          <t>4efcb79ae710a68f5f272a2f9030937499117f9d</t>
         </is>
       </c>
     </row>
@@ -24679,13 +24681,13 @@
         </is>
       </c>
       <c r="C104" s="17" t="n">
-        <v>1645</v>
+        <v>2120</v>
       </c>
       <c r="D104" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E104" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F104" s="8" t="inlineStr">
         <is>
@@ -24703,7 +24705,7 @@
         </is>
       </c>
       <c r="I104" s="8" t="n">
-        <v>517</v>
+        <v>705</v>
       </c>
       <c r="J104" s="8" t="n"/>
       <c r="K104" s="8" t="n"/>
@@ -24718,7 +24720,7 @@
       <c r="P104" s="8" t="n"/>
       <c r="Q104" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="R104" s="8" t="inlineStr">
@@ -24740,7 +24742,7 @@
       <c r="V104" s="7" t="inlineStr"/>
       <c r="W104" s="8" t="inlineStr">
         <is>
-          <t>4efcb79ae710a68f5f272a2f9030937499117f9d</t>
+          <t>c5c1741357dfce3547bdab7d4d5a0e7602846192</t>
         </is>
       </c>
     </row>
@@ -24754,13 +24756,13 @@
         </is>
       </c>
       <c r="C105" s="17" t="n">
-        <v>2120</v>
+        <v>1645</v>
       </c>
       <c r="D105" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E105" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F105" s="8" t="inlineStr">
         <is>
@@ -24778,7 +24780,7 @@
         </is>
       </c>
       <c r="I105" s="8" t="n">
-        <v>705</v>
+        <v>571</v>
       </c>
       <c r="J105" s="8" t="n"/>
       <c r="K105" s="8" t="n"/>
@@ -24815,7 +24817,7 @@
       <c r="V105" s="7" t="inlineStr"/>
       <c r="W105" s="8" t="inlineStr">
         <is>
-          <t>c5c1741357dfce3547bdab7d4d5a0e7602846192</t>
+          <t>487e67b2d6680ebaabfcc49d4d33e21cb65cca6d</t>
         </is>
       </c>
     </row>
@@ -24829,10 +24831,10 @@
         </is>
       </c>
       <c r="C106" s="17" t="n">
-        <v>1645</v>
+        <v>2250</v>
       </c>
       <c r="D106" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E106" s="8" t="n">
         <v>1</v>
@@ -24844,7 +24846,7 @@
       </c>
       <c r="G106" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Apartments, Bristol, BS1</t>
         </is>
       </c>
       <c r="H106" s="8" t="inlineStr">
@@ -24852,15 +24854,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I106" s="8" t="n">
-        <v>571</v>
-      </c>
+      <c r="I106" s="8" t="n"/>
       <c r="J106" s="8" t="n"/>
       <c r="K106" s="8" t="n"/>
       <c r="L106" s="8" t="n"/>
       <c r="M106" s="8" t="n"/>
       <c r="N106" s="8" t="n">
-        <v>20820</v>
+        <v>22132</v>
       </c>
       <c r="O106" s="8" t="n">
         <v>0</v>
@@ -24873,7 +24873,7 @@
       </c>
       <c r="R106" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S106" s="9" t="inlineStr"/>
@@ -24890,7 +24890,7 @@
       <c r="V106" s="7" t="inlineStr"/>
       <c r="W106" s="8" t="inlineStr">
         <is>
-          <t>487e67b2d6680ebaabfcc49d4d33e21cb65cca6d</t>
+          <t>b3bc6f44f28301ca7ff059723f3c836424cd082f</t>
         </is>
       </c>
     </row>
@@ -24904,7 +24904,7 @@
         </is>
       </c>
       <c r="C107" s="17" t="n">
-        <v>2250</v>
+        <v>1600</v>
       </c>
       <c r="D107" s="8" t="n">
         <v>2</v>
@@ -24919,12 +24919,12 @@
       </c>
       <c r="G107" s="9" t="inlineStr">
         <is>
-          <t>Apartments, Bristol, BS1</t>
+          <t>Stapleton Road, Bristol, BS5</t>
         </is>
       </c>
       <c r="H107" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS5</t>
         </is>
       </c>
       <c r="I107" s="8" t="n"/>
@@ -24933,7 +24933,7 @@
       <c r="L107" s="8" t="n"/>
       <c r="M107" s="8" t="n"/>
       <c r="N107" s="8" t="n">
-        <v>22132</v>
+        <v>19576</v>
       </c>
       <c r="O107" s="8" t="n">
         <v>0</v>
@@ -24941,7 +24941,7 @@
       <c r="P107" s="8" t="n"/>
       <c r="Q107" s="8" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="R107" s="8" t="inlineStr">
@@ -24963,7 +24963,7 @@
       <c r="V107" s="7" t="inlineStr"/>
       <c r="W107" s="8" t="inlineStr">
         <is>
-          <t>b3bc6f44f28301ca7ff059723f3c836424cd082f</t>
+          <t>41184aca0a094a13f0cf944554fa6ab5b6f9b761</t>
         </is>
       </c>
     </row>
@@ -24983,7 +24983,7 @@
         <v>2</v>
       </c>
       <c r="E108" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F108" s="8" t="inlineStr">
         <is>
@@ -24992,12 +24992,12 @@
       </c>
       <c r="G108" s="9" t="inlineStr">
         <is>
-          <t>Stapleton Road, Bristol, BS5</t>
+          <t>Ratcliffe Court, Bristol, BS2</t>
         </is>
       </c>
       <c r="H108" s="8" t="inlineStr">
         <is>
-          <t>BS5</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I108" s="8" t="n"/>
@@ -25006,7 +25006,7 @@
       <c r="L108" s="8" t="n"/>
       <c r="M108" s="8" t="n"/>
       <c r="N108" s="8" t="n">
-        <v>19576</v>
+        <v>20124</v>
       </c>
       <c r="O108" s="8" t="n">
         <v>0</v>
@@ -25014,7 +25014,7 @@
       <c r="P108" s="8" t="n"/>
       <c r="Q108" s="8" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R108" s="8" t="inlineStr">
@@ -25036,7 +25036,7 @@
       <c r="V108" s="7" t="inlineStr"/>
       <c r="W108" s="8" t="inlineStr">
         <is>
-          <t>41184aca0a094a13f0cf944554fa6ab5b6f9b761</t>
+          <t>e9219c4f68722ad3bdeee0c4c4cb31134f26af57</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
House search data from run 21
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -19242,7 +19242,7 @@
         </is>
       </c>
       <c r="C31" s="17" t="n">
-        <v>1555</v>
+        <v>1300</v>
       </c>
       <c r="D31" s="8" t="n">
         <v>1</v>
@@ -19257,7 +19257,7 @@
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>Lombard Street, Bristol, BS3</t>
+          <t>St. Johns Lane, Bedminster, BS3</t>
         </is>
       </c>
       <c r="H31" s="8" t="inlineStr">
@@ -19271,7 +19271,7 @@
       <c r="L31" s="8" t="n"/>
       <c r="M31" s="8" t="n"/>
       <c r="N31" s="8" t="n">
-        <v>12036</v>
+        <v>7112</v>
       </c>
       <c r="O31" s="8" t="n">
         <v>0</v>
@@ -19279,12 +19279,12 @@
       <c r="P31" s="8" t="n"/>
       <c r="Q31" s="8" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Taylors Lettings, Bedminster</t>
         </is>
       </c>
       <c r="S31" s="9" t="inlineStr">
@@ -19305,7 +19305,7 @@
       <c r="V31" s="7" t="inlineStr"/>
       <c r="W31" s="8" t="inlineStr">
         <is>
-          <t>4d3990c67ed2848296e2aa2fa362730e0557bd43</t>
+          <t>91339ed58a9e4347ac017823b498695129a40922</t>
         </is>
       </c>
     </row>
@@ -19319,7 +19319,7 @@
         </is>
       </c>
       <c r="C32" s="17" t="n">
-        <v>1300</v>
+        <v>1495</v>
       </c>
       <c r="D32" s="8" t="n">
         <v>1</v>
@@ -19334,12 +19334,12 @@
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>St. Johns Lane, Bedminster, BS3</t>
+          <t>Baldwin Street, Bristol, Somerset, BS1</t>
         </is>
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>BS3</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I32" s="8" t="n"/>
@@ -19348,7 +19348,7 @@
       <c r="L32" s="8" t="n"/>
       <c r="M32" s="8" t="n"/>
       <c r="N32" s="8" t="n">
-        <v>7112</v>
+        <v>20848</v>
       </c>
       <c r="O32" s="8" t="n">
         <v>0</v>
@@ -19356,17 +19356,17 @@
       <c r="P32" s="8" t="n"/>
       <c r="Q32" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
-          <t>Taylors Lettings, Bedminster</t>
+          <t>Romans, Clifton</t>
         </is>
       </c>
       <c r="S32" s="9" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T32" s="12" t="inlineStr">
@@ -19382,7 +19382,7 @@
       <c r="V32" s="7" t="inlineStr"/>
       <c r="W32" s="8" t="inlineStr">
         <is>
-          <t>91339ed58a9e4347ac017823b498695129a40922</t>
+          <t>21a50ee847cce4668d3bf6b9117fdfe0f1917533</t>
         </is>
       </c>
     </row>
@@ -19396,7 +19396,7 @@
         </is>
       </c>
       <c r="C33" s="17" t="n">
-        <v>1495</v>
+        <v>1733</v>
       </c>
       <c r="D33" s="8" t="n">
         <v>1</v>
@@ -19411,7 +19411,7 @@
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
-          <t>Baldwin Street, Bristol, Somerset, BS1</t>
+          <t>Cheltenham House, Clare Street, Bristol</t>
         </is>
       </c>
       <c r="H33" s="8" t="inlineStr">
@@ -19419,26 +19419,26 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I33" s="8" t="n"/>
+      <c r="I33" s="8" t="n">
+        <v>455</v>
+      </c>
       <c r="J33" s="8" t="n"/>
       <c r="K33" s="8" t="n"/>
       <c r="L33" s="8" t="n"/>
       <c r="M33" s="8" t="n"/>
-      <c r="N33" s="8" t="n">
-        <v>20848</v>
-      </c>
+      <c r="N33" s="8" t="n"/>
       <c r="O33" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P33" s="8" t="n"/>
       <c r="Q33" s="8" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
-          <t>Romans, Clifton</t>
+          <t>Mariana Real Estate, London</t>
         </is>
       </c>
       <c r="S33" s="9" t="inlineStr">
@@ -19459,7 +19459,7 @@
       <c r="V33" s="7" t="inlineStr"/>
       <c r="W33" s="8" t="inlineStr">
         <is>
-          <t>21a50ee847cce4668d3bf6b9117fdfe0f1917533</t>
+          <t>7aeb8331a46bbe8acd8189d3a63f58f7e3892936</t>
         </is>
       </c>
     </row>
@@ -19473,7 +19473,7 @@
         </is>
       </c>
       <c r="C34" s="17" t="n">
-        <v>1733</v>
+        <v>1400</v>
       </c>
       <c r="D34" s="8" t="n">
         <v>1</v>
@@ -19488,7 +19488,7 @@
       </c>
       <c r="G34" s="9" t="inlineStr">
         <is>
-          <t>Cheltenham House, Clare Street, Bristol</t>
+          <t>City Centre, Number One Bristol, BS1 2NR</t>
         </is>
       </c>
       <c r="H34" s="8" t="inlineStr">
@@ -19497,30 +19497,32 @@
         </is>
       </c>
       <c r="I34" s="8" t="n">
-        <v>455</v>
+        <v>527</v>
       </c>
       <c r="J34" s="8" t="n"/>
       <c r="K34" s="8" t="n"/>
       <c r="L34" s="8" t="n"/>
       <c r="M34" s="8" t="n"/>
-      <c r="N34" s="8" t="n"/>
+      <c r="N34" s="8" t="n">
+        <v>21804</v>
+      </c>
       <c r="O34" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P34" s="8" t="n"/>
       <c r="Q34" s="8" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
-          <t>Mariana Real Estate, London</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S34" s="9" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T34" s="12" t="inlineStr">
@@ -19536,7 +19538,7 @@
       <c r="V34" s="7" t="inlineStr"/>
       <c r="W34" s="8" t="inlineStr">
         <is>
-          <t>7aeb8331a46bbe8acd8189d3a63f58f7e3892936</t>
+          <t>27b085b9bcbec967c008845a19f54e272fc12b87</t>
         </is>
       </c>
     </row>
@@ -19550,13 +19552,13 @@
         </is>
       </c>
       <c r="C35" s="17" t="n">
-        <v>1400</v>
+        <v>2200</v>
       </c>
       <c r="D35" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F35" s="8" t="inlineStr">
         <is>
@@ -19565,23 +19567,21 @@
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
-          <t>City Centre, Number One Bristol, BS1 2NR</t>
+          <t>Stillhouse lane</t>
         </is>
       </c>
       <c r="H35" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I35" s="8" t="n">
-        <v>527</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="n"/>
       <c r="J35" s="8" t="n"/>
       <c r="K35" s="8" t="n"/>
       <c r="L35" s="8" t="n"/>
       <c r="M35" s="8" t="n"/>
       <c r="N35" s="8" t="n">
-        <v>21804</v>
+        <v>14304</v>
       </c>
       <c r="O35" s="8" t="n">
         <v>0</v>
@@ -19589,17 +19589,17 @@
       <c r="P35" s="8" t="n"/>
       <c r="Q35" s="8" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R35" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>Connells Lettings, Southville</t>
         </is>
       </c>
       <c r="S35" s="9" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T35" s="12" t="inlineStr">
@@ -19615,7 +19615,7 @@
       <c r="V35" s="7" t="inlineStr"/>
       <c r="W35" s="8" t="inlineStr">
         <is>
-          <t>27b085b9bcbec967c008845a19f54e272fc12b87</t>
+          <t>5cd63c65fc4cff6a9795b3661298e348456cd9ae</t>
         </is>
       </c>
     </row>
@@ -19629,13 +19629,13 @@
         </is>
       </c>
       <c r="C36" s="17" t="n">
-        <v>2200</v>
+        <v>3200</v>
       </c>
       <c r="D36" s="8" t="n">
         <v>3</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F36" s="8" t="inlineStr">
         <is>
@@ -19644,21 +19644,23 @@
       </c>
       <c r="G36" s="9" t="inlineStr">
         <is>
-          <t>Stillhouse lane</t>
+          <t>Redcliff Backs, The Custom House Redcliff Backs, BS1</t>
         </is>
       </c>
       <c r="H36" s="8" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I36" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="n">
+        <v>1033</v>
+      </c>
       <c r="J36" s="8" t="n"/>
       <c r="K36" s="8" t="n"/>
       <c r="L36" s="8" t="n"/>
       <c r="M36" s="8" t="n"/>
       <c r="N36" s="8" t="n">
-        <v>14304</v>
+        <v>20348</v>
       </c>
       <c r="O36" s="8" t="n">
         <v>0</v>
@@ -19671,7 +19673,7 @@
       </c>
       <c r="R36" s="8" t="inlineStr">
         <is>
-          <t>Connells Lettings, Southville</t>
+          <t>Acen Properties, Bristol</t>
         </is>
       </c>
       <c r="S36" s="9" t="inlineStr">
@@ -19692,7 +19694,7 @@
       <c r="V36" s="7" t="inlineStr"/>
       <c r="W36" s="8" t="inlineStr">
         <is>
-          <t>5cd63c65fc4cff6a9795b3661298e348456cd9ae</t>
+          <t>dc59104b573c7cdb75e715aaeca492455c19e7d4</t>
         </is>
       </c>
     </row>
@@ -19706,13 +19708,13 @@
         </is>
       </c>
       <c r="C37" s="17" t="n">
-        <v>3200</v>
+        <v>1200</v>
       </c>
       <c r="D37" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E37" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F37" s="8" t="inlineStr">
         <is>
@@ -19721,23 +19723,23 @@
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>Redcliff Backs, The Custom House Redcliff Backs, BS1</t>
+          <t>North Road, St. Andrews, BS6</t>
         </is>
       </c>
       <c r="H37" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS6</t>
         </is>
       </c>
       <c r="I37" s="8" t="n">
-        <v>1033</v>
+        <v>420</v>
       </c>
       <c r="J37" s="8" t="n"/>
       <c r="K37" s="8" t="n"/>
       <c r="L37" s="8" t="n"/>
       <c r="M37" s="8" t="n"/>
       <c r="N37" s="8" t="n">
-        <v>20348</v>
+        <v>8012</v>
       </c>
       <c r="O37" s="8" t="n">
         <v>0</v>
@@ -19745,12 +19747,12 @@
       <c r="P37" s="8" t="n"/>
       <c r="Q37" s="8" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="R37" s="8" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>Bristol Property Centre, Bristol</t>
         </is>
       </c>
       <c r="S37" s="9" t="inlineStr">
@@ -19771,7 +19773,7 @@
       <c r="V37" s="7" t="inlineStr"/>
       <c r="W37" s="8" t="inlineStr">
         <is>
-          <t>dc59104b573c7cdb75e715aaeca492455c19e7d4</t>
+          <t>a8afb5f086b1cf94d7c3bca118dd00b4440ca1b3</t>
         </is>
       </c>
     </row>
@@ -19800,23 +19802,21 @@
       </c>
       <c r="G38" s="9" t="inlineStr">
         <is>
-          <t>North Road, St. Andrews, BS6</t>
+          <t>Boot Lane - Bedminster</t>
         </is>
       </c>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t>BS6</t>
-        </is>
-      </c>
-      <c r="I38" s="8" t="n">
-        <v>420</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="n"/>
       <c r="J38" s="8" t="n"/>
       <c r="K38" s="8" t="n"/>
       <c r="L38" s="8" t="n"/>
       <c r="M38" s="8" t="n"/>
       <c r="N38" s="8" t="n">
-        <v>8012</v>
+        <v>15180</v>
       </c>
       <c r="O38" s="8" t="n">
         <v>0</v>
@@ -19824,12 +19824,12 @@
       <c r="P38" s="8" t="n"/>
       <c r="Q38" s="8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="R38" s="8" t="inlineStr">
         <is>
-          <t>Bristol Property Centre, Bristol</t>
+          <t>Ocean, Southville</t>
         </is>
       </c>
       <c r="S38" s="9" t="inlineStr">
@@ -19850,7 +19850,7 @@
       <c r="V38" s="7" t="inlineStr"/>
       <c r="W38" s="8" t="inlineStr">
         <is>
-          <t>a8afb5f086b1cf94d7c3bca118dd00b4440ca1b3</t>
+          <t>d0acdc25c6b4269d541e14519dfdbb42337f1828</t>
         </is>
       </c>
     </row>
@@ -19864,7 +19864,7 @@
         </is>
       </c>
       <c r="C39" s="17" t="n">
-        <v>1200</v>
+        <v>1150</v>
       </c>
       <c r="D39" s="8" t="n">
         <v>1</v>
@@ -19879,12 +19879,12 @@
       </c>
       <c r="G39" s="9" t="inlineStr">
         <is>
-          <t>Boot Lane - Bedminster</t>
+          <t>Church Road, Redfield, Bristol</t>
         </is>
       </c>
       <c r="H39" s="8" t="inlineStr">
         <is>
-          <t>BS3</t>
+          <t>BS5</t>
         </is>
       </c>
       <c r="I39" s="8" t="n"/>
@@ -19893,7 +19893,7 @@
       <c r="L39" s="8" t="n"/>
       <c r="M39" s="8" t="n"/>
       <c r="N39" s="8" t="n">
-        <v>15180</v>
+        <v>9192</v>
       </c>
       <c r="O39" s="8" t="n">
         <v>0</v>
@@ -19906,12 +19906,12 @@
       </c>
       <c r="R39" s="8" t="inlineStr">
         <is>
-          <t>Ocean, Southville</t>
+          <t>House + Co Property, Bristol</t>
         </is>
       </c>
       <c r="S39" s="9" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T39" s="12" t="inlineStr">
@@ -19927,7 +19927,7 @@
       <c r="V39" s="7" t="inlineStr"/>
       <c r="W39" s="8" t="inlineStr">
         <is>
-          <t>d0acdc25c6b4269d541e14519dfdbb42337f1828</t>
+          <t>7a41aac9e360b75a3e49c55b3cf8e321e60f6e4c</t>
         </is>
       </c>
     </row>
@@ -19941,7 +19941,7 @@
         </is>
       </c>
       <c r="C40" s="17" t="n">
-        <v>1150</v>
+        <v>1200</v>
       </c>
       <c r="D40" s="8" t="n">
         <v>1</v>
@@ -19956,7 +19956,7 @@
       </c>
       <c r="G40" s="9" t="inlineStr">
         <is>
-          <t>Church Road, Redfield, Bristol</t>
+          <t>Butlers Close, Crew's Hole, Bristol, BS5</t>
         </is>
       </c>
       <c r="H40" s="8" t="inlineStr">
@@ -19970,7 +19970,7 @@
       <c r="L40" s="8" t="n"/>
       <c r="M40" s="8" t="n"/>
       <c r="N40" s="8" t="n">
-        <v>9192</v>
+        <v>4996</v>
       </c>
       <c r="O40" s="8" t="n">
         <v>0</v>
@@ -19978,17 +19978,17 @@
       <c r="P40" s="8" t="n"/>
       <c r="Q40" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R40" s="8" t="inlineStr">
         <is>
-          <t>House + Co Property, Bristol</t>
+          <t>CJ Hole, Kingswood</t>
         </is>
       </c>
       <c r="S40" s="9" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T40" s="12" t="inlineStr">
@@ -20004,7 +20004,7 @@
       <c r="V40" s="7" t="inlineStr"/>
       <c r="W40" s="8" t="inlineStr">
         <is>
-          <t>7a41aac9e360b75a3e49c55b3cf8e321e60f6e4c</t>
+          <t>b41de22f35bcc18a3460e5242a89db630aea48eb</t>
         </is>
       </c>
     </row>
@@ -20018,7 +20018,7 @@
         </is>
       </c>
       <c r="C41" s="17" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="D41" s="8" t="n">
         <v>1</v>
@@ -20033,7 +20033,7 @@
       </c>
       <c r="G41" s="9" t="inlineStr">
         <is>
-          <t>Butlers Close, Crew's Hole, Bristol, BS5</t>
+          <t>Butlers Close, Bristol, BS5</t>
         </is>
       </c>
       <c r="H41" s="8" t="inlineStr">
@@ -20055,12 +20055,12 @@
       <c r="P41" s="8" t="n"/>
       <c r="Q41" s="8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="R41" s="8" t="inlineStr">
         <is>
-          <t>CJ Hole, Kingswood</t>
+          <t>Parks Estate Agents, Bristol</t>
         </is>
       </c>
       <c r="S41" s="9" t="inlineStr">
@@ -20081,7 +20081,7 @@
       <c r="V41" s="7" t="inlineStr"/>
       <c r="W41" s="8" t="inlineStr">
         <is>
-          <t>b41de22f35bcc18a3460e5242a89db630aea48eb</t>
+          <t>7cdb078ade9559511282395915101ace88ed6ee0</t>
         </is>
       </c>
     </row>
@@ -20110,12 +20110,12 @@
       </c>
       <c r="G42" s="9" t="inlineStr">
         <is>
-          <t>Butlers Close, Bristol, BS5</t>
+          <t>Manor Road, Bishopston, Bristol</t>
         </is>
       </c>
       <c r="H42" s="8" t="inlineStr">
         <is>
-          <t>BS5</t>
+          <t>BS7</t>
         </is>
       </c>
       <c r="I42" s="8" t="n"/>
@@ -20124,7 +20124,7 @@
       <c r="L42" s="8" t="n"/>
       <c r="M42" s="8" t="n"/>
       <c r="N42" s="8" t="n">
-        <v>4996</v>
+        <v>5396</v>
       </c>
       <c r="O42" s="8" t="n">
         <v>0</v>
@@ -20132,12 +20132,12 @@
       <c r="P42" s="8" t="n"/>
       <c r="Q42" s="8" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="R42" s="8" t="inlineStr">
         <is>
-          <t>Parks Estate Agents, Bristol</t>
+          <t>Connells Lettings, Southville</t>
         </is>
       </c>
       <c r="S42" s="9" t="inlineStr">
@@ -20158,7 +20158,7 @@
       <c r="V42" s="7" t="inlineStr"/>
       <c r="W42" s="8" t="inlineStr">
         <is>
-          <t>7cdb078ade9559511282395915101ace88ed6ee0</t>
+          <t>c5162861f3e11f0b7ccc2c9cecdfe5e060141029</t>
         </is>
       </c>
     </row>
@@ -20172,7 +20172,7 @@
         </is>
       </c>
       <c r="C43" s="17" t="n">
-        <v>1100</v>
+        <v>1200</v>
       </c>
       <c r="D43" s="8" t="n">
         <v>1</v>
@@ -20187,21 +20187,23 @@
       </c>
       <c r="G43" s="9" t="inlineStr">
         <is>
-          <t>Manor Road, Bishopston, Bristol</t>
+          <t>Marlborough Street, Eastville, Bristol</t>
         </is>
       </c>
       <c r="H43" s="8" t="inlineStr">
         <is>
-          <t>BS7</t>
-        </is>
-      </c>
-      <c r="I43" s="8" t="n"/>
+          <t>BS5</t>
+        </is>
+      </c>
+      <c r="I43" s="8" t="n">
+        <v>366</v>
+      </c>
       <c r="J43" s="8" t="n"/>
       <c r="K43" s="8" t="n"/>
       <c r="L43" s="8" t="n"/>
       <c r="M43" s="8" t="n"/>
       <c r="N43" s="8" t="n">
-        <v>5396</v>
+        <v>7920</v>
       </c>
       <c r="O43" s="8" t="n">
         <v>0</v>
@@ -20209,17 +20211,17 @@
       <c r="P43" s="8" t="n"/>
       <c r="Q43" s="8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="R43" s="8" t="inlineStr">
         <is>
-          <t>Connells Lettings, Southville</t>
+          <t>Hopewell, Bristol</t>
         </is>
       </c>
       <c r="S43" s="9" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T43" s="12" t="inlineStr">
@@ -20235,7 +20237,7 @@
       <c r="V43" s="7" t="inlineStr"/>
       <c r="W43" s="8" t="inlineStr">
         <is>
-          <t>c5162861f3e11f0b7ccc2c9cecdfe5e060141029</t>
+          <t>c9ead95c194e86c58ad819b434342e19c802a4f6</t>
         </is>
       </c>
     </row>
@@ -20249,7 +20251,7 @@
         </is>
       </c>
       <c r="C44" s="17" t="n">
-        <v>1200</v>
+        <v>975</v>
       </c>
       <c r="D44" s="8" t="n">
         <v>1</v>
@@ -20264,7 +20266,7 @@
       </c>
       <c r="G44" s="9" t="inlineStr">
         <is>
-          <t>Marlborough Street, Eastville, Bristol</t>
+          <t>Hudd's Vale Road, St George, Bristol, BS5</t>
         </is>
       </c>
       <c r="H44" s="8" t="inlineStr">
@@ -20272,15 +20274,13 @@
           <t>BS5</t>
         </is>
       </c>
-      <c r="I44" s="8" t="n">
-        <v>366</v>
-      </c>
+      <c r="I44" s="8" t="n"/>
       <c r="J44" s="8" t="n"/>
       <c r="K44" s="8" t="n"/>
       <c r="L44" s="8" t="n"/>
       <c r="M44" s="8" t="n"/>
       <c r="N44" s="8" t="n">
-        <v>7920</v>
+        <v>7804</v>
       </c>
       <c r="O44" s="8" t="n">
         <v>0</v>
@@ -20293,12 +20293,12 @@
       </c>
       <c r="R44" s="8" t="inlineStr">
         <is>
-          <t>Hopewell, Bristol</t>
+          <t>Northwood, Bristol</t>
         </is>
       </c>
       <c r="S44" s="9" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T44" s="12" t="inlineStr">
@@ -20314,7 +20314,7 @@
       <c r="V44" s="7" t="inlineStr"/>
       <c r="W44" s="8" t="inlineStr">
         <is>
-          <t>c9ead95c194e86c58ad819b434342e19c802a4f6</t>
+          <t>395007b279a3467e781f0aa9438723752e1eb50f</t>
         </is>
       </c>
     </row>
@@ -20343,7 +20343,7 @@
       </c>
       <c r="G45" s="9" t="inlineStr">
         <is>
-          <t>Hudd's Vale Road, St George, Bristol, BS5</t>
+          <t>Roseberry Park, Roseberry Mews Roseberry Park, BS5</t>
         </is>
       </c>
       <c r="H45" s="8" t="inlineStr">
@@ -20357,7 +20357,7 @@
       <c r="L45" s="8" t="n"/>
       <c r="M45" s="8" t="n"/>
       <c r="N45" s="8" t="n">
-        <v>7804</v>
+        <v>8640</v>
       </c>
       <c r="O45" s="8" t="n">
         <v>0</v>
@@ -20365,17 +20365,17 @@
       <c r="P45" s="8" t="n"/>
       <c r="Q45" s="8" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="R45" s="8" t="inlineStr">
         <is>
-          <t>Northwood, Bristol</t>
+          <t>Nook Lettings, Bristol</t>
         </is>
       </c>
       <c r="S45" s="9" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T45" s="12" t="inlineStr">
@@ -20391,7 +20391,7 @@
       <c r="V45" s="7" t="inlineStr"/>
       <c r="W45" s="8" t="inlineStr">
         <is>
-          <t>395007b279a3467e781f0aa9438723752e1eb50f</t>
+          <t>6b0cdf0711902be9b117a15d1a608cca17cc2d3f</t>
         </is>
       </c>
     </row>
@@ -20405,7 +20405,7 @@
         </is>
       </c>
       <c r="C46" s="17" t="n">
-        <v>975</v>
+        <v>1100</v>
       </c>
       <c r="D46" s="8" t="n">
         <v>1</v>
@@ -20420,12 +20420,12 @@
       </c>
       <c r="G46" s="9" t="inlineStr">
         <is>
-          <t>Roseberry Park, Roseberry Mews Roseberry Park, BS5</t>
+          <t>Ravenswood Road, Bristol, BS6</t>
         </is>
       </c>
       <c r="H46" s="8" t="inlineStr">
         <is>
-          <t>BS5</t>
+          <t>BS6</t>
         </is>
       </c>
       <c r="I46" s="8" t="n"/>
@@ -20434,7 +20434,7 @@
       <c r="L46" s="8" t="n"/>
       <c r="M46" s="8" t="n"/>
       <c r="N46" s="8" t="n">
-        <v>8640</v>
+        <v>16556</v>
       </c>
       <c r="O46" s="8" t="n">
         <v>0</v>
@@ -20442,17 +20442,17 @@
       <c r="P46" s="8" t="n"/>
       <c r="Q46" s="8" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="R46" s="8" t="inlineStr">
         <is>
-          <t>Nook Lettings, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S46" s="9" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>bills included</t>
         </is>
       </c>
       <c r="T46" s="12" t="inlineStr">
@@ -20468,13 +20468,13 @@
       <c r="V46" s="7" t="inlineStr"/>
       <c r="W46" s="8" t="inlineStr">
         <is>
-          <t>6b0cdf0711902be9b117a15d1a608cca17cc2d3f</t>
+          <t>1c315268eed469425b8c480540e07721a1a3c908</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="n">
-        <v>3.7</v>
+        <v>2</v>
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
@@ -20482,7 +20482,7 @@
         </is>
       </c>
       <c r="C47" s="17" t="n">
-        <v>1100</v>
+        <v>1200</v>
       </c>
       <c r="D47" s="8" t="n">
         <v>1</v>
@@ -20497,12 +20497,12 @@
       </c>
       <c r="G47" s="9" t="inlineStr">
         <is>
-          <t>Ravenswood Road, Bristol, BS6</t>
+          <t>Talavera Close, Bristol</t>
         </is>
       </c>
       <c r="H47" s="8" t="inlineStr">
         <is>
-          <t>BS6</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I47" s="8" t="n"/>
@@ -20511,7 +20511,7 @@
       <c r="L47" s="8" t="n"/>
       <c r="M47" s="8" t="n"/>
       <c r="N47" s="8" t="n">
-        <v>16556</v>
+        <v>19980</v>
       </c>
       <c r="O47" s="8" t="n">
         <v>0</v>
@@ -20519,19 +20519,15 @@
       <c r="P47" s="8" t="n"/>
       <c r="Q47" s="8" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="R47" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
-        </is>
-      </c>
-      <c r="S47" s="9" t="inlineStr">
-        <is>
-          <t>bills included</t>
-        </is>
-      </c>
+          <t>Campions Property Lettings &amp; Management Ltd, National</t>
+        </is>
+      </c>
+      <c r="S47" s="9" t="inlineStr"/>
       <c r="T47" s="12" t="inlineStr">
         <is>
           <t>View listing</t>
@@ -20545,7 +20541,7 @@
       <c r="V47" s="7" t="inlineStr"/>
       <c r="W47" s="8" t="inlineStr">
         <is>
-          <t>1c315268eed469425b8c480540e07721a1a3c908</t>
+          <t>e0a93f8e75c81900b60248c526509a97c04a5289</t>
         </is>
       </c>
     </row>
@@ -20559,7 +20555,7 @@
         </is>
       </c>
       <c r="C48" s="17" t="n">
-        <v>1200</v>
+        <v>1150</v>
       </c>
       <c r="D48" s="8" t="n">
         <v>1</v>
@@ -20574,12 +20570,12 @@
       </c>
       <c r="G48" s="9" t="inlineStr">
         <is>
-          <t>Talavera Close, Bristol</t>
+          <t>Bedminster Parade Bedminster, Bristol, BS3</t>
         </is>
       </c>
       <c r="H48" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS3</t>
         </is>
       </c>
       <c r="I48" s="8" t="n"/>
@@ -20588,7 +20584,7 @@
       <c r="L48" s="8" t="n"/>
       <c r="M48" s="8" t="n"/>
       <c r="N48" s="8" t="n">
-        <v>19980</v>
+        <v>15212</v>
       </c>
       <c r="O48" s="8" t="n">
         <v>0</v>
@@ -20596,12 +20592,12 @@
       <c r="P48" s="8" t="n"/>
       <c r="Q48" s="8" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="R48" s="8" t="inlineStr">
         <is>
-          <t>Campions Property Lettings &amp; Management Ltd, National</t>
+          <t>Accommodation Unlimited, Bristol</t>
         </is>
       </c>
       <c r="S48" s="9" t="inlineStr"/>
@@ -20618,7 +20614,7 @@
       <c r="V48" s="7" t="inlineStr"/>
       <c r="W48" s="8" t="inlineStr">
         <is>
-          <t>e0a93f8e75c81900b60248c526509a97c04a5289</t>
+          <t>50cb5f4990ae3655c686a0bb94886a0f25eb2ec9</t>
         </is>
       </c>
     </row>
@@ -20632,7 +20628,7 @@
         </is>
       </c>
       <c r="C49" s="17" t="n">
-        <v>1150</v>
+        <v>1200</v>
       </c>
       <c r="D49" s="8" t="n">
         <v>1</v>
@@ -20647,12 +20643,12 @@
       </c>
       <c r="G49" s="9" t="inlineStr">
         <is>
-          <t>Bedminster Parade Bedminster, Bristol, BS3</t>
+          <t>Knowle Road, Bristol, BS4</t>
         </is>
       </c>
       <c r="H49" s="8" t="inlineStr">
         <is>
-          <t>BS3</t>
+          <t>BS4</t>
         </is>
       </c>
       <c r="I49" s="8" t="n"/>
@@ -20661,7 +20657,7 @@
       <c r="L49" s="8" t="n"/>
       <c r="M49" s="8" t="n"/>
       <c r="N49" s="8" t="n">
-        <v>15212</v>
+        <v>6852</v>
       </c>
       <c r="O49" s="8" t="n">
         <v>0</v>
@@ -20669,12 +20665,12 @@
       <c r="P49" s="8" t="n"/>
       <c r="Q49" s="8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R49" s="8" t="inlineStr">
         <is>
-          <t>Accommodation Unlimited, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S49" s="9" t="inlineStr"/>
@@ -20691,7 +20687,7 @@
       <c r="V49" s="7" t="inlineStr"/>
       <c r="W49" s="8" t="inlineStr">
         <is>
-          <t>50cb5f4990ae3655c686a0bb94886a0f25eb2ec9</t>
+          <t>bbb9b81c216b0de31ba8859ef50a78ed36377871</t>
         </is>
       </c>
     </row>
@@ -20705,7 +20701,7 @@
         </is>
       </c>
       <c r="C50" s="17" t="n">
-        <v>1200</v>
+        <v>1640</v>
       </c>
       <c r="D50" s="8" t="n">
         <v>1</v>
@@ -20720,21 +20716,23 @@
       </c>
       <c r="G50" s="9" t="inlineStr">
         <is>
-          <t>Knowle Road, Bristol, BS4</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H50" s="8" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I50" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I50" s="8" t="n">
+        <v>484</v>
+      </c>
       <c r="J50" s="8" t="n"/>
       <c r="K50" s="8" t="n"/>
       <c r="L50" s="8" t="n"/>
       <c r="M50" s="8" t="n"/>
       <c r="N50" s="8" t="n">
-        <v>6852</v>
+        <v>21504</v>
       </c>
       <c r="O50" s="8" t="n">
         <v>0</v>
@@ -20742,12 +20740,12 @@
       <c r="P50" s="8" t="n"/>
       <c r="Q50" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="R50" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S50" s="9" t="inlineStr"/>
@@ -20764,7 +20762,7 @@
       <c r="V50" s="7" t="inlineStr"/>
       <c r="W50" s="8" t="inlineStr">
         <is>
-          <t>bbb9b81c216b0de31ba8859ef50a78ed36377871</t>
+          <t>5d39df649daaa86eebac0b90b2a33fa18f365ed3</t>
         </is>
       </c>
     </row>
@@ -20778,7 +20776,7 @@
         </is>
       </c>
       <c r="C51" s="17" t="n">
-        <v>1640</v>
+        <v>1600</v>
       </c>
       <c r="D51" s="8" t="n">
         <v>1</v>
@@ -20793,7 +20791,7 @@
       </c>
       <c r="G51" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Hope Quay, Wapping Wharf</t>
         </is>
       </c>
       <c r="H51" s="8" t="inlineStr">
@@ -20801,15 +20799,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I51" s="8" t="n">
-        <v>484</v>
-      </c>
+      <c r="I51" s="8" t="n"/>
       <c r="J51" s="8" t="n"/>
       <c r="K51" s="8" t="n"/>
       <c r="L51" s="8" t="n"/>
       <c r="M51" s="8" t="n"/>
       <c r="N51" s="8" t="n">
-        <v>21504</v>
+        <v>16708</v>
       </c>
       <c r="O51" s="8" t="n">
         <v>0</v>
@@ -20817,12 +20813,12 @@
       <c r="P51" s="8" t="n"/>
       <c r="Q51" s="8" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R51" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S51" s="9" t="inlineStr"/>
@@ -20839,7 +20835,7 @@
       <c r="V51" s="7" t="inlineStr"/>
       <c r="W51" s="8" t="inlineStr">
         <is>
-          <t>5d39df649daaa86eebac0b90b2a33fa18f365ed3</t>
+          <t>0dbbb656d8ffbae712c9077ec0f7c1849746bd0b</t>
         </is>
       </c>
     </row>
@@ -20853,7 +20849,7 @@
         </is>
       </c>
       <c r="C52" s="17" t="n">
-        <v>1600</v>
+        <v>1300</v>
       </c>
       <c r="D52" s="8" t="n">
         <v>1</v>
@@ -20868,12 +20864,12 @@
       </c>
       <c r="G52" s="9" t="inlineStr">
         <is>
-          <t>Hope Quay, Wapping Wharf</t>
+          <t>Hamilton Court - City Centre</t>
         </is>
       </c>
       <c r="H52" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I52" s="8" t="n"/>
@@ -20882,7 +20878,7 @@
       <c r="L52" s="8" t="n"/>
       <c r="M52" s="8" t="n"/>
       <c r="N52" s="8" t="n">
-        <v>16708</v>
+        <v>21616</v>
       </c>
       <c r="O52" s="8" t="n">
         <v>0</v>
@@ -20895,7 +20891,7 @@
       </c>
       <c r="R52" s="8" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>Ocean, Clifton</t>
         </is>
       </c>
       <c r="S52" s="9" t="inlineStr"/>
@@ -20912,7 +20908,7 @@
       <c r="V52" s="7" t="inlineStr"/>
       <c r="W52" s="8" t="inlineStr">
         <is>
-          <t>0dbbb656d8ffbae712c9077ec0f7c1849746bd0b</t>
+          <t>8bd3f395f80d9e75d404d499c9b227ed567374e3</t>
         </is>
       </c>
     </row>
@@ -20926,10 +20922,10 @@
         </is>
       </c>
       <c r="C53" s="17" t="n">
-        <v>1300</v>
+        <v>2200</v>
       </c>
       <c r="D53" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E53" s="8" t="n">
         <v>1</v>
@@ -20941,7 +20937,7 @@
       </c>
       <c r="G53" s="9" t="inlineStr">
         <is>
-          <t>Hamilton Court - City Centre</t>
+          <t>Castle Park View, Castle Street, Bristol</t>
         </is>
       </c>
       <c r="H53" s="8" t="inlineStr">
@@ -20955,7 +20951,7 @@
       <c r="L53" s="8" t="n"/>
       <c r="M53" s="8" t="n"/>
       <c r="N53" s="8" t="n">
-        <v>21616</v>
+        <v>21984</v>
       </c>
       <c r="O53" s="8" t="n">
         <v>0</v>
@@ -20963,12 +20959,12 @@
       <c r="P53" s="8" t="n"/>
       <c r="Q53" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="R53" s="8" t="inlineStr">
         <is>
-          <t>Ocean, Clifton</t>
+          <t>Savills Lettings, CPV</t>
         </is>
       </c>
       <c r="S53" s="9" t="inlineStr"/>
@@ -20985,7 +20981,7 @@
       <c r="V53" s="7" t="inlineStr"/>
       <c r="W53" s="8" t="inlineStr">
         <is>
-          <t>8bd3f395f80d9e75d404d499c9b227ed567374e3</t>
+          <t>406fab2577557efdd9382cee302acdc7a788c3d8</t>
         </is>
       </c>
     </row>
@@ -20999,13 +20995,13 @@
         </is>
       </c>
       <c r="C54" s="17" t="n">
-        <v>2200</v>
+        <v>2300</v>
       </c>
       <c r="D54" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E54" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F54" s="8" t="inlineStr">
         <is>
@@ -21022,7 +21018,9 @@
           <t>BS2</t>
         </is>
       </c>
-      <c r="I54" s="8" t="n"/>
+      <c r="I54" s="8" t="n">
+        <v>757</v>
+      </c>
       <c r="J54" s="8" t="n"/>
       <c r="K54" s="8" t="n"/>
       <c r="L54" s="8" t="n"/>
@@ -21058,7 +21056,7 @@
       <c r="V54" s="7" t="inlineStr"/>
       <c r="W54" s="8" t="inlineStr">
         <is>
-          <t>406fab2577557efdd9382cee302acdc7a788c3d8</t>
+          <t>82dded0955660a8ec4af3acb8db470436bdc522b</t>
         </is>
       </c>
     </row>
@@ -21087,7 +21085,7 @@
       </c>
       <c r="G55" s="9" t="inlineStr">
         <is>
-          <t>Castle Park View, Castle Street, Bristol</t>
+          <t>Castle Park View, Castle Street, Bristol, BS2 0ND</t>
         </is>
       </c>
       <c r="H55" s="8" t="inlineStr">
@@ -21095,9 +21093,7 @@
           <t>BS2</t>
         </is>
       </c>
-      <c r="I55" s="8" t="n">
-        <v>757</v>
-      </c>
+      <c r="I55" s="8" t="n"/>
       <c r="J55" s="8" t="n"/>
       <c r="K55" s="8" t="n"/>
       <c r="L55" s="8" t="n"/>
@@ -21133,7 +21129,7 @@
       <c r="V55" s="7" t="inlineStr"/>
       <c r="W55" s="8" t="inlineStr">
         <is>
-          <t>82dded0955660a8ec4af3acb8db470436bdc522b</t>
+          <t>fc4abec405a6b435cb290523f6e7784fc2de1099</t>
         </is>
       </c>
     </row>
@@ -21147,13 +21143,13 @@
         </is>
       </c>
       <c r="C56" s="17" t="n">
-        <v>2300</v>
+        <v>2095</v>
       </c>
       <c r="D56" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E56" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F56" s="8" t="inlineStr">
         <is>
@@ -21162,7 +21158,7 @@
       </c>
       <c r="G56" s="9" t="inlineStr">
         <is>
-          <t>Castle Park View, Castle Street, Bristol, BS2 0ND</t>
+          <t>Castle Park View, Castle Street, BS2 0ND, Bristol</t>
         </is>
       </c>
       <c r="H56" s="8" t="inlineStr">
@@ -21206,7 +21202,7 @@
       <c r="V56" s="7" t="inlineStr"/>
       <c r="W56" s="8" t="inlineStr">
         <is>
-          <t>fc4abec405a6b435cb290523f6e7784fc2de1099</t>
+          <t>7a4bff96a8fb36d99cc3d7825e84bee85f8c5ba7</t>
         </is>
       </c>
     </row>
@@ -21220,10 +21216,10 @@
         </is>
       </c>
       <c r="C57" s="17" t="n">
-        <v>2095</v>
+        <v>1400</v>
       </c>
       <c r="D57" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E57" s="8" t="n">
         <v>1</v>
@@ -21235,12 +21231,12 @@
       </c>
       <c r="G57" s="9" t="inlineStr">
         <is>
-          <t>Castle Park View, Castle Street, BS2 0ND, Bristol</t>
+          <t>Jessop Court Ferry Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H57" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I57" s="8" t="n"/>
@@ -21249,7 +21245,7 @@
       <c r="L57" s="8" t="n"/>
       <c r="M57" s="8" t="n"/>
       <c r="N57" s="8" t="n">
-        <v>21984</v>
+        <v>20908</v>
       </c>
       <c r="O57" s="8" t="n">
         <v>0</v>
@@ -21257,12 +21253,12 @@
       <c r="P57" s="8" t="n"/>
       <c r="Q57" s="8" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="R57" s="8" t="inlineStr">
         <is>
-          <t>Savills Lettings, CPV</t>
+          <t>Accommodation Unlimited, Bristol</t>
         </is>
       </c>
       <c r="S57" s="9" t="inlineStr"/>
@@ -21279,7 +21275,7 @@
       <c r="V57" s="7" t="inlineStr"/>
       <c r="W57" s="8" t="inlineStr">
         <is>
-          <t>7a4bff96a8fb36d99cc3d7825e84bee85f8c5ba7</t>
+          <t>45f17f505657c6333c92b921a50f7641e02f2c2f</t>
         </is>
       </c>
     </row>
@@ -21293,10 +21289,10 @@
         </is>
       </c>
       <c r="C58" s="17" t="n">
-        <v>1400</v>
+        <v>1500</v>
       </c>
       <c r="D58" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E58" s="8" t="n">
         <v>1</v>
@@ -21308,12 +21304,12 @@
       </c>
       <c r="G58" s="9" t="inlineStr">
         <is>
-          <t>Jessop Court Ferry Street, Bristol, BS1</t>
+          <t>St Clements Court, Wilson Street, Bristol</t>
         </is>
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I58" s="8" t="n"/>
@@ -21322,7 +21318,7 @@
       <c r="L58" s="8" t="n"/>
       <c r="M58" s="8" t="n"/>
       <c r="N58" s="8" t="n">
-        <v>20908</v>
+        <v>21600</v>
       </c>
       <c r="O58" s="8" t="n">
         <v>0</v>
@@ -21330,12 +21326,12 @@
       <c r="P58" s="8" t="n"/>
       <c r="Q58" s="8" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="R58" s="8" t="inlineStr">
         <is>
-          <t>Accommodation Unlimited, Bristol</t>
+          <t>Kendall Harper, Bishopston</t>
         </is>
       </c>
       <c r="S58" s="9" t="inlineStr"/>
@@ -21352,7 +21348,7 @@
       <c r="V58" s="7" t="inlineStr"/>
       <c r="W58" s="8" t="inlineStr">
         <is>
-          <t>45f17f505657c6333c92b921a50f7641e02f2c2f</t>
+          <t>b3bf3a18fe9e3595ef643379d979e59ee826fcbc</t>
         </is>
       </c>
     </row>
@@ -21366,7 +21362,7 @@
         </is>
       </c>
       <c r="C59" s="17" t="n">
-        <v>1500</v>
+        <v>1600</v>
       </c>
       <c r="D59" s="8" t="n">
         <v>2</v>
@@ -21381,7 +21377,7 @@
       </c>
       <c r="G59" s="9" t="inlineStr">
         <is>
-          <t>St Clements Court, Wilson Street, Bristol</t>
+          <t>Waterloo Road, Midland Mews, BS2</t>
         </is>
       </c>
       <c r="H59" s="8" t="inlineStr">
@@ -21389,13 +21385,15 @@
           <t>BS2</t>
         </is>
       </c>
-      <c r="I59" s="8" t="n"/>
+      <c r="I59" s="8" t="n">
+        <v>721</v>
+      </c>
       <c r="J59" s="8" t="n"/>
       <c r="K59" s="8" t="n"/>
       <c r="L59" s="8" t="n"/>
       <c r="M59" s="8" t="n"/>
       <c r="N59" s="8" t="n">
-        <v>21600</v>
+        <v>20856</v>
       </c>
       <c r="O59" s="8" t="n">
         <v>0</v>
@@ -21403,12 +21401,12 @@
       <c r="P59" s="8" t="n"/>
       <c r="Q59" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R59" s="8" t="inlineStr">
         <is>
-          <t>Kendall Harper, Bishopston</t>
+          <t>Acen Properties, Bristol</t>
         </is>
       </c>
       <c r="S59" s="9" t="inlineStr"/>
@@ -21425,7 +21423,7 @@
       <c r="V59" s="7" t="inlineStr"/>
       <c r="W59" s="8" t="inlineStr">
         <is>
-          <t>b3bf3a18fe9e3595ef643379d979e59ee826fcbc</t>
+          <t>cf8a979c7c13e868d74a6828d64c93a46d2e7209</t>
         </is>
       </c>
     </row>
@@ -21439,7 +21437,7 @@
         </is>
       </c>
       <c r="C60" s="17" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="D60" s="8" t="n">
         <v>2</v>
@@ -21454,7 +21452,7 @@
       </c>
       <c r="G60" s="9" t="inlineStr">
         <is>
-          <t>Waterloo Road, Midland Mews, BS2</t>
+          <t>Midland Mews Waterloo Road Old Market, Bristol, BS2</t>
         </is>
       </c>
       <c r="H60" s="8" t="inlineStr">
@@ -21462,9 +21460,7 @@
           <t>BS2</t>
         </is>
       </c>
-      <c r="I60" s="8" t="n">
-        <v>721</v>
-      </c>
+      <c r="I60" s="8" t="n"/>
       <c r="J60" s="8" t="n"/>
       <c r="K60" s="8" t="n"/>
       <c r="L60" s="8" t="n"/>
@@ -21478,12 +21474,12 @@
       <c r="P60" s="8" t="n"/>
       <c r="Q60" s="8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="R60" s="8" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>Accommodation Unlimited, Bristol</t>
         </is>
       </c>
       <c r="S60" s="9" t="inlineStr"/>
@@ -21500,7 +21496,7 @@
       <c r="V60" s="7" t="inlineStr"/>
       <c r="W60" s="8" t="inlineStr">
         <is>
-          <t>cf8a979c7c13e868d74a6828d64c93a46d2e7209</t>
+          <t>f83555c1dc6f03087d999787a76db9b49794ddb4</t>
         </is>
       </c>
     </row>
@@ -21514,13 +21510,13 @@
         </is>
       </c>
       <c r="C61" s="17" t="n">
-        <v>2085</v>
+        <v>1300</v>
       </c>
       <c r="D61" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E61" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F61" s="8" t="inlineStr">
         <is>
@@ -21529,7 +21525,7 @@
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>City Centre, Queen Square Apartments, BS1</t>
         </is>
       </c>
       <c r="H61" s="8" t="inlineStr">
@@ -21538,14 +21534,14 @@
         </is>
       </c>
       <c r="I61" s="8" t="n">
-        <v>722</v>
+        <v>405</v>
       </c>
       <c r="J61" s="8" t="n"/>
       <c r="K61" s="8" t="n"/>
       <c r="L61" s="8" t="n"/>
       <c r="M61" s="8" t="n"/>
       <c r="N61" s="8" t="n">
-        <v>21504</v>
+        <v>20316</v>
       </c>
       <c r="O61" s="8" t="n">
         <v>0</v>
@@ -21558,7 +21554,7 @@
       </c>
       <c r="R61" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S61" s="9" t="inlineStr"/>
@@ -21575,7 +21571,7 @@
       <c r="V61" s="7" t="inlineStr"/>
       <c r="W61" s="8" t="inlineStr">
         <is>
-          <t>12a5f2c4f1be2a8f1a9b2c6cbe66191abf1d7975</t>
+          <t>9ad2c7bc90885b9a9e65b462b952842a964f1d35</t>
         </is>
       </c>
     </row>
@@ -21589,13 +21585,13 @@
         </is>
       </c>
       <c r="C62" s="17" t="n">
-        <v>1640</v>
+        <v>2020</v>
       </c>
       <c r="D62" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E62" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
@@ -21613,14 +21609,14 @@
         </is>
       </c>
       <c r="I62" s="8" t="n">
-        <v>570</v>
+        <v>764</v>
       </c>
       <c r="J62" s="8" t="n"/>
       <c r="K62" s="8" t="n"/>
       <c r="L62" s="8" t="n"/>
       <c r="M62" s="8" t="n"/>
       <c r="N62" s="8" t="n">
-        <v>20820</v>
+        <v>20856</v>
       </c>
       <c r="O62" s="8" t="n">
         <v>0</v>
@@ -21628,7 +21624,7 @@
       <c r="P62" s="8" t="n"/>
       <c r="Q62" s="8" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="R62" s="8" t="inlineStr">
@@ -21650,7 +21646,7 @@
       <c r="V62" s="7" t="inlineStr"/>
       <c r="W62" s="8" t="inlineStr">
         <is>
-          <t>f7afd1bbb106a22d180a78614dde509c1dbfa8c1</t>
+          <t>6140b74b7d83ae5918fdabb6f9371e2f4b63a9c2</t>
         </is>
       </c>
     </row>
@@ -21664,13 +21660,13 @@
         </is>
       </c>
       <c r="C63" s="17" t="n">
-        <v>1500</v>
+        <v>2145</v>
       </c>
       <c r="D63" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E63" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F63" s="8" t="inlineStr">
         <is>
@@ -21679,21 +21675,23 @@
       </c>
       <c r="G63" s="9" t="inlineStr">
         <is>
-          <t>Midland Mews Waterloo Road Old Market, Bristol, BS2</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H63" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I63" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I63" s="8" t="n">
+        <v>815</v>
+      </c>
       <c r="J63" s="8" t="n"/>
       <c r="K63" s="8" t="n"/>
       <c r="L63" s="8" t="n"/>
       <c r="M63" s="8" t="n"/>
       <c r="N63" s="8" t="n">
-        <v>20856</v>
+        <v>21504</v>
       </c>
       <c r="O63" s="8" t="n">
         <v>0</v>
@@ -21701,12 +21699,12 @@
       <c r="P63" s="8" t="n"/>
       <c r="Q63" s="8" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="R63" s="8" t="inlineStr">
         <is>
-          <t>Accommodation Unlimited, Bristol</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S63" s="9" t="inlineStr"/>
@@ -21723,7 +21721,7 @@
       <c r="V63" s="7" t="inlineStr"/>
       <c r="W63" s="8" t="inlineStr">
         <is>
-          <t>f83555c1dc6f03087d999787a76db9b49794ddb4</t>
+          <t>24009eb3414633bf24b3b69631ba405866a1e5c9</t>
         </is>
       </c>
     </row>
@@ -21737,7 +21735,7 @@
         </is>
       </c>
       <c r="C64" s="17" t="n">
-        <v>1300</v>
+        <v>1635</v>
       </c>
       <c r="D64" s="8" t="n">
         <v>1</v>
@@ -21752,7 +21750,7 @@
       </c>
       <c r="G64" s="9" t="inlineStr">
         <is>
-          <t>City Centre, Queen Square Apartments, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H64" s="8" t="inlineStr">
@@ -21761,14 +21759,14 @@
         </is>
       </c>
       <c r="I64" s="8" t="n">
-        <v>405</v>
+        <v>486</v>
       </c>
       <c r="J64" s="8" t="n"/>
       <c r="K64" s="8" t="n"/>
       <c r="L64" s="8" t="n"/>
       <c r="M64" s="8" t="n"/>
       <c r="N64" s="8" t="n">
-        <v>20316</v>
+        <v>21504</v>
       </c>
       <c r="O64" s="8" t="n">
         <v>0</v>
@@ -21776,12 +21774,12 @@
       <c r="P64" s="8" t="n"/>
       <c r="Q64" s="8" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="R64" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S64" s="9" t="inlineStr"/>
@@ -21798,7 +21796,7 @@
       <c r="V64" s="7" t="inlineStr"/>
       <c r="W64" s="8" t="inlineStr">
         <is>
-          <t>9ad2c7bc90885b9a9e65b462b952842a964f1d35</t>
+          <t>bbf6e42784b6e4b7dae8d6bef9900115d0f3056e</t>
         </is>
       </c>
     </row>
@@ -21812,7 +21810,7 @@
         </is>
       </c>
       <c r="C65" s="17" t="n">
-        <v>2020</v>
+        <v>1750</v>
       </c>
       <c r="D65" s="8" t="n">
         <v>2</v>
@@ -21827,23 +21825,23 @@
       </c>
       <c r="G65" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Arnos Vale, Paintworks, BS4</t>
         </is>
       </c>
       <c r="H65" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS4</t>
         </is>
       </c>
       <c r="I65" s="8" t="n">
-        <v>764</v>
+        <v>731</v>
       </c>
       <c r="J65" s="8" t="n"/>
       <c r="K65" s="8" t="n"/>
       <c r="L65" s="8" t="n"/>
       <c r="M65" s="8" t="n"/>
       <c r="N65" s="8" t="n">
-        <v>20856</v>
+        <v>4680</v>
       </c>
       <c r="O65" s="8" t="n">
         <v>0</v>
@@ -21856,7 +21854,7 @@
       </c>
       <c r="R65" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S65" s="9" t="inlineStr"/>
@@ -21873,7 +21871,7 @@
       <c r="V65" s="7" t="inlineStr"/>
       <c r="W65" s="8" t="inlineStr">
         <is>
-          <t>6140b74b7d83ae5918fdabb6f9371e2f4b63a9c2</t>
+          <t>1c0acc4cbbc0f239d4843e9eb56c0d04ca3a6278</t>
         </is>
       </c>
     </row>
@@ -21887,13 +21885,13 @@
         </is>
       </c>
       <c r="C66" s="17" t="n">
-        <v>2145</v>
+        <v>2100</v>
       </c>
       <c r="D66" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E66" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F66" s="8" t="inlineStr">
         <is>
@@ -21902,7 +21900,7 @@
       </c>
       <c r="G66" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Baldwin St, Bristol, BS1</t>
         </is>
       </c>
       <c r="H66" s="8" t="inlineStr">
@@ -21910,15 +21908,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I66" s="8" t="n">
-        <v>815</v>
-      </c>
+      <c r="I66" s="8" t="n"/>
       <c r="J66" s="8" t="n"/>
       <c r="K66" s="8" t="n"/>
       <c r="L66" s="8" t="n"/>
       <c r="M66" s="8" t="n"/>
       <c r="N66" s="8" t="n">
-        <v>21504</v>
+        <v>21148</v>
       </c>
       <c r="O66" s="8" t="n">
         <v>0</v>
@@ -21926,12 +21922,12 @@
       <c r="P66" s="8" t="n"/>
       <c r="Q66" s="8" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R66" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S66" s="9" t="inlineStr"/>
@@ -21948,7 +21944,7 @@
       <c r="V66" s="7" t="inlineStr"/>
       <c r="W66" s="8" t="inlineStr">
         <is>
-          <t>24009eb3414633bf24b3b69631ba405866a1e5c9</t>
+          <t>ba1c1abaa5dbfd6e19c20fa9df1e66799d9c2462</t>
         </is>
       </c>
     </row>
@@ -21962,13 +21958,13 @@
         </is>
       </c>
       <c r="C67" s="17" t="n">
-        <v>1635</v>
+        <v>2220</v>
       </c>
       <c r="D67" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E67" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F67" s="8" t="inlineStr">
         <is>
@@ -21977,7 +21973,7 @@
       </c>
       <c r="G67" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H67" s="8" t="inlineStr">
@@ -21986,14 +21982,14 @@
         </is>
       </c>
       <c r="I67" s="8" t="n">
-        <v>486</v>
+        <v>697</v>
       </c>
       <c r="J67" s="8" t="n"/>
       <c r="K67" s="8" t="n"/>
       <c r="L67" s="8" t="n"/>
       <c r="M67" s="8" t="n"/>
       <c r="N67" s="8" t="n">
-        <v>21504</v>
+        <v>20820</v>
       </c>
       <c r="O67" s="8" t="n">
         <v>0</v>
@@ -22001,12 +21997,12 @@
       <c r="P67" s="8" t="n"/>
       <c r="Q67" s="8" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R67" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S67" s="9" t="inlineStr"/>
@@ -22023,7 +22019,7 @@
       <c r="V67" s="7" t="inlineStr"/>
       <c r="W67" s="8" t="inlineStr">
         <is>
-          <t>bbf6e42784b6e4b7dae8d6bef9900115d0f3056e</t>
+          <t>5870266ee1b15bf20f0a085f56358c762e522fa8</t>
         </is>
       </c>
     </row>
@@ -22037,13 +22033,13 @@
         </is>
       </c>
       <c r="C68" s="17" t="n">
-        <v>1750</v>
+        <v>1300</v>
       </c>
       <c r="D68" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E68" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
@@ -22052,23 +22048,21 @@
       </c>
       <c r="G68" s="9" t="inlineStr">
         <is>
-          <t>Arnos Vale, Paintworks, BS4</t>
+          <t>Bristol City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H68" s="8" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I68" s="8" t="n">
-        <v>731</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I68" s="8" t="n"/>
       <c r="J68" s="8" t="n"/>
       <c r="K68" s="8" t="n"/>
       <c r="L68" s="8" t="n"/>
       <c r="M68" s="8" t="n"/>
       <c r="N68" s="8" t="n">
-        <v>4680</v>
+        <v>21428</v>
       </c>
       <c r="O68" s="8" t="n">
         <v>0</v>
@@ -22076,12 +22070,12 @@
       <c r="P68" s="8" t="n"/>
       <c r="Q68" s="8" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="R68" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S68" s="9" t="inlineStr"/>
@@ -22098,7 +22092,7 @@
       <c r="V68" s="7" t="inlineStr"/>
       <c r="W68" s="8" t="inlineStr">
         <is>
-          <t>1c0acc4cbbc0f239d4843e9eb56c0d04ca3a6278</t>
+          <t>317e9ab29cad2381c41672743d877feba2c14e45</t>
         </is>
       </c>
     </row>
@@ -22112,7 +22106,7 @@
         </is>
       </c>
       <c r="C69" s="17" t="n">
-        <v>2100</v>
+        <v>1500</v>
       </c>
       <c r="D69" s="8" t="n">
         <v>1</v>
@@ -22127,7 +22121,7 @@
       </c>
       <c r="G69" s="9" t="inlineStr">
         <is>
-          <t>Baldwin St, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H69" s="8" t="inlineStr">
@@ -22135,13 +22129,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I69" s="8" t="n"/>
+      <c r="I69" s="8" t="n">
+        <v>548</v>
+      </c>
       <c r="J69" s="8" t="n"/>
       <c r="K69" s="8" t="n"/>
       <c r="L69" s="8" t="n"/>
       <c r="M69" s="8" t="n"/>
       <c r="N69" s="8" t="n">
-        <v>21148</v>
+        <v>21504</v>
       </c>
       <c r="O69" s="8" t="n">
         <v>0</v>
@@ -22149,12 +22145,12 @@
       <c r="P69" s="8" t="n"/>
       <c r="Q69" s="8" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R69" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S69" s="9" t="inlineStr"/>
@@ -22171,7 +22167,7 @@
       <c r="V69" s="7" t="inlineStr"/>
       <c r="W69" s="8" t="inlineStr">
         <is>
-          <t>ba1c1abaa5dbfd6e19c20fa9df1e66799d9c2462</t>
+          <t>bad1e4584285201ef9995d2b437343fca870009c</t>
         </is>
       </c>
     </row>
@@ -22185,13 +22181,13 @@
         </is>
       </c>
       <c r="C70" s="17" t="n">
-        <v>2220</v>
+        <v>1615</v>
       </c>
       <c r="D70" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E70" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F70" s="8" t="inlineStr">
         <is>
@@ -22200,7 +22196,7 @@
       </c>
       <c r="G70" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H70" s="8" t="inlineStr">
@@ -22209,14 +22205,14 @@
         </is>
       </c>
       <c r="I70" s="8" t="n">
-        <v>697</v>
+        <v>486</v>
       </c>
       <c r="J70" s="8" t="n"/>
       <c r="K70" s="8" t="n"/>
       <c r="L70" s="8" t="n"/>
       <c r="M70" s="8" t="n"/>
       <c r="N70" s="8" t="n">
-        <v>20820</v>
+        <v>21504</v>
       </c>
       <c r="O70" s="8" t="n">
         <v>0</v>
@@ -22224,12 +22220,12 @@
       <c r="P70" s="8" t="n"/>
       <c r="Q70" s="8" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R70" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S70" s="9" t="inlineStr"/>
@@ -22246,7 +22242,7 @@
       <c r="V70" s="7" t="inlineStr"/>
       <c r="W70" s="8" t="inlineStr">
         <is>
-          <t>5870266ee1b15bf20f0a085f56358c762e522fa8</t>
+          <t>67ff71428df47b0eb7f7da47600378ffdad1f97c</t>
         </is>
       </c>
     </row>
@@ -22260,10 +22256,10 @@
         </is>
       </c>
       <c r="C71" s="17" t="n">
-        <v>1300</v>
+        <v>1965</v>
       </c>
       <c r="D71" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E71" s="8" t="n">
         <v>1</v>
@@ -22275,7 +22271,7 @@
       </c>
       <c r="G71" s="9" t="inlineStr">
         <is>
-          <t>Bristol City Centre, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H71" s="8" t="inlineStr">
@@ -22283,13 +22279,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I71" s="8" t="n"/>
+      <c r="I71" s="8" t="n">
+        <v>655</v>
+      </c>
       <c r="J71" s="8" t="n"/>
       <c r="K71" s="8" t="n"/>
       <c r="L71" s="8" t="n"/>
       <c r="M71" s="8" t="n"/>
       <c r="N71" s="8" t="n">
-        <v>21428</v>
+        <v>21504</v>
       </c>
       <c r="O71" s="8" t="n">
         <v>0</v>
@@ -22297,12 +22295,12 @@
       <c r="P71" s="8" t="n"/>
       <c r="Q71" s="8" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="R71" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S71" s="9" t="inlineStr"/>
@@ -22319,7 +22317,7 @@
       <c r="V71" s="7" t="inlineStr"/>
       <c r="W71" s="8" t="inlineStr">
         <is>
-          <t>317e9ab29cad2381c41672743d877feba2c14e45</t>
+          <t>1a5b509e1606992acea1736489630b2bc57cc717</t>
         </is>
       </c>
     </row>
@@ -22333,13 +22331,13 @@
         </is>
       </c>
       <c r="C72" s="17" t="n">
-        <v>1500</v>
+        <v>2080</v>
       </c>
       <c r="D72" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E72" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F72" s="8" t="inlineStr">
         <is>
@@ -22348,7 +22346,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
@@ -22357,14 +22355,14 @@
         </is>
       </c>
       <c r="I72" s="8" t="n">
-        <v>548</v>
+        <v>705</v>
       </c>
       <c r="J72" s="8" t="n"/>
       <c r="K72" s="8" t="n"/>
       <c r="L72" s="8" t="n"/>
       <c r="M72" s="8" t="n"/>
       <c r="N72" s="8" t="n">
-        <v>21504</v>
+        <v>20820</v>
       </c>
       <c r="O72" s="8" t="n">
         <v>0</v>
@@ -22372,12 +22370,12 @@
       <c r="P72" s="8" t="n"/>
       <c r="Q72" s="8" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="R72" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S72" s="9" t="inlineStr"/>
@@ -22394,7 +22392,7 @@
       <c r="V72" s="7" t="inlineStr"/>
       <c r="W72" s="8" t="inlineStr">
         <is>
-          <t>bad1e4584285201ef9995d2b437343fca870009c</t>
+          <t>0453e07b653a16ada93327f26a41e0b204d289a4</t>
         </is>
       </c>
     </row>
@@ -22408,7 +22406,7 @@
         </is>
       </c>
       <c r="C73" s="17" t="n">
-        <v>1615</v>
+        <v>1400</v>
       </c>
       <c r="D73" s="8" t="n">
         <v>1</v>
@@ -22423,7 +22421,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Redcliffe Parade West, Flat 3, City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H73" s="8" t="inlineStr">
@@ -22431,15 +22429,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I73" s="8" t="n">
-        <v>486</v>
-      </c>
+      <c r="I73" s="8" t="n"/>
       <c r="J73" s="8" t="n"/>
       <c r="K73" s="8" t="n"/>
       <c r="L73" s="8" t="n"/>
       <c r="M73" s="8" t="n"/>
       <c r="N73" s="8" t="n">
-        <v>21504</v>
+        <v>19484</v>
       </c>
       <c r="O73" s="8" t="n">
         <v>0</v>
@@ -22447,12 +22443,12 @@
       <c r="P73" s="8" t="n"/>
       <c r="Q73" s="8" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="R73" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S73" s="9" t="inlineStr"/>
@@ -22469,7 +22465,7 @@
       <c r="V73" s="7" t="inlineStr"/>
       <c r="W73" s="8" t="inlineStr">
         <is>
-          <t>67ff71428df47b0eb7f7da47600378ffdad1f97c</t>
+          <t>9b65e5a0fb0bc8fc27d566eae912cddf76828cc9</t>
         </is>
       </c>
     </row>
@@ -22483,13 +22479,13 @@
         </is>
       </c>
       <c r="C74" s="17" t="n">
-        <v>1965</v>
+        <v>2000</v>
       </c>
       <c r="D74" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E74" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F74" s="8" t="inlineStr">
         <is>
@@ -22498,7 +22494,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Welsh Back, Bristol, BS1</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr">
@@ -22507,15 +22503,13 @@
         </is>
       </c>
       <c r="I74" s="8" t="n">
-        <v>655</v>
+        <v>908</v>
       </c>
       <c r="J74" s="8" t="n"/>
       <c r="K74" s="8" t="n"/>
       <c r="L74" s="8" t="n"/>
       <c r="M74" s="8" t="n"/>
-      <c r="N74" s="8" t="n">
-        <v>21504</v>
-      </c>
+      <c r="N74" s="8" t="n"/>
       <c r="O74" s="8" t="n">
         <v>0</v>
       </c>
@@ -22527,7 +22521,7 @@
       </c>
       <c r="R74" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Hello Neighbour, London</t>
         </is>
       </c>
       <c r="S74" s="9" t="inlineStr"/>
@@ -22544,7 +22538,7 @@
       <c r="V74" s="7" t="inlineStr"/>
       <c r="W74" s="8" t="inlineStr">
         <is>
-          <t>1a5b509e1606992acea1736489630b2bc57cc717</t>
+          <t>65ed2520fdf37e6dde4abe0097cc3edbbbeff957</t>
         </is>
       </c>
     </row>
@@ -22558,7 +22552,7 @@
         </is>
       </c>
       <c r="C75" s="17" t="n">
-        <v>2080</v>
+        <v>2020</v>
       </c>
       <c r="D75" s="8" t="n">
         <v>2</v>
@@ -22588,16 +22582,14 @@
       <c r="K75" s="8" t="n"/>
       <c r="L75" s="8" t="n"/>
       <c r="M75" s="8" t="n"/>
-      <c r="N75" s="8" t="n">
-        <v>20820</v>
-      </c>
+      <c r="N75" s="8" t="n"/>
       <c r="O75" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P75" s="8" t="n"/>
       <c r="Q75" s="8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="R75" s="8" t="inlineStr">
@@ -22619,7 +22611,7 @@
       <c r="V75" s="7" t="inlineStr"/>
       <c r="W75" s="8" t="inlineStr">
         <is>
-          <t>0453e07b653a16ada93327f26a41e0b204d289a4</t>
+          <t>75b3ee81b8ecb4015a80108f6d509e4156f4e8e4</t>
         </is>
       </c>
     </row>
@@ -22633,13 +22625,13 @@
         </is>
       </c>
       <c r="C76" s="17" t="n">
-        <v>1400</v>
+        <v>2000</v>
       </c>
       <c r="D76" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E76" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
@@ -22648,7 +22640,7 @@
       </c>
       <c r="G76" s="9" t="inlineStr">
         <is>
-          <t>Redcliffe Parade West, Flat 3, City Centre, Bristol, BS1</t>
+          <t>Eclipse - City Centre</t>
         </is>
       </c>
       <c r="H76" s="8" t="inlineStr">
@@ -22661,21 +22653,19 @@
       <c r="K76" s="8" t="n"/>
       <c r="L76" s="8" t="n"/>
       <c r="M76" s="8" t="n"/>
-      <c r="N76" s="8" t="n">
-        <v>19484</v>
-      </c>
+      <c r="N76" s="8" t="n"/>
       <c r="O76" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P76" s="8" t="n"/>
       <c r="Q76" s="8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="R76" s="8" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>Ocean, Clifton</t>
         </is>
       </c>
       <c r="S76" s="9" t="inlineStr"/>
@@ -22692,7 +22682,7 @@
       <c r="V76" s="7" t="inlineStr"/>
       <c r="W76" s="8" t="inlineStr">
         <is>
-          <t>9b65e5a0fb0bc8fc27d566eae912cddf76828cc9</t>
+          <t>638ecbe81729048ffda61524ca9b06c4a208ce7b</t>
         </is>
       </c>
     </row>
@@ -22706,13 +22696,13 @@
         </is>
       </c>
       <c r="C77" s="17" t="n">
-        <v>2000</v>
+        <v>2085</v>
       </c>
       <c r="D77" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E77" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F77" s="8" t="inlineStr">
         <is>
@@ -22721,7 +22711,7 @@
       </c>
       <c r="G77" s="9" t="inlineStr">
         <is>
-          <t>Welsh Back, Bristol, BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H77" s="8" t="inlineStr">
@@ -22730,7 +22720,7 @@
         </is>
       </c>
       <c r="I77" s="8" t="n">
-        <v>908</v>
+        <v>705</v>
       </c>
       <c r="J77" s="8" t="n"/>
       <c r="K77" s="8" t="n"/>
@@ -22743,12 +22733,12 @@
       <c r="P77" s="8" t="n"/>
       <c r="Q77" s="8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="R77" s="8" t="inlineStr">
         <is>
-          <t>Hello Neighbour, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S77" s="9" t="inlineStr"/>
@@ -22765,7 +22755,7 @@
       <c r="V77" s="7" t="inlineStr"/>
       <c r="W77" s="8" t="inlineStr">
         <is>
-          <t>65ed2520fdf37e6dde4abe0097cc3edbbbeff957</t>
+          <t>16c89eb9a4cdeb57ddb3fd1201b7084ea2f3c007</t>
         </is>
       </c>
     </row>
@@ -22779,13 +22769,13 @@
         </is>
       </c>
       <c r="C78" s="17" t="n">
-        <v>2020</v>
+        <v>1615</v>
       </c>
       <c r="D78" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E78" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F78" s="8" t="inlineStr">
         <is>
@@ -22794,7 +22784,7 @@
       </c>
       <c r="G78" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H78" s="8" t="inlineStr">
@@ -22803,7 +22793,7 @@
         </is>
       </c>
       <c r="I78" s="8" t="n">
-        <v>705</v>
+        <v>487</v>
       </c>
       <c r="J78" s="8" t="n"/>
       <c r="K78" s="8" t="n"/>
@@ -22816,12 +22806,12 @@
       <c r="P78" s="8" t="n"/>
       <c r="Q78" s="8" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="R78" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S78" s="9" t="inlineStr"/>
@@ -22838,7 +22828,7 @@
       <c r="V78" s="7" t="inlineStr"/>
       <c r="W78" s="8" t="inlineStr">
         <is>
-          <t>75b3ee81b8ecb4015a80108f6d509e4156f4e8e4</t>
+          <t>cd57661c8d996d20c5c1c7c34b12787f40073ec9</t>
         </is>
       </c>
     </row>
@@ -22852,7 +22842,7 @@
         </is>
       </c>
       <c r="C79" s="17" t="n">
-        <v>2000</v>
+        <v>2065</v>
       </c>
       <c r="D79" s="8" t="n">
         <v>2</v>
@@ -22867,7 +22857,7 @@
       </c>
       <c r="G79" s="9" t="inlineStr">
         <is>
-          <t>Eclipse - City Centre</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H79" s="8" t="inlineStr">
@@ -22875,7 +22865,9 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I79" s="8" t="n"/>
+      <c r="I79" s="8" t="n">
+        <v>641</v>
+      </c>
       <c r="J79" s="8" t="n"/>
       <c r="K79" s="8" t="n"/>
       <c r="L79" s="8" t="n"/>
@@ -22887,12 +22879,12 @@
       <c r="P79" s="8" t="n"/>
       <c r="Q79" s="8" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="R79" s="8" t="inlineStr">
         <is>
-          <t>Ocean, Clifton</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S79" s="9" t="inlineStr"/>
@@ -22909,7 +22901,7 @@
       <c r="V79" s="7" t="inlineStr"/>
       <c r="W79" s="8" t="inlineStr">
         <is>
-          <t>638ecbe81729048ffda61524ca9b06c4a208ce7b</t>
+          <t>d23eb397c84a723416c257acf4e25973ede40bc5</t>
         </is>
       </c>
     </row>
@@ -22923,13 +22915,13 @@
         </is>
       </c>
       <c r="C80" s="17" t="n">
-        <v>1595</v>
+        <v>2185</v>
       </c>
       <c r="D80" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E80" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F80" s="8" t="inlineStr">
         <is>
@@ -22938,7 +22930,7 @@
       </c>
       <c r="G80" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H80" s="8" t="inlineStr">
@@ -22947,7 +22939,7 @@
         </is>
       </c>
       <c r="I80" s="8" t="n">
-        <v>499</v>
+        <v>721</v>
       </c>
       <c r="J80" s="8" t="n"/>
       <c r="K80" s="8" t="n"/>
@@ -22960,12 +22952,12 @@
       <c r="P80" s="8" t="n"/>
       <c r="Q80" s="8" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="R80" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S80" s="9" t="inlineStr"/>
@@ -22982,7 +22974,7 @@
       <c r="V80" s="7" t="inlineStr"/>
       <c r="W80" s="8" t="inlineStr">
         <is>
-          <t>f2f3afa9f34b35c1d7d84b8e8f6c80b9a91340b1</t>
+          <t>6446e0c7d9c4f21f9eb6239caeeeee0599a68101</t>
         </is>
       </c>
     </row>
@@ -22996,13 +22988,13 @@
         </is>
       </c>
       <c r="C81" s="17" t="n">
-        <v>2085</v>
+        <v>1565</v>
       </c>
       <c r="D81" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E81" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F81" s="8" t="inlineStr">
         <is>
@@ -23011,7 +23003,7 @@
       </c>
       <c r="G81" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H81" s="8" t="inlineStr">
@@ -23020,7 +23012,7 @@
         </is>
       </c>
       <c r="I81" s="8" t="n">
-        <v>705</v>
+        <v>484</v>
       </c>
       <c r="J81" s="8" t="n"/>
       <c r="K81" s="8" t="n"/>
@@ -23033,12 +23025,12 @@
       <c r="P81" s="8" t="n"/>
       <c r="Q81" s="8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="R81" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S81" s="9" t="inlineStr"/>
@@ -23055,7 +23047,7 @@
       <c r="V81" s="7" t="inlineStr"/>
       <c r="W81" s="8" t="inlineStr">
         <is>
-          <t>16c89eb9a4cdeb57ddb3fd1201b7084ea2f3c007</t>
+          <t>34d9877a23c82be120784d9dd55c23c17584c91a</t>
         </is>
       </c>
     </row>
@@ -23069,7 +23061,7 @@
         </is>
       </c>
       <c r="C82" s="17" t="n">
-        <v>1615</v>
+        <v>1650</v>
       </c>
       <c r="D82" s="8" t="n">
         <v>1</v>
@@ -23084,7 +23076,7 @@
       </c>
       <c r="G82" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Horizon, Broad Weir, Bristol, BS1</t>
         </is>
       </c>
       <c r="H82" s="8" t="inlineStr">
@@ -23092,9 +23084,7 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I82" s="8" t="n">
-        <v>487</v>
-      </c>
+      <c r="I82" s="8" t="n"/>
       <c r="J82" s="8" t="n"/>
       <c r="K82" s="8" t="n"/>
       <c r="L82" s="8" t="n"/>
@@ -23106,12 +23096,12 @@
       <c r="P82" s="8" t="n"/>
       <c r="Q82" s="8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="R82" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>CJ Hole, Bishopston</t>
         </is>
       </c>
       <c r="S82" s="9" t="inlineStr"/>
@@ -23128,7 +23118,7 @@
       <c r="V82" s="7" t="inlineStr"/>
       <c r="W82" s="8" t="inlineStr">
         <is>
-          <t>cd57661c8d996d20c5c1c7c34b12787f40073ec9</t>
+          <t>aa3cf620ad25601a026424157bd8c0abb746373f</t>
         </is>
       </c>
     </row>
@@ -23142,13 +23132,13 @@
         </is>
       </c>
       <c r="C83" s="17" t="n">
-        <v>2065</v>
+        <v>2100</v>
       </c>
       <c r="D83" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E83" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F83" s="8" t="inlineStr">
         <is>
@@ -23157,7 +23147,7 @@
       </c>
       <c r="G83" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>The Three Kings Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H83" s="8" t="inlineStr">
@@ -23165,9 +23155,7 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I83" s="8" t="n">
-        <v>641</v>
-      </c>
+      <c r="I83" s="8" t="n"/>
       <c r="J83" s="8" t="n"/>
       <c r="K83" s="8" t="n"/>
       <c r="L83" s="8" t="n"/>
@@ -23179,12 +23167,12 @@
       <c r="P83" s="8" t="n"/>
       <c r="Q83" s="8" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="R83" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S83" s="9" t="inlineStr"/>
@@ -23201,7 +23189,7 @@
       <c r="V83" s="7" t="inlineStr"/>
       <c r="W83" s="8" t="inlineStr">
         <is>
-          <t>d23eb397c84a723416c257acf4e25973ede40bc5</t>
+          <t>954007c82f6f3a495c465b72c9a1c44c0c84713e</t>
         </is>
       </c>
     </row>
@@ -23215,13 +23203,13 @@
         </is>
       </c>
       <c r="C84" s="17" t="n">
-        <v>2185</v>
+        <v>1660</v>
       </c>
       <c r="D84" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E84" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F84" s="8" t="inlineStr">
         <is>
@@ -23239,20 +23227,22 @@
         </is>
       </c>
       <c r="I84" s="8" t="n">
-        <v>721</v>
+        <v>486</v>
       </c>
       <c r="J84" s="8" t="n"/>
       <c r="K84" s="8" t="n"/>
       <c r="L84" s="8" t="n"/>
       <c r="M84" s="8" t="n"/>
-      <c r="N84" s="8" t="n"/>
+      <c r="N84" s="8" t="n">
+        <v>21504</v>
+      </c>
       <c r="O84" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P84" s="8" t="n"/>
       <c r="Q84" s="8" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R84" s="8" t="inlineStr">
@@ -23274,7 +23264,7 @@
       <c r="V84" s="7" t="inlineStr"/>
       <c r="W84" s="8" t="inlineStr">
         <is>
-          <t>6446e0c7d9c4f21f9eb6239caeeeee0599a68101</t>
+          <t>c2c660e4e8cefc047b4bc72bf19b48ce9ef7ec99</t>
         </is>
       </c>
     </row>
@@ -23288,13 +23278,13 @@
         </is>
       </c>
       <c r="C85" s="17" t="n">
-        <v>1565</v>
+        <v>2175</v>
       </c>
       <c r="D85" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E85" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F85" s="8" t="inlineStr">
         <is>
@@ -23303,7 +23293,7 @@
       </c>
       <c r="G85" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H85" s="8" t="inlineStr">
@@ -23312,25 +23302,27 @@
         </is>
       </c>
       <c r="I85" s="8" t="n">
-        <v>484</v>
+        <v>814</v>
       </c>
       <c r="J85" s="8" t="n"/>
       <c r="K85" s="8" t="n"/>
       <c r="L85" s="8" t="n"/>
       <c r="M85" s="8" t="n"/>
-      <c r="N85" s="8" t="n"/>
+      <c r="N85" s="8" t="n">
+        <v>21504</v>
+      </c>
       <c r="O85" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P85" s="8" t="n"/>
       <c r="Q85" s="8" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R85" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S85" s="9" t="inlineStr"/>
@@ -23347,7 +23339,7 @@
       <c r="V85" s="7" t="inlineStr"/>
       <c r="W85" s="8" t="inlineStr">
         <is>
-          <t>34d9877a23c82be120784d9dd55c23c17584c91a</t>
+          <t>83406f05c9aded812a566cc6806036dda0d45fc0</t>
         </is>
       </c>
     </row>
@@ -23361,13 +23353,13 @@
         </is>
       </c>
       <c r="C86" s="17" t="n">
-        <v>1650</v>
+        <v>1500</v>
       </c>
       <c r="D86" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E86" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F86" s="8" t="inlineStr">
         <is>
@@ -23376,7 +23368,7 @@
       </c>
       <c r="G86" s="9" t="inlineStr">
         <is>
-          <t>Horizon, Broad Weir, Bristol, BS1</t>
+          <t>Small Street - City Centre</t>
         </is>
       </c>
       <c r="H86" s="8" t="inlineStr">
@@ -23389,19 +23381,21 @@
       <c r="K86" s="8" t="n"/>
       <c r="L86" s="8" t="n"/>
       <c r="M86" s="8" t="n"/>
-      <c r="N86" s="8" t="n"/>
+      <c r="N86" s="8" t="n">
+        <v>21816</v>
+      </c>
       <c r="O86" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P86" s="8" t="n"/>
       <c r="Q86" s="8" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R86" s="8" t="inlineStr">
         <is>
-          <t>CJ Hole, Bishopston</t>
+          <t>Ocean, Clifton</t>
         </is>
       </c>
       <c r="S86" s="9" t="inlineStr"/>
@@ -23418,7 +23412,7 @@
       <c r="V86" s="7" t="inlineStr"/>
       <c r="W86" s="8" t="inlineStr">
         <is>
-          <t>aa3cf620ad25601a026424157bd8c0abb746373f</t>
+          <t>cb4b1af676ff54ae12ad7bf4fa94acd8ef94a533</t>
         </is>
       </c>
     </row>
@@ -23432,13 +23426,13 @@
         </is>
       </c>
       <c r="C87" s="17" t="n">
-        <v>1625</v>
+        <v>2115</v>
       </c>
       <c r="D87" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E87" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F87" s="8" t="inlineStr">
         <is>
@@ -23447,7 +23441,7 @@
       </c>
       <c r="G87" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H87" s="8" t="inlineStr">
@@ -23456,25 +23450,27 @@
         </is>
       </c>
       <c r="I87" s="8" t="n">
-        <v>485</v>
+        <v>823</v>
       </c>
       <c r="J87" s="8" t="n"/>
       <c r="K87" s="8" t="n"/>
       <c r="L87" s="8" t="n"/>
       <c r="M87" s="8" t="n"/>
-      <c r="N87" s="8" t="n"/>
+      <c r="N87" s="8" t="n">
+        <v>20820</v>
+      </c>
       <c r="O87" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P87" s="8" t="n"/>
       <c r="Q87" s="8" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="R87" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S87" s="9" t="inlineStr"/>
@@ -23491,7 +23487,7 @@
       <c r="V87" s="7" t="inlineStr"/>
       <c r="W87" s="8" t="inlineStr">
         <is>
-          <t>ea3758a9fd1b4190b4e5ae17519645f00d2e6a8f</t>
+          <t>0b78c6e29d96ae73c643d0d50d50949797b02893</t>
         </is>
       </c>
     </row>
@@ -23505,13 +23501,13 @@
         </is>
       </c>
       <c r="C88" s="17" t="n">
-        <v>2175</v>
+        <v>1660</v>
       </c>
       <c r="D88" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E88" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F88" s="8" t="inlineStr">
         <is>
@@ -23529,20 +23525,22 @@
         </is>
       </c>
       <c r="I88" s="8" t="n">
-        <v>722</v>
+        <v>486</v>
       </c>
       <c r="J88" s="8" t="n"/>
       <c r="K88" s="8" t="n"/>
       <c r="L88" s="8" t="n"/>
       <c r="M88" s="8" t="n"/>
-      <c r="N88" s="8" t="n"/>
+      <c r="N88" s="8" t="n">
+        <v>21504</v>
+      </c>
       <c r="O88" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P88" s="8" t="n"/>
       <c r="Q88" s="8" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="R88" s="8" t="inlineStr">
@@ -23564,7 +23562,7 @@
       <c r="V88" s="7" t="inlineStr"/>
       <c r="W88" s="8" t="inlineStr">
         <is>
-          <t>ab566c9b065047cd166a2ad3ae56e88704bc1358</t>
+          <t>c798c669d03fa2e42fd418ff0916de022d3380ad</t>
         </is>
       </c>
     </row>
@@ -23578,13 +23576,13 @@
         </is>
       </c>
       <c r="C89" s="17" t="n">
-        <v>2100</v>
+        <v>1915</v>
       </c>
       <c r="D89" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E89" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F89" s="8" t="inlineStr">
         <is>
@@ -23593,7 +23591,7 @@
       </c>
       <c r="G89" s="9" t="inlineStr">
         <is>
-          <t>The Three Kings Court, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H89" s="8" t="inlineStr">
@@ -23601,24 +23599,28 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I89" s="8" t="n"/>
+      <c r="I89" s="8" t="n">
+        <v>746</v>
+      </c>
       <c r="J89" s="8" t="n"/>
       <c r="K89" s="8" t="n"/>
       <c r="L89" s="8" t="n"/>
       <c r="M89" s="8" t="n"/>
-      <c r="N89" s="8" t="n"/>
+      <c r="N89" s="8" t="n">
+        <v>21680</v>
+      </c>
       <c r="O89" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P89" s="8" t="n"/>
       <c r="Q89" s="8" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="R89" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S89" s="9" t="inlineStr"/>
@@ -23635,7 +23637,7 @@
       <c r="V89" s="7" t="inlineStr"/>
       <c r="W89" s="8" t="inlineStr">
         <is>
-          <t>954007c82f6f3a495c465b72c9a1c44c0c84713e</t>
+          <t>36797023cff0095f1bf764fa2f176d5595124854</t>
         </is>
       </c>
     </row>
@@ -23649,13 +23651,13 @@
         </is>
       </c>
       <c r="C90" s="17" t="n">
-        <v>1900</v>
+        <v>1150</v>
       </c>
       <c r="D90" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E90" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F90" s="8" t="inlineStr">
         <is>
@@ -23664,12 +23666,12 @@
       </c>
       <c r="G90" s="9" t="inlineStr">
         <is>
-          <t>The Granary, Queen Charlotte Street, BRISTOL, BS1</t>
+          <t>Knowle Road, Bristol</t>
         </is>
       </c>
       <c r="H90" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS4</t>
         </is>
       </c>
       <c r="I90" s="8" t="n"/>
@@ -23677,19 +23679,21 @@
       <c r="K90" s="8" t="n"/>
       <c r="L90" s="8" t="n"/>
       <c r="M90" s="8" t="n"/>
-      <c r="N90" s="8" t="n"/>
+      <c r="N90" s="8" t="n">
+        <v>6872</v>
+      </c>
       <c r="O90" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P90" s="8" t="n"/>
       <c r="Q90" s="8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R90" s="8" t="inlineStr">
         <is>
-          <t>Andrews Letting and Management, Clifton</t>
+          <t>Hopewell, Bristol</t>
         </is>
       </c>
       <c r="S90" s="9" t="inlineStr"/>
@@ -23706,7 +23710,7 @@
       <c r="V90" s="7" t="inlineStr"/>
       <c r="W90" s="8" t="inlineStr">
         <is>
-          <t>b19bc62dddbc90526344a15be65fbc2e74a96d22</t>
+          <t>edac1b499f84e07ce85894b488f82dc5cd104202</t>
         </is>
       </c>
     </row>
@@ -23720,13 +23724,13 @@
         </is>
       </c>
       <c r="C91" s="17" t="n">
-        <v>1660</v>
+        <v>2450</v>
       </c>
       <c r="D91" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E91" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F91" s="8" t="inlineStr">
         <is>
@@ -23735,7 +23739,7 @@
       </c>
       <c r="G91" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>The Herbert Ashman Building, Bristol, BS1</t>
         </is>
       </c>
       <c r="H91" s="8" t="inlineStr">
@@ -23743,15 +23747,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I91" s="8" t="n">
-        <v>486</v>
-      </c>
+      <c r="I91" s="8" t="n"/>
       <c r="J91" s="8" t="n"/>
       <c r="K91" s="8" t="n"/>
       <c r="L91" s="8" t="n"/>
       <c r="M91" s="8" t="n"/>
       <c r="N91" s="8" t="n">
-        <v>21504</v>
+        <v>21788</v>
       </c>
       <c r="O91" s="8" t="n">
         <v>0</v>
@@ -23759,12 +23761,12 @@
       <c r="P91" s="8" t="n"/>
       <c r="Q91" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R91" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S91" s="9" t="inlineStr"/>
@@ -23781,7 +23783,7 @@
       <c r="V91" s="7" t="inlineStr"/>
       <c r="W91" s="8" t="inlineStr">
         <is>
-          <t>c2c660e4e8cefc047b4bc72bf19b48ce9ef7ec99</t>
+          <t>4cd4fdc09f26b6316c31aa22f38853db44d1ea9a</t>
         </is>
       </c>
     </row>
@@ -23795,7 +23797,7 @@
         </is>
       </c>
       <c r="C92" s="17" t="n">
-        <v>2175</v>
+        <v>1700</v>
       </c>
       <c r="D92" s="8" t="n">
         <v>2</v>
@@ -23810,7 +23812,7 @@
       </c>
       <c r="G92" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>The Crescent</t>
         </is>
       </c>
       <c r="H92" s="8" t="inlineStr">
@@ -23818,15 +23820,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I92" s="8" t="n">
-        <v>814</v>
-      </c>
+      <c r="I92" s="8" t="n"/>
       <c r="J92" s="8" t="n"/>
       <c r="K92" s="8" t="n"/>
       <c r="L92" s="8" t="n"/>
       <c r="M92" s="8" t="n"/>
       <c r="N92" s="8" t="n">
-        <v>21504</v>
+        <v>16368</v>
       </c>
       <c r="O92" s="8" t="n">
         <v>0</v>
@@ -23834,12 +23834,12 @@
       <c r="P92" s="8" t="n"/>
       <c r="Q92" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R92" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S92" s="9" t="inlineStr"/>
@@ -23856,7 +23856,7 @@
       <c r="V92" s="7" t="inlineStr"/>
       <c r="W92" s="8" t="inlineStr">
         <is>
-          <t>83406f05c9aded812a566cc6806036dda0d45fc0</t>
+          <t>8a8446c119238f7a042580aed1922ef6cfd79ae2</t>
         </is>
       </c>
     </row>
@@ -23870,13 +23870,13 @@
         </is>
       </c>
       <c r="C93" s="17" t="n">
-        <v>1500</v>
+        <v>1250</v>
       </c>
       <c r="D93" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E93" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F93" s="8" t="inlineStr">
         <is>
@@ -23885,7 +23885,7 @@
       </c>
       <c r="G93" s="9" t="inlineStr">
         <is>
-          <t>Small Street - City Centre</t>
+          <t>Victoria Street, Bristol, BS1 6DR</t>
         </is>
       </c>
       <c r="H93" s="8" t="inlineStr">
@@ -23899,7 +23899,7 @@
       <c r="L93" s="8" t="n"/>
       <c r="M93" s="8" t="n"/>
       <c r="N93" s="8" t="n">
-        <v>21816</v>
+        <v>21160</v>
       </c>
       <c r="O93" s="8" t="n">
         <v>0</v>
@@ -23907,12 +23907,12 @@
       <c r="P93" s="8" t="n"/>
       <c r="Q93" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R93" s="8" t="inlineStr">
         <is>
-          <t>Ocean, Clifton</t>
+          <t>Visum, Nationwide</t>
         </is>
       </c>
       <c r="S93" s="9" t="inlineStr"/>
@@ -23929,7 +23929,7 @@
       <c r="V93" s="7" t="inlineStr"/>
       <c r="W93" s="8" t="inlineStr">
         <is>
-          <t>cb4b1af676ff54ae12ad7bf4fa94acd8ef94a533</t>
+          <t>78fe8e0511ccc37f104368075238c845f57d7864</t>
         </is>
       </c>
     </row>
@@ -23943,13 +23943,13 @@
         </is>
       </c>
       <c r="C94" s="17" t="n">
-        <v>2115</v>
+        <v>1999</v>
       </c>
       <c r="D94" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E94" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F94" s="8" t="inlineStr">
         <is>
@@ -23958,7 +23958,7 @@
       </c>
       <c r="G94" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Swann House, Bristol, BS1</t>
         </is>
       </c>
       <c r="H94" s="8" t="inlineStr">
@@ -23966,15 +23966,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I94" s="8" t="n">
-        <v>823</v>
-      </c>
+      <c r="I94" s="8" t="n"/>
       <c r="J94" s="8" t="n"/>
       <c r="K94" s="8" t="n"/>
       <c r="L94" s="8" t="n"/>
       <c r="M94" s="8" t="n"/>
       <c r="N94" s="8" t="n">
-        <v>20820</v>
+        <v>20800</v>
       </c>
       <c r="O94" s="8" t="n">
         <v>0</v>
@@ -23982,12 +23980,12 @@
       <c r="P94" s="8" t="n"/>
       <c r="Q94" s="8" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R94" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S94" s="9" t="inlineStr"/>
@@ -24004,7 +24002,7 @@
       <c r="V94" s="7" t="inlineStr"/>
       <c r="W94" s="8" t="inlineStr">
         <is>
-          <t>0b78c6e29d96ae73c643d0d50d50949797b02893</t>
+          <t>5cec67aa8ba885c4c8f85e47d3354d187da9d897</t>
         </is>
       </c>
     </row>
@@ -24018,7 +24016,7 @@
         </is>
       </c>
       <c r="C95" s="17" t="n">
-        <v>1660</v>
+        <v>1670</v>
       </c>
       <c r="D95" s="8" t="n">
         <v>1</v>
@@ -24042,7 +24040,7 @@
         </is>
       </c>
       <c r="I95" s="8" t="n">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="J95" s="8" t="n"/>
       <c r="K95" s="8" t="n"/>
@@ -24057,7 +24055,7 @@
       <c r="P95" s="8" t="n"/>
       <c r="Q95" s="8" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R95" s="8" t="inlineStr">
@@ -24079,7 +24077,7 @@
       <c r="V95" s="7" t="inlineStr"/>
       <c r="W95" s="8" t="inlineStr">
         <is>
-          <t>c798c669d03fa2e42fd418ff0916de022d3380ad</t>
+          <t>73f3509a6c69eef7af4c6b9ff0dc69b97478c20a</t>
         </is>
       </c>
     </row>
@@ -24093,13 +24091,13 @@
         </is>
       </c>
       <c r="C96" s="17" t="n">
-        <v>1915</v>
+        <v>1645</v>
       </c>
       <c r="D96" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E96" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F96" s="8" t="inlineStr">
         <is>
@@ -24108,7 +24106,7 @@
       </c>
       <c r="G96" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H96" s="8" t="inlineStr">
@@ -24117,14 +24115,14 @@
         </is>
       </c>
       <c r="I96" s="8" t="n">
-        <v>746</v>
+        <v>517</v>
       </c>
       <c r="J96" s="8" t="n"/>
       <c r="K96" s="8" t="n"/>
       <c r="L96" s="8" t="n"/>
       <c r="M96" s="8" t="n"/>
       <c r="N96" s="8" t="n">
-        <v>21680</v>
+        <v>20820</v>
       </c>
       <c r="O96" s="8" t="n">
         <v>0</v>
@@ -24132,12 +24130,12 @@
       <c r="P96" s="8" t="n"/>
       <c r="Q96" s="8" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R96" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S96" s="9" t="inlineStr"/>
@@ -24154,7 +24152,7 @@
       <c r="V96" s="7" t="inlineStr"/>
       <c r="W96" s="8" t="inlineStr">
         <is>
-          <t>36797023cff0095f1bf764fa2f176d5595124854</t>
+          <t>4efcb79ae710a68f5f272a2f9030937499117f9d</t>
         </is>
       </c>
     </row>
@@ -24168,13 +24166,13 @@
         </is>
       </c>
       <c r="C97" s="17" t="n">
-        <v>1150</v>
+        <v>2120</v>
       </c>
       <c r="D97" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E97" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F97" s="8" t="inlineStr">
         <is>
@@ -24183,21 +24181,23 @@
       </c>
       <c r="G97" s="9" t="inlineStr">
         <is>
-          <t>Knowle Road, Bristol</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H97" s="8" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I97" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I97" s="8" t="n">
+        <v>705</v>
+      </c>
       <c r="J97" s="8" t="n"/>
       <c r="K97" s="8" t="n"/>
       <c r="L97" s="8" t="n"/>
       <c r="M97" s="8" t="n"/>
       <c r="N97" s="8" t="n">
-        <v>6872</v>
+        <v>20820</v>
       </c>
       <c r="O97" s="8" t="n">
         <v>0</v>
@@ -24205,12 +24205,12 @@
       <c r="P97" s="8" t="n"/>
       <c r="Q97" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="R97" s="8" t="inlineStr">
         <is>
-          <t>Hopewell, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S97" s="9" t="inlineStr"/>
@@ -24227,7 +24227,7 @@
       <c r="V97" s="7" t="inlineStr"/>
       <c r="W97" s="8" t="inlineStr">
         <is>
-          <t>edac1b499f84e07ce85894b488f82dc5cd104202</t>
+          <t>c5c1741357dfce3547bdab7d4d5a0e7602846192</t>
         </is>
       </c>
     </row>
@@ -24241,13 +24241,13 @@
         </is>
       </c>
       <c r="C98" s="17" t="n">
-        <v>2450</v>
+        <v>1645</v>
       </c>
       <c r="D98" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E98" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F98" s="8" t="inlineStr">
         <is>
@@ -24256,7 +24256,7 @@
       </c>
       <c r="G98" s="9" t="inlineStr">
         <is>
-          <t>The Herbert Ashman Building, Bristol, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H98" s="8" t="inlineStr">
@@ -24264,13 +24264,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I98" s="8" t="n"/>
+      <c r="I98" s="8" t="n">
+        <v>571</v>
+      </c>
       <c r="J98" s="8" t="n"/>
       <c r="K98" s="8" t="n"/>
       <c r="L98" s="8" t="n"/>
       <c r="M98" s="8" t="n"/>
       <c r="N98" s="8" t="n">
-        <v>21788</v>
+        <v>20820</v>
       </c>
       <c r="O98" s="8" t="n">
         <v>0</v>
@@ -24278,12 +24280,12 @@
       <c r="P98" s="8" t="n"/>
       <c r="Q98" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="R98" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S98" s="9" t="inlineStr"/>
@@ -24300,7 +24302,7 @@
       <c r="V98" s="7" t="inlineStr"/>
       <c r="W98" s="8" t="inlineStr">
         <is>
-          <t>4cd4fdc09f26b6316c31aa22f38853db44d1ea9a</t>
+          <t>487e67b2d6680ebaabfcc49d4d33e21cb65cca6d</t>
         </is>
       </c>
     </row>
@@ -24314,13 +24316,13 @@
         </is>
       </c>
       <c r="C99" s="17" t="n">
-        <v>1700</v>
+        <v>1950</v>
       </c>
       <c r="D99" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E99" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F99" s="8" t="inlineStr">
         <is>
@@ -24329,7 +24331,7 @@
       </c>
       <c r="G99" s="9" t="inlineStr">
         <is>
-          <t>The Crescent</t>
+          <t>Apartments, Bristol, BS1</t>
         </is>
       </c>
       <c r="H99" s="8" t="inlineStr">
@@ -24343,7 +24345,7 @@
       <c r="L99" s="8" t="n"/>
       <c r="M99" s="8" t="n"/>
       <c r="N99" s="8" t="n">
-        <v>16368</v>
+        <v>22132</v>
       </c>
       <c r="O99" s="8" t="n">
         <v>0</v>
@@ -24351,12 +24353,12 @@
       <c r="P99" s="8" t="n"/>
       <c r="Q99" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="R99" s="8" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S99" s="9" t="inlineStr"/>
@@ -24373,7 +24375,7 @@
       <c r="V99" s="7" t="inlineStr"/>
       <c r="W99" s="8" t="inlineStr">
         <is>
-          <t>8a8446c119238f7a042580aed1922ef6cfd79ae2</t>
+          <t>b3bc6f44f28301ca7ff059723f3c836424cd082f</t>
         </is>
       </c>
     </row>
@@ -24387,10 +24389,10 @@
         </is>
       </c>
       <c r="C100" s="17" t="n">
-        <v>1250</v>
+        <v>1600</v>
       </c>
       <c r="D100" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E100" s="8" t="n">
         <v>1</v>
@@ -24402,12 +24404,12 @@
       </c>
       <c r="G100" s="9" t="inlineStr">
         <is>
-          <t>Victoria Street, Bristol, BS1 6DR</t>
+          <t>Stapleton Road, Bristol, BS5</t>
         </is>
       </c>
       <c r="H100" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS5</t>
         </is>
       </c>
       <c r="I100" s="8" t="n"/>
@@ -24416,7 +24418,7 @@
       <c r="L100" s="8" t="n"/>
       <c r="M100" s="8" t="n"/>
       <c r="N100" s="8" t="n">
-        <v>21160</v>
+        <v>19576</v>
       </c>
       <c r="O100" s="8" t="n">
         <v>0</v>
@@ -24424,12 +24426,12 @@
       <c r="P100" s="8" t="n"/>
       <c r="Q100" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="R100" s="8" t="inlineStr">
         <is>
-          <t>Visum, Nationwide</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S100" s="9" t="inlineStr"/>
@@ -24446,7 +24448,7 @@
       <c r="V100" s="7" t="inlineStr"/>
       <c r="W100" s="8" t="inlineStr">
         <is>
-          <t>78fe8e0511ccc37f104368075238c845f57d7864</t>
+          <t>41184aca0a094a13f0cf944554fa6ab5b6f9b761</t>
         </is>
       </c>
     </row>
@@ -24460,13 +24462,13 @@
         </is>
       </c>
       <c r="C101" s="17" t="n">
-        <v>2145</v>
+        <v>1555</v>
       </c>
       <c r="D101" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E101" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F101" s="8" t="inlineStr">
         <is>
@@ -24475,23 +24477,21 @@
       </c>
       <c r="G101" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Lombard Street, Bristol, BS3</t>
         </is>
       </c>
       <c r="H101" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I101" s="8" t="n">
-        <v>796</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I101" s="8" t="n"/>
       <c r="J101" s="8" t="n"/>
       <c r="K101" s="8" t="n"/>
       <c r="L101" s="8" t="n"/>
       <c r="M101" s="8" t="n"/>
       <c r="N101" s="8" t="n">
-        <v>20820</v>
+        <v>12036</v>
       </c>
       <c r="O101" s="8" t="n">
         <v>0</v>
@@ -24499,12 +24499,12 @@
       <c r="P101" s="8" t="n"/>
       <c r="Q101" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="R101" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S101" s="9" t="inlineStr"/>
@@ -24521,7 +24521,7 @@
       <c r="V101" s="7" t="inlineStr"/>
       <c r="W101" s="8" t="inlineStr">
         <is>
-          <t>898ba227d5b949e4e7f18b49536b3c908560d145</t>
+          <t>4d3990c67ed2848296e2aa2fa362730e0557bd43</t>
         </is>
       </c>
     </row>
@@ -24535,13 +24535,13 @@
         </is>
       </c>
       <c r="C102" s="17" t="n">
-        <v>1999</v>
+        <v>2085</v>
       </c>
       <c r="D102" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E102" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F102" s="8" t="inlineStr">
         <is>
@@ -24550,7 +24550,7 @@
       </c>
       <c r="G102" s="9" t="inlineStr">
         <is>
-          <t>Swann House, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H102" s="8" t="inlineStr">
@@ -24558,13 +24558,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I102" s="8" t="n"/>
+      <c r="I102" s="8" t="n">
+        <v>722</v>
+      </c>
       <c r="J102" s="8" t="n"/>
       <c r="K102" s="8" t="n"/>
       <c r="L102" s="8" t="n"/>
       <c r="M102" s="8" t="n"/>
       <c r="N102" s="8" t="n">
-        <v>20800</v>
+        <v>21504</v>
       </c>
       <c r="O102" s="8" t="n">
         <v>0</v>
@@ -24572,12 +24574,12 @@
       <c r="P102" s="8" t="n"/>
       <c r="Q102" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="R102" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S102" s="9" t="inlineStr"/>
@@ -24594,7 +24596,7 @@
       <c r="V102" s="7" t="inlineStr"/>
       <c r="W102" s="8" t="inlineStr">
         <is>
-          <t>5cec67aa8ba885c4c8f85e47d3354d187da9d897</t>
+          <t>12a5f2c4f1be2a8f1a9b2c6cbe66191abf1d7975</t>
         </is>
       </c>
     </row>
@@ -24608,7 +24610,7 @@
         </is>
       </c>
       <c r="C103" s="17" t="n">
-        <v>1670</v>
+        <v>1640</v>
       </c>
       <c r="D103" s="8" t="n">
         <v>1</v>
@@ -24623,7 +24625,7 @@
       </c>
       <c r="G103" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H103" s="8" t="inlineStr">
@@ -24632,14 +24634,14 @@
         </is>
       </c>
       <c r="I103" s="8" t="n">
-        <v>485</v>
+        <v>570</v>
       </c>
       <c r="J103" s="8" t="n"/>
       <c r="K103" s="8" t="n"/>
       <c r="L103" s="8" t="n"/>
       <c r="M103" s="8" t="n"/>
       <c r="N103" s="8" t="n">
-        <v>21504</v>
+        <v>20820</v>
       </c>
       <c r="O103" s="8" t="n">
         <v>0</v>
@@ -24647,12 +24649,12 @@
       <c r="P103" s="8" t="n"/>
       <c r="Q103" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="R103" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S103" s="9" t="inlineStr"/>
@@ -24669,7 +24671,7 @@
       <c r="V103" s="7" t="inlineStr"/>
       <c r="W103" s="8" t="inlineStr">
         <is>
-          <t>73f3509a6c69eef7af4c6b9ff0dc69b97478c20a</t>
+          <t>f7afd1bbb106a22d180a78614dde509c1dbfa8c1</t>
         </is>
       </c>
     </row>
@@ -24683,7 +24685,7 @@
         </is>
       </c>
       <c r="C104" s="17" t="n">
-        <v>1645</v>
+        <v>1595</v>
       </c>
       <c r="D104" s="8" t="n">
         <v>1</v>
@@ -24698,7 +24700,7 @@
       </c>
       <c r="G104" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H104" s="8" t="inlineStr">
@@ -24707,27 +24709,25 @@
         </is>
       </c>
       <c r="I104" s="8" t="n">
-        <v>517</v>
+        <v>499</v>
       </c>
       <c r="J104" s="8" t="n"/>
       <c r="K104" s="8" t="n"/>
       <c r="L104" s="8" t="n"/>
       <c r="M104" s="8" t="n"/>
-      <c r="N104" s="8" t="n">
-        <v>20820</v>
-      </c>
+      <c r="N104" s="8" t="n"/>
       <c r="O104" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P104" s="8" t="n"/>
       <c r="Q104" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="R104" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S104" s="9" t="inlineStr"/>
@@ -24744,7 +24744,7 @@
       <c r="V104" s="7" t="inlineStr"/>
       <c r="W104" s="8" t="inlineStr">
         <is>
-          <t>4efcb79ae710a68f5f272a2f9030937499117f9d</t>
+          <t>f2f3afa9f34b35c1d7d84b8e8f6c80b9a91340b1</t>
         </is>
       </c>
     </row>
@@ -24758,13 +24758,13 @@
         </is>
       </c>
       <c r="C105" s="17" t="n">
-        <v>2120</v>
+        <v>1625</v>
       </c>
       <c r="D105" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E105" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F105" s="8" t="inlineStr">
         <is>
@@ -24773,7 +24773,7 @@
       </c>
       <c r="G105" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H105" s="8" t="inlineStr">
@@ -24782,27 +24782,25 @@
         </is>
       </c>
       <c r="I105" s="8" t="n">
-        <v>705</v>
+        <v>485</v>
       </c>
       <c r="J105" s="8" t="n"/>
       <c r="K105" s="8" t="n"/>
       <c r="L105" s="8" t="n"/>
       <c r="M105" s="8" t="n"/>
-      <c r="N105" s="8" t="n">
-        <v>20820</v>
-      </c>
+      <c r="N105" s="8" t="n"/>
       <c r="O105" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P105" s="8" t="n"/>
       <c r="Q105" s="8" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="R105" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S105" s="9" t="inlineStr"/>
@@ -24819,7 +24817,7 @@
       <c r="V105" s="7" t="inlineStr"/>
       <c r="W105" s="8" t="inlineStr">
         <is>
-          <t>c5c1741357dfce3547bdab7d4d5a0e7602846192</t>
+          <t>ea3758a9fd1b4190b4e5ae17519645f00d2e6a8f</t>
         </is>
       </c>
     </row>
@@ -24833,13 +24831,13 @@
         </is>
       </c>
       <c r="C106" s="17" t="n">
-        <v>1645</v>
+        <v>2175</v>
       </c>
       <c r="D106" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E106" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F106" s="8" t="inlineStr">
         <is>
@@ -24848,7 +24846,7 @@
       </c>
       <c r="G106" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H106" s="8" t="inlineStr">
@@ -24857,27 +24855,25 @@
         </is>
       </c>
       <c r="I106" s="8" t="n">
-        <v>571</v>
+        <v>722</v>
       </c>
       <c r="J106" s="8" t="n"/>
       <c r="K106" s="8" t="n"/>
       <c r="L106" s="8" t="n"/>
       <c r="M106" s="8" t="n"/>
-      <c r="N106" s="8" t="n">
-        <v>20820</v>
-      </c>
+      <c r="N106" s="8" t="n"/>
       <c r="O106" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P106" s="8" t="n"/>
       <c r="Q106" s="8" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="R106" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S106" s="9" t="inlineStr"/>
@@ -24894,7 +24890,7 @@
       <c r="V106" s="7" t="inlineStr"/>
       <c r="W106" s="8" t="inlineStr">
         <is>
-          <t>487e67b2d6680ebaabfcc49d4d33e21cb65cca6d</t>
+          <t>ab566c9b065047cd166a2ad3ae56e88704bc1358</t>
         </is>
       </c>
     </row>
@@ -24908,13 +24904,13 @@
         </is>
       </c>
       <c r="C107" s="17" t="n">
-        <v>2250</v>
+        <v>1900</v>
       </c>
       <c r="D107" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E107" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F107" s="8" t="inlineStr">
         <is>
@@ -24923,7 +24919,7 @@
       </c>
       <c r="G107" s="9" t="inlineStr">
         <is>
-          <t>Apartments, Bristol, BS1</t>
+          <t>The Granary, Queen Charlotte Street, BRISTOL, BS1</t>
         </is>
       </c>
       <c r="H107" s="8" t="inlineStr">
@@ -24936,21 +24932,19 @@
       <c r="K107" s="8" t="n"/>
       <c r="L107" s="8" t="n"/>
       <c r="M107" s="8" t="n"/>
-      <c r="N107" s="8" t="n">
-        <v>22132</v>
-      </c>
+      <c r="N107" s="8" t="n"/>
       <c r="O107" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P107" s="8" t="n"/>
       <c r="Q107" s="8" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="R107" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Andrews Letting and Management, Clifton</t>
         </is>
       </c>
       <c r="S107" s="9" t="inlineStr"/>
@@ -24967,7 +24961,7 @@
       <c r="V107" s="7" t="inlineStr"/>
       <c r="W107" s="8" t="inlineStr">
         <is>
-          <t>b3bc6f44f28301ca7ff059723f3c836424cd082f</t>
+          <t>b19bc62dddbc90526344a15be65fbc2e74a96d22</t>
         </is>
       </c>
     </row>
@@ -24981,13 +24975,13 @@
         </is>
       </c>
       <c r="C108" s="17" t="n">
-        <v>1600</v>
+        <v>2145</v>
       </c>
       <c r="D108" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E108" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F108" s="8" t="inlineStr">
         <is>
@@ -24996,21 +24990,23 @@
       </c>
       <c r="G108" s="9" t="inlineStr">
         <is>
-          <t>Stapleton Road, Bristol, BS5</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H108" s="8" t="inlineStr">
         <is>
-          <t>BS5</t>
-        </is>
-      </c>
-      <c r="I108" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I108" s="8" t="n">
+        <v>796</v>
+      </c>
       <c r="J108" s="8" t="n"/>
       <c r="K108" s="8" t="n"/>
       <c r="L108" s="8" t="n"/>
       <c r="M108" s="8" t="n"/>
       <c r="N108" s="8" t="n">
-        <v>19576</v>
+        <v>20820</v>
       </c>
       <c r="O108" s="8" t="n">
         <v>0</v>
@@ -25018,12 +25014,12 @@
       <c r="P108" s="8" t="n"/>
       <c r="Q108" s="8" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R108" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S108" s="9" t="inlineStr"/>
@@ -25040,7 +25036,7 @@
       <c r="V108" s="7" t="inlineStr"/>
       <c r="W108" s="8" t="inlineStr">
         <is>
-          <t>41184aca0a094a13f0cf944554fa6ab5b6f9b761</t>
+          <t>898ba227d5b949e4e7f18b49536b3c908560d145</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
House search data from run 23
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -17064,10 +17064,10 @@
         </is>
       </c>
       <c r="C3" s="17" t="n">
-        <v>1200</v>
+        <v>1900</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" s="8" t="n">
         <v>1</v>
@@ -17079,7 +17079,7 @@
       </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
-          <t>Caslon Court, Somerset Street, BS1</t>
+          <t>Redcliff Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H3" s="8" t="inlineStr">
@@ -17087,13 +17087,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I3" s="8" t="n"/>
+      <c r="I3" s="8" t="n">
+        <v>731</v>
+      </c>
       <c r="J3" s="8" t="n"/>
       <c r="K3" s="8" t="n"/>
       <c r="L3" s="8" t="n"/>
       <c r="M3" s="8" t="n"/>
       <c r="N3" s="8" t="n">
-        <v>18424</v>
+        <v>20892</v>
       </c>
       <c r="O3" s="8" t="n">
         <v>0</v>
@@ -17101,12 +17103,12 @@
       <c r="P3" s="8" t="n"/>
       <c r="Q3" s="8" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="R3" s="8" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>A2Dominion Group, A2Dominion Lettings</t>
         </is>
       </c>
       <c r="S3" s="9" t="inlineStr">
@@ -17127,7 +17129,7 @@
       <c r="V3" s="7" t="inlineStr"/>
       <c r="W3" s="8" t="inlineStr">
         <is>
-          <t>f6187d8c2bb085d8ddb57c1f8b8dc96ceada86aa</t>
+          <t>c11b7a868ede7c3b0a3d524aa4d4e8f661494706</t>
         </is>
       </c>
     </row>
@@ -17141,10 +17143,10 @@
         </is>
       </c>
       <c r="C4" s="17" t="n">
-        <v>1900</v>
+        <v>1395</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" s="8" t="n">
         <v>1</v>
@@ -17156,23 +17158,21 @@
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>Redcliff Street, Bristol, BS1</t>
+          <t>Hamilton Court, Bristol, BS2</t>
         </is>
       </c>
       <c r="H4" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I4" s="8" t="n">
-        <v>731</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="n"/>
       <c r="J4" s="8" t="n"/>
       <c r="K4" s="8" t="n"/>
       <c r="L4" s="8" t="n"/>
       <c r="M4" s="8" t="n"/>
       <c r="N4" s="8" t="n">
-        <v>20892</v>
+        <v>21660</v>
       </c>
       <c r="O4" s="8" t="n">
         <v>0</v>
@@ -17180,17 +17180,17 @@
       <c r="P4" s="8" t="n"/>
       <c r="Q4" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R4" s="8" t="inlineStr">
         <is>
-          <t>A2Dominion Group, A2Dominion Lettings</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S4" s="9" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T4" s="12" t="inlineStr">
@@ -17206,7 +17206,7 @@
       <c r="V4" s="7" t="inlineStr"/>
       <c r="W4" s="8" t="inlineStr">
         <is>
-          <t>c11b7a868ede7c3b0a3d524aa4d4e8f661494706</t>
+          <t>55512167c7894bf9991618275f495f9b5aa0a1af</t>
         </is>
       </c>
     </row>
@@ -17220,13 +17220,13 @@
         </is>
       </c>
       <c r="C5" s="17" t="n">
-        <v>1395</v>
+        <v>2000</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
@@ -17235,12 +17235,12 @@
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>Hamilton Court, Bristol, BS2</t>
+          <t>Deanery Road, Bristol, BS1</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I5" s="8" t="n"/>
@@ -17249,7 +17249,7 @@
       <c r="L5" s="8" t="n"/>
       <c r="M5" s="8" t="n"/>
       <c r="N5" s="8" t="n">
-        <v>21660</v>
+        <v>18292</v>
       </c>
       <c r="O5" s="8" t="n">
         <v>0</v>
@@ -17262,12 +17262,12 @@
       </c>
       <c r="R5" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Howard, Bristol</t>
         </is>
       </c>
       <c r="S5" s="9" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T5" s="12" t="inlineStr">
@@ -17283,7 +17283,7 @@
       <c r="V5" s="7" t="inlineStr"/>
       <c r="W5" s="8" t="inlineStr">
         <is>
-          <t>55512167c7894bf9991618275f495f9b5aa0a1af</t>
+          <t>591cc261a1f5973aaa4a7b3adbcbe4699bcc6440</t>
         </is>
       </c>
     </row>
@@ -17297,13 +17297,13 @@
         </is>
       </c>
       <c r="C6" s="17" t="n">
-        <v>2000</v>
+        <v>1550</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
@@ -17312,12 +17312,12 @@
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>Deanery Road, Bristol, BS1</t>
+          <t>Beaufort Street, Stapleton, Bristol</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS5</t>
         </is>
       </c>
       <c r="I6" s="8" t="n"/>
@@ -17326,7 +17326,7 @@
       <c r="L6" s="8" t="n"/>
       <c r="M6" s="8" t="n"/>
       <c r="N6" s="8" t="n">
-        <v>18292</v>
+        <v>19400</v>
       </c>
       <c r="O6" s="8" t="n">
         <v>0</v>
@@ -17339,7 +17339,7 @@
       </c>
       <c r="R6" s="8" t="inlineStr">
         <is>
-          <t>Howard, Bristol</t>
+          <t>Taylors Lettings, Bradley Stoke</t>
         </is>
       </c>
       <c r="S6" s="9" t="inlineStr">
@@ -17360,7 +17360,7 @@
       <c r="V6" s="7" t="inlineStr"/>
       <c r="W6" s="8" t="inlineStr">
         <is>
-          <t>591cc261a1f5973aaa4a7b3adbcbe4699bcc6440</t>
+          <t>81712a02a3a8827c0a71232c3b582e0d2b990a2a</t>
         </is>
       </c>
     </row>
@@ -17374,13 +17374,13 @@
         </is>
       </c>
       <c r="C7" s="17" t="n">
-        <v>1550</v>
+        <v>1900</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
@@ -17389,21 +17389,23 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>Beaufort Street, Stapleton, Bristol</t>
+          <t>Arnos Vale, Paintworks, BS4</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>BS5</t>
-        </is>
-      </c>
-      <c r="I7" s="8" t="n"/>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>783</v>
+      </c>
       <c r="J7" s="8" t="n"/>
       <c r="K7" s="8" t="n"/>
       <c r="L7" s="8" t="n"/>
       <c r="M7" s="8" t="n"/>
       <c r="N7" s="8" t="n">
-        <v>19400</v>
+        <v>4680</v>
       </c>
       <c r="O7" s="8" t="n">
         <v>0</v>
@@ -17411,12 +17413,12 @@
       <c r="P7" s="8" t="n"/>
       <c r="Q7" s="8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="R7" s="8" t="inlineStr">
         <is>
-          <t>Taylors Lettings, Bradley Stoke</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S7" s="9" t="inlineStr">
@@ -17437,7 +17439,7 @@
       <c r="V7" s="7" t="inlineStr"/>
       <c r="W7" s="8" t="inlineStr">
         <is>
-          <t>81712a02a3a8827c0a71232c3b582e0d2b990a2a</t>
+          <t>ec80bfb810dff72d9cbd21b8e12b70951ce557a7</t>
         </is>
       </c>
     </row>
@@ -17451,7 +17453,7 @@
         </is>
       </c>
       <c r="C8" s="17" t="n">
-        <v>1900</v>
+        <v>2170</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>2</v>
@@ -17466,23 +17468,23 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>Arnos Vale, Paintworks, BS4</t>
+          <t>522 Rosewood, Box Makers Yard, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>BS4</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I8" s="8" t="n">
-        <v>783</v>
+        <v>799</v>
       </c>
       <c r="J8" s="8" t="n"/>
       <c r="K8" s="8" t="n"/>
       <c r="L8" s="8" t="n"/>
       <c r="M8" s="8" t="n"/>
       <c r="N8" s="8" t="n">
-        <v>4680</v>
+        <v>20800</v>
       </c>
       <c r="O8" s="8" t="n">
         <v>0</v>
@@ -17490,12 +17492,12 @@
       <c r="P8" s="8" t="n"/>
       <c r="Q8" s="8" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R8" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S8" s="9" t="inlineStr">
@@ -17516,7 +17518,7 @@
       <c r="V8" s="7" t="inlineStr"/>
       <c r="W8" s="8" t="inlineStr">
         <is>
-          <t>ec80bfb810dff72d9cbd21b8e12b70951ce557a7</t>
+          <t>c0573087585d4e3e5716cf3f127e0ed418364345</t>
         </is>
       </c>
     </row>
@@ -17530,7 +17532,7 @@
         </is>
       </c>
       <c r="C9" s="17" t="n">
-        <v>2170</v>
+        <v>2195</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>2</v>
@@ -17545,7 +17547,7 @@
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>522 Rosewood, Box Makers Yard, New Kingsley Road, Bristol, BS2</t>
+          <t>802 Rosewood, Box Makers Yard, New Kingsley Road, Bristol, BS2 0GJ</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
@@ -17554,7 +17556,7 @@
         </is>
       </c>
       <c r="I9" s="8" t="n">
-        <v>799</v>
+        <v>809</v>
       </c>
       <c r="J9" s="8" t="n"/>
       <c r="K9" s="8" t="n"/>
@@ -17595,7 +17597,7 @@
       <c r="V9" s="7" t="inlineStr"/>
       <c r="W9" s="8" t="inlineStr">
         <is>
-          <t>c0573087585d4e3e5716cf3f127e0ed418364345</t>
+          <t>ad6f591658988c13d13881686e197fa878817439</t>
         </is>
       </c>
     </row>
@@ -17609,7 +17611,7 @@
         </is>
       </c>
       <c r="C10" s="17" t="n">
-        <v>2195</v>
+        <v>1995</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>2</v>
@@ -17624,23 +17626,21 @@
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>802 Rosewood, Box Makers Yard, New Kingsley Road, Bristol, BS2 0GJ</t>
+          <t>Sugar House, French Yard, City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I10" s="8" t="n">
-        <v>809</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="n"/>
       <c r="J10" s="8" t="n"/>
       <c r="K10" s="8" t="n"/>
       <c r="L10" s="8" t="n"/>
       <c r="M10" s="8" t="n"/>
       <c r="N10" s="8" t="n">
-        <v>20800</v>
+        <v>18544</v>
       </c>
       <c r="O10" s="8" t="n">
         <v>0</v>
@@ -17653,7 +17653,7 @@
       </c>
       <c r="R10" s="8" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S10" s="9" t="inlineStr">
@@ -17674,7 +17674,7 @@
       <c r="V10" s="7" t="inlineStr"/>
       <c r="W10" s="8" t="inlineStr">
         <is>
-          <t>ad6f591658988c13d13881686e197fa878817439</t>
+          <t>f829bfa651ebc050b5c2fa24aea7bca4147d62c3</t>
         </is>
       </c>
     </row>
@@ -17688,13 +17688,13 @@
         </is>
       </c>
       <c r="C11" s="17" t="n">
-        <v>1995</v>
+        <v>1655</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
@@ -17703,21 +17703,23 @@
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>Sugar House, French Yard, City Centre, Bristol, BS1</t>
+          <t>New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I11" s="8" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>547</v>
+      </c>
       <c r="J11" s="8" t="n"/>
       <c r="K11" s="8" t="n"/>
       <c r="L11" s="8" t="n"/>
       <c r="M11" s="8" t="n"/>
       <c r="N11" s="8" t="n">
-        <v>18544</v>
+        <v>20800</v>
       </c>
       <c r="O11" s="8" t="n">
         <v>0</v>
@@ -17725,12 +17727,12 @@
       <c r="P11" s="8" t="n"/>
       <c r="Q11" s="8" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R11" s="8" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S11" s="9" t="inlineStr">
@@ -17751,7 +17753,7 @@
       <c r="V11" s="7" t="inlineStr"/>
       <c r="W11" s="8" t="inlineStr">
         <is>
-          <t>f829bfa651ebc050b5c2fa24aea7bca4147d62c3</t>
+          <t>1f8489d296d842011bdf7a2ca1f952e6b948c3d3</t>
         </is>
       </c>
     </row>
@@ -17765,13 +17767,13 @@
         </is>
       </c>
       <c r="C12" s="17" t="n">
-        <v>1450</v>
+        <v>2500</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
@@ -17780,23 +17782,21 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>Bedminster, Berkeley Place, BS3</t>
+          <t>Electricity House, Colston Avenue, BS1</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I12" s="8" t="n">
-        <v>7685</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="n"/>
       <c r="J12" s="8" t="n"/>
       <c r="K12" s="8" t="n"/>
       <c r="L12" s="8" t="n"/>
       <c r="M12" s="8" t="n"/>
       <c r="N12" s="8" t="n">
-        <v>7648</v>
+        <v>21876</v>
       </c>
       <c r="O12" s="8" t="n">
         <v>0</v>
@@ -17804,12 +17804,12 @@
       <c r="P12" s="8" t="n"/>
       <c r="Q12" s="8" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R12" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S12" s="9" t="inlineStr">
@@ -17830,7 +17830,7 @@
       <c r="V12" s="7" t="inlineStr"/>
       <c r="W12" s="8" t="inlineStr">
         <is>
-          <t>4855da62cb452e8973968307d05f937e5ab76b6c</t>
+          <t>b2e83643f78121776465be4134c64aa64f0141c3</t>
         </is>
       </c>
     </row>
@@ -17844,7 +17844,7 @@
         </is>
       </c>
       <c r="C13" s="17" t="n">
-        <v>1655</v>
+        <v>1500</v>
       </c>
       <c r="D13" s="8" t="n">
         <v>1</v>
@@ -17859,23 +17859,21 @@
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>New Kingsley Road, Bristol, BS2</t>
+          <t>The Crescent, Hannover Quay, BS1</t>
         </is>
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I13" s="8" t="n">
-        <v>547</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="n"/>
       <c r="J13" s="8" t="n"/>
       <c r="K13" s="8" t="n"/>
       <c r="L13" s="8" t="n"/>
       <c r="M13" s="8" t="n"/>
       <c r="N13" s="8" t="n">
-        <v>20800</v>
+        <v>16232</v>
       </c>
       <c r="O13" s="8" t="n">
         <v>0</v>
@@ -17888,7 +17886,7 @@
       </c>
       <c r="R13" s="8" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S13" s="9" t="inlineStr">
@@ -17909,7 +17907,7 @@
       <c r="V13" s="7" t="inlineStr"/>
       <c r="W13" s="8" t="inlineStr">
         <is>
-          <t>1f8489d296d842011bdf7a2ca1f952e6b948c3d3</t>
+          <t>6bb8673e1999d1e987f72fb4720f3d7b072fa45e</t>
         </is>
       </c>
     </row>
@@ -17923,7 +17921,7 @@
         </is>
       </c>
       <c r="C14" s="17" t="n">
-        <v>2500</v>
+        <v>1850</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>2</v>
@@ -17938,7 +17936,7 @@
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>Electricity House, Colston Avenue, BS1</t>
+          <t>Park Row, Bristol, BS1</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
@@ -17946,26 +17944,26 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I14" s="8" t="n"/>
+      <c r="I14" s="8" t="n">
+        <v>797</v>
+      </c>
       <c r="J14" s="8" t="n"/>
       <c r="K14" s="8" t="n"/>
       <c r="L14" s="8" t="n"/>
       <c r="M14" s="8" t="n"/>
-      <c r="N14" s="8" t="n">
-        <v>21876</v>
-      </c>
+      <c r="N14" s="8" t="n"/>
       <c r="O14" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P14" s="8" t="n"/>
       <c r="Q14" s="8" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="R14" s="8" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>CJ Hole, Bishopston</t>
         </is>
       </c>
       <c r="S14" s="9" t="inlineStr">
@@ -17986,7 +17984,7 @@
       <c r="V14" s="7" t="inlineStr"/>
       <c r="W14" s="8" t="inlineStr">
         <is>
-          <t>b2e83643f78121776465be4134c64aa64f0141c3</t>
+          <t>50b953f0114e0c02556c27be640db0024cba0be6</t>
         </is>
       </c>
     </row>
@@ -18000,13 +17998,13 @@
         </is>
       </c>
       <c r="C15" s="17" t="n">
-        <v>1500</v>
+        <v>2975</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
@@ -18015,21 +18013,23 @@
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>The Crescent, Hannover Quay, BS1</t>
+          <t>Capricorn Place, Hotwells</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I15" s="8" t="n"/>
+          <t>BS8</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="n">
+        <v>1615</v>
+      </c>
       <c r="J15" s="8" t="n"/>
       <c r="K15" s="8" t="n"/>
       <c r="L15" s="8" t="n"/>
       <c r="M15" s="8" t="n"/>
       <c r="N15" s="8" t="n">
-        <v>16232</v>
+        <v>15104</v>
       </c>
       <c r="O15" s="8" t="n">
         <v>0</v>
@@ -18037,12 +18037,12 @@
       <c r="P15" s="8" t="n"/>
       <c r="Q15" s="8" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="R15" s="8" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>Sarah Kenny Residential Lettings, Bristol</t>
         </is>
       </c>
       <c r="S15" s="9" t="inlineStr">
@@ -18063,7 +18063,7 @@
       <c r="V15" s="7" t="inlineStr"/>
       <c r="W15" s="8" t="inlineStr">
         <is>
-          <t>6bb8673e1999d1e987f72fb4720f3d7b072fa45e</t>
+          <t>24fea285cbc5f197ed72b50a372f175ddb5fa732</t>
         </is>
       </c>
     </row>
@@ -18077,7 +18077,7 @@
         </is>
       </c>
       <c r="C16" s="17" t="n">
-        <v>1850</v>
+        <v>2000</v>
       </c>
       <c r="D16" s="8" t="n">
         <v>2</v>
@@ -18092,7 +18092,7 @@
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>Park Row, Bristol, BS1</t>
+          <t>Horizon - City Centre</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
@@ -18100,31 +18100,31 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I16" s="8" t="n">
-        <v>797</v>
-      </c>
+      <c r="I16" s="8" t="n"/>
       <c r="J16" s="8" t="n"/>
       <c r="K16" s="8" t="n"/>
       <c r="L16" s="8" t="n"/>
       <c r="M16" s="8" t="n"/>
-      <c r="N16" s="8" t="n"/>
+      <c r="N16" s="8" t="n">
+        <v>22020</v>
+      </c>
       <c r="O16" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P16" s="8" t="n"/>
       <c r="Q16" s="8" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R16" s="8" t="inlineStr">
         <is>
-          <t>CJ Hole, Bishopston</t>
+          <t>Ocean, Clifton</t>
         </is>
       </c>
       <c r="S16" s="9" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T16" s="12" t="inlineStr">
@@ -18140,7 +18140,7 @@
       <c r="V16" s="7" t="inlineStr"/>
       <c r="W16" s="8" t="inlineStr">
         <is>
-          <t>50b953f0114e0c02556c27be640db0024cba0be6</t>
+          <t>8988913a4580793e64d3ae8351174e2d71317d16</t>
         </is>
       </c>
     </row>
@@ -18154,13 +18154,13 @@
         </is>
       </c>
       <c r="C17" s="17" t="n">
-        <v>2975</v>
+        <v>1400</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
@@ -18169,23 +18169,21 @@
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>Capricorn Place, Hotwells</t>
+          <t>The Crescent, Harbourside, Bristol</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>BS8</t>
-        </is>
-      </c>
-      <c r="I17" s="8" t="n">
-        <v>1615</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="n"/>
       <c r="J17" s="8" t="n"/>
       <c r="K17" s="8" t="n"/>
       <c r="L17" s="8" t="n"/>
       <c r="M17" s="8" t="n"/>
       <c r="N17" s="8" t="n">
-        <v>15104</v>
+        <v>16368</v>
       </c>
       <c r="O17" s="8" t="n">
         <v>0</v>
@@ -18193,12 +18191,12 @@
       <c r="P17" s="8" t="n"/>
       <c r="Q17" s="8" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R17" s="8" t="inlineStr">
         <is>
-          <t>Sarah Kenny Residential Lettings, Bristol</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S17" s="9" t="inlineStr">
@@ -18219,7 +18217,7 @@
       <c r="V17" s="7" t="inlineStr"/>
       <c r="W17" s="8" t="inlineStr">
         <is>
-          <t>24fea285cbc5f197ed72b50a372f175ddb5fa732</t>
+          <t>59af10441dff618517a35c62d6a67a8485c2f2fa</t>
         </is>
       </c>
     </row>
@@ -18233,7 +18231,7 @@
         </is>
       </c>
       <c r="C18" s="17" t="n">
-        <v>2000</v>
+        <v>1900</v>
       </c>
       <c r="D18" s="8" t="n">
         <v>2</v>
@@ -18248,7 +18246,7 @@
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>Horizon - City Centre</t>
+          <t>51.02 - St James Barton</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
@@ -18262,7 +18260,7 @@
       <c r="L18" s="8" t="n"/>
       <c r="M18" s="8" t="n"/>
       <c r="N18" s="8" t="n">
-        <v>22020</v>
+        <v>22132</v>
       </c>
       <c r="O18" s="8" t="n">
         <v>0</v>
@@ -18280,7 +18278,7 @@
       </c>
       <c r="S18" s="9" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T18" s="12" t="inlineStr">
@@ -18296,7 +18294,7 @@
       <c r="V18" s="7" t="inlineStr"/>
       <c r="W18" s="8" t="inlineStr">
         <is>
-          <t>8988913a4580793e64d3ae8351174e2d71317d16</t>
+          <t>1d421f07eb2d142471d3e293f8cb751813656c56</t>
         </is>
       </c>
     </row>
@@ -18310,13 +18308,13 @@
         </is>
       </c>
       <c r="C19" s="17" t="n">
-        <v>1400</v>
+        <v>1700</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
@@ -18325,7 +18323,7 @@
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>The Crescent, Harbourside, Bristol</t>
+          <t>Steamship House, Gas Ferry Road, BS1</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
@@ -18339,7 +18337,7 @@
       <c r="L19" s="8" t="n"/>
       <c r="M19" s="8" t="n"/>
       <c r="N19" s="8" t="n">
-        <v>16368</v>
+        <v>14420</v>
       </c>
       <c r="O19" s="8" t="n">
         <v>0</v>
@@ -18347,7 +18345,7 @@
       <c r="P19" s="8" t="n"/>
       <c r="Q19" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R19" s="8" t="inlineStr">
@@ -18373,7 +18371,7 @@
       <c r="V19" s="7" t="inlineStr"/>
       <c r="W19" s="8" t="inlineStr">
         <is>
-          <t>59af10441dff618517a35c62d6a67a8485c2f2fa</t>
+          <t>f7b6312c22af08d7f7e765adf92d9a3fb0f82781</t>
         </is>
       </c>
     </row>
@@ -18387,7 +18385,7 @@
         </is>
       </c>
       <c r="C20" s="17" t="n">
-        <v>1900</v>
+        <v>1950</v>
       </c>
       <c r="D20" s="8" t="n">
         <v>2</v>
@@ -18402,7 +18400,7 @@
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>51.02 - St James Barton</t>
+          <t>Harbourside, The Crescent, BS1 5JP</t>
         </is>
       </c>
       <c r="H20" s="8" t="inlineStr">
@@ -18410,13 +18408,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I20" s="8" t="n"/>
+      <c r="I20" s="8" t="n">
+        <v>969</v>
+      </c>
       <c r="J20" s="8" t="n"/>
       <c r="K20" s="8" t="n"/>
       <c r="L20" s="8" t="n"/>
       <c r="M20" s="8" t="n"/>
       <c r="N20" s="8" t="n">
-        <v>22132</v>
+        <v>16368</v>
       </c>
       <c r="O20" s="8" t="n">
         <v>0</v>
@@ -18424,12 +18424,12 @@
       <c r="P20" s="8" t="n"/>
       <c r="Q20" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R20" s="8" t="inlineStr">
         <is>
-          <t>Ocean, Clifton</t>
+          <t>The Bristol Residential Letting Co, Clifton</t>
         </is>
       </c>
       <c r="S20" s="9" t="inlineStr">
@@ -18450,7 +18450,7 @@
       <c r="V20" s="7" t="inlineStr"/>
       <c r="W20" s="8" t="inlineStr">
         <is>
-          <t>1d421f07eb2d142471d3e293f8cb751813656c56</t>
+          <t>384c19ad899eb10f0c99305f716bbf9cc2030cb0</t>
         </is>
       </c>
     </row>
@@ -18464,13 +18464,13 @@
         </is>
       </c>
       <c r="C21" s="17" t="n">
-        <v>1700</v>
+        <v>1350</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
@@ -18479,7 +18479,7 @@
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>Steamship House, Gas Ferry Road, BS1</t>
+          <t>Millennium Promenade, Bristol, BS1</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
@@ -18487,13 +18487,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I21" s="8" t="n"/>
+      <c r="I21" s="8" t="n">
+        <v>491</v>
+      </c>
       <c r="J21" s="8" t="n"/>
       <c r="K21" s="8" t="n"/>
       <c r="L21" s="8" t="n"/>
       <c r="M21" s="8" t="n"/>
       <c r="N21" s="8" t="n">
-        <v>14420</v>
+        <v>17096</v>
       </c>
       <c r="O21" s="8" t="n">
         <v>0</v>
@@ -18506,7 +18508,7 @@
       </c>
       <c r="R21" s="8" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>A2Dominion Group, A2Dominion Lettings</t>
         </is>
       </c>
       <c r="S21" s="9" t="inlineStr">
@@ -18527,7 +18529,7 @@
       <c r="V21" s="7" t="inlineStr"/>
       <c r="W21" s="8" t="inlineStr">
         <is>
-          <t>f7b6312c22af08d7f7e765adf92d9a3fb0f82781</t>
+          <t>3ab86f4fbffd37f02afac44cadd6ec8a27da6f0a</t>
         </is>
       </c>
     </row>
@@ -18541,7 +18543,7 @@
         </is>
       </c>
       <c r="C22" s="17" t="n">
-        <v>1950</v>
+        <v>2000</v>
       </c>
       <c r="D22" s="8" t="n">
         <v>2</v>
@@ -18556,7 +18558,7 @@
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>Harbourside, The Crescent, BS1 5JP</t>
+          <t>Caledonian Road, Bristol, BS1</t>
         </is>
       </c>
       <c r="H22" s="8" t="inlineStr">
@@ -18564,15 +18566,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I22" s="8" t="n">
-        <v>969</v>
-      </c>
+      <c r="I22" s="8" t="n"/>
       <c r="J22" s="8" t="n"/>
       <c r="K22" s="8" t="n"/>
       <c r="L22" s="8" t="n"/>
       <c r="M22" s="8" t="n"/>
       <c r="N22" s="8" t="n">
-        <v>16368</v>
+        <v>14632</v>
       </c>
       <c r="O22" s="8" t="n">
         <v>0</v>
@@ -18585,7 +18585,7 @@
       </c>
       <c r="R22" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Clifton</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S22" s="9" t="inlineStr">
@@ -18606,7 +18606,7 @@
       <c r="V22" s="7" t="inlineStr"/>
       <c r="W22" s="8" t="inlineStr">
         <is>
-          <t>384c19ad899eb10f0c99305f716bbf9cc2030cb0</t>
+          <t>9a270cf54e31627246aef21daa26a60bb5f977ad</t>
         </is>
       </c>
     </row>
@@ -18620,13 +18620,13 @@
         </is>
       </c>
       <c r="C23" s="17" t="n">
-        <v>1350</v>
+        <v>1650</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
@@ -18635,23 +18635,21 @@
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>Millennium Promenade, Bristol, BS1</t>
+          <t>Sweetman Place, Bristol, BS2</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I23" s="8" t="n">
-        <v>491</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="n"/>
       <c r="J23" s="8" t="n"/>
       <c r="K23" s="8" t="n"/>
       <c r="L23" s="8" t="n"/>
       <c r="M23" s="8" t="n"/>
       <c r="N23" s="8" t="n">
-        <v>17096</v>
+        <v>20416</v>
       </c>
       <c r="O23" s="8" t="n">
         <v>0</v>
@@ -18664,7 +18662,7 @@
       </c>
       <c r="R23" s="8" t="inlineStr">
         <is>
-          <t>A2Dominion Group, A2Dominion Lettings</t>
+          <t>Andrews Letting and Management, Clifton</t>
         </is>
       </c>
       <c r="S23" s="9" t="inlineStr">
@@ -18685,7 +18683,7 @@
       <c r="V23" s="7" t="inlineStr"/>
       <c r="W23" s="8" t="inlineStr">
         <is>
-          <t>3ab86f4fbffd37f02afac44cadd6ec8a27da6f0a</t>
+          <t>54fa42ef8d0349a295f45392644c43dec3321c5b</t>
         </is>
       </c>
     </row>
@@ -18699,13 +18697,13 @@
         </is>
       </c>
       <c r="C24" s="17" t="n">
-        <v>2000</v>
+        <v>1200</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
@@ -18714,7 +18712,7 @@
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>Caledonian Road, Bristol, BS1</t>
+          <t>City Centre, Corinthian Court, BS1</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr">
@@ -18722,13 +18720,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I24" s="8" t="n"/>
+      <c r="I24" s="8" t="n">
+        <v>389</v>
+      </c>
       <c r="J24" s="8" t="n"/>
       <c r="K24" s="8" t="n"/>
       <c r="L24" s="8" t="n"/>
       <c r="M24" s="8" t="n"/>
       <c r="N24" s="8" t="n">
-        <v>14632</v>
+        <v>18820</v>
       </c>
       <c r="O24" s="8" t="n">
         <v>0</v>
@@ -18736,12 +18736,12 @@
       <c r="P24" s="8" t="n"/>
       <c r="Q24" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="R24" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S24" s="9" t="inlineStr">
@@ -18762,7 +18762,7 @@
       <c r="V24" s="7" t="inlineStr"/>
       <c r="W24" s="8" t="inlineStr">
         <is>
-          <t>9a270cf54e31627246aef21daa26a60bb5f977ad</t>
+          <t>5aed40eba285a7fa0266bfe8eb49613bb2f96c97</t>
         </is>
       </c>
     </row>
@@ -18776,13 +18776,13 @@
         </is>
       </c>
       <c r="C25" s="17" t="n">
-        <v>1650</v>
+        <v>1500</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
@@ -18791,21 +18791,23 @@
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>Sweetman Place, Bristol, BS2</t>
+          <t>Harbourside, Steamship House, BS1 6GL</t>
         </is>
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I25" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="n">
+        <v>506</v>
+      </c>
       <c r="J25" s="8" t="n"/>
       <c r="K25" s="8" t="n"/>
       <c r="L25" s="8" t="n"/>
       <c r="M25" s="8" t="n"/>
       <c r="N25" s="8" t="n">
-        <v>20416</v>
+        <v>14420</v>
       </c>
       <c r="O25" s="8" t="n">
         <v>0</v>
@@ -18813,12 +18815,12 @@
       <c r="P25" s="8" t="n"/>
       <c r="Q25" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="R25" s="8" t="inlineStr">
         <is>
-          <t>Andrews Letting and Management, Clifton</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S25" s="9" t="inlineStr">
@@ -18839,7 +18841,7 @@
       <c r="V25" s="7" t="inlineStr"/>
       <c r="W25" s="8" t="inlineStr">
         <is>
-          <t>54fa42ef8d0349a295f45392644c43dec3321c5b</t>
+          <t>bf329b73db0d1de077d78cddc284f1017fcfc43a</t>
         </is>
       </c>
     </row>
@@ -18853,7 +18855,7 @@
         </is>
       </c>
       <c r="C26" s="17" t="n">
-        <v>1200</v>
+        <v>1400</v>
       </c>
       <c r="D26" s="8" t="n">
         <v>1</v>
@@ -18868,7 +18870,7 @@
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>City Centre, Corinthian Court, BS1</t>
+          <t>St. James Barton, Bristol, Somerset, BS1</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">
@@ -18876,15 +18878,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I26" s="8" t="n">
-        <v>389</v>
-      </c>
+      <c r="I26" s="8" t="n"/>
       <c r="J26" s="8" t="n"/>
       <c r="K26" s="8" t="n"/>
       <c r="L26" s="8" t="n"/>
       <c r="M26" s="8" t="n"/>
       <c r="N26" s="8" t="n">
-        <v>18820</v>
+        <v>22132</v>
       </c>
       <c r="O26" s="8" t="n">
         <v>0</v>
@@ -18897,7 +18897,7 @@
       </c>
       <c r="R26" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Balloon Letting Company, Bristol</t>
         </is>
       </c>
       <c r="S26" s="9" t="inlineStr">
@@ -18918,7 +18918,7 @@
       <c r="V26" s="7" t="inlineStr"/>
       <c r="W26" s="8" t="inlineStr">
         <is>
-          <t>5aed40eba285a7fa0266bfe8eb49613bb2f96c97</t>
+          <t>f2c75a0f99c7c358be96a67019a6c639e60845fb</t>
         </is>
       </c>
     </row>
@@ -18932,10 +18932,10 @@
         </is>
       </c>
       <c r="C27" s="17" t="n">
-        <v>1500</v>
+        <v>1950</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E27" s="8" t="n">
         <v>1</v>
@@ -18947,7 +18947,7 @@
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>Harbourside, Steamship House, BS1 6GL</t>
+          <t>Apartments, Bristol, BS1</t>
         </is>
       </c>
       <c r="H27" s="8" t="inlineStr">
@@ -18955,15 +18955,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I27" s="8" t="n">
-        <v>506</v>
-      </c>
+      <c r="I27" s="8" t="n"/>
       <c r="J27" s="8" t="n"/>
       <c r="K27" s="8" t="n"/>
       <c r="L27" s="8" t="n"/>
       <c r="M27" s="8" t="n"/>
       <c r="N27" s="8" t="n">
-        <v>14420</v>
+        <v>22132</v>
       </c>
       <c r="O27" s="8" t="n">
         <v>0</v>
@@ -18976,12 +18974,12 @@
       </c>
       <c r="R27" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S27" s="9" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>bills included</t>
         </is>
       </c>
       <c r="T27" s="12" t="inlineStr">
@@ -18997,7 +18995,7 @@
       <c r="V27" s="7" t="inlineStr"/>
       <c r="W27" s="8" t="inlineStr">
         <is>
-          <t>bf329b73db0d1de077d78cddc284f1017fcfc43a</t>
+          <t>b3bc6f44f28301ca7ff059723f3c836424cd082f</t>
         </is>
       </c>
     </row>
@@ -19011,27 +19009,27 @@
         </is>
       </c>
       <c r="C28" s="17" t="n">
-        <v>1400</v>
+        <v>3750</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>St. James Barton, Bristol, Somerset, BS1</t>
+          <t>Dove Street, Bristol, BS2</t>
         </is>
       </c>
       <c r="H28" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I28" s="8" t="n"/>
@@ -19040,7 +19038,7 @@
       <c r="L28" s="8" t="n"/>
       <c r="M28" s="8" t="n"/>
       <c r="N28" s="8" t="n">
-        <v>22132</v>
+        <v>21288</v>
       </c>
       <c r="O28" s="8" t="n">
         <v>0</v>
@@ -19053,12 +19051,12 @@
       </c>
       <c r="R28" s="8" t="inlineStr">
         <is>
-          <t>Balloon Letting Company, Bristol</t>
+          <t>Phoenix Property Company, Bristol</t>
         </is>
       </c>
       <c r="S28" s="9" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T28" s="12" t="inlineStr">
@@ -19074,7 +19072,7 @@
       <c r="V28" s="7" t="inlineStr"/>
       <c r="W28" s="8" t="inlineStr">
         <is>
-          <t>f2c75a0f99c7c358be96a67019a6c639e60845fb</t>
+          <t>1bcb0667c3a3efe864816ea971273f0e1ff48f01</t>
         </is>
       </c>
     </row>
@@ -19088,10 +19086,10 @@
         </is>
       </c>
       <c r="C29" s="17" t="n">
-        <v>1950</v>
+        <v>1300</v>
       </c>
       <c r="D29" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E29" s="8" t="n">
         <v>1</v>
@@ -19103,7 +19101,7 @@
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>Apartments, Bristol, BS1</t>
+          <t>Three Queens Lane, Bristol, BS1</t>
         </is>
       </c>
       <c r="H29" s="8" t="inlineStr">
@@ -19117,7 +19115,7 @@
       <c r="L29" s="8" t="n"/>
       <c r="M29" s="8" t="n"/>
       <c r="N29" s="8" t="n">
-        <v>22132</v>
+        <v>20608</v>
       </c>
       <c r="O29" s="8" t="n">
         <v>0</v>
@@ -19125,17 +19123,17 @@
       <c r="P29" s="8" t="n"/>
       <c r="Q29" s="8" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="R29" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Romans, Clifton</t>
         </is>
       </c>
       <c r="S29" s="9" t="inlineStr">
         <is>
-          <t>bills included</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T29" s="12" t="inlineStr">
@@ -19151,7 +19149,7 @@
       <c r="V29" s="7" t="inlineStr"/>
       <c r="W29" s="8" t="inlineStr">
         <is>
-          <t>b3bc6f44f28301ca7ff059723f3c836424cd082f</t>
+          <t>7c9f52e17d949cd3dc79f3eb8c1020a81c729d66</t>
         </is>
       </c>
     </row>
@@ -19165,27 +19163,27 @@
         </is>
       </c>
       <c r="C30" s="17" t="n">
-        <v>3750</v>
+        <v>2200</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E30" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>Dove Street, Bristol, BS2</t>
+          <t>Lewins Mead, Bristol</t>
         </is>
       </c>
       <c r="H30" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I30" s="8" t="n"/>
@@ -19193,26 +19191,24 @@
       <c r="K30" s="8" t="n"/>
       <c r="L30" s="8" t="n"/>
       <c r="M30" s="8" t="n"/>
-      <c r="N30" s="8" t="n">
-        <v>21288</v>
-      </c>
+      <c r="N30" s="8" t="n"/>
       <c r="O30" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P30" s="8" t="n"/>
       <c r="Q30" s="8" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
-          <t>Phoenix Property Company, Bristol</t>
+          <t>Airsat Real Estate, Bristol</t>
         </is>
       </c>
       <c r="S30" s="9" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T30" s="12" t="inlineStr">
@@ -19228,7 +19224,7 @@
       <c r="V30" s="7" t="inlineStr"/>
       <c r="W30" s="8" t="inlineStr">
         <is>
-          <t>1bcb0667c3a3efe864816ea971273f0e1ff48f01</t>
+          <t>2d3387df3c55adfe44b18dbc94a6511d536c9187</t>
         </is>
       </c>
     </row>
@@ -19242,7 +19238,7 @@
         </is>
       </c>
       <c r="C31" s="17" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="D31" s="8" t="n">
         <v>1</v>
@@ -19257,7 +19253,7 @@
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>Three Queens Lane, Bristol, BS1</t>
+          <t>Caslon Court, Somerset Street, BS1</t>
         </is>
       </c>
       <c r="H31" s="8" t="inlineStr">
@@ -19271,7 +19267,7 @@
       <c r="L31" s="8" t="n"/>
       <c r="M31" s="8" t="n"/>
       <c r="N31" s="8" t="n">
-        <v>20608</v>
+        <v>18424</v>
       </c>
       <c r="O31" s="8" t="n">
         <v>0</v>
@@ -19279,12 +19275,12 @@
       <c r="P31" s="8" t="n"/>
       <c r="Q31" s="8" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
-          <t>Romans, Clifton</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S31" s="9" t="inlineStr">
@@ -19305,7 +19301,7 @@
       <c r="V31" s="7" t="inlineStr"/>
       <c r="W31" s="8" t="inlineStr">
         <is>
-          <t>7c9f52e17d949cd3dc79f3eb8c1020a81c729d66</t>
+          <t>f6187d8c2bb085d8ddb57c1f8b8dc96ceada86aa</t>
         </is>
       </c>
     </row>
@@ -19319,13 +19315,13 @@
         </is>
       </c>
       <c r="C32" s="17" t="n">
-        <v>2200</v>
+        <v>1450</v>
       </c>
       <c r="D32" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
@@ -19334,32 +19330,36 @@
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>Lewins Mead, Bristol</t>
+          <t>Bedminster, Berkeley Place, BS3</t>
         </is>
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I32" s="8" t="n"/>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="n">
+        <v>7685</v>
+      </c>
       <c r="J32" s="8" t="n"/>
       <c r="K32" s="8" t="n"/>
       <c r="L32" s="8" t="n"/>
       <c r="M32" s="8" t="n"/>
-      <c r="N32" s="8" t="n"/>
+      <c r="N32" s="8" t="n">
+        <v>7648</v>
+      </c>
       <c r="O32" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P32" s="8" t="n"/>
       <c r="Q32" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
-          <t>Airsat Real Estate, Bristol</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S32" s="9" t="inlineStr">
@@ -19380,7 +19380,7 @@
       <c r="V32" s="7" t="inlineStr"/>
       <c r="W32" s="8" t="inlineStr">
         <is>
-          <t>2d3387df3c55adfe44b18dbc94a6511d536c9187</t>
+          <t>4855da62cb452e8973968307d05f937e5ab76b6c</t>
         </is>
       </c>
     </row>
@@ -21662,13 +21662,13 @@
         </is>
       </c>
       <c r="C63" s="17" t="n">
-        <v>1300</v>
+        <v>2020</v>
       </c>
       <c r="D63" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E63" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F63" s="8" t="inlineStr">
         <is>
@@ -21677,7 +21677,7 @@
       </c>
       <c r="G63" s="9" t="inlineStr">
         <is>
-          <t>City Centre, Queen Square Apartments, BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H63" s="8" t="inlineStr">
@@ -21686,14 +21686,14 @@
         </is>
       </c>
       <c r="I63" s="8" t="n">
-        <v>405</v>
+        <v>764</v>
       </c>
       <c r="J63" s="8" t="n"/>
       <c r="K63" s="8" t="n"/>
       <c r="L63" s="8" t="n"/>
       <c r="M63" s="8" t="n"/>
       <c r="N63" s="8" t="n">
-        <v>20316</v>
+        <v>20856</v>
       </c>
       <c r="O63" s="8" t="n">
         <v>0</v>
@@ -21701,12 +21701,12 @@
       <c r="P63" s="8" t="n"/>
       <c r="Q63" s="8" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="R63" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S63" s="9" t="inlineStr"/>
@@ -21723,7 +21723,7 @@
       <c r="V63" s="7" t="inlineStr"/>
       <c r="W63" s="8" t="inlineStr">
         <is>
-          <t>9ad2c7bc90885b9a9e65b462b952842a964f1d35</t>
+          <t>6140b74b7d83ae5918fdabb6f9371e2f4b63a9c2</t>
         </is>
       </c>
     </row>
@@ -21737,7 +21737,7 @@
         </is>
       </c>
       <c r="C64" s="17" t="n">
-        <v>2020</v>
+        <v>2145</v>
       </c>
       <c r="D64" s="8" t="n">
         <v>2</v>
@@ -21752,7 +21752,7 @@
       </c>
       <c r="G64" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H64" s="8" t="inlineStr">
@@ -21761,14 +21761,14 @@
         </is>
       </c>
       <c r="I64" s="8" t="n">
-        <v>764</v>
+        <v>815</v>
       </c>
       <c r="J64" s="8" t="n"/>
       <c r="K64" s="8" t="n"/>
       <c r="L64" s="8" t="n"/>
       <c r="M64" s="8" t="n"/>
       <c r="N64" s="8" t="n">
-        <v>20856</v>
+        <v>21504</v>
       </c>
       <c r="O64" s="8" t="n">
         <v>0</v>
@@ -21781,7 +21781,7 @@
       </c>
       <c r="R64" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S64" s="9" t="inlineStr"/>
@@ -21798,7 +21798,7 @@
       <c r="V64" s="7" t="inlineStr"/>
       <c r="W64" s="8" t="inlineStr">
         <is>
-          <t>6140b74b7d83ae5918fdabb6f9371e2f4b63a9c2</t>
+          <t>24009eb3414633bf24b3b69631ba405866a1e5c9</t>
         </is>
       </c>
     </row>
@@ -21812,13 +21812,13 @@
         </is>
       </c>
       <c r="C65" s="17" t="n">
-        <v>2145</v>
+        <v>1635</v>
       </c>
       <c r="D65" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E65" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F65" s="8" t="inlineStr">
         <is>
@@ -21827,7 +21827,7 @@
       </c>
       <c r="G65" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H65" s="8" t="inlineStr">
@@ -21836,7 +21836,7 @@
         </is>
       </c>
       <c r="I65" s="8" t="n">
-        <v>815</v>
+        <v>486</v>
       </c>
       <c r="J65" s="8" t="n"/>
       <c r="K65" s="8" t="n"/>
@@ -21856,7 +21856,7 @@
       </c>
       <c r="R65" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S65" s="9" t="inlineStr"/>
@@ -21873,7 +21873,7 @@
       <c r="V65" s="7" t="inlineStr"/>
       <c r="W65" s="8" t="inlineStr">
         <is>
-          <t>24009eb3414633bf24b3b69631ba405866a1e5c9</t>
+          <t>bbf6e42784b6e4b7dae8d6bef9900115d0f3056e</t>
         </is>
       </c>
     </row>
@@ -21887,13 +21887,13 @@
         </is>
       </c>
       <c r="C66" s="17" t="n">
-        <v>1635</v>
+        <v>1750</v>
       </c>
       <c r="D66" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E66" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F66" s="8" t="inlineStr">
         <is>
@@ -21902,23 +21902,23 @@
       </c>
       <c r="G66" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Arnos Vale, Paintworks, BS4</t>
         </is>
       </c>
       <c r="H66" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS4</t>
         </is>
       </c>
       <c r="I66" s="8" t="n">
-        <v>486</v>
+        <v>731</v>
       </c>
       <c r="J66" s="8" t="n"/>
       <c r="K66" s="8" t="n"/>
       <c r="L66" s="8" t="n"/>
       <c r="M66" s="8" t="n"/>
       <c r="N66" s="8" t="n">
-        <v>21504</v>
+        <v>4680</v>
       </c>
       <c r="O66" s="8" t="n">
         <v>0</v>
@@ -21931,7 +21931,7 @@
       </c>
       <c r="R66" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S66" s="9" t="inlineStr"/>
@@ -21948,7 +21948,7 @@
       <c r="V66" s="7" t="inlineStr"/>
       <c r="W66" s="8" t="inlineStr">
         <is>
-          <t>bbf6e42784b6e4b7dae8d6bef9900115d0f3056e</t>
+          <t>1c0acc4cbbc0f239d4843e9eb56c0d04ca3a6278</t>
         </is>
       </c>
     </row>
@@ -21962,13 +21962,13 @@
         </is>
       </c>
       <c r="C67" s="17" t="n">
-        <v>1750</v>
+        <v>2100</v>
       </c>
       <c r="D67" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E67" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F67" s="8" t="inlineStr">
         <is>
@@ -21977,23 +21977,21 @@
       </c>
       <c r="G67" s="9" t="inlineStr">
         <is>
-          <t>Arnos Vale, Paintworks, BS4</t>
+          <t>Baldwin St, Bristol, BS1</t>
         </is>
       </c>
       <c r="H67" s="8" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I67" s="8" t="n">
-        <v>731</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I67" s="8" t="n"/>
       <c r="J67" s="8" t="n"/>
       <c r="K67" s="8" t="n"/>
       <c r="L67" s="8" t="n"/>
       <c r="M67" s="8" t="n"/>
       <c r="N67" s="8" t="n">
-        <v>4680</v>
+        <v>21148</v>
       </c>
       <c r="O67" s="8" t="n">
         <v>0</v>
@@ -22001,12 +21999,12 @@
       <c r="P67" s="8" t="n"/>
       <c r="Q67" s="8" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R67" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S67" s="9" t="inlineStr"/>
@@ -22023,7 +22021,7 @@
       <c r="V67" s="7" t="inlineStr"/>
       <c r="W67" s="8" t="inlineStr">
         <is>
-          <t>1c0acc4cbbc0f239d4843e9eb56c0d04ca3a6278</t>
+          <t>ba1c1abaa5dbfd6e19c20fa9df1e66799d9c2462</t>
         </is>
       </c>
     </row>
@@ -22037,13 +22035,13 @@
         </is>
       </c>
       <c r="C68" s="17" t="n">
-        <v>2100</v>
+        <v>2220</v>
       </c>
       <c r="D68" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E68" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
@@ -22052,7 +22050,7 @@
       </c>
       <c r="G68" s="9" t="inlineStr">
         <is>
-          <t>Baldwin St, Bristol, BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H68" s="8" t="inlineStr">
@@ -22060,13 +22058,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I68" s="8" t="n"/>
+      <c r="I68" s="8" t="n">
+        <v>697</v>
+      </c>
       <c r="J68" s="8" t="n"/>
       <c r="K68" s="8" t="n"/>
       <c r="L68" s="8" t="n"/>
       <c r="M68" s="8" t="n"/>
       <c r="N68" s="8" t="n">
-        <v>21148</v>
+        <v>20820</v>
       </c>
       <c r="O68" s="8" t="n">
         <v>0</v>
@@ -22079,7 +22079,7 @@
       </c>
       <c r="R68" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S68" s="9" t="inlineStr"/>
@@ -22096,7 +22096,7 @@
       <c r="V68" s="7" t="inlineStr"/>
       <c r="W68" s="8" t="inlineStr">
         <is>
-          <t>ba1c1abaa5dbfd6e19c20fa9df1e66799d9c2462</t>
+          <t>5870266ee1b15bf20f0a085f56358c762e522fa8</t>
         </is>
       </c>
     </row>
@@ -22110,13 +22110,13 @@
         </is>
       </c>
       <c r="C69" s="17" t="n">
-        <v>2220</v>
+        <v>1300</v>
       </c>
       <c r="D69" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E69" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F69" s="8" t="inlineStr">
         <is>
@@ -22125,7 +22125,7 @@
       </c>
       <c r="G69" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Bristol City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H69" s="8" t="inlineStr">
@@ -22133,15 +22133,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I69" s="8" t="n">
-        <v>697</v>
-      </c>
+      <c r="I69" s="8" t="n"/>
       <c r="J69" s="8" t="n"/>
       <c r="K69" s="8" t="n"/>
       <c r="L69" s="8" t="n"/>
       <c r="M69" s="8" t="n"/>
       <c r="N69" s="8" t="n">
-        <v>20820</v>
+        <v>21428</v>
       </c>
       <c r="O69" s="8" t="n">
         <v>0</v>
@@ -22149,12 +22147,12 @@
       <c r="P69" s="8" t="n"/>
       <c r="Q69" s="8" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="R69" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S69" s="9" t="inlineStr"/>
@@ -22171,7 +22169,7 @@
       <c r="V69" s="7" t="inlineStr"/>
       <c r="W69" s="8" t="inlineStr">
         <is>
-          <t>5870266ee1b15bf20f0a085f56358c762e522fa8</t>
+          <t>317e9ab29cad2381c41672743d877feba2c14e45</t>
         </is>
       </c>
     </row>
@@ -22185,7 +22183,7 @@
         </is>
       </c>
       <c r="C70" s="17" t="n">
-        <v>1300</v>
+        <v>1500</v>
       </c>
       <c r="D70" s="8" t="n">
         <v>1</v>
@@ -22200,7 +22198,7 @@
       </c>
       <c r="G70" s="9" t="inlineStr">
         <is>
-          <t>Bristol City Centre, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H70" s="8" t="inlineStr">
@@ -22208,13 +22206,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I70" s="8" t="n"/>
+      <c r="I70" s="8" t="n">
+        <v>548</v>
+      </c>
       <c r="J70" s="8" t="n"/>
       <c r="K70" s="8" t="n"/>
       <c r="L70" s="8" t="n"/>
       <c r="M70" s="8" t="n"/>
       <c r="N70" s="8" t="n">
-        <v>21428</v>
+        <v>21504</v>
       </c>
       <c r="O70" s="8" t="n">
         <v>0</v>
@@ -22222,12 +22222,12 @@
       <c r="P70" s="8" t="n"/>
       <c r="Q70" s="8" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R70" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S70" s="9" t="inlineStr"/>
@@ -22244,7 +22244,7 @@
       <c r="V70" s="7" t="inlineStr"/>
       <c r="W70" s="8" t="inlineStr">
         <is>
-          <t>317e9ab29cad2381c41672743d877feba2c14e45</t>
+          <t>bad1e4584285201ef9995d2b437343fca870009c</t>
         </is>
       </c>
     </row>
@@ -22258,7 +22258,7 @@
         </is>
       </c>
       <c r="C71" s="17" t="n">
-        <v>1500</v>
+        <v>1615</v>
       </c>
       <c r="D71" s="8" t="n">
         <v>1</v>
@@ -22273,7 +22273,7 @@
       </c>
       <c r="G71" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H71" s="8" t="inlineStr">
@@ -22282,7 +22282,7 @@
         </is>
       </c>
       <c r="I71" s="8" t="n">
-        <v>548</v>
+        <v>486</v>
       </c>
       <c r="J71" s="8" t="n"/>
       <c r="K71" s="8" t="n"/>
@@ -22302,7 +22302,7 @@
       </c>
       <c r="R71" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S71" s="9" t="inlineStr"/>
@@ -22319,7 +22319,7 @@
       <c r="V71" s="7" t="inlineStr"/>
       <c r="W71" s="8" t="inlineStr">
         <is>
-          <t>bad1e4584285201ef9995d2b437343fca870009c</t>
+          <t>67ff71428df47b0eb7f7da47600378ffdad1f97c</t>
         </is>
       </c>
     </row>
@@ -22333,10 +22333,10 @@
         </is>
       </c>
       <c r="C72" s="17" t="n">
-        <v>1615</v>
+        <v>1965</v>
       </c>
       <c r="D72" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E72" s="8" t="n">
         <v>1</v>
@@ -22348,7 +22348,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
@@ -22357,7 +22357,7 @@
         </is>
       </c>
       <c r="I72" s="8" t="n">
-        <v>486</v>
+        <v>655</v>
       </c>
       <c r="J72" s="8" t="n"/>
       <c r="K72" s="8" t="n"/>
@@ -22372,12 +22372,12 @@
       <c r="P72" s="8" t="n"/>
       <c r="Q72" s="8" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="R72" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S72" s="9" t="inlineStr"/>
@@ -22394,7 +22394,7 @@
       <c r="V72" s="7" t="inlineStr"/>
       <c r="W72" s="8" t="inlineStr">
         <is>
-          <t>67ff71428df47b0eb7f7da47600378ffdad1f97c</t>
+          <t>1a5b509e1606992acea1736489630b2bc57cc717</t>
         </is>
       </c>
     </row>
@@ -22408,13 +22408,13 @@
         </is>
       </c>
       <c r="C73" s="17" t="n">
-        <v>1965</v>
+        <v>2080</v>
       </c>
       <c r="D73" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E73" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F73" s="8" t="inlineStr">
         <is>
@@ -22423,7 +22423,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H73" s="8" t="inlineStr">
@@ -22432,14 +22432,14 @@
         </is>
       </c>
       <c r="I73" s="8" t="n">
-        <v>655</v>
+        <v>705</v>
       </c>
       <c r="J73" s="8" t="n"/>
       <c r="K73" s="8" t="n"/>
       <c r="L73" s="8" t="n"/>
       <c r="M73" s="8" t="n"/>
       <c r="N73" s="8" t="n">
-        <v>21504</v>
+        <v>20820</v>
       </c>
       <c r="O73" s="8" t="n">
         <v>0</v>
@@ -22452,7 +22452,7 @@
       </c>
       <c r="R73" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S73" s="9" t="inlineStr"/>
@@ -22469,7 +22469,7 @@
       <c r="V73" s="7" t="inlineStr"/>
       <c r="W73" s="8" t="inlineStr">
         <is>
-          <t>1a5b509e1606992acea1736489630b2bc57cc717</t>
+          <t>0453e07b653a16ada93327f26a41e0b204d289a4</t>
         </is>
       </c>
     </row>
@@ -22483,13 +22483,13 @@
         </is>
       </c>
       <c r="C74" s="17" t="n">
-        <v>2080</v>
+        <v>2000</v>
       </c>
       <c r="D74" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E74" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F74" s="8" t="inlineStr">
         <is>
@@ -22498,7 +22498,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Welsh Back, Bristol, BS1</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr">
@@ -22507,15 +22507,13 @@
         </is>
       </c>
       <c r="I74" s="8" t="n">
-        <v>705</v>
+        <v>908</v>
       </c>
       <c r="J74" s="8" t="n"/>
       <c r="K74" s="8" t="n"/>
       <c r="L74" s="8" t="n"/>
       <c r="M74" s="8" t="n"/>
-      <c r="N74" s="8" t="n">
-        <v>20820</v>
-      </c>
+      <c r="N74" s="8" t="n"/>
       <c r="O74" s="8" t="n">
         <v>0</v>
       </c>
@@ -22527,7 +22525,7 @@
       </c>
       <c r="R74" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Hello Neighbour, London</t>
         </is>
       </c>
       <c r="S74" s="9" t="inlineStr"/>
@@ -22544,7 +22542,7 @@
       <c r="V74" s="7" t="inlineStr"/>
       <c r="W74" s="8" t="inlineStr">
         <is>
-          <t>0453e07b653a16ada93327f26a41e0b204d289a4</t>
+          <t>65ed2520fdf37e6dde4abe0097cc3edbbbeff957</t>
         </is>
       </c>
     </row>
@@ -22558,13 +22556,13 @@
         </is>
       </c>
       <c r="C75" s="17" t="n">
-        <v>1400</v>
+        <v>2020</v>
       </c>
       <c r="D75" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E75" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F75" s="8" t="inlineStr">
         <is>
@@ -22573,7 +22571,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>Redcliffe Parade West, Flat 3, City Centre, Bristol, BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr">
@@ -22581,26 +22579,26 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I75" s="8" t="n"/>
+      <c r="I75" s="8" t="n">
+        <v>705</v>
+      </c>
       <c r="J75" s="8" t="n"/>
       <c r="K75" s="8" t="n"/>
       <c r="L75" s="8" t="n"/>
       <c r="M75" s="8" t="n"/>
-      <c r="N75" s="8" t="n">
-        <v>19484</v>
-      </c>
+      <c r="N75" s="8" t="n"/>
       <c r="O75" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P75" s="8" t="n"/>
       <c r="Q75" s="8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="R75" s="8" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S75" s="9" t="inlineStr"/>
@@ -22617,7 +22615,7 @@
       <c r="V75" s="7" t="inlineStr"/>
       <c r="W75" s="8" t="inlineStr">
         <is>
-          <t>9b65e5a0fb0bc8fc27d566eae912cddf76828cc9</t>
+          <t>75b3ee81b8ecb4015a80108f6d509e4156f4e8e4</t>
         </is>
       </c>
     </row>
@@ -22637,7 +22635,7 @@
         <v>2</v>
       </c>
       <c r="E76" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
@@ -22646,7 +22644,7 @@
       </c>
       <c r="G76" s="9" t="inlineStr">
         <is>
-          <t>Welsh Back, Bristol, BS1</t>
+          <t>Eclipse - City Centre</t>
         </is>
       </c>
       <c r="H76" s="8" t="inlineStr">
@@ -22654,9 +22652,7 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I76" s="8" t="n">
-        <v>908</v>
-      </c>
+      <c r="I76" s="8" t="n"/>
       <c r="J76" s="8" t="n"/>
       <c r="K76" s="8" t="n"/>
       <c r="L76" s="8" t="n"/>
@@ -22668,12 +22664,12 @@
       <c r="P76" s="8" t="n"/>
       <c r="Q76" s="8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="R76" s="8" t="inlineStr">
         <is>
-          <t>Hello Neighbour, London</t>
+          <t>Ocean, Clifton</t>
         </is>
       </c>
       <c r="S76" s="9" t="inlineStr"/>
@@ -22690,7 +22686,7 @@
       <c r="V76" s="7" t="inlineStr"/>
       <c r="W76" s="8" t="inlineStr">
         <is>
-          <t>65ed2520fdf37e6dde4abe0097cc3edbbbeff957</t>
+          <t>638ecbe81729048ffda61524ca9b06c4a208ce7b</t>
         </is>
       </c>
     </row>
@@ -22704,7 +22700,7 @@
         </is>
       </c>
       <c r="C77" s="17" t="n">
-        <v>2020</v>
+        <v>2085</v>
       </c>
       <c r="D77" s="8" t="n">
         <v>2</v>
@@ -22741,7 +22737,7 @@
       <c r="P77" s="8" t="n"/>
       <c r="Q77" s="8" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="R77" s="8" t="inlineStr">
@@ -22763,7 +22759,7 @@
       <c r="V77" s="7" t="inlineStr"/>
       <c r="W77" s="8" t="inlineStr">
         <is>
-          <t>75b3ee81b8ecb4015a80108f6d509e4156f4e8e4</t>
+          <t>16c89eb9a4cdeb57ddb3fd1201b7084ea2f3c007</t>
         </is>
       </c>
     </row>
@@ -22777,13 +22773,13 @@
         </is>
       </c>
       <c r="C78" s="17" t="n">
-        <v>2000</v>
+        <v>1615</v>
       </c>
       <c r="D78" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E78" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F78" s="8" t="inlineStr">
         <is>
@@ -22792,7 +22788,7 @@
       </c>
       <c r="G78" s="9" t="inlineStr">
         <is>
-          <t>Eclipse - City Centre</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H78" s="8" t="inlineStr">
@@ -22800,7 +22796,9 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I78" s="8" t="n"/>
+      <c r="I78" s="8" t="n">
+        <v>487</v>
+      </c>
       <c r="J78" s="8" t="n"/>
       <c r="K78" s="8" t="n"/>
       <c r="L78" s="8" t="n"/>
@@ -22812,12 +22810,12 @@
       <c r="P78" s="8" t="n"/>
       <c r="Q78" s="8" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="R78" s="8" t="inlineStr">
         <is>
-          <t>Ocean, Clifton</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S78" s="9" t="inlineStr"/>
@@ -22834,7 +22832,7 @@
       <c r="V78" s="7" t="inlineStr"/>
       <c r="W78" s="8" t="inlineStr">
         <is>
-          <t>638ecbe81729048ffda61524ca9b06c4a208ce7b</t>
+          <t>cd57661c8d996d20c5c1c7c34b12787f40073ec9</t>
         </is>
       </c>
     </row>
@@ -22848,7 +22846,7 @@
         </is>
       </c>
       <c r="C79" s="17" t="n">
-        <v>2085</v>
+        <v>2065</v>
       </c>
       <c r="D79" s="8" t="n">
         <v>2</v>
@@ -22863,7 +22861,7 @@
       </c>
       <c r="G79" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H79" s="8" t="inlineStr">
@@ -22872,7 +22870,7 @@
         </is>
       </c>
       <c r="I79" s="8" t="n">
-        <v>705</v>
+        <v>641</v>
       </c>
       <c r="J79" s="8" t="n"/>
       <c r="K79" s="8" t="n"/>
@@ -22885,12 +22883,12 @@
       <c r="P79" s="8" t="n"/>
       <c r="Q79" s="8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="R79" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S79" s="9" t="inlineStr"/>
@@ -22907,7 +22905,7 @@
       <c r="V79" s="7" t="inlineStr"/>
       <c r="W79" s="8" t="inlineStr">
         <is>
-          <t>16c89eb9a4cdeb57ddb3fd1201b7084ea2f3c007</t>
+          <t>d23eb397c84a723416c257acf4e25973ede40bc5</t>
         </is>
       </c>
     </row>
@@ -22921,13 +22919,13 @@
         </is>
       </c>
       <c r="C80" s="17" t="n">
-        <v>1615</v>
+        <v>2185</v>
       </c>
       <c r="D80" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E80" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F80" s="8" t="inlineStr">
         <is>
@@ -22945,7 +22943,7 @@
         </is>
       </c>
       <c r="I80" s="8" t="n">
-        <v>487</v>
+        <v>721</v>
       </c>
       <c r="J80" s="8" t="n"/>
       <c r="K80" s="8" t="n"/>
@@ -22958,7 +22956,7 @@
       <c r="P80" s="8" t="n"/>
       <c r="Q80" s="8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="R80" s="8" t="inlineStr">
@@ -22980,7 +22978,7 @@
       <c r="V80" s="7" t="inlineStr"/>
       <c r="W80" s="8" t="inlineStr">
         <is>
-          <t>cd57661c8d996d20c5c1c7c34b12787f40073ec9</t>
+          <t>6446e0c7d9c4f21f9eb6239caeeeee0599a68101</t>
         </is>
       </c>
     </row>
@@ -22994,13 +22992,13 @@
         </is>
       </c>
       <c r="C81" s="17" t="n">
-        <v>2065</v>
+        <v>1565</v>
       </c>
       <c r="D81" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E81" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F81" s="8" t="inlineStr">
         <is>
@@ -23009,7 +23007,7 @@
       </c>
       <c r="G81" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H81" s="8" t="inlineStr">
@@ -23018,7 +23016,7 @@
         </is>
       </c>
       <c r="I81" s="8" t="n">
-        <v>641</v>
+        <v>484</v>
       </c>
       <c r="J81" s="8" t="n"/>
       <c r="K81" s="8" t="n"/>
@@ -23036,7 +23034,7 @@
       </c>
       <c r="R81" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S81" s="9" t="inlineStr"/>
@@ -23053,7 +23051,7 @@
       <c r="V81" s="7" t="inlineStr"/>
       <c r="W81" s="8" t="inlineStr">
         <is>
-          <t>d23eb397c84a723416c257acf4e25973ede40bc5</t>
+          <t>34d9877a23c82be120784d9dd55c23c17584c91a</t>
         </is>
       </c>
     </row>
@@ -23067,13 +23065,13 @@
         </is>
       </c>
       <c r="C82" s="17" t="n">
-        <v>2185</v>
+        <v>2100</v>
       </c>
       <c r="D82" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E82" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F82" s="8" t="inlineStr">
         <is>
@@ -23082,7 +23080,7 @@
       </c>
       <c r="G82" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>The Three Kings Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H82" s="8" t="inlineStr">
@@ -23090,9 +23088,7 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I82" s="8" t="n">
-        <v>721</v>
-      </c>
+      <c r="I82" s="8" t="n"/>
       <c r="J82" s="8" t="n"/>
       <c r="K82" s="8" t="n"/>
       <c r="L82" s="8" t="n"/>
@@ -23104,12 +23100,12 @@
       <c r="P82" s="8" t="n"/>
       <c r="Q82" s="8" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="R82" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S82" s="9" t="inlineStr"/>
@@ -23126,7 +23122,7 @@
       <c r="V82" s="7" t="inlineStr"/>
       <c r="W82" s="8" t="inlineStr">
         <is>
-          <t>6446e0c7d9c4f21f9eb6239caeeeee0599a68101</t>
+          <t>954007c82f6f3a495c465b72c9a1c44c0c84713e</t>
         </is>
       </c>
     </row>
@@ -23140,7 +23136,7 @@
         </is>
       </c>
       <c r="C83" s="17" t="n">
-        <v>1565</v>
+        <v>1660</v>
       </c>
       <c r="D83" s="8" t="n">
         <v>1</v>
@@ -23164,20 +23160,22 @@
         </is>
       </c>
       <c r="I83" s="8" t="n">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="J83" s="8" t="n"/>
       <c r="K83" s="8" t="n"/>
       <c r="L83" s="8" t="n"/>
       <c r="M83" s="8" t="n"/>
-      <c r="N83" s="8" t="n"/>
+      <c r="N83" s="8" t="n">
+        <v>21504</v>
+      </c>
       <c r="O83" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P83" s="8" t="n"/>
       <c r="Q83" s="8" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R83" s="8" t="inlineStr">
@@ -23199,7 +23197,7 @@
       <c r="V83" s="7" t="inlineStr"/>
       <c r="W83" s="8" t="inlineStr">
         <is>
-          <t>34d9877a23c82be120784d9dd55c23c17584c91a</t>
+          <t>c2c660e4e8cefc047b4bc72bf19b48ce9ef7ec99</t>
         </is>
       </c>
     </row>
@@ -23213,13 +23211,13 @@
         </is>
       </c>
       <c r="C84" s="17" t="n">
-        <v>1650</v>
+        <v>2175</v>
       </c>
       <c r="D84" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E84" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F84" s="8" t="inlineStr">
         <is>
@@ -23228,7 +23226,7 @@
       </c>
       <c r="G84" s="9" t="inlineStr">
         <is>
-          <t>Horizon, Broad Weir, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H84" s="8" t="inlineStr">
@@ -23236,24 +23234,28 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I84" s="8" t="n"/>
+      <c r="I84" s="8" t="n">
+        <v>814</v>
+      </c>
       <c r="J84" s="8" t="n"/>
       <c r="K84" s="8" t="n"/>
       <c r="L84" s="8" t="n"/>
       <c r="M84" s="8" t="n"/>
-      <c r="N84" s="8" t="n"/>
+      <c r="N84" s="8" t="n">
+        <v>21504</v>
+      </c>
       <c r="O84" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P84" s="8" t="n"/>
       <c r="Q84" s="8" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R84" s="8" t="inlineStr">
         <is>
-          <t>CJ Hole, Bishopston</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S84" s="9" t="inlineStr"/>
@@ -23270,7 +23272,7 @@
       <c r="V84" s="7" t="inlineStr"/>
       <c r="W84" s="8" t="inlineStr">
         <is>
-          <t>aa3cf620ad25601a026424157bd8c0abb746373f</t>
+          <t>83406f05c9aded812a566cc6806036dda0d45fc0</t>
         </is>
       </c>
     </row>
@@ -23284,13 +23286,13 @@
         </is>
       </c>
       <c r="C85" s="17" t="n">
-        <v>2100</v>
+        <v>2115</v>
       </c>
       <c r="D85" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E85" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F85" s="8" t="inlineStr">
         <is>
@@ -23299,7 +23301,7 @@
       </c>
       <c r="G85" s="9" t="inlineStr">
         <is>
-          <t>The Three Kings Court, Bristol, BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H85" s="8" t="inlineStr">
@@ -23307,24 +23309,28 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I85" s="8" t="n"/>
+      <c r="I85" s="8" t="n">
+        <v>823</v>
+      </c>
       <c r="J85" s="8" t="n"/>
       <c r="K85" s="8" t="n"/>
       <c r="L85" s="8" t="n"/>
       <c r="M85" s="8" t="n"/>
-      <c r="N85" s="8" t="n"/>
+      <c r="N85" s="8" t="n">
+        <v>20820</v>
+      </c>
       <c r="O85" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P85" s="8" t="n"/>
       <c r="Q85" s="8" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="R85" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S85" s="9" t="inlineStr"/>
@@ -23341,7 +23347,7 @@
       <c r="V85" s="7" t="inlineStr"/>
       <c r="W85" s="8" t="inlineStr">
         <is>
-          <t>954007c82f6f3a495c465b72c9a1c44c0c84713e</t>
+          <t>0b78c6e29d96ae73c643d0d50d50949797b02893</t>
         </is>
       </c>
     </row>
@@ -23394,7 +23400,7 @@
       <c r="P86" s="8" t="n"/>
       <c r="Q86" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="R86" s="8" t="inlineStr">
@@ -23416,7 +23422,7 @@
       <c r="V86" s="7" t="inlineStr"/>
       <c r="W86" s="8" t="inlineStr">
         <is>
-          <t>c2c660e4e8cefc047b4bc72bf19b48ce9ef7ec99</t>
+          <t>c798c669d03fa2e42fd418ff0916de022d3380ad</t>
         </is>
       </c>
     </row>
@@ -23430,7 +23436,7 @@
         </is>
       </c>
       <c r="C87" s="17" t="n">
-        <v>2175</v>
+        <v>1915</v>
       </c>
       <c r="D87" s="8" t="n">
         <v>2</v>
@@ -23454,14 +23460,14 @@
         </is>
       </c>
       <c r="I87" s="8" t="n">
-        <v>814</v>
+        <v>746</v>
       </c>
       <c r="J87" s="8" t="n"/>
       <c r="K87" s="8" t="n"/>
       <c r="L87" s="8" t="n"/>
       <c r="M87" s="8" t="n"/>
       <c r="N87" s="8" t="n">
-        <v>21504</v>
+        <v>21680</v>
       </c>
       <c r="O87" s="8" t="n">
         <v>0</v>
@@ -23469,7 +23475,7 @@
       <c r="P87" s="8" t="n"/>
       <c r="Q87" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="R87" s="8" t="inlineStr">
@@ -23491,7 +23497,7 @@
       <c r="V87" s="7" t="inlineStr"/>
       <c r="W87" s="8" t="inlineStr">
         <is>
-          <t>83406f05c9aded812a566cc6806036dda0d45fc0</t>
+          <t>36797023cff0095f1bf764fa2f176d5595124854</t>
         </is>
       </c>
     </row>
@@ -23505,10 +23511,10 @@
         </is>
       </c>
       <c r="C88" s="17" t="n">
-        <v>1500</v>
+        <v>2450</v>
       </c>
       <c r="D88" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E88" s="8" t="n">
         <v>2</v>
@@ -23520,7 +23526,7 @@
       </c>
       <c r="G88" s="9" t="inlineStr">
         <is>
-          <t>Small Street - City Centre</t>
+          <t>The Herbert Ashman Building, Bristol, BS1</t>
         </is>
       </c>
       <c r="H88" s="8" t="inlineStr">
@@ -23534,7 +23540,7 @@
       <c r="L88" s="8" t="n"/>
       <c r="M88" s="8" t="n"/>
       <c r="N88" s="8" t="n">
-        <v>21816</v>
+        <v>21788</v>
       </c>
       <c r="O88" s="8" t="n">
         <v>0</v>
@@ -23542,12 +23548,12 @@
       <c r="P88" s="8" t="n"/>
       <c r="Q88" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R88" s="8" t="inlineStr">
         <is>
-          <t>Ocean, Clifton</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S88" s="9" t="inlineStr"/>
@@ -23564,7 +23570,7 @@
       <c r="V88" s="7" t="inlineStr"/>
       <c r="W88" s="8" t="inlineStr">
         <is>
-          <t>cb4b1af676ff54ae12ad7bf4fa94acd8ef94a533</t>
+          <t>4cd4fdc09f26b6316c31aa22f38853db44d1ea9a</t>
         </is>
       </c>
     </row>
@@ -23578,7 +23584,7 @@
         </is>
       </c>
       <c r="C89" s="17" t="n">
-        <v>2115</v>
+        <v>1700</v>
       </c>
       <c r="D89" s="8" t="n">
         <v>2</v>
@@ -23593,7 +23599,7 @@
       </c>
       <c r="G89" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>The Crescent</t>
         </is>
       </c>
       <c r="H89" s="8" t="inlineStr">
@@ -23601,15 +23607,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I89" s="8" t="n">
-        <v>823</v>
-      </c>
+      <c r="I89" s="8" t="n"/>
       <c r="J89" s="8" t="n"/>
       <c r="K89" s="8" t="n"/>
       <c r="L89" s="8" t="n"/>
       <c r="M89" s="8" t="n"/>
       <c r="N89" s="8" t="n">
-        <v>20820</v>
+        <v>16368</v>
       </c>
       <c r="O89" s="8" t="n">
         <v>0</v>
@@ -23617,12 +23621,12 @@
       <c r="P89" s="8" t="n"/>
       <c r="Q89" s="8" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R89" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S89" s="9" t="inlineStr"/>
@@ -23639,7 +23643,7 @@
       <c r="V89" s="7" t="inlineStr"/>
       <c r="W89" s="8" t="inlineStr">
         <is>
-          <t>0b78c6e29d96ae73c643d0d50d50949797b02893</t>
+          <t>8a8446c119238f7a042580aed1922ef6cfd79ae2</t>
         </is>
       </c>
     </row>
@@ -23653,7 +23657,7 @@
         </is>
       </c>
       <c r="C90" s="17" t="n">
-        <v>1660</v>
+        <v>1250</v>
       </c>
       <c r="D90" s="8" t="n">
         <v>1</v>
@@ -23668,7 +23672,7 @@
       </c>
       <c r="G90" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Victoria Street, Bristol, BS1 6DR</t>
         </is>
       </c>
       <c r="H90" s="8" t="inlineStr">
@@ -23676,15 +23680,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I90" s="8" t="n">
-        <v>486</v>
-      </c>
+      <c r="I90" s="8" t="n"/>
       <c r="J90" s="8" t="n"/>
       <c r="K90" s="8" t="n"/>
       <c r="L90" s="8" t="n"/>
       <c r="M90" s="8" t="n"/>
       <c r="N90" s="8" t="n">
-        <v>21504</v>
+        <v>21160</v>
       </c>
       <c r="O90" s="8" t="n">
         <v>0</v>
@@ -23692,12 +23694,12 @@
       <c r="P90" s="8" t="n"/>
       <c r="Q90" s="8" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R90" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Visum, Nationwide</t>
         </is>
       </c>
       <c r="S90" s="9" t="inlineStr"/>
@@ -23714,7 +23716,7 @@
       <c r="V90" s="7" t="inlineStr"/>
       <c r="W90" s="8" t="inlineStr">
         <is>
-          <t>c798c669d03fa2e42fd418ff0916de022d3380ad</t>
+          <t>78fe8e0511ccc37f104368075238c845f57d7864</t>
         </is>
       </c>
     </row>
@@ -23728,13 +23730,13 @@
         </is>
       </c>
       <c r="C91" s="17" t="n">
-        <v>1915</v>
+        <v>1999</v>
       </c>
       <c r="D91" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E91" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F91" s="8" t="inlineStr">
         <is>
@@ -23743,7 +23745,7 @@
       </c>
       <c r="G91" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Swann House, Bristol, BS1</t>
         </is>
       </c>
       <c r="H91" s="8" t="inlineStr">
@@ -23751,15 +23753,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I91" s="8" t="n">
-        <v>746</v>
-      </c>
+      <c r="I91" s="8" t="n"/>
       <c r="J91" s="8" t="n"/>
       <c r="K91" s="8" t="n"/>
       <c r="L91" s="8" t="n"/>
       <c r="M91" s="8" t="n"/>
       <c r="N91" s="8" t="n">
-        <v>21680</v>
+        <v>20800</v>
       </c>
       <c r="O91" s="8" t="n">
         <v>0</v>
@@ -23767,12 +23767,12 @@
       <c r="P91" s="8" t="n"/>
       <c r="Q91" s="8" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R91" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S91" s="9" t="inlineStr"/>
@@ -23789,7 +23789,7 @@
       <c r="V91" s="7" t="inlineStr"/>
       <c r="W91" s="8" t="inlineStr">
         <is>
-          <t>36797023cff0095f1bf764fa2f176d5595124854</t>
+          <t>5cec67aa8ba885c4c8f85e47d3354d187da9d897</t>
         </is>
       </c>
     </row>
@@ -23803,7 +23803,7 @@
         </is>
       </c>
       <c r="C92" s="17" t="n">
-        <v>1150</v>
+        <v>1670</v>
       </c>
       <c r="D92" s="8" t="n">
         <v>1</v>
@@ -23818,21 +23818,23 @@
       </c>
       <c r="G92" s="9" t="inlineStr">
         <is>
-          <t>Knowle Road, Bristol</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H92" s="8" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I92" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I92" s="8" t="n">
+        <v>485</v>
+      </c>
       <c r="J92" s="8" t="n"/>
       <c r="K92" s="8" t="n"/>
       <c r="L92" s="8" t="n"/>
       <c r="M92" s="8" t="n"/>
       <c r="N92" s="8" t="n">
-        <v>6872</v>
+        <v>21504</v>
       </c>
       <c r="O92" s="8" t="n">
         <v>0</v>
@@ -23840,12 +23842,12 @@
       <c r="P92" s="8" t="n"/>
       <c r="Q92" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R92" s="8" t="inlineStr">
         <is>
-          <t>Hopewell, Bristol</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S92" s="9" t="inlineStr"/>
@@ -23862,7 +23864,7 @@
       <c r="V92" s="7" t="inlineStr"/>
       <c r="W92" s="8" t="inlineStr">
         <is>
-          <t>edac1b499f84e07ce85894b488f82dc5cd104202</t>
+          <t>73f3509a6c69eef7af4c6b9ff0dc69b97478c20a</t>
         </is>
       </c>
     </row>
@@ -23876,13 +23878,13 @@
         </is>
       </c>
       <c r="C93" s="17" t="n">
-        <v>2450</v>
+        <v>1645</v>
       </c>
       <c r="D93" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E93" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F93" s="8" t="inlineStr">
         <is>
@@ -23891,7 +23893,7 @@
       </c>
       <c r="G93" s="9" t="inlineStr">
         <is>
-          <t>The Herbert Ashman Building, Bristol, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H93" s="8" t="inlineStr">
@@ -23899,13 +23901,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I93" s="8" t="n"/>
+      <c r="I93" s="8" t="n">
+        <v>517</v>
+      </c>
       <c r="J93" s="8" t="n"/>
       <c r="K93" s="8" t="n"/>
       <c r="L93" s="8" t="n"/>
       <c r="M93" s="8" t="n"/>
       <c r="N93" s="8" t="n">
-        <v>21788</v>
+        <v>20820</v>
       </c>
       <c r="O93" s="8" t="n">
         <v>0</v>
@@ -23913,12 +23917,12 @@
       <c r="P93" s="8" t="n"/>
       <c r="Q93" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R93" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S93" s="9" t="inlineStr"/>
@@ -23935,7 +23939,7 @@
       <c r="V93" s="7" t="inlineStr"/>
       <c r="W93" s="8" t="inlineStr">
         <is>
-          <t>4cd4fdc09f26b6316c31aa22f38853db44d1ea9a</t>
+          <t>4efcb79ae710a68f5f272a2f9030937499117f9d</t>
         </is>
       </c>
     </row>
@@ -23949,7 +23953,7 @@
         </is>
       </c>
       <c r="C94" s="17" t="n">
-        <v>1700</v>
+        <v>2120</v>
       </c>
       <c r="D94" s="8" t="n">
         <v>2</v>
@@ -23964,7 +23968,7 @@
       </c>
       <c r="G94" s="9" t="inlineStr">
         <is>
-          <t>The Crescent</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H94" s="8" t="inlineStr">
@@ -23972,13 +23976,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I94" s="8" t="n"/>
+      <c r="I94" s="8" t="n">
+        <v>705</v>
+      </c>
       <c r="J94" s="8" t="n"/>
       <c r="K94" s="8" t="n"/>
       <c r="L94" s="8" t="n"/>
       <c r="M94" s="8" t="n"/>
       <c r="N94" s="8" t="n">
-        <v>16368</v>
+        <v>20820</v>
       </c>
       <c r="O94" s="8" t="n">
         <v>0</v>
@@ -23986,12 +23992,12 @@
       <c r="P94" s="8" t="n"/>
       <c r="Q94" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="R94" s="8" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S94" s="9" t="inlineStr"/>
@@ -24008,7 +24014,7 @@
       <c r="V94" s="7" t="inlineStr"/>
       <c r="W94" s="8" t="inlineStr">
         <is>
-          <t>8a8446c119238f7a042580aed1922ef6cfd79ae2</t>
+          <t>c5c1741357dfce3547bdab7d4d5a0e7602846192</t>
         </is>
       </c>
     </row>
@@ -24022,7 +24028,7 @@
         </is>
       </c>
       <c r="C95" s="17" t="n">
-        <v>1250</v>
+        <v>1645</v>
       </c>
       <c r="D95" s="8" t="n">
         <v>1</v>
@@ -24037,7 +24043,7 @@
       </c>
       <c r="G95" s="9" t="inlineStr">
         <is>
-          <t>Victoria Street, Bristol, BS1 6DR</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H95" s="8" t="inlineStr">
@@ -24045,13 +24051,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I95" s="8" t="n"/>
+      <c r="I95" s="8" t="n">
+        <v>571</v>
+      </c>
       <c r="J95" s="8" t="n"/>
       <c r="K95" s="8" t="n"/>
       <c r="L95" s="8" t="n"/>
       <c r="M95" s="8" t="n"/>
       <c r="N95" s="8" t="n">
-        <v>21160</v>
+        <v>20820</v>
       </c>
       <c r="O95" s="8" t="n">
         <v>0</v>
@@ -24059,12 +24067,12 @@
       <c r="P95" s="8" t="n"/>
       <c r="Q95" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="R95" s="8" t="inlineStr">
         <is>
-          <t>Visum, Nationwide</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S95" s="9" t="inlineStr"/>
@@ -24081,7 +24089,7 @@
       <c r="V95" s="7" t="inlineStr"/>
       <c r="W95" s="8" t="inlineStr">
         <is>
-          <t>78fe8e0511ccc37f104368075238c845f57d7864</t>
+          <t>487e67b2d6680ebaabfcc49d4d33e21cb65cca6d</t>
         </is>
       </c>
     </row>
@@ -24095,7 +24103,7 @@
         </is>
       </c>
       <c r="C96" s="17" t="n">
-        <v>1999</v>
+        <v>1600</v>
       </c>
       <c r="D96" s="8" t="n">
         <v>2</v>
@@ -24110,12 +24118,12 @@
       </c>
       <c r="G96" s="9" t="inlineStr">
         <is>
-          <t>Swann House, Bristol, BS1</t>
+          <t>Stapleton Road, Bristol, BS5</t>
         </is>
       </c>
       <c r="H96" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS5</t>
         </is>
       </c>
       <c r="I96" s="8" t="n"/>
@@ -24124,7 +24132,7 @@
       <c r="L96" s="8" t="n"/>
       <c r="M96" s="8" t="n"/>
       <c r="N96" s="8" t="n">
-        <v>20800</v>
+        <v>19576</v>
       </c>
       <c r="O96" s="8" t="n">
         <v>0</v>
@@ -24132,7 +24140,7 @@
       <c r="P96" s="8" t="n"/>
       <c r="Q96" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="R96" s="8" t="inlineStr">
@@ -24154,7 +24162,7 @@
       <c r="V96" s="7" t="inlineStr"/>
       <c r="W96" s="8" t="inlineStr">
         <is>
-          <t>5cec67aa8ba885c4c8f85e47d3354d187da9d897</t>
+          <t>41184aca0a094a13f0cf944554fa6ab5b6f9b761</t>
         </is>
       </c>
     </row>
@@ -24168,13 +24176,13 @@
         </is>
       </c>
       <c r="C97" s="17" t="n">
-        <v>1670</v>
+        <v>1550</v>
       </c>
       <c r="D97" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E97" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F97" s="8" t="inlineStr">
         <is>
@@ -24183,7 +24191,7 @@
       </c>
       <c r="G97" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>City Centre, Waverley House, BS1 5LW</t>
         </is>
       </c>
       <c r="H97" s="8" t="inlineStr">
@@ -24192,14 +24200,14 @@
         </is>
       </c>
       <c r="I97" s="8" t="n">
-        <v>485</v>
+        <v>775</v>
       </c>
       <c r="J97" s="8" t="n"/>
       <c r="K97" s="8" t="n"/>
       <c r="L97" s="8" t="n"/>
       <c r="M97" s="8" t="n"/>
       <c r="N97" s="8" t="n">
-        <v>21504</v>
+        <v>17744</v>
       </c>
       <c r="O97" s="8" t="n">
         <v>0</v>
@@ -24207,12 +24215,12 @@
       <c r="P97" s="8" t="n"/>
       <c r="Q97" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="R97" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>The Bristol Residential Letting Co, Clifton</t>
         </is>
       </c>
       <c r="S97" s="9" t="inlineStr"/>
@@ -24229,7 +24237,7 @@
       <c r="V97" s="7" t="inlineStr"/>
       <c r="W97" s="8" t="inlineStr">
         <is>
-          <t>73f3509a6c69eef7af4c6b9ff0dc69b97478c20a</t>
+          <t>ac4ae9e8b18bae38c431398f0f633dd1691dd454</t>
         </is>
       </c>
     </row>
@@ -24243,13 +24251,13 @@
         </is>
       </c>
       <c r="C98" s="17" t="n">
-        <v>1645</v>
+        <v>2125</v>
       </c>
       <c r="D98" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E98" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F98" s="8" t="inlineStr">
         <is>
@@ -24267,7 +24275,7 @@
         </is>
       </c>
       <c r="I98" s="8" t="n">
-        <v>517</v>
+        <v>705</v>
       </c>
       <c r="J98" s="8" t="n"/>
       <c r="K98" s="8" t="n"/>
@@ -24282,7 +24290,7 @@
       <c r="P98" s="8" t="n"/>
       <c r="Q98" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="R98" s="8" t="inlineStr">
@@ -24304,7 +24312,7 @@
       <c r="V98" s="7" t="inlineStr"/>
       <c r="W98" s="8" t="inlineStr">
         <is>
-          <t>4efcb79ae710a68f5f272a2f9030937499117f9d</t>
+          <t>98852e60433cf90995df068fb3ceec727903a8f0</t>
         </is>
       </c>
     </row>
@@ -24318,13 +24326,13 @@
         </is>
       </c>
       <c r="C99" s="17" t="n">
-        <v>2120</v>
+        <v>1580</v>
       </c>
       <c r="D99" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E99" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F99" s="8" t="inlineStr">
         <is>
@@ -24333,7 +24341,7 @@
       </c>
       <c r="G99" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H99" s="8" t="inlineStr">
@@ -24342,14 +24350,14 @@
         </is>
       </c>
       <c r="I99" s="8" t="n">
-        <v>705</v>
+        <v>486</v>
       </c>
       <c r="J99" s="8" t="n"/>
       <c r="K99" s="8" t="n"/>
       <c r="L99" s="8" t="n"/>
       <c r="M99" s="8" t="n"/>
       <c r="N99" s="8" t="n">
-        <v>20820</v>
+        <v>21504</v>
       </c>
       <c r="O99" s="8" t="n">
         <v>0</v>
@@ -24357,12 +24365,12 @@
       <c r="P99" s="8" t="n"/>
       <c r="Q99" s="8" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="R99" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S99" s="9" t="inlineStr"/>
@@ -24379,7 +24387,7 @@
       <c r="V99" s="7" t="inlineStr"/>
       <c r="W99" s="8" t="inlineStr">
         <is>
-          <t>c5c1741357dfce3547bdab7d4d5a0e7602846192</t>
+          <t>75f9f4931bb794ff7a8be9528691bace351a0d13</t>
         </is>
       </c>
     </row>
@@ -24393,7 +24401,7 @@
         </is>
       </c>
       <c r="C100" s="17" t="n">
-        <v>1645</v>
+        <v>1500</v>
       </c>
       <c r="D100" s="8" t="n">
         <v>1</v>
@@ -24408,23 +24416,23 @@
       </c>
       <c r="G100" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Bedminster, Regent House, BS3 1FT</t>
         </is>
       </c>
       <c r="H100" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS3</t>
         </is>
       </c>
       <c r="I100" s="8" t="n">
-        <v>571</v>
+        <v>527</v>
       </c>
       <c r="J100" s="8" t="n"/>
       <c r="K100" s="8" t="n"/>
       <c r="L100" s="8" t="n"/>
       <c r="M100" s="8" t="n"/>
       <c r="N100" s="8" t="n">
-        <v>20820</v>
+        <v>13548</v>
       </c>
       <c r="O100" s="8" t="n">
         <v>0</v>
@@ -24432,12 +24440,12 @@
       <c r="P100" s="8" t="n"/>
       <c r="Q100" s="8" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="R100" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S100" s="9" t="inlineStr"/>
@@ -24454,7 +24462,7 @@
       <c r="V100" s="7" t="inlineStr"/>
       <c r="W100" s="8" t="inlineStr">
         <is>
-          <t>487e67b2d6680ebaabfcc49d4d33e21cb65cca6d</t>
+          <t>b5574d3457f97017e231a45d57df860c0d54fe3d</t>
         </is>
       </c>
     </row>
@@ -24468,10 +24476,10 @@
         </is>
       </c>
       <c r="C101" s="17" t="n">
-        <v>1600</v>
+        <v>1350</v>
       </c>
       <c r="D101" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E101" s="8" t="n">
         <v>1</v>
@@ -24483,21 +24491,23 @@
       </c>
       <c r="G101" s="9" t="inlineStr">
         <is>
-          <t>Stapleton Road, Bristol, BS5</t>
+          <t>Baldwin Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H101" s="8" t="inlineStr">
         <is>
-          <t>BS5</t>
-        </is>
-      </c>
-      <c r="I101" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I101" s="8" t="n">
+        <v>413</v>
+      </c>
       <c r="J101" s="8" t="n"/>
       <c r="K101" s="8" t="n"/>
       <c r="L101" s="8" t="n"/>
       <c r="M101" s="8" t="n"/>
       <c r="N101" s="8" t="n">
-        <v>19576</v>
+        <v>21148</v>
       </c>
       <c r="O101" s="8" t="n">
         <v>0</v>
@@ -24505,12 +24515,12 @@
       <c r="P101" s="8" t="n"/>
       <c r="Q101" s="8" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="R101" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Savills Lettings, Clifton</t>
         </is>
       </c>
       <c r="S101" s="9" t="inlineStr"/>
@@ -24527,7 +24537,7 @@
       <c r="V101" s="7" t="inlineStr"/>
       <c r="W101" s="8" t="inlineStr">
         <is>
-          <t>41184aca0a094a13f0cf944554fa6ab5b6f9b761</t>
+          <t>ca58d4891f705dc219b7ca74ef59637a2959afb0</t>
         </is>
       </c>
     </row>
@@ -24541,7 +24551,7 @@
         </is>
       </c>
       <c r="C102" s="17" t="n">
-        <v>1555</v>
+        <v>1620</v>
       </c>
       <c r="D102" s="8" t="n">
         <v>1</v>
@@ -24556,21 +24566,23 @@
       </c>
       <c r="G102" s="9" t="inlineStr">
         <is>
-          <t>Lombard Street, Bristol, BS3</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H102" s="8" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I102" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I102" s="8" t="n">
+        <v>494</v>
+      </c>
       <c r="J102" s="8" t="n"/>
       <c r="K102" s="8" t="n"/>
       <c r="L102" s="8" t="n"/>
       <c r="M102" s="8" t="n"/>
       <c r="N102" s="8" t="n">
-        <v>12036</v>
+        <v>20820</v>
       </c>
       <c r="O102" s="8" t="n">
         <v>0</v>
@@ -24578,12 +24590,12 @@
       <c r="P102" s="8" t="n"/>
       <c r="Q102" s="8" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="R102" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S102" s="9" t="inlineStr"/>
@@ -24600,7 +24612,7 @@
       <c r="V102" s="7" t="inlineStr"/>
       <c r="W102" s="8" t="inlineStr">
         <is>
-          <t>4d3990c67ed2848296e2aa2fa362730e0557bd43</t>
+          <t>b9cdcc0c4daa02ab2447615be3746df090f8a759</t>
         </is>
       </c>
     </row>
@@ -24614,7 +24626,7 @@
         </is>
       </c>
       <c r="C103" s="17" t="n">
-        <v>1550</v>
+        <v>2110</v>
       </c>
       <c r="D103" s="8" t="n">
         <v>2</v>
@@ -24629,7 +24641,7 @@
       </c>
       <c r="G103" s="9" t="inlineStr">
         <is>
-          <t>City Centre, Waverley House, BS1 5LW</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H103" s="8" t="inlineStr">
@@ -24638,15 +24650,13 @@
         </is>
       </c>
       <c r="I103" s="8" t="n">
-        <v>775</v>
+        <v>722</v>
       </c>
       <c r="J103" s="8" t="n"/>
       <c r="K103" s="8" t="n"/>
       <c r="L103" s="8" t="n"/>
       <c r="M103" s="8" t="n"/>
-      <c r="N103" s="8" t="n">
-        <v>17744</v>
-      </c>
+      <c r="N103" s="8" t="n"/>
       <c r="O103" s="8" t="n">
         <v>0</v>
       </c>
@@ -24658,7 +24668,7 @@
       </c>
       <c r="R103" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Clifton</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S103" s="9" t="inlineStr"/>
@@ -24675,7 +24685,7 @@
       <c r="V103" s="7" t="inlineStr"/>
       <c r="W103" s="8" t="inlineStr">
         <is>
-          <t>ac4ae9e8b18bae38c431398f0f633dd1691dd454</t>
+          <t>1fc314f1a5b51f6a42142e88d789000861f8e441</t>
         </is>
       </c>
     </row>
@@ -24689,13 +24699,13 @@
         </is>
       </c>
       <c r="C104" s="17" t="n">
-        <v>2125</v>
+        <v>1300</v>
       </c>
       <c r="D104" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E104" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F104" s="8" t="inlineStr">
         <is>
@@ -24704,7 +24714,7 @@
       </c>
       <c r="G104" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>City Centre, Queen Square Apartments, BS1</t>
         </is>
       </c>
       <c r="H104" s="8" t="inlineStr">
@@ -24713,14 +24723,14 @@
         </is>
       </c>
       <c r="I104" s="8" t="n">
-        <v>705</v>
+        <v>405</v>
       </c>
       <c r="J104" s="8" t="n"/>
       <c r="K104" s="8" t="n"/>
       <c r="L104" s="8" t="n"/>
       <c r="M104" s="8" t="n"/>
       <c r="N104" s="8" t="n">
-        <v>20820</v>
+        <v>20316</v>
       </c>
       <c r="O104" s="8" t="n">
         <v>0</v>
@@ -24728,12 +24738,12 @@
       <c r="P104" s="8" t="n"/>
       <c r="Q104" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="R104" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S104" s="9" t="inlineStr"/>
@@ -24750,7 +24760,7 @@
       <c r="V104" s="7" t="inlineStr"/>
       <c r="W104" s="8" t="inlineStr">
         <is>
-          <t>98852e60433cf90995df068fb3ceec727903a8f0</t>
+          <t>9ad2c7bc90885b9a9e65b462b952842a964f1d35</t>
         </is>
       </c>
     </row>
@@ -24764,7 +24774,7 @@
         </is>
       </c>
       <c r="C105" s="17" t="n">
-        <v>1580</v>
+        <v>1400</v>
       </c>
       <c r="D105" s="8" t="n">
         <v>1</v>
@@ -24779,7 +24789,7 @@
       </c>
       <c r="G105" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Redcliffe Parade West, Flat 3, City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H105" s="8" t="inlineStr">
@@ -24787,15 +24797,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I105" s="8" t="n">
-        <v>486</v>
-      </c>
+      <c r="I105" s="8" t="n"/>
       <c r="J105" s="8" t="n"/>
       <c r="K105" s="8" t="n"/>
       <c r="L105" s="8" t="n"/>
       <c r="M105" s="8" t="n"/>
       <c r="N105" s="8" t="n">
-        <v>21504</v>
+        <v>19484</v>
       </c>
       <c r="O105" s="8" t="n">
         <v>0</v>
@@ -24803,12 +24811,12 @@
       <c r="P105" s="8" t="n"/>
       <c r="Q105" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="R105" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S105" s="9" t="inlineStr"/>
@@ -24825,7 +24833,7 @@
       <c r="V105" s="7" t="inlineStr"/>
       <c r="W105" s="8" t="inlineStr">
         <is>
-          <t>75f9f4931bb794ff7a8be9528691bace351a0d13</t>
+          <t>9b65e5a0fb0bc8fc27d566eae912cddf76828cc9</t>
         </is>
       </c>
     </row>
@@ -24839,7 +24847,7 @@
         </is>
       </c>
       <c r="C106" s="17" t="n">
-        <v>1500</v>
+        <v>1650</v>
       </c>
       <c r="D106" s="8" t="n">
         <v>1</v>
@@ -24854,36 +24862,32 @@
       </c>
       <c r="G106" s="9" t="inlineStr">
         <is>
-          <t>Bedminster, Regent House, BS3 1FT</t>
+          <t>Horizon, Broad Weir, Bristol, BS1</t>
         </is>
       </c>
       <c r="H106" s="8" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I106" s="8" t="n">
-        <v>527</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I106" s="8" t="n"/>
       <c r="J106" s="8" t="n"/>
       <c r="K106" s="8" t="n"/>
       <c r="L106" s="8" t="n"/>
       <c r="M106" s="8" t="n"/>
-      <c r="N106" s="8" t="n">
-        <v>13548</v>
-      </c>
+      <c r="N106" s="8" t="n"/>
       <c r="O106" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P106" s="8" t="n"/>
       <c r="Q106" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="R106" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>CJ Hole, Bishopston</t>
         </is>
       </c>
       <c r="S106" s="9" t="inlineStr"/>
@@ -24900,7 +24904,7 @@
       <c r="V106" s="7" t="inlineStr"/>
       <c r="W106" s="8" t="inlineStr">
         <is>
-          <t>b5574d3457f97017e231a45d57df860c0d54fe3d</t>
+          <t>aa3cf620ad25601a026424157bd8c0abb746373f</t>
         </is>
       </c>
     </row>
@@ -24914,13 +24918,13 @@
         </is>
       </c>
       <c r="C107" s="17" t="n">
-        <v>1350</v>
+        <v>1500</v>
       </c>
       <c r="D107" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E107" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F107" s="8" t="inlineStr">
         <is>
@@ -24929,7 +24933,7 @@
       </c>
       <c r="G107" s="9" t="inlineStr">
         <is>
-          <t>Baldwin Street, Bristol, BS1</t>
+          <t>Small Street - City Centre</t>
         </is>
       </c>
       <c r="H107" s="8" t="inlineStr">
@@ -24937,15 +24941,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I107" s="8" t="n">
-        <v>413</v>
-      </c>
+      <c r="I107" s="8" t="n"/>
       <c r="J107" s="8" t="n"/>
       <c r="K107" s="8" t="n"/>
       <c r="L107" s="8" t="n"/>
       <c r="M107" s="8" t="n"/>
       <c r="N107" s="8" t="n">
-        <v>21148</v>
+        <v>21816</v>
       </c>
       <c r="O107" s="8" t="n">
         <v>0</v>
@@ -24953,12 +24955,12 @@
       <c r="P107" s="8" t="n"/>
       <c r="Q107" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R107" s="8" t="inlineStr">
         <is>
-          <t>Savills Lettings, Clifton</t>
+          <t>Ocean, Clifton</t>
         </is>
       </c>
       <c r="S107" s="9" t="inlineStr"/>
@@ -24975,7 +24977,7 @@
       <c r="V107" s="7" t="inlineStr"/>
       <c r="W107" s="8" t="inlineStr">
         <is>
-          <t>ca58d4891f705dc219b7ca74ef59637a2959afb0</t>
+          <t>cb4b1af676ff54ae12ad7bf4fa94acd8ef94a533</t>
         </is>
       </c>
     </row>
@@ -24989,7 +24991,7 @@
         </is>
       </c>
       <c r="C108" s="17" t="n">
-        <v>1620</v>
+        <v>1150</v>
       </c>
       <c r="D108" s="8" t="n">
         <v>1</v>
@@ -25004,23 +25006,21 @@
       </c>
       <c r="G108" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Knowle Road, Bristol</t>
         </is>
       </c>
       <c r="H108" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I108" s="8" t="n">
-        <v>494</v>
-      </c>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I108" s="8" t="n"/>
       <c r="J108" s="8" t="n"/>
       <c r="K108" s="8" t="n"/>
       <c r="L108" s="8" t="n"/>
       <c r="M108" s="8" t="n"/>
       <c r="N108" s="8" t="n">
-        <v>20820</v>
+        <v>6872</v>
       </c>
       <c r="O108" s="8" t="n">
         <v>0</v>
@@ -25028,12 +25028,12 @@
       <c r="P108" s="8" t="n"/>
       <c r="Q108" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R108" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Hopewell, Bristol</t>
         </is>
       </c>
       <c r="S108" s="9" t="inlineStr"/>
@@ -25050,7 +25050,7 @@
       <c r="V108" s="7" t="inlineStr"/>
       <c r="W108" s="8" t="inlineStr">
         <is>
-          <t>b9cdcc0c4daa02ab2447615be3746df090f8a759</t>
+          <t>edac1b499f84e07ce85894b488f82dc5cd104202</t>
         </is>
       </c>
     </row>
@@ -25064,13 +25064,13 @@
         </is>
       </c>
       <c r="C109" s="17" t="n">
-        <v>2110</v>
+        <v>1555</v>
       </c>
       <c r="D109" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E109" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F109" s="8" t="inlineStr">
         <is>
@@ -25079,34 +25079,34 @@
       </c>
       <c r="G109" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Lombard Street, Bristol, BS3</t>
         </is>
       </c>
       <c r="H109" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I109" s="8" t="n">
-        <v>722</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I109" s="8" t="n"/>
       <c r="J109" s="8" t="n"/>
       <c r="K109" s="8" t="n"/>
       <c r="L109" s="8" t="n"/>
       <c r="M109" s="8" t="n"/>
-      <c r="N109" s="8" t="n"/>
+      <c r="N109" s="8" t="n">
+        <v>12036</v>
+      </c>
       <c r="O109" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P109" s="8" t="n"/>
       <c r="Q109" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="R109" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S109" s="9" t="inlineStr"/>
@@ -25123,7 +25123,7 @@
       <c r="V109" s="7" t="inlineStr"/>
       <c r="W109" s="8" t="inlineStr">
         <is>
-          <t>1fc314f1a5b51f6a42142e88d789000861f8e441</t>
+          <t>4d3990c67ed2848296e2aa2fa362730e0557bd43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
House search data from run 25
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -17172,7 +17172,7 @@
       <c r="L4" s="8" t="n"/>
       <c r="M4" s="8" t="n"/>
       <c r="N4" s="8" t="n">
-        <v>21660</v>
+        <v>21616</v>
       </c>
       <c r="O4" s="8" t="n">
         <v>0</v>
@@ -21074,13 +21074,13 @@
         </is>
       </c>
       <c r="C55" s="17" t="n">
-        <v>2200</v>
+        <v>2300</v>
       </c>
       <c r="D55" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E55" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F55" s="8" t="inlineStr">
         <is>
@@ -21133,7 +21133,7 @@
       <c r="V55" s="7" t="inlineStr"/>
       <c r="W55" s="8" t="inlineStr">
         <is>
-          <t>406fab2577557efdd9382cee302acdc7a788c3d8</t>
+          <t>82dded0955660a8ec4af3acb8db470436bdc522b</t>
         </is>
       </c>
     </row>
@@ -21162,7 +21162,7 @@
       </c>
       <c r="G56" s="9" t="inlineStr">
         <is>
-          <t>Castle Park View, Castle Street, Bristol</t>
+          <t>Castle Park View, Castle Street, Bristol, BS2 0ND</t>
         </is>
       </c>
       <c r="H56" s="8" t="inlineStr">
@@ -21206,7 +21206,7 @@
       <c r="V56" s="7" t="inlineStr"/>
       <c r="W56" s="8" t="inlineStr">
         <is>
-          <t>82dded0955660a8ec4af3acb8db470436bdc522b</t>
+          <t>fc4abec405a6b435cb290523f6e7784fc2de1099</t>
         </is>
       </c>
     </row>
@@ -21220,13 +21220,13 @@
         </is>
       </c>
       <c r="C57" s="17" t="n">
-        <v>2300</v>
+        <v>2095</v>
       </c>
       <c r="D57" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E57" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F57" s="8" t="inlineStr">
         <is>
@@ -21235,7 +21235,7 @@
       </c>
       <c r="G57" s="9" t="inlineStr">
         <is>
-          <t>Castle Park View, Castle Street, Bristol, BS2 0ND</t>
+          <t>Castle Park View, Castle Street, BS2 0ND, Bristol</t>
         </is>
       </c>
       <c r="H57" s="8" t="inlineStr">
@@ -21279,7 +21279,7 @@
       <c r="V57" s="7" t="inlineStr"/>
       <c r="W57" s="8" t="inlineStr">
         <is>
-          <t>fc4abec405a6b435cb290523f6e7784fc2de1099</t>
+          <t>7a4bff96a8fb36d99cc3d7825e84bee85f8c5ba7</t>
         </is>
       </c>
     </row>
@@ -21293,10 +21293,10 @@
         </is>
       </c>
       <c r="C58" s="17" t="n">
-        <v>2095</v>
+        <v>1400</v>
       </c>
       <c r="D58" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E58" s="8" t="n">
         <v>1</v>
@@ -21308,12 +21308,12 @@
       </c>
       <c r="G58" s="9" t="inlineStr">
         <is>
-          <t>Castle Park View, Castle Street, BS2 0ND, Bristol</t>
+          <t>Jessop Court Ferry Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I58" s="8" t="n"/>
@@ -21322,7 +21322,7 @@
       <c r="L58" s="8" t="n"/>
       <c r="M58" s="8" t="n"/>
       <c r="N58" s="8" t="n">
-        <v>21984</v>
+        <v>20908</v>
       </c>
       <c r="O58" s="8" t="n">
         <v>0</v>
@@ -21330,12 +21330,12 @@
       <c r="P58" s="8" t="n"/>
       <c r="Q58" s="8" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="R58" s="8" t="inlineStr">
         <is>
-          <t>Savills Lettings, CPV</t>
+          <t>Accommodation Unlimited, Bristol</t>
         </is>
       </c>
       <c r="S58" s="9" t="inlineStr"/>
@@ -21352,7 +21352,7 @@
       <c r="V58" s="7" t="inlineStr"/>
       <c r="W58" s="8" t="inlineStr">
         <is>
-          <t>7a4bff96a8fb36d99cc3d7825e84bee85f8c5ba7</t>
+          <t>45f17f505657c6333c92b921a50f7641e02f2c2f</t>
         </is>
       </c>
     </row>
@@ -21366,10 +21366,10 @@
         </is>
       </c>
       <c r="C59" s="17" t="n">
-        <v>1400</v>
+        <v>1500</v>
       </c>
       <c r="D59" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E59" s="8" t="n">
         <v>1</v>
@@ -21381,12 +21381,12 @@
       </c>
       <c r="G59" s="9" t="inlineStr">
         <is>
-          <t>Jessop Court Ferry Street, Bristol, BS1</t>
+          <t>St Clements Court, Wilson Street, Bristol</t>
         </is>
       </c>
       <c r="H59" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I59" s="8" t="n"/>
@@ -21395,7 +21395,7 @@
       <c r="L59" s="8" t="n"/>
       <c r="M59" s="8" t="n"/>
       <c r="N59" s="8" t="n">
-        <v>20908</v>
+        <v>21600</v>
       </c>
       <c r="O59" s="8" t="n">
         <v>0</v>
@@ -21403,12 +21403,12 @@
       <c r="P59" s="8" t="n"/>
       <c r="Q59" s="8" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="R59" s="8" t="inlineStr">
         <is>
-          <t>Accommodation Unlimited, Bristol</t>
+          <t>Kendall Harper, Bishopston</t>
         </is>
       </c>
       <c r="S59" s="9" t="inlineStr"/>
@@ -21425,7 +21425,7 @@
       <c r="V59" s="7" t="inlineStr"/>
       <c r="W59" s="8" t="inlineStr">
         <is>
-          <t>45f17f505657c6333c92b921a50f7641e02f2c2f</t>
+          <t>b3bf3a18fe9e3595ef643379d979e59ee826fcbc</t>
         </is>
       </c>
     </row>
@@ -21454,7 +21454,7 @@
       </c>
       <c r="G60" s="9" t="inlineStr">
         <is>
-          <t>St Clements Court, Wilson Street, Bristol</t>
+          <t>Midland Mews Waterloo Road Old Market, Bristol, BS2</t>
         </is>
       </c>
       <c r="H60" s="8" t="inlineStr">
@@ -21468,7 +21468,7 @@
       <c r="L60" s="8" t="n"/>
       <c r="M60" s="8" t="n"/>
       <c r="N60" s="8" t="n">
-        <v>21600</v>
+        <v>20856</v>
       </c>
       <c r="O60" s="8" t="n">
         <v>0</v>
@@ -21476,12 +21476,12 @@
       <c r="P60" s="8" t="n"/>
       <c r="Q60" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="R60" s="8" t="inlineStr">
         <is>
-          <t>Kendall Harper, Bishopston</t>
+          <t>Accommodation Unlimited, Bristol</t>
         </is>
       </c>
       <c r="S60" s="9" t="inlineStr"/>
@@ -21498,7 +21498,7 @@
       <c r="V60" s="7" t="inlineStr"/>
       <c r="W60" s="8" t="inlineStr">
         <is>
-          <t>b3bf3a18fe9e3595ef643379d979e59ee826fcbc</t>
+          <t>f83555c1dc6f03087d999787a76db9b49794ddb4</t>
         </is>
       </c>
     </row>
@@ -21512,13 +21512,13 @@
         </is>
       </c>
       <c r="C61" s="17" t="n">
-        <v>1600</v>
+        <v>2020</v>
       </c>
       <c r="D61" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E61" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F61" s="8" t="inlineStr">
         <is>
@@ -21527,16 +21527,16 @@
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
-          <t>Waterloo Road, Midland Mews, BS2</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H61" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I61" s="8" t="n">
-        <v>721</v>
+        <v>764</v>
       </c>
       <c r="J61" s="8" t="n"/>
       <c r="K61" s="8" t="n"/>
@@ -21551,12 +21551,12 @@
       <c r="P61" s="8" t="n"/>
       <c r="Q61" s="8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="R61" s="8" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S61" s="9" t="inlineStr"/>
@@ -21573,7 +21573,7 @@
       <c r="V61" s="7" t="inlineStr"/>
       <c r="W61" s="8" t="inlineStr">
         <is>
-          <t>cf8a979c7c13e868d74a6828d64c93a46d2e7209</t>
+          <t>6140b74b7d83ae5918fdabb6f9371e2f4b63a9c2</t>
         </is>
       </c>
     </row>
@@ -21587,13 +21587,13 @@
         </is>
       </c>
       <c r="C62" s="17" t="n">
-        <v>1500</v>
+        <v>2145</v>
       </c>
       <c r="D62" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E62" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
@@ -21602,21 +21602,23 @@
       </c>
       <c r="G62" s="9" t="inlineStr">
         <is>
-          <t>Midland Mews Waterloo Road Old Market, Bristol, BS2</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H62" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I62" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I62" s="8" t="n">
+        <v>815</v>
+      </c>
       <c r="J62" s="8" t="n"/>
       <c r="K62" s="8" t="n"/>
       <c r="L62" s="8" t="n"/>
       <c r="M62" s="8" t="n"/>
       <c r="N62" s="8" t="n">
-        <v>20856</v>
+        <v>21504</v>
       </c>
       <c r="O62" s="8" t="n">
         <v>0</v>
@@ -21624,12 +21626,12 @@
       <c r="P62" s="8" t="n"/>
       <c r="Q62" s="8" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="R62" s="8" t="inlineStr">
         <is>
-          <t>Accommodation Unlimited, Bristol</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S62" s="9" t="inlineStr"/>
@@ -21646,7 +21648,7 @@
       <c r="V62" s="7" t="inlineStr"/>
       <c r="W62" s="8" t="inlineStr">
         <is>
-          <t>f83555c1dc6f03087d999787a76db9b49794ddb4</t>
+          <t>24009eb3414633bf24b3b69631ba405866a1e5c9</t>
         </is>
       </c>
     </row>
@@ -21660,13 +21662,13 @@
         </is>
       </c>
       <c r="C63" s="17" t="n">
-        <v>2020</v>
+        <v>1635</v>
       </c>
       <c r="D63" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E63" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F63" s="8" t="inlineStr">
         <is>
@@ -21675,7 +21677,7 @@
       </c>
       <c r="G63" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H63" s="8" t="inlineStr">
@@ -21684,14 +21686,14 @@
         </is>
       </c>
       <c r="I63" s="8" t="n">
-        <v>764</v>
+        <v>486</v>
       </c>
       <c r="J63" s="8" t="n"/>
       <c r="K63" s="8" t="n"/>
       <c r="L63" s="8" t="n"/>
       <c r="M63" s="8" t="n"/>
       <c r="N63" s="8" t="n">
-        <v>20856</v>
+        <v>21504</v>
       </c>
       <c r="O63" s="8" t="n">
         <v>0</v>
@@ -21704,7 +21706,7 @@
       </c>
       <c r="R63" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S63" s="9" t="inlineStr"/>
@@ -21721,7 +21723,7 @@
       <c r="V63" s="7" t="inlineStr"/>
       <c r="W63" s="8" t="inlineStr">
         <is>
-          <t>6140b74b7d83ae5918fdabb6f9371e2f4b63a9c2</t>
+          <t>bbf6e42784b6e4b7dae8d6bef9900115d0f3056e</t>
         </is>
       </c>
     </row>
@@ -21735,7 +21737,7 @@
         </is>
       </c>
       <c r="C64" s="17" t="n">
-        <v>2145</v>
+        <v>1750</v>
       </c>
       <c r="D64" s="8" t="n">
         <v>2</v>
@@ -21750,23 +21752,23 @@
       </c>
       <c r="G64" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Arnos Vale, Paintworks, BS4</t>
         </is>
       </c>
       <c r="H64" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS4</t>
         </is>
       </c>
       <c r="I64" s="8" t="n">
-        <v>815</v>
+        <v>731</v>
       </c>
       <c r="J64" s="8" t="n"/>
       <c r="K64" s="8" t="n"/>
       <c r="L64" s="8" t="n"/>
       <c r="M64" s="8" t="n"/>
       <c r="N64" s="8" t="n">
-        <v>21504</v>
+        <v>4680</v>
       </c>
       <c r="O64" s="8" t="n">
         <v>0</v>
@@ -21779,7 +21781,7 @@
       </c>
       <c r="R64" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S64" s="9" t="inlineStr"/>
@@ -21796,7 +21798,7 @@
       <c r="V64" s="7" t="inlineStr"/>
       <c r="W64" s="8" t="inlineStr">
         <is>
-          <t>24009eb3414633bf24b3b69631ba405866a1e5c9</t>
+          <t>1c0acc4cbbc0f239d4843e9eb56c0d04ca3a6278</t>
         </is>
       </c>
     </row>
@@ -21810,7 +21812,7 @@
         </is>
       </c>
       <c r="C65" s="17" t="n">
-        <v>1635</v>
+        <v>2100</v>
       </c>
       <c r="D65" s="8" t="n">
         <v>1</v>
@@ -21825,7 +21827,7 @@
       </c>
       <c r="G65" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Baldwin St, Bristol, BS1</t>
         </is>
       </c>
       <c r="H65" s="8" t="inlineStr">
@@ -21833,15 +21835,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I65" s="8" t="n">
-        <v>486</v>
-      </c>
+      <c r="I65" s="8" t="n"/>
       <c r="J65" s="8" t="n"/>
       <c r="K65" s="8" t="n"/>
       <c r="L65" s="8" t="n"/>
       <c r="M65" s="8" t="n"/>
       <c r="N65" s="8" t="n">
-        <v>21504</v>
+        <v>21148</v>
       </c>
       <c r="O65" s="8" t="n">
         <v>0</v>
@@ -21849,12 +21849,12 @@
       <c r="P65" s="8" t="n"/>
       <c r="Q65" s="8" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R65" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S65" s="9" t="inlineStr"/>
@@ -21871,7 +21871,7 @@
       <c r="V65" s="7" t="inlineStr"/>
       <c r="W65" s="8" t="inlineStr">
         <is>
-          <t>bbf6e42784b6e4b7dae8d6bef9900115d0f3056e</t>
+          <t>ba1c1abaa5dbfd6e19c20fa9df1e66799d9c2462</t>
         </is>
       </c>
     </row>
@@ -21885,7 +21885,7 @@
         </is>
       </c>
       <c r="C66" s="17" t="n">
-        <v>1750</v>
+        <v>2220</v>
       </c>
       <c r="D66" s="8" t="n">
         <v>2</v>
@@ -21900,23 +21900,23 @@
       </c>
       <c r="G66" s="9" t="inlineStr">
         <is>
-          <t>Arnos Vale, Paintworks, BS4</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H66" s="8" t="inlineStr">
         <is>
-          <t>BS4</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I66" s="8" t="n">
-        <v>731</v>
+        <v>697</v>
       </c>
       <c r="J66" s="8" t="n"/>
       <c r="K66" s="8" t="n"/>
       <c r="L66" s="8" t="n"/>
       <c r="M66" s="8" t="n"/>
       <c r="N66" s="8" t="n">
-        <v>4680</v>
+        <v>20820</v>
       </c>
       <c r="O66" s="8" t="n">
         <v>0</v>
@@ -21924,12 +21924,12 @@
       <c r="P66" s="8" t="n"/>
       <c r="Q66" s="8" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R66" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S66" s="9" t="inlineStr"/>
@@ -21946,7 +21946,7 @@
       <c r="V66" s="7" t="inlineStr"/>
       <c r="W66" s="8" t="inlineStr">
         <is>
-          <t>1c0acc4cbbc0f239d4843e9eb56c0d04ca3a6278</t>
+          <t>5870266ee1b15bf20f0a085f56358c762e522fa8</t>
         </is>
       </c>
     </row>
@@ -21960,7 +21960,7 @@
         </is>
       </c>
       <c r="C67" s="17" t="n">
-        <v>2100</v>
+        <v>1300</v>
       </c>
       <c r="D67" s="8" t="n">
         <v>1</v>
@@ -21975,7 +21975,7 @@
       </c>
       <c r="G67" s="9" t="inlineStr">
         <is>
-          <t>Baldwin St, Bristol, BS1</t>
+          <t>Bristol City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H67" s="8" t="inlineStr">
@@ -21989,7 +21989,7 @@
       <c r="L67" s="8" t="n"/>
       <c r="M67" s="8" t="n"/>
       <c r="N67" s="8" t="n">
-        <v>21148</v>
+        <v>21428</v>
       </c>
       <c r="O67" s="8" t="n">
         <v>0</v>
@@ -21997,7 +21997,7 @@
       <c r="P67" s="8" t="n"/>
       <c r="Q67" s="8" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="R67" s="8" t="inlineStr">
@@ -22019,7 +22019,7 @@
       <c r="V67" s="7" t="inlineStr"/>
       <c r="W67" s="8" t="inlineStr">
         <is>
-          <t>ba1c1abaa5dbfd6e19c20fa9df1e66799d9c2462</t>
+          <t>317e9ab29cad2381c41672743d877feba2c14e45</t>
         </is>
       </c>
     </row>
@@ -22033,13 +22033,13 @@
         </is>
       </c>
       <c r="C68" s="17" t="n">
-        <v>2220</v>
+        <v>1500</v>
       </c>
       <c r="D68" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E68" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
@@ -22048,7 +22048,7 @@
       </c>
       <c r="G68" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H68" s="8" t="inlineStr">
@@ -22057,14 +22057,14 @@
         </is>
       </c>
       <c r="I68" s="8" t="n">
-        <v>697</v>
+        <v>548</v>
       </c>
       <c r="J68" s="8" t="n"/>
       <c r="K68" s="8" t="n"/>
       <c r="L68" s="8" t="n"/>
       <c r="M68" s="8" t="n"/>
       <c r="N68" s="8" t="n">
-        <v>20820</v>
+        <v>21504</v>
       </c>
       <c r="O68" s="8" t="n">
         <v>0</v>
@@ -22072,12 +22072,12 @@
       <c r="P68" s="8" t="n"/>
       <c r="Q68" s="8" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R68" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S68" s="9" t="inlineStr"/>
@@ -22094,7 +22094,7 @@
       <c r="V68" s="7" t="inlineStr"/>
       <c r="W68" s="8" t="inlineStr">
         <is>
-          <t>5870266ee1b15bf20f0a085f56358c762e522fa8</t>
+          <t>bad1e4584285201ef9995d2b437343fca870009c</t>
         </is>
       </c>
     </row>
@@ -22108,7 +22108,7 @@
         </is>
       </c>
       <c r="C69" s="17" t="n">
-        <v>1300</v>
+        <v>1615</v>
       </c>
       <c r="D69" s="8" t="n">
         <v>1</v>
@@ -22123,7 +22123,7 @@
       </c>
       <c r="G69" s="9" t="inlineStr">
         <is>
-          <t>Bristol City Centre, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H69" s="8" t="inlineStr">
@@ -22131,13 +22131,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I69" s="8" t="n"/>
+      <c r="I69" s="8" t="n">
+        <v>486</v>
+      </c>
       <c r="J69" s="8" t="n"/>
       <c r="K69" s="8" t="n"/>
       <c r="L69" s="8" t="n"/>
       <c r="M69" s="8" t="n"/>
       <c r="N69" s="8" t="n">
-        <v>21428</v>
+        <v>21504</v>
       </c>
       <c r="O69" s="8" t="n">
         <v>0</v>
@@ -22145,12 +22147,12 @@
       <c r="P69" s="8" t="n"/>
       <c r="Q69" s="8" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R69" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S69" s="9" t="inlineStr"/>
@@ -22167,7 +22169,7 @@
       <c r="V69" s="7" t="inlineStr"/>
       <c r="W69" s="8" t="inlineStr">
         <is>
-          <t>317e9ab29cad2381c41672743d877feba2c14e45</t>
+          <t>67ff71428df47b0eb7f7da47600378ffdad1f97c</t>
         </is>
       </c>
     </row>
@@ -22181,10 +22183,10 @@
         </is>
       </c>
       <c r="C70" s="17" t="n">
-        <v>1500</v>
+        <v>1965</v>
       </c>
       <c r="D70" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E70" s="8" t="n">
         <v>1</v>
@@ -22205,7 +22207,7 @@
         </is>
       </c>
       <c r="I70" s="8" t="n">
-        <v>548</v>
+        <v>655</v>
       </c>
       <c r="J70" s="8" t="n"/>
       <c r="K70" s="8" t="n"/>
@@ -22220,7 +22222,7 @@
       <c r="P70" s="8" t="n"/>
       <c r="Q70" s="8" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="R70" s="8" t="inlineStr">
@@ -22242,7 +22244,7 @@
       <c r="V70" s="7" t="inlineStr"/>
       <c r="W70" s="8" t="inlineStr">
         <is>
-          <t>bad1e4584285201ef9995d2b437343fca870009c</t>
+          <t>1a5b509e1606992acea1736489630b2bc57cc717</t>
         </is>
       </c>
     </row>
@@ -22256,13 +22258,13 @@
         </is>
       </c>
       <c r="C71" s="17" t="n">
-        <v>1615</v>
+        <v>2080</v>
       </c>
       <c r="D71" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E71" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F71" s="8" t="inlineStr">
         <is>
@@ -22271,7 +22273,7 @@
       </c>
       <c r="G71" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H71" s="8" t="inlineStr">
@@ -22280,14 +22282,14 @@
         </is>
       </c>
       <c r="I71" s="8" t="n">
-        <v>486</v>
+        <v>705</v>
       </c>
       <c r="J71" s="8" t="n"/>
       <c r="K71" s="8" t="n"/>
       <c r="L71" s="8" t="n"/>
       <c r="M71" s="8" t="n"/>
       <c r="N71" s="8" t="n">
-        <v>21504</v>
+        <v>20820</v>
       </c>
       <c r="O71" s="8" t="n">
         <v>0</v>
@@ -22295,12 +22297,12 @@
       <c r="P71" s="8" t="n"/>
       <c r="Q71" s="8" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="R71" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S71" s="9" t="inlineStr"/>
@@ -22317,7 +22319,7 @@
       <c r="V71" s="7" t="inlineStr"/>
       <c r="W71" s="8" t="inlineStr">
         <is>
-          <t>67ff71428df47b0eb7f7da47600378ffdad1f97c</t>
+          <t>0453e07b653a16ada93327f26a41e0b204d289a4</t>
         </is>
       </c>
     </row>
@@ -22331,13 +22333,13 @@
         </is>
       </c>
       <c r="C72" s="17" t="n">
-        <v>1965</v>
+        <v>2020</v>
       </c>
       <c r="D72" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E72" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F72" s="8" t="inlineStr">
         <is>
@@ -22346,7 +22348,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
@@ -22355,27 +22357,25 @@
         </is>
       </c>
       <c r="I72" s="8" t="n">
-        <v>655</v>
+        <v>705</v>
       </c>
       <c r="J72" s="8" t="n"/>
       <c r="K72" s="8" t="n"/>
       <c r="L72" s="8" t="n"/>
       <c r="M72" s="8" t="n"/>
-      <c r="N72" s="8" t="n">
-        <v>21504</v>
-      </c>
+      <c r="N72" s="8" t="n"/>
       <c r="O72" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P72" s="8" t="n"/>
       <c r="Q72" s="8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="R72" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S72" s="9" t="inlineStr"/>
@@ -22392,7 +22392,7 @@
       <c r="V72" s="7" t="inlineStr"/>
       <c r="W72" s="8" t="inlineStr">
         <is>
-          <t>1a5b509e1606992acea1736489630b2bc57cc717</t>
+          <t>75b3ee81b8ecb4015a80108f6d509e4156f4e8e4</t>
         </is>
       </c>
     </row>
@@ -22406,7 +22406,7 @@
         </is>
       </c>
       <c r="C73" s="17" t="n">
-        <v>2080</v>
+        <v>2000</v>
       </c>
       <c r="D73" s="8" t="n">
         <v>2</v>
@@ -22421,7 +22421,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Eclipse - City Centre</t>
         </is>
       </c>
       <c r="H73" s="8" t="inlineStr">
@@ -22429,28 +22429,24 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I73" s="8" t="n">
-        <v>705</v>
-      </c>
+      <c r="I73" s="8" t="n"/>
       <c r="J73" s="8" t="n"/>
       <c r="K73" s="8" t="n"/>
       <c r="L73" s="8" t="n"/>
       <c r="M73" s="8" t="n"/>
-      <c r="N73" s="8" t="n">
-        <v>20820</v>
-      </c>
+      <c r="N73" s="8" t="n"/>
       <c r="O73" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P73" s="8" t="n"/>
       <c r="Q73" s="8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="R73" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Ocean, Clifton</t>
         </is>
       </c>
       <c r="S73" s="9" t="inlineStr"/>
@@ -22467,7 +22463,7 @@
       <c r="V73" s="7" t="inlineStr"/>
       <c r="W73" s="8" t="inlineStr">
         <is>
-          <t>0453e07b653a16ada93327f26a41e0b204d289a4</t>
+          <t>638ecbe81729048ffda61524ca9b06c4a208ce7b</t>
         </is>
       </c>
     </row>
@@ -22481,13 +22477,13 @@
         </is>
       </c>
       <c r="C74" s="17" t="n">
-        <v>2000</v>
+        <v>2085</v>
       </c>
       <c r="D74" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E74" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F74" s="8" t="inlineStr">
         <is>
@@ -22496,7 +22492,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>Welsh Back, Bristol, BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr">
@@ -22505,7 +22501,7 @@
         </is>
       </c>
       <c r="I74" s="8" t="n">
-        <v>908</v>
+        <v>705</v>
       </c>
       <c r="J74" s="8" t="n"/>
       <c r="K74" s="8" t="n"/>
@@ -22518,12 +22514,12 @@
       <c r="P74" s="8" t="n"/>
       <c r="Q74" s="8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="R74" s="8" t="inlineStr">
         <is>
-          <t>Hello Neighbour, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S74" s="9" t="inlineStr"/>
@@ -22540,7 +22536,7 @@
       <c r="V74" s="7" t="inlineStr"/>
       <c r="W74" s="8" t="inlineStr">
         <is>
-          <t>65ed2520fdf37e6dde4abe0097cc3edbbbeff957</t>
+          <t>16c89eb9a4cdeb57ddb3fd1201b7084ea2f3c007</t>
         </is>
       </c>
     </row>
@@ -22554,13 +22550,13 @@
         </is>
       </c>
       <c r="C75" s="17" t="n">
-        <v>2020</v>
+        <v>1615</v>
       </c>
       <c r="D75" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E75" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F75" s="8" t="inlineStr">
         <is>
@@ -22569,7 +22565,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr">
@@ -22578,7 +22574,7 @@
         </is>
       </c>
       <c r="I75" s="8" t="n">
-        <v>705</v>
+        <v>487</v>
       </c>
       <c r="J75" s="8" t="n"/>
       <c r="K75" s="8" t="n"/>
@@ -22591,12 +22587,12 @@
       <c r="P75" s="8" t="n"/>
       <c r="Q75" s="8" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="R75" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S75" s="9" t="inlineStr"/>
@@ -22613,7 +22609,7 @@
       <c r="V75" s="7" t="inlineStr"/>
       <c r="W75" s="8" t="inlineStr">
         <is>
-          <t>75b3ee81b8ecb4015a80108f6d509e4156f4e8e4</t>
+          <t>cd57661c8d996d20c5c1c7c34b12787f40073ec9</t>
         </is>
       </c>
     </row>
@@ -22627,7 +22623,7 @@
         </is>
       </c>
       <c r="C76" s="17" t="n">
-        <v>2000</v>
+        <v>2065</v>
       </c>
       <c r="D76" s="8" t="n">
         <v>2</v>
@@ -22642,7 +22638,7 @@
       </c>
       <c r="G76" s="9" t="inlineStr">
         <is>
-          <t>Eclipse - City Centre</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H76" s="8" t="inlineStr">
@@ -22650,7 +22646,9 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I76" s="8" t="n"/>
+      <c r="I76" s="8" t="n">
+        <v>641</v>
+      </c>
       <c r="J76" s="8" t="n"/>
       <c r="K76" s="8" t="n"/>
       <c r="L76" s="8" t="n"/>
@@ -22662,12 +22660,12 @@
       <c r="P76" s="8" t="n"/>
       <c r="Q76" s="8" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="R76" s="8" t="inlineStr">
         <is>
-          <t>Ocean, Clifton</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S76" s="9" t="inlineStr"/>
@@ -22684,7 +22682,7 @@
       <c r="V76" s="7" t="inlineStr"/>
       <c r="W76" s="8" t="inlineStr">
         <is>
-          <t>638ecbe81729048ffda61524ca9b06c4a208ce7b</t>
+          <t>d23eb397c84a723416c257acf4e25973ede40bc5</t>
         </is>
       </c>
     </row>
@@ -22698,7 +22696,7 @@
         </is>
       </c>
       <c r="C77" s="17" t="n">
-        <v>2085</v>
+        <v>2185</v>
       </c>
       <c r="D77" s="8" t="n">
         <v>2</v>
@@ -22713,7 +22711,7 @@
       </c>
       <c r="G77" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H77" s="8" t="inlineStr">
@@ -22722,7 +22720,7 @@
         </is>
       </c>
       <c r="I77" s="8" t="n">
-        <v>705</v>
+        <v>721</v>
       </c>
       <c r="J77" s="8" t="n"/>
       <c r="K77" s="8" t="n"/>
@@ -22735,12 +22733,12 @@
       <c r="P77" s="8" t="n"/>
       <c r="Q77" s="8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="R77" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S77" s="9" t="inlineStr"/>
@@ -22757,7 +22755,7 @@
       <c r="V77" s="7" t="inlineStr"/>
       <c r="W77" s="8" t="inlineStr">
         <is>
-          <t>16c89eb9a4cdeb57ddb3fd1201b7084ea2f3c007</t>
+          <t>6446e0c7d9c4f21f9eb6239caeeeee0599a68101</t>
         </is>
       </c>
     </row>
@@ -22771,7 +22769,7 @@
         </is>
       </c>
       <c r="C78" s="17" t="n">
-        <v>1615</v>
+        <v>1565</v>
       </c>
       <c r="D78" s="8" t="n">
         <v>1</v>
@@ -22795,7 +22793,7 @@
         </is>
       </c>
       <c r="I78" s="8" t="n">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="J78" s="8" t="n"/>
       <c r="K78" s="8" t="n"/>
@@ -22808,7 +22806,7 @@
       <c r="P78" s="8" t="n"/>
       <c r="Q78" s="8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="R78" s="8" t="inlineStr">
@@ -22830,7 +22828,7 @@
       <c r="V78" s="7" t="inlineStr"/>
       <c r="W78" s="8" t="inlineStr">
         <is>
-          <t>cd57661c8d996d20c5c1c7c34b12787f40073ec9</t>
+          <t>34d9877a23c82be120784d9dd55c23c17584c91a</t>
         </is>
       </c>
     </row>
@@ -22844,13 +22842,13 @@
         </is>
       </c>
       <c r="C79" s="17" t="n">
-        <v>2065</v>
+        <v>2100</v>
       </c>
       <c r="D79" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E79" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F79" s="8" t="inlineStr">
         <is>
@@ -22859,7 +22857,7 @@
       </c>
       <c r="G79" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>The Three Kings Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H79" s="8" t="inlineStr">
@@ -22867,9 +22865,7 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I79" s="8" t="n">
-        <v>641</v>
-      </c>
+      <c r="I79" s="8" t="n"/>
       <c r="J79" s="8" t="n"/>
       <c r="K79" s="8" t="n"/>
       <c r="L79" s="8" t="n"/>
@@ -22881,12 +22877,12 @@
       <c r="P79" s="8" t="n"/>
       <c r="Q79" s="8" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="R79" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S79" s="9" t="inlineStr"/>
@@ -22903,7 +22899,7 @@
       <c r="V79" s="7" t="inlineStr"/>
       <c r="W79" s="8" t="inlineStr">
         <is>
-          <t>d23eb397c84a723416c257acf4e25973ede40bc5</t>
+          <t>954007c82f6f3a495c465b72c9a1c44c0c84713e</t>
         </is>
       </c>
     </row>
@@ -22917,13 +22913,13 @@
         </is>
       </c>
       <c r="C80" s="17" t="n">
-        <v>2185</v>
+        <v>1660</v>
       </c>
       <c r="D80" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E80" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F80" s="8" t="inlineStr">
         <is>
@@ -22941,20 +22937,22 @@
         </is>
       </c>
       <c r="I80" s="8" t="n">
-        <v>721</v>
+        <v>486</v>
       </c>
       <c r="J80" s="8" t="n"/>
       <c r="K80" s="8" t="n"/>
       <c r="L80" s="8" t="n"/>
       <c r="M80" s="8" t="n"/>
-      <c r="N80" s="8" t="n"/>
+      <c r="N80" s="8" t="n">
+        <v>21504</v>
+      </c>
       <c r="O80" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P80" s="8" t="n"/>
       <c r="Q80" s="8" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R80" s="8" t="inlineStr">
@@ -22976,7 +22974,7 @@
       <c r="V80" s="7" t="inlineStr"/>
       <c r="W80" s="8" t="inlineStr">
         <is>
-          <t>6446e0c7d9c4f21f9eb6239caeeeee0599a68101</t>
+          <t>c2c660e4e8cefc047b4bc72bf19b48ce9ef7ec99</t>
         </is>
       </c>
     </row>
@@ -22990,13 +22988,13 @@
         </is>
       </c>
       <c r="C81" s="17" t="n">
-        <v>1565</v>
+        <v>2175</v>
       </c>
       <c r="D81" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E81" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F81" s="8" t="inlineStr">
         <is>
@@ -23005,7 +23003,7 @@
       </c>
       <c r="G81" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H81" s="8" t="inlineStr">
@@ -23014,25 +23012,27 @@
         </is>
       </c>
       <c r="I81" s="8" t="n">
-        <v>484</v>
+        <v>814</v>
       </c>
       <c r="J81" s="8" t="n"/>
       <c r="K81" s="8" t="n"/>
       <c r="L81" s="8" t="n"/>
       <c r="M81" s="8" t="n"/>
-      <c r="N81" s="8" t="n"/>
+      <c r="N81" s="8" t="n">
+        <v>21504</v>
+      </c>
       <c r="O81" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P81" s="8" t="n"/>
       <c r="Q81" s="8" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="R81" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S81" s="9" t="inlineStr"/>
@@ -23049,7 +23049,7 @@
       <c r="V81" s="7" t="inlineStr"/>
       <c r="W81" s="8" t="inlineStr">
         <is>
-          <t>34d9877a23c82be120784d9dd55c23c17584c91a</t>
+          <t>83406f05c9aded812a566cc6806036dda0d45fc0</t>
         </is>
       </c>
     </row>
@@ -23063,13 +23063,13 @@
         </is>
       </c>
       <c r="C82" s="17" t="n">
-        <v>2100</v>
+        <v>2115</v>
       </c>
       <c r="D82" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E82" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F82" s="8" t="inlineStr">
         <is>
@@ -23078,7 +23078,7 @@
       </c>
       <c r="G82" s="9" t="inlineStr">
         <is>
-          <t>The Three Kings Court, Bristol, BS1</t>
+          <t>Glasshouse Square Bristol BS1</t>
         </is>
       </c>
       <c r="H82" s="8" t="inlineStr">
@@ -23086,24 +23086,28 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I82" s="8" t="n"/>
+      <c r="I82" s="8" t="n">
+        <v>823</v>
+      </c>
       <c r="J82" s="8" t="n"/>
       <c r="K82" s="8" t="n"/>
       <c r="L82" s="8" t="n"/>
       <c r="M82" s="8" t="n"/>
-      <c r="N82" s="8" t="n"/>
+      <c r="N82" s="8" t="n">
+        <v>20820</v>
+      </c>
       <c r="O82" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P82" s="8" t="n"/>
       <c r="Q82" s="8" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="R82" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S82" s="9" t="inlineStr"/>
@@ -23120,7 +23124,7 @@
       <c r="V82" s="7" t="inlineStr"/>
       <c r="W82" s="8" t="inlineStr">
         <is>
-          <t>954007c82f6f3a495c465b72c9a1c44c0c84713e</t>
+          <t>0b78c6e29d96ae73c643d0d50d50949797b02893</t>
         </is>
       </c>
     </row>
@@ -23173,7 +23177,7 @@
       <c r="P83" s="8" t="n"/>
       <c r="Q83" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="R83" s="8" t="inlineStr">
@@ -23195,7 +23199,7 @@
       <c r="V83" s="7" t="inlineStr"/>
       <c r="W83" s="8" t="inlineStr">
         <is>
-          <t>c2c660e4e8cefc047b4bc72bf19b48ce9ef7ec99</t>
+          <t>c798c669d03fa2e42fd418ff0916de022d3380ad</t>
         </is>
       </c>
     </row>
@@ -23209,7 +23213,7 @@
         </is>
       </c>
       <c r="C84" s="17" t="n">
-        <v>2175</v>
+        <v>1915</v>
       </c>
       <c r="D84" s="8" t="n">
         <v>2</v>
@@ -23233,14 +23237,14 @@
         </is>
       </c>
       <c r="I84" s="8" t="n">
-        <v>814</v>
+        <v>746</v>
       </c>
       <c r="J84" s="8" t="n"/>
       <c r="K84" s="8" t="n"/>
       <c r="L84" s="8" t="n"/>
       <c r="M84" s="8" t="n"/>
       <c r="N84" s="8" t="n">
-        <v>21504</v>
+        <v>21680</v>
       </c>
       <c r="O84" s="8" t="n">
         <v>0</v>
@@ -23248,7 +23252,7 @@
       <c r="P84" s="8" t="n"/>
       <c r="Q84" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="R84" s="8" t="inlineStr">
@@ -23270,7 +23274,7 @@
       <c r="V84" s="7" t="inlineStr"/>
       <c r="W84" s="8" t="inlineStr">
         <is>
-          <t>83406f05c9aded812a566cc6806036dda0d45fc0</t>
+          <t>36797023cff0095f1bf764fa2f176d5595124854</t>
         </is>
       </c>
     </row>
@@ -23284,10 +23288,10 @@
         </is>
       </c>
       <c r="C85" s="17" t="n">
-        <v>2115</v>
+        <v>2450</v>
       </c>
       <c r="D85" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E85" s="8" t="n">
         <v>2</v>
@@ -23299,7 +23303,7 @@
       </c>
       <c r="G85" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square Bristol BS1</t>
+          <t>The Herbert Ashman Building, Bristol, BS1</t>
         </is>
       </c>
       <c r="H85" s="8" t="inlineStr">
@@ -23307,15 +23311,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I85" s="8" t="n">
-        <v>823</v>
-      </c>
+      <c r="I85" s="8" t="n"/>
       <c r="J85" s="8" t="n"/>
       <c r="K85" s="8" t="n"/>
       <c r="L85" s="8" t="n"/>
       <c r="M85" s="8" t="n"/>
       <c r="N85" s="8" t="n">
-        <v>20820</v>
+        <v>21788</v>
       </c>
       <c r="O85" s="8" t="n">
         <v>0</v>
@@ -23323,12 +23325,12 @@
       <c r="P85" s="8" t="n"/>
       <c r="Q85" s="8" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R85" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S85" s="9" t="inlineStr"/>
@@ -23345,7 +23347,7 @@
       <c r="V85" s="7" t="inlineStr"/>
       <c r="W85" s="8" t="inlineStr">
         <is>
-          <t>0b78c6e29d96ae73c643d0d50d50949797b02893</t>
+          <t>4cd4fdc09f26b6316c31aa22f38853db44d1ea9a</t>
         </is>
       </c>
     </row>
@@ -23359,7 +23361,7 @@
         </is>
       </c>
       <c r="C86" s="17" t="n">
-        <v>1660</v>
+        <v>1250</v>
       </c>
       <c r="D86" s="8" t="n">
         <v>1</v>
@@ -23374,7 +23376,7 @@
       </c>
       <c r="G86" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Victoria Street, Bristol, BS1 6DR</t>
         </is>
       </c>
       <c r="H86" s="8" t="inlineStr">
@@ -23382,15 +23384,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I86" s="8" t="n">
-        <v>486</v>
-      </c>
+      <c r="I86" s="8" t="n"/>
       <c r="J86" s="8" t="n"/>
       <c r="K86" s="8" t="n"/>
       <c r="L86" s="8" t="n"/>
       <c r="M86" s="8" t="n"/>
       <c r="N86" s="8" t="n">
-        <v>21504</v>
+        <v>21160</v>
       </c>
       <c r="O86" s="8" t="n">
         <v>0</v>
@@ -23398,12 +23398,12 @@
       <c r="P86" s="8" t="n"/>
       <c r="Q86" s="8" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R86" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Visum, Nationwide</t>
         </is>
       </c>
       <c r="S86" s="9" t="inlineStr"/>
@@ -23420,7 +23420,7 @@
       <c r="V86" s="7" t="inlineStr"/>
       <c r="W86" s="8" t="inlineStr">
         <is>
-          <t>c798c669d03fa2e42fd418ff0916de022d3380ad</t>
+          <t>78fe8e0511ccc37f104368075238c845f57d7864</t>
         </is>
       </c>
     </row>
@@ -23434,13 +23434,13 @@
         </is>
       </c>
       <c r="C87" s="17" t="n">
-        <v>1915</v>
+        <v>1999</v>
       </c>
       <c r="D87" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E87" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F87" s="8" t="inlineStr">
         <is>
@@ -23449,7 +23449,7 @@
       </c>
       <c r="G87" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Swann House, Bristol, BS1</t>
         </is>
       </c>
       <c r="H87" s="8" t="inlineStr">
@@ -23457,15 +23457,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I87" s="8" t="n">
-        <v>746</v>
-      </c>
+      <c r="I87" s="8" t="n"/>
       <c r="J87" s="8" t="n"/>
       <c r="K87" s="8" t="n"/>
       <c r="L87" s="8" t="n"/>
       <c r="M87" s="8" t="n"/>
       <c r="N87" s="8" t="n">
-        <v>21680</v>
+        <v>20800</v>
       </c>
       <c r="O87" s="8" t="n">
         <v>0</v>
@@ -23473,12 +23471,12 @@
       <c r="P87" s="8" t="n"/>
       <c r="Q87" s="8" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R87" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S87" s="9" t="inlineStr"/>
@@ -23495,7 +23493,7 @@
       <c r="V87" s="7" t="inlineStr"/>
       <c r="W87" s="8" t="inlineStr">
         <is>
-          <t>36797023cff0095f1bf764fa2f176d5595124854</t>
+          <t>5cec67aa8ba885c4c8f85e47d3354d187da9d897</t>
         </is>
       </c>
     </row>
@@ -23509,13 +23507,13 @@
         </is>
       </c>
       <c r="C88" s="17" t="n">
-        <v>2450</v>
+        <v>1670</v>
       </c>
       <c r="D88" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E88" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F88" s="8" t="inlineStr">
         <is>
@@ -23524,7 +23522,7 @@
       </c>
       <c r="G88" s="9" t="inlineStr">
         <is>
-          <t>The Herbert Ashman Building, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H88" s="8" t="inlineStr">
@@ -23532,13 +23530,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I88" s="8" t="n"/>
+      <c r="I88" s="8" t="n">
+        <v>485</v>
+      </c>
       <c r="J88" s="8" t="n"/>
       <c r="K88" s="8" t="n"/>
       <c r="L88" s="8" t="n"/>
       <c r="M88" s="8" t="n"/>
       <c r="N88" s="8" t="n">
-        <v>21788</v>
+        <v>21504</v>
       </c>
       <c r="O88" s="8" t="n">
         <v>0</v>
@@ -23546,12 +23546,12 @@
       <c r="P88" s="8" t="n"/>
       <c r="Q88" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R88" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S88" s="9" t="inlineStr"/>
@@ -23568,7 +23568,7 @@
       <c r="V88" s="7" t="inlineStr"/>
       <c r="W88" s="8" t="inlineStr">
         <is>
-          <t>4cd4fdc09f26b6316c31aa22f38853db44d1ea9a</t>
+          <t>73f3509a6c69eef7af4c6b9ff0dc69b97478c20a</t>
         </is>
       </c>
     </row>
@@ -23582,13 +23582,13 @@
         </is>
       </c>
       <c r="C89" s="17" t="n">
-        <v>1700</v>
+        <v>1645</v>
       </c>
       <c r="D89" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E89" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F89" s="8" t="inlineStr">
         <is>
@@ -23597,7 +23597,7 @@
       </c>
       <c r="G89" s="9" t="inlineStr">
         <is>
-          <t>The Crescent</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H89" s="8" t="inlineStr">
@@ -23605,13 +23605,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I89" s="8" t="n"/>
+      <c r="I89" s="8" t="n">
+        <v>517</v>
+      </c>
       <c r="J89" s="8" t="n"/>
       <c r="K89" s="8" t="n"/>
       <c r="L89" s="8" t="n"/>
       <c r="M89" s="8" t="n"/>
       <c r="N89" s="8" t="n">
-        <v>16368</v>
+        <v>20820</v>
       </c>
       <c r="O89" s="8" t="n">
         <v>0</v>
@@ -23619,12 +23621,12 @@
       <c r="P89" s="8" t="n"/>
       <c r="Q89" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R89" s="8" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S89" s="9" t="inlineStr"/>
@@ -23641,7 +23643,7 @@
       <c r="V89" s="7" t="inlineStr"/>
       <c r="W89" s="8" t="inlineStr">
         <is>
-          <t>8a8446c119238f7a042580aed1922ef6cfd79ae2</t>
+          <t>4efcb79ae710a68f5f272a2f9030937499117f9d</t>
         </is>
       </c>
     </row>
@@ -23655,13 +23657,13 @@
         </is>
       </c>
       <c r="C90" s="17" t="n">
-        <v>1250</v>
+        <v>2120</v>
       </c>
       <c r="D90" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E90" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F90" s="8" t="inlineStr">
         <is>
@@ -23670,7 +23672,7 @@
       </c>
       <c r="G90" s="9" t="inlineStr">
         <is>
-          <t>Victoria Street, Bristol, BS1 6DR</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H90" s="8" t="inlineStr">
@@ -23678,13 +23680,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I90" s="8" t="n"/>
+      <c r="I90" s="8" t="n">
+        <v>705</v>
+      </c>
       <c r="J90" s="8" t="n"/>
       <c r="K90" s="8" t="n"/>
       <c r="L90" s="8" t="n"/>
       <c r="M90" s="8" t="n"/>
       <c r="N90" s="8" t="n">
-        <v>21160</v>
+        <v>20820</v>
       </c>
       <c r="O90" s="8" t="n">
         <v>0</v>
@@ -23692,12 +23696,12 @@
       <c r="P90" s="8" t="n"/>
       <c r="Q90" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="R90" s="8" t="inlineStr">
         <is>
-          <t>Visum, Nationwide</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S90" s="9" t="inlineStr"/>
@@ -23714,7 +23718,7 @@
       <c r="V90" s="7" t="inlineStr"/>
       <c r="W90" s="8" t="inlineStr">
         <is>
-          <t>78fe8e0511ccc37f104368075238c845f57d7864</t>
+          <t>c5c1741357dfce3547bdab7d4d5a0e7602846192</t>
         </is>
       </c>
     </row>
@@ -23728,10 +23732,10 @@
         </is>
       </c>
       <c r="C91" s="17" t="n">
-        <v>1999</v>
+        <v>1645</v>
       </c>
       <c r="D91" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E91" s="8" t="n">
         <v>1</v>
@@ -23743,7 +23747,7 @@
       </c>
       <c r="G91" s="9" t="inlineStr">
         <is>
-          <t>Swann House, Bristol, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H91" s="8" t="inlineStr">
@@ -23751,13 +23755,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I91" s="8" t="n"/>
+      <c r="I91" s="8" t="n">
+        <v>571</v>
+      </c>
       <c r="J91" s="8" t="n"/>
       <c r="K91" s="8" t="n"/>
       <c r="L91" s="8" t="n"/>
       <c r="M91" s="8" t="n"/>
       <c r="N91" s="8" t="n">
-        <v>20800</v>
+        <v>20820</v>
       </c>
       <c r="O91" s="8" t="n">
         <v>0</v>
@@ -23765,12 +23771,12 @@
       <c r="P91" s="8" t="n"/>
       <c r="Q91" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="R91" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S91" s="9" t="inlineStr"/>
@@ -23787,7 +23793,7 @@
       <c r="V91" s="7" t="inlineStr"/>
       <c r="W91" s="8" t="inlineStr">
         <is>
-          <t>5cec67aa8ba885c4c8f85e47d3354d187da9d897</t>
+          <t>487e67b2d6680ebaabfcc49d4d33e21cb65cca6d</t>
         </is>
       </c>
     </row>
@@ -23801,10 +23807,10 @@
         </is>
       </c>
       <c r="C92" s="17" t="n">
-        <v>1670</v>
+        <v>1600</v>
       </c>
       <c r="D92" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E92" s="8" t="n">
         <v>1</v>
@@ -23816,23 +23822,21 @@
       </c>
       <c r="G92" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Stapleton Road, Bristol, BS5</t>
         </is>
       </c>
       <c r="H92" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I92" s="8" t="n">
-        <v>485</v>
-      </c>
+          <t>BS5</t>
+        </is>
+      </c>
+      <c r="I92" s="8" t="n"/>
       <c r="J92" s="8" t="n"/>
       <c r="K92" s="8" t="n"/>
       <c r="L92" s="8" t="n"/>
       <c r="M92" s="8" t="n"/>
       <c r="N92" s="8" t="n">
-        <v>21504</v>
+        <v>19576</v>
       </c>
       <c r="O92" s="8" t="n">
         <v>0</v>
@@ -23840,12 +23844,12 @@
       <c r="P92" s="8" t="n"/>
       <c r="Q92" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="R92" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S92" s="9" t="inlineStr"/>
@@ -23862,7 +23866,7 @@
       <c r="V92" s="7" t="inlineStr"/>
       <c r="W92" s="8" t="inlineStr">
         <is>
-          <t>73f3509a6c69eef7af4c6b9ff0dc69b97478c20a</t>
+          <t>41184aca0a094a13f0cf944554fa6ab5b6f9b761</t>
         </is>
       </c>
     </row>
@@ -23876,13 +23880,13 @@
         </is>
       </c>
       <c r="C93" s="17" t="n">
-        <v>1645</v>
+        <v>1550</v>
       </c>
       <c r="D93" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E93" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F93" s="8" t="inlineStr">
         <is>
@@ -23891,7 +23895,7 @@
       </c>
       <c r="G93" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>City Centre, Waverley House, BS1 5LW</t>
         </is>
       </c>
       <c r="H93" s="8" t="inlineStr">
@@ -23900,14 +23904,14 @@
         </is>
       </c>
       <c r="I93" s="8" t="n">
-        <v>517</v>
+        <v>775</v>
       </c>
       <c r="J93" s="8" t="n"/>
       <c r="K93" s="8" t="n"/>
       <c r="L93" s="8" t="n"/>
       <c r="M93" s="8" t="n"/>
       <c r="N93" s="8" t="n">
-        <v>20820</v>
+        <v>17744</v>
       </c>
       <c r="O93" s="8" t="n">
         <v>0</v>
@@ -23915,12 +23919,12 @@
       <c r="P93" s="8" t="n"/>
       <c r="Q93" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="R93" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>The Bristol Residential Letting Co, Clifton</t>
         </is>
       </c>
       <c r="S93" s="9" t="inlineStr"/>
@@ -23937,7 +23941,7 @@
       <c r="V93" s="7" t="inlineStr"/>
       <c r="W93" s="8" t="inlineStr">
         <is>
-          <t>4efcb79ae710a68f5f272a2f9030937499117f9d</t>
+          <t>ac4ae9e8b18bae38c431398f0f633dd1691dd454</t>
         </is>
       </c>
     </row>
@@ -23951,7 +23955,7 @@
         </is>
       </c>
       <c r="C94" s="17" t="n">
-        <v>2120</v>
+        <v>2125</v>
       </c>
       <c r="D94" s="8" t="n">
         <v>2</v>
@@ -23990,7 +23994,7 @@
       <c r="P94" s="8" t="n"/>
       <c r="Q94" s="8" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="R94" s="8" t="inlineStr">
@@ -24012,7 +24016,7 @@
       <c r="V94" s="7" t="inlineStr"/>
       <c r="W94" s="8" t="inlineStr">
         <is>
-          <t>c5c1741357dfce3547bdab7d4d5a0e7602846192</t>
+          <t>98852e60433cf90995df068fb3ceec727903a8f0</t>
         </is>
       </c>
     </row>
@@ -24026,7 +24030,7 @@
         </is>
       </c>
       <c r="C95" s="17" t="n">
-        <v>1645</v>
+        <v>1580</v>
       </c>
       <c r="D95" s="8" t="n">
         <v>1</v>
@@ -24041,7 +24045,7 @@
       </c>
       <c r="G95" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H95" s="8" t="inlineStr">
@@ -24050,14 +24054,14 @@
         </is>
       </c>
       <c r="I95" s="8" t="n">
-        <v>571</v>
+        <v>486</v>
       </c>
       <c r="J95" s="8" t="n"/>
       <c r="K95" s="8" t="n"/>
       <c r="L95" s="8" t="n"/>
       <c r="M95" s="8" t="n"/>
       <c r="N95" s="8" t="n">
-        <v>20820</v>
+        <v>21504</v>
       </c>
       <c r="O95" s="8" t="n">
         <v>0</v>
@@ -24065,12 +24069,12 @@
       <c r="P95" s="8" t="n"/>
       <c r="Q95" s="8" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="R95" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S95" s="9" t="inlineStr"/>
@@ -24087,7 +24091,7 @@
       <c r="V95" s="7" t="inlineStr"/>
       <c r="W95" s="8" t="inlineStr">
         <is>
-          <t>487e67b2d6680ebaabfcc49d4d33e21cb65cca6d</t>
+          <t>75f9f4931bb794ff7a8be9528691bace351a0d13</t>
         </is>
       </c>
     </row>
@@ -24101,10 +24105,10 @@
         </is>
       </c>
       <c r="C96" s="17" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="D96" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E96" s="8" t="n">
         <v>1</v>
@@ -24116,21 +24120,23 @@
       </c>
       <c r="G96" s="9" t="inlineStr">
         <is>
-          <t>Stapleton Road, Bristol, BS5</t>
+          <t>Bedminster, Regent House, BS3 1FT</t>
         </is>
       </c>
       <c r="H96" s="8" t="inlineStr">
         <is>
-          <t>BS5</t>
-        </is>
-      </c>
-      <c r="I96" s="8" t="n"/>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I96" s="8" t="n">
+        <v>527</v>
+      </c>
       <c r="J96" s="8" t="n"/>
       <c r="K96" s="8" t="n"/>
       <c r="L96" s="8" t="n"/>
       <c r="M96" s="8" t="n"/>
       <c r="N96" s="8" t="n">
-        <v>19576</v>
+        <v>13548</v>
       </c>
       <c r="O96" s="8" t="n">
         <v>0</v>
@@ -24138,12 +24144,12 @@
       <c r="P96" s="8" t="n"/>
       <c r="Q96" s="8" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="R96" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S96" s="9" t="inlineStr"/>
@@ -24160,7 +24166,7 @@
       <c r="V96" s="7" t="inlineStr"/>
       <c r="W96" s="8" t="inlineStr">
         <is>
-          <t>41184aca0a094a13f0cf944554fa6ab5b6f9b761</t>
+          <t>b5574d3457f97017e231a45d57df860c0d54fe3d</t>
         </is>
       </c>
     </row>
@@ -24174,13 +24180,13 @@
         </is>
       </c>
       <c r="C97" s="17" t="n">
-        <v>1550</v>
+        <v>1350</v>
       </c>
       <c r="D97" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E97" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F97" s="8" t="inlineStr">
         <is>
@@ -24189,7 +24195,7 @@
       </c>
       <c r="G97" s="9" t="inlineStr">
         <is>
-          <t>City Centre, Waverley House, BS1 5LW</t>
+          <t>Baldwin Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H97" s="8" t="inlineStr">
@@ -24198,14 +24204,14 @@
         </is>
       </c>
       <c r="I97" s="8" t="n">
-        <v>775</v>
+        <v>413</v>
       </c>
       <c r="J97" s="8" t="n"/>
       <c r="K97" s="8" t="n"/>
       <c r="L97" s="8" t="n"/>
       <c r="M97" s="8" t="n"/>
       <c r="N97" s="8" t="n">
-        <v>17744</v>
+        <v>21148</v>
       </c>
       <c r="O97" s="8" t="n">
         <v>0</v>
@@ -24218,7 +24224,7 @@
       </c>
       <c r="R97" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Clifton</t>
+          <t>Savills Lettings, Clifton</t>
         </is>
       </c>
       <c r="S97" s="9" t="inlineStr"/>
@@ -24235,7 +24241,7 @@
       <c r="V97" s="7" t="inlineStr"/>
       <c r="W97" s="8" t="inlineStr">
         <is>
-          <t>ac4ae9e8b18bae38c431398f0f633dd1691dd454</t>
+          <t>ca58d4891f705dc219b7ca74ef59637a2959afb0</t>
         </is>
       </c>
     </row>
@@ -24249,13 +24255,13 @@
         </is>
       </c>
       <c r="C98" s="17" t="n">
-        <v>2125</v>
+        <v>1620</v>
       </c>
       <c r="D98" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E98" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F98" s="8" t="inlineStr">
         <is>
@@ -24273,7 +24279,7 @@
         </is>
       </c>
       <c r="I98" s="8" t="n">
-        <v>705</v>
+        <v>494</v>
       </c>
       <c r="J98" s="8" t="n"/>
       <c r="K98" s="8" t="n"/>
@@ -24310,7 +24316,7 @@
       <c r="V98" s="7" t="inlineStr"/>
       <c r="W98" s="8" t="inlineStr">
         <is>
-          <t>98852e60433cf90995df068fb3ceec727903a8f0</t>
+          <t>b9cdcc0c4daa02ab2447615be3746df090f8a759</t>
         </is>
       </c>
     </row>
@@ -24324,13 +24330,13 @@
         </is>
       </c>
       <c r="C99" s="17" t="n">
-        <v>1580</v>
+        <v>2110</v>
       </c>
       <c r="D99" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E99" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F99" s="8" t="inlineStr">
         <is>
@@ -24348,15 +24354,13 @@
         </is>
       </c>
       <c r="I99" s="8" t="n">
-        <v>486</v>
+        <v>722</v>
       </c>
       <c r="J99" s="8" t="n"/>
       <c r="K99" s="8" t="n"/>
       <c r="L99" s="8" t="n"/>
       <c r="M99" s="8" t="n"/>
-      <c r="N99" s="8" t="n">
-        <v>21504</v>
-      </c>
+      <c r="N99" s="8" t="n"/>
       <c r="O99" s="8" t="n">
         <v>0</v>
       </c>
@@ -24385,7 +24389,7 @@
       <c r="V99" s="7" t="inlineStr"/>
       <c r="W99" s="8" t="inlineStr">
         <is>
-          <t>75f9f4931bb794ff7a8be9528691bace351a0d13</t>
+          <t>1fc314f1a5b51f6a42142e88d789000861f8e441</t>
         </is>
       </c>
     </row>
@@ -24399,13 +24403,13 @@
         </is>
       </c>
       <c r="C100" s="17" t="n">
-        <v>1500</v>
+        <v>2075</v>
       </c>
       <c r="D100" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E100" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F100" s="8" t="inlineStr">
         <is>
@@ -24414,23 +24418,23 @@
       </c>
       <c r="G100" s="9" t="inlineStr">
         <is>
-          <t>Bedminster, Regent House, BS3 1FT</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H100" s="8" t="inlineStr">
         <is>
-          <t>BS3</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I100" s="8" t="n">
-        <v>527</v>
+        <v>673</v>
       </c>
       <c r="J100" s="8" t="n"/>
       <c r="K100" s="8" t="n"/>
       <c r="L100" s="8" t="n"/>
       <c r="M100" s="8" t="n"/>
       <c r="N100" s="8" t="n">
-        <v>13548</v>
+        <v>20820</v>
       </c>
       <c r="O100" s="8" t="n">
         <v>0</v>
@@ -24438,12 +24442,12 @@
       <c r="P100" s="8" t="n"/>
       <c r="Q100" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="R100" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S100" s="9" t="inlineStr"/>
@@ -24460,7 +24464,7 @@
       <c r="V100" s="7" t="inlineStr"/>
       <c r="W100" s="8" t="inlineStr">
         <is>
-          <t>b5574d3457f97017e231a45d57df860c0d54fe3d</t>
+          <t>8c622e84bc80db890ad79fd8aced6eff3e7b71c5</t>
         </is>
       </c>
     </row>
@@ -24474,7 +24478,7 @@
         </is>
       </c>
       <c r="C101" s="17" t="n">
-        <v>1350</v>
+        <v>1645</v>
       </c>
       <c r="D101" s="8" t="n">
         <v>1</v>
@@ -24489,7 +24493,7 @@
       </c>
       <c r="G101" s="9" t="inlineStr">
         <is>
-          <t>Baldwin Street, Bristol, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H101" s="8" t="inlineStr">
@@ -24498,14 +24502,14 @@
         </is>
       </c>
       <c r="I101" s="8" t="n">
-        <v>413</v>
+        <v>546</v>
       </c>
       <c r="J101" s="8" t="n"/>
       <c r="K101" s="8" t="n"/>
       <c r="L101" s="8" t="n"/>
       <c r="M101" s="8" t="n"/>
       <c r="N101" s="8" t="n">
-        <v>21148</v>
+        <v>20820</v>
       </c>
       <c r="O101" s="8" t="n">
         <v>0</v>
@@ -24513,12 +24517,12 @@
       <c r="P101" s="8" t="n"/>
       <c r="Q101" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="R101" s="8" t="inlineStr">
         <is>
-          <t>Savills Lettings, Clifton</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S101" s="9" t="inlineStr"/>
@@ -24535,7 +24539,7 @@
       <c r="V101" s="7" t="inlineStr"/>
       <c r="W101" s="8" t="inlineStr">
         <is>
-          <t>ca58d4891f705dc219b7ca74ef59637a2959afb0</t>
+          <t>97965ef25d5084c20bb1be86ca100fd603557ea5</t>
         </is>
       </c>
     </row>
@@ -24549,10 +24553,10 @@
         </is>
       </c>
       <c r="C102" s="17" t="n">
-        <v>1620</v>
+        <v>1600</v>
       </c>
       <c r="D102" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E102" s="8" t="n">
         <v>1</v>
@@ -24564,23 +24568,21 @@
       </c>
       <c r="G102" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Portland Square, City Centre</t>
         </is>
       </c>
       <c r="H102" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I102" s="8" t="n">
-        <v>494</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I102" s="8" t="n"/>
       <c r="J102" s="8" t="n"/>
       <c r="K102" s="8" t="n"/>
       <c r="L102" s="8" t="n"/>
       <c r="M102" s="8" t="n"/>
       <c r="N102" s="8" t="n">
-        <v>20820</v>
+        <v>21392</v>
       </c>
       <c r="O102" s="8" t="n">
         <v>0</v>
@@ -24588,12 +24590,12 @@
       <c r="P102" s="8" t="n"/>
       <c r="Q102" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="R102" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S102" s="9" t="inlineStr"/>
@@ -24610,7 +24612,7 @@
       <c r="V102" s="7" t="inlineStr"/>
       <c r="W102" s="8" t="inlineStr">
         <is>
-          <t>b9cdcc0c4daa02ab2447615be3746df090f8a759</t>
+          <t>5c6702e019e22ae6a63f958f13da168b2a7871d1</t>
         </is>
       </c>
     </row>
@@ -24624,13 +24626,13 @@
         </is>
       </c>
       <c r="C103" s="17" t="n">
-        <v>2110</v>
+        <v>1630</v>
       </c>
       <c r="D103" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E103" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F103" s="8" t="inlineStr">
         <is>
@@ -24648,20 +24650,22 @@
         </is>
       </c>
       <c r="I103" s="8" t="n">
-        <v>722</v>
+        <v>486</v>
       </c>
       <c r="J103" s="8" t="n"/>
       <c r="K103" s="8" t="n"/>
       <c r="L103" s="8" t="n"/>
       <c r="M103" s="8" t="n"/>
-      <c r="N103" s="8" t="n"/>
+      <c r="N103" s="8" t="n">
+        <v>21504</v>
+      </c>
       <c r="O103" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P103" s="8" t="n"/>
       <c r="Q103" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="R103" s="8" t="inlineStr">
@@ -24683,7 +24687,7 @@
       <c r="V103" s="7" t="inlineStr"/>
       <c r="W103" s="8" t="inlineStr">
         <is>
-          <t>1fc314f1a5b51f6a42142e88d789000861f8e441</t>
+          <t>0d149e26cf43428bfa175140c03d2088b6cd6bed</t>
         </is>
       </c>
     </row>
@@ -24697,13 +24701,13 @@
         </is>
       </c>
       <c r="C104" s="17" t="n">
-        <v>2075</v>
+        <v>2200</v>
       </c>
       <c r="D104" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E104" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F104" s="8" t="inlineStr">
         <is>
@@ -24712,23 +24716,21 @@
       </c>
       <c r="G104" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Castle Park View, Castle Street, Bristol</t>
         </is>
       </c>
       <c r="H104" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I104" s="8" t="n">
-        <v>673</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I104" s="8" t="n"/>
       <c r="J104" s="8" t="n"/>
       <c r="K104" s="8" t="n"/>
       <c r="L104" s="8" t="n"/>
       <c r="M104" s="8" t="n"/>
       <c r="N104" s="8" t="n">
-        <v>20820</v>
+        <v>21984</v>
       </c>
       <c r="O104" s="8" t="n">
         <v>0</v>
@@ -24736,12 +24738,12 @@
       <c r="P104" s="8" t="n"/>
       <c r="Q104" s="8" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="R104" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Savills Lettings, CPV</t>
         </is>
       </c>
       <c r="S104" s="9" t="inlineStr"/>
@@ -24758,7 +24760,7 @@
       <c r="V104" s="7" t="inlineStr"/>
       <c r="W104" s="8" t="inlineStr">
         <is>
-          <t>8c622e84bc80db890ad79fd8aced6eff3e7b71c5</t>
+          <t>406fab2577557efdd9382cee302acdc7a788c3d8</t>
         </is>
       </c>
     </row>
@@ -24772,10 +24774,10 @@
         </is>
       </c>
       <c r="C105" s="17" t="n">
-        <v>1645</v>
+        <v>1600</v>
       </c>
       <c r="D105" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E105" s="8" t="n">
         <v>1</v>
@@ -24787,23 +24789,23 @@
       </c>
       <c r="G105" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Waterloo Road, Midland Mews, BS2</t>
         </is>
       </c>
       <c r="H105" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I105" s="8" t="n">
-        <v>546</v>
+        <v>721</v>
       </c>
       <c r="J105" s="8" t="n"/>
       <c r="K105" s="8" t="n"/>
       <c r="L105" s="8" t="n"/>
       <c r="M105" s="8" t="n"/>
       <c r="N105" s="8" t="n">
-        <v>20820</v>
+        <v>20856</v>
       </c>
       <c r="O105" s="8" t="n">
         <v>0</v>
@@ -24811,12 +24813,12 @@
       <c r="P105" s="8" t="n"/>
       <c r="Q105" s="8" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R105" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Acen Properties, Bristol</t>
         </is>
       </c>
       <c r="S105" s="9" t="inlineStr"/>
@@ -24833,7 +24835,7 @@
       <c r="V105" s="7" t="inlineStr"/>
       <c r="W105" s="8" t="inlineStr">
         <is>
-          <t>97965ef25d5084c20bb1be86ca100fd603557ea5</t>
+          <t>cf8a979c7c13e868d74a6828d64c93a46d2e7209</t>
         </is>
       </c>
     </row>
@@ -24847,13 +24849,13 @@
         </is>
       </c>
       <c r="C106" s="17" t="n">
-        <v>1600</v>
+        <v>2000</v>
       </c>
       <c r="D106" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E106" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F106" s="8" t="inlineStr">
         <is>
@@ -24862,34 +24864,34 @@
       </c>
       <c r="G106" s="9" t="inlineStr">
         <is>
-          <t>Portland Square, City Centre</t>
+          <t>Welsh Back, Bristol, BS1</t>
         </is>
       </c>
       <c r="H106" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I106" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I106" s="8" t="n">
+        <v>908</v>
+      </c>
       <c r="J106" s="8" t="n"/>
       <c r="K106" s="8" t="n"/>
       <c r="L106" s="8" t="n"/>
       <c r="M106" s="8" t="n"/>
-      <c r="N106" s="8" t="n">
-        <v>21392</v>
-      </c>
+      <c r="N106" s="8" t="n"/>
       <c r="O106" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P106" s="8" t="n"/>
       <c r="Q106" s="8" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="R106" s="8" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>Hello Neighbour, London</t>
         </is>
       </c>
       <c r="S106" s="9" t="inlineStr"/>
@@ -24906,7 +24908,7 @@
       <c r="V106" s="7" t="inlineStr"/>
       <c r="W106" s="8" t="inlineStr">
         <is>
-          <t>5c6702e019e22ae6a63f958f13da168b2a7871d1</t>
+          <t>65ed2520fdf37e6dde4abe0097cc3edbbbeff957</t>
         </is>
       </c>
     </row>
@@ -24920,13 +24922,13 @@
         </is>
       </c>
       <c r="C107" s="17" t="n">
-        <v>1630</v>
+        <v>1700</v>
       </c>
       <c r="D107" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E107" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F107" s="8" t="inlineStr">
         <is>
@@ -24935,7 +24937,7 @@
       </c>
       <c r="G107" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>The Crescent</t>
         </is>
       </c>
       <c r="H107" s="8" t="inlineStr">
@@ -24943,15 +24945,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I107" s="8" t="n">
-        <v>486</v>
-      </c>
+      <c r="I107" s="8" t="n"/>
       <c r="J107" s="8" t="n"/>
       <c r="K107" s="8" t="n"/>
       <c r="L107" s="8" t="n"/>
       <c r="M107" s="8" t="n"/>
       <c r="N107" s="8" t="n">
-        <v>21504</v>
+        <v>16368</v>
       </c>
       <c r="O107" s="8" t="n">
         <v>0</v>
@@ -24959,12 +24959,12 @@
       <c r="P107" s="8" t="n"/>
       <c r="Q107" s="8" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R107" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S107" s="9" t="inlineStr"/>
@@ -24981,7 +24981,7 @@
       <c r="V107" s="7" t="inlineStr"/>
       <c r="W107" s="8" t="inlineStr">
         <is>
-          <t>0d149e26cf43428bfa175140c03d2088b6cd6bed</t>
+          <t>8a8446c119238f7a042580aed1922ef6cfd79ae2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
House search data from run 45
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -17297,13 +17297,13 @@
         </is>
       </c>
       <c r="C6" s="17" t="n">
-        <v>1655</v>
+        <v>2500</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
@@ -17312,23 +17312,21 @@
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>712 Rosewood New Kingsley Road, Bristol, BS2</t>
+          <t>Electricity House, Colston Avenue, BS1</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I6" s="8" t="n">
-        <v>547</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="n"/>
       <c r="J6" s="8" t="n"/>
       <c r="K6" s="8" t="n"/>
       <c r="L6" s="8" t="n"/>
       <c r="M6" s="8" t="n"/>
       <c r="N6" s="8" t="n">
-        <v>20800</v>
+        <v>21876</v>
       </c>
       <c r="O6" s="8" t="n">
         <v>0</v>
@@ -17341,7 +17339,7 @@
       </c>
       <c r="R6" s="8" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S6" s="9" t="inlineStr">
@@ -17362,7 +17360,7 @@
       <c r="V6" s="7" t="inlineStr"/>
       <c r="W6" s="8" t="inlineStr">
         <is>
-          <t>1f8489d296d842011bdf7a2ca1f952e6b948c3d3</t>
+          <t>b2e83643f78121776465be4134c64aa64f0141c3</t>
         </is>
       </c>
     </row>
@@ -17376,13 +17374,13 @@
         </is>
       </c>
       <c r="C7" s="17" t="n">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
@@ -17391,7 +17389,7 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>Electricity House, Colston Avenue, BS1</t>
+          <t>The Crescent, Hannover Quay, BS1</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr">
@@ -17405,7 +17403,7 @@
       <c r="L7" s="8" t="n"/>
       <c r="M7" s="8" t="n"/>
       <c r="N7" s="8" t="n">
-        <v>21876</v>
+        <v>16232</v>
       </c>
       <c r="O7" s="8" t="n">
         <v>0</v>
@@ -17439,7 +17437,7 @@
       <c r="V7" s="7" t="inlineStr"/>
       <c r="W7" s="8" t="inlineStr">
         <is>
-          <t>b2e83643f78121776465be4134c64aa64f0141c3</t>
+          <t>6bb8673e1999d1e987f72fb4720f3d7b072fa45e</t>
         </is>
       </c>
     </row>
@@ -17453,13 +17451,13 @@
         </is>
       </c>
       <c r="C8" s="17" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
@@ -17468,7 +17466,7 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>The Crescent, Hannover Quay, BS1</t>
+          <t>Horizon - City Centre</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
@@ -17482,7 +17480,7 @@
       <c r="L8" s="8" t="n"/>
       <c r="M8" s="8" t="n"/>
       <c r="N8" s="8" t="n">
-        <v>16232</v>
+        <v>22020</v>
       </c>
       <c r="O8" s="8" t="n">
         <v>0</v>
@@ -17490,17 +17488,17 @@
       <c r="P8" s="8" t="n"/>
       <c r="Q8" s="8" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R8" s="8" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>Ocean, Clifton</t>
         </is>
       </c>
       <c r="S8" s="9" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T8" s="12" t="inlineStr">
@@ -17516,7 +17514,7 @@
       <c r="V8" s="7" t="inlineStr"/>
       <c r="W8" s="8" t="inlineStr">
         <is>
-          <t>6bb8673e1999d1e987f72fb4720f3d7b072fa45e</t>
+          <t>8988913a4580793e64d3ae8351174e2d71317d16</t>
         </is>
       </c>
     </row>
@@ -17530,13 +17528,13 @@
         </is>
       </c>
       <c r="C9" s="17" t="n">
-        <v>2000</v>
+        <v>1400</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
@@ -17545,7 +17543,7 @@
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>Horizon - City Centre</t>
+          <t>The Crescent, Harbourside, Bristol</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
@@ -17559,7 +17557,7 @@
       <c r="L9" s="8" t="n"/>
       <c r="M9" s="8" t="n"/>
       <c r="N9" s="8" t="n">
-        <v>22020</v>
+        <v>16368</v>
       </c>
       <c r="O9" s="8" t="n">
         <v>0</v>
@@ -17572,12 +17570,12 @@
       </c>
       <c r="R9" s="8" t="inlineStr">
         <is>
-          <t>Ocean, Clifton</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S9" s="9" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T9" s="12" t="inlineStr">
@@ -17593,7 +17591,7 @@
       <c r="V9" s="7" t="inlineStr"/>
       <c r="W9" s="8" t="inlineStr">
         <is>
-          <t>8988913a4580793e64d3ae8351174e2d71317d16</t>
+          <t>59af10441dff618517a35c62d6a67a8485c2f2fa</t>
         </is>
       </c>
     </row>
@@ -17607,13 +17605,13 @@
         </is>
       </c>
       <c r="C10" s="17" t="n">
-        <v>1400</v>
+        <v>1900</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
@@ -17622,7 +17620,7 @@
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>The Crescent, Harbourside, Bristol</t>
+          <t>51.02 - St James Barton</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
@@ -17636,7 +17634,7 @@
       <c r="L10" s="8" t="n"/>
       <c r="M10" s="8" t="n"/>
       <c r="N10" s="8" t="n">
-        <v>16368</v>
+        <v>22132</v>
       </c>
       <c r="O10" s="8" t="n">
         <v>0</v>
@@ -17649,7 +17647,7 @@
       </c>
       <c r="R10" s="8" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>Ocean, Clifton</t>
         </is>
       </c>
       <c r="S10" s="9" t="inlineStr">
@@ -17670,7 +17668,7 @@
       <c r="V10" s="7" t="inlineStr"/>
       <c r="W10" s="8" t="inlineStr">
         <is>
-          <t>59af10441dff618517a35c62d6a67a8485c2f2fa</t>
+          <t>1d421f07eb2d142471d3e293f8cb751813656c56</t>
         </is>
       </c>
     </row>
@@ -17684,7 +17682,7 @@
         </is>
       </c>
       <c r="C11" s="17" t="n">
-        <v>1900</v>
+        <v>2000</v>
       </c>
       <c r="D11" s="8" t="n">
         <v>2</v>
@@ -17699,7 +17697,7 @@
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>51.02 - St James Barton</t>
+          <t>Caledonian Road, Bristol, BS1</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr">
@@ -17713,7 +17711,7 @@
       <c r="L11" s="8" t="n"/>
       <c r="M11" s="8" t="n"/>
       <c r="N11" s="8" t="n">
-        <v>22132</v>
+        <v>14632</v>
       </c>
       <c r="O11" s="8" t="n">
         <v>0</v>
@@ -17721,12 +17719,12 @@
       <c r="P11" s="8" t="n"/>
       <c r="Q11" s="8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R11" s="8" t="inlineStr">
         <is>
-          <t>Ocean, Clifton</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S11" s="9" t="inlineStr">
@@ -17747,7 +17745,7 @@
       <c r="V11" s="7" t="inlineStr"/>
       <c r="W11" s="8" t="inlineStr">
         <is>
-          <t>1d421f07eb2d142471d3e293f8cb751813656c56</t>
+          <t>9a270cf54e31627246aef21daa26a60bb5f977ad</t>
         </is>
       </c>
     </row>
@@ -17761,7 +17759,7 @@
         </is>
       </c>
       <c r="C12" s="17" t="n">
-        <v>2000</v>
+        <v>1650</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>2</v>
@@ -17776,12 +17774,12 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>Caledonian Road, Bristol, BS1</t>
+          <t>Sweetman Place, Bristol, BS2</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I12" s="8" t="n"/>
@@ -17790,7 +17788,7 @@
       <c r="L12" s="8" t="n"/>
       <c r="M12" s="8" t="n"/>
       <c r="N12" s="8" t="n">
-        <v>14632</v>
+        <v>20416</v>
       </c>
       <c r="O12" s="8" t="n">
         <v>0</v>
@@ -17803,7 +17801,7 @@
       </c>
       <c r="R12" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Andrews Letting and Management, Clifton</t>
         </is>
       </c>
       <c r="S12" s="9" t="inlineStr">
@@ -17824,7 +17822,7 @@
       <c r="V12" s="7" t="inlineStr"/>
       <c r="W12" s="8" t="inlineStr">
         <is>
-          <t>9a270cf54e31627246aef21daa26a60bb5f977ad</t>
+          <t>54fa42ef8d0349a295f45392644c43dec3321c5b</t>
         </is>
       </c>
     </row>
@@ -17838,7 +17836,7 @@
         </is>
       </c>
       <c r="C13" s="17" t="n">
-        <v>1650</v>
+        <v>2000</v>
       </c>
       <c r="D13" s="8" t="n">
         <v>2</v>
@@ -17853,21 +17851,23 @@
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>Sweetman Place, Bristol, BS2</t>
+          <t>Chatfield House, Marsh Street, Bristol</t>
         </is>
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I13" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="n">
+        <v>705</v>
+      </c>
       <c r="J13" s="8" t="n"/>
       <c r="K13" s="8" t="n"/>
       <c r="L13" s="8" t="n"/>
       <c r="M13" s="8" t="n"/>
       <c r="N13" s="8" t="n">
-        <v>20416</v>
+        <v>20932</v>
       </c>
       <c r="O13" s="8" t="n">
         <v>0</v>
@@ -17875,12 +17875,12 @@
       <c r="P13" s="8" t="n"/>
       <c r="Q13" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="R13" s="8" t="inlineStr">
         <is>
-          <t>Andrews Letting and Management, Clifton</t>
+          <t>Mariana Real Estate, London</t>
         </is>
       </c>
       <c r="S13" s="9" t="inlineStr">
@@ -17901,7 +17901,7 @@
       <c r="V13" s="7" t="inlineStr"/>
       <c r="W13" s="8" t="inlineStr">
         <is>
-          <t>54fa42ef8d0349a295f45392644c43dec3321c5b</t>
+          <t>be4fdd18faf2bcf44d894da42e9c874b7d868fbe</t>
         </is>
       </c>
     </row>
@@ -17915,13 +17915,13 @@
         </is>
       </c>
       <c r="C14" s="17" t="n">
-        <v>2000</v>
+        <v>1600</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
@@ -17930,7 +17930,7 @@
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>Chatfield House, Marsh Street, Bristol</t>
+          <t>St. Stephens Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
@@ -17938,15 +17938,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I14" s="8" t="n">
-        <v>705</v>
-      </c>
+      <c r="I14" s="8" t="n"/>
       <c r="J14" s="8" t="n"/>
       <c r="K14" s="8" t="n"/>
       <c r="L14" s="8" t="n"/>
       <c r="M14" s="8" t="n"/>
       <c r="N14" s="8" t="n">
-        <v>20932</v>
+        <v>21428</v>
       </c>
       <c r="O14" s="8" t="n">
         <v>0</v>
@@ -17959,7 +17957,7 @@
       </c>
       <c r="R14" s="8" t="inlineStr">
         <is>
-          <t>Mariana Real Estate, London</t>
+          <t>Romans, Clifton</t>
         </is>
       </c>
       <c r="S14" s="9" t="inlineStr">
@@ -17980,7 +17978,7 @@
       <c r="V14" s="7" t="inlineStr"/>
       <c r="W14" s="8" t="inlineStr">
         <is>
-          <t>be4fdd18faf2bcf44d894da42e9c874b7d868fbe</t>
+          <t>cd770dd603af2e6f4f23a72c9685c7468c731a6d</t>
         </is>
       </c>
     </row>
@@ -17994,10 +17992,10 @@
         </is>
       </c>
       <c r="C15" s="17" t="n">
-        <v>1600</v>
+        <v>1200</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E15" s="8" t="n">
         <v>1</v>
@@ -18009,12 +18007,12 @@
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>St. Stephens Street, Bristol, BS1</t>
+          <t>Union Road, Bristol BS2 0FN</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I15" s="8" t="n"/>
@@ -18023,7 +18021,7 @@
       <c r="L15" s="8" t="n"/>
       <c r="M15" s="8" t="n"/>
       <c r="N15" s="8" t="n">
-        <v>21428</v>
+        <v>20144</v>
       </c>
       <c r="O15" s="8" t="n">
         <v>0</v>
@@ -18031,12 +18029,12 @@
       <c r="P15" s="8" t="n"/>
       <c r="Q15" s="8" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="R15" s="8" t="inlineStr">
         <is>
-          <t>Romans, Clifton</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S15" s="9" t="inlineStr">
@@ -18057,7 +18055,7 @@
       <c r="V15" s="7" t="inlineStr"/>
       <c r="W15" s="8" t="inlineStr">
         <is>
-          <t>cd770dd603af2e6f4f23a72c9685c7468c731a6d</t>
+          <t>2b2295e0c22bd50658835eb43d2eb433f6d1cd1b</t>
         </is>
       </c>
     </row>
@@ -18071,13 +18069,13 @@
         </is>
       </c>
       <c r="C16" s="17" t="n">
-        <v>1200</v>
+        <v>2850</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
@@ -18086,21 +18084,23 @@
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>Union Road, Bristol BS2 0FN</t>
+          <t>Capricorn Place, Hotwells, BS8</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I16" s="8" t="n"/>
+          <t>BS8</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="n">
+        <v>1615</v>
+      </c>
       <c r="J16" s="8" t="n"/>
       <c r="K16" s="8" t="n"/>
       <c r="L16" s="8" t="n"/>
       <c r="M16" s="8" t="n"/>
       <c r="N16" s="8" t="n">
-        <v>20144</v>
+        <v>15104</v>
       </c>
       <c r="O16" s="8" t="n">
         <v>0</v>
@@ -18113,7 +18113,7 @@
       </c>
       <c r="R16" s="8" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Sarah Kenny Residential Lettings, Bristol</t>
         </is>
       </c>
       <c r="S16" s="9" t="inlineStr">
@@ -18134,7 +18134,7 @@
       <c r="V16" s="7" t="inlineStr"/>
       <c r="W16" s="8" t="inlineStr">
         <is>
-          <t>2b2295e0c22bd50658835eb43d2eb433f6d1cd1b</t>
+          <t>11c93771b8963d430763c083c575b56042e71418</t>
         </is>
       </c>
     </row>
@@ -18148,7 +18148,7 @@
         </is>
       </c>
       <c r="C17" s="17" t="n">
-        <v>2850</v>
+        <v>2050</v>
       </c>
       <c r="D17" s="8" t="n">
         <v>2</v>
@@ -18163,23 +18163,23 @@
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>Capricorn Place, Hotwells, BS8</t>
+          <t>421 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>BS8</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I17" s="8" t="n">
-        <v>1615</v>
+        <v>802</v>
       </c>
       <c r="J17" s="8" t="n"/>
       <c r="K17" s="8" t="n"/>
       <c r="L17" s="8" t="n"/>
       <c r="M17" s="8" t="n"/>
       <c r="N17" s="8" t="n">
-        <v>15104</v>
+        <v>20800</v>
       </c>
       <c r="O17" s="8" t="n">
         <v>0</v>
@@ -18187,12 +18187,12 @@
       <c r="P17" s="8" t="n"/>
       <c r="Q17" s="8" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="R17" s="8" t="inlineStr">
         <is>
-          <t>Sarah Kenny Residential Lettings, Bristol</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S17" s="9" t="inlineStr">
@@ -18213,7 +18213,7 @@
       <c r="V17" s="7" t="inlineStr"/>
       <c r="W17" s="8" t="inlineStr">
         <is>
-          <t>11c93771b8963d430763c083c575b56042e71418</t>
+          <t>b7d86b41b199aaf040e0304048e519e961081fd2</t>
         </is>
       </c>
     </row>
@@ -18227,14 +18227,12 @@
         </is>
       </c>
       <c r="C18" s="17" t="n">
-        <v>1665</v>
+        <v>2100</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="8" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="E18" s="8" t="n"/>
       <c r="F18" s="8" t="inlineStr">
         <is>
           <t>flat</t>
@@ -18242,7 +18240,7 @@
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>425 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>526 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
@@ -18251,7 +18249,7 @@
         </is>
       </c>
       <c r="I18" s="8" t="n">
-        <v>548</v>
+        <v>800</v>
       </c>
       <c r="J18" s="8" t="n"/>
       <c r="K18" s="8" t="n"/>
@@ -18292,7 +18290,7 @@
       <c r="V18" s="7" t="inlineStr"/>
       <c r="W18" s="8" t="inlineStr">
         <is>
-          <t>c340a6dabc6dc987b590f784ea30b8d4f34f9e0c</t>
+          <t>74d41470c07849b906ad0a12b07a1745551d8e6f</t>
         </is>
       </c>
     </row>
@@ -18306,7 +18304,7 @@
         </is>
       </c>
       <c r="C19" s="17" t="n">
-        <v>2050</v>
+        <v>2120</v>
       </c>
       <c r="D19" s="8" t="n">
         <v>2</v>
@@ -18321,7 +18319,7 @@
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>421 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>522 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
@@ -18330,7 +18328,7 @@
         </is>
       </c>
       <c r="I19" s="8" t="n">
-        <v>802</v>
+        <v>799</v>
       </c>
       <c r="J19" s="8" t="n"/>
       <c r="K19" s="8" t="n"/>
@@ -18371,7 +18369,7 @@
       <c r="V19" s="7" t="inlineStr"/>
       <c r="W19" s="8" t="inlineStr">
         <is>
-          <t>b7d86b41b199aaf040e0304048e519e961081fd2</t>
+          <t>4a3dbf2b76e61d3a02d3b62cb6a5a56affeadff0</t>
         </is>
       </c>
     </row>
@@ -18385,12 +18383,14 @@
         </is>
       </c>
       <c r="C20" s="17" t="n">
-        <v>2100</v>
+        <v>2150</v>
       </c>
       <c r="D20" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="E20" s="8" t="n"/>
+      <c r="E20" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
           <t>flat</t>
@@ -18398,7 +18398,7 @@
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>526 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>802 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H20" s="8" t="inlineStr">
@@ -18407,7 +18407,7 @@
         </is>
       </c>
       <c r="I20" s="8" t="n">
-        <v>800</v>
+        <v>809</v>
       </c>
       <c r="J20" s="8" t="n"/>
       <c r="K20" s="8" t="n"/>
@@ -18448,7 +18448,7 @@
       <c r="V20" s="7" t="inlineStr"/>
       <c r="W20" s="8" t="inlineStr">
         <is>
-          <t>74d41470c07849b906ad0a12b07a1745551d8e6f</t>
+          <t>fcdcdd1da915be6f6b065ad9cbeea66062d00301</t>
         </is>
       </c>
     </row>
@@ -18462,10 +18462,10 @@
         </is>
       </c>
       <c r="C21" s="17" t="n">
-        <v>2120</v>
+        <v>2830</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E21" s="8" t="n">
         <v>2</v>
@@ -18477,7 +18477,7 @@
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>522 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>315 Dovetail, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
@@ -18486,7 +18486,7 @@
         </is>
       </c>
       <c r="I21" s="8" t="n">
-        <v>799</v>
+        <v>1120</v>
       </c>
       <c r="J21" s="8" t="n"/>
       <c r="K21" s="8" t="n"/>
@@ -18501,7 +18501,7 @@
       <c r="P21" s="8" t="n"/>
       <c r="Q21" s="8" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="R21" s="8" t="inlineStr">
@@ -18527,7 +18527,7 @@
       <c r="V21" s="7" t="inlineStr"/>
       <c r="W21" s="8" t="inlineStr">
         <is>
-          <t>4a3dbf2b76e61d3a02d3b62cb6a5a56affeadff0</t>
+          <t>e4f6deef9389498e73820b4056b013ac2b6ff363</t>
         </is>
       </c>
     </row>
@@ -18541,13 +18541,13 @@
         </is>
       </c>
       <c r="C22" s="17" t="n">
-        <v>2150</v>
+        <v>1950</v>
       </c>
       <c r="D22" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
@@ -18556,23 +18556,23 @@
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>802 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>Cheltenham House, 24A Clare Street, Bristol</t>
         </is>
       </c>
       <c r="H22" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I22" s="8" t="n">
-        <v>809</v>
+        <v>668</v>
       </c>
       <c r="J22" s="8" t="n"/>
       <c r="K22" s="8" t="n"/>
       <c r="L22" s="8" t="n"/>
       <c r="M22" s="8" t="n"/>
       <c r="N22" s="8" t="n">
-        <v>20800</v>
+        <v>21044</v>
       </c>
       <c r="O22" s="8" t="n">
         <v>0</v>
@@ -18580,12 +18580,12 @@
       <c r="P22" s="8" t="n"/>
       <c r="Q22" s="8" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="R22" s="8" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>Mariana Real Estate, London</t>
         </is>
       </c>
       <c r="S22" s="9" t="inlineStr">
@@ -18606,7 +18606,7 @@
       <c r="V22" s="7" t="inlineStr"/>
       <c r="W22" s="8" t="inlineStr">
         <is>
-          <t>fcdcdd1da915be6f6b065ad9cbeea66062d00301</t>
+          <t>9bdc8fdc90a88180cfd80c66940dfb5055afd30b</t>
         </is>
       </c>
     </row>
@@ -18620,13 +18620,13 @@
         </is>
       </c>
       <c r="C23" s="17" t="n">
-        <v>2830</v>
+        <v>1500</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
@@ -18635,23 +18635,21 @@
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>315 Dovetail, New Kingsley Road, Bristol, BS2</t>
+          <t>The Metropolitan, Redcliff Backs, BRISTOL, BS1</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I23" s="8" t="n">
-        <v>1120</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="n"/>
       <c r="J23" s="8" t="n"/>
       <c r="K23" s="8" t="n"/>
       <c r="L23" s="8" t="n"/>
       <c r="M23" s="8" t="n"/>
       <c r="N23" s="8" t="n">
-        <v>20800</v>
+        <v>20320</v>
       </c>
       <c r="O23" s="8" t="n">
         <v>0</v>
@@ -18659,12 +18657,12 @@
       <c r="P23" s="8" t="n"/>
       <c r="Q23" s="8" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="R23" s="8" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>Andrews Letting and Management, Clifton</t>
         </is>
       </c>
       <c r="S23" s="9" t="inlineStr">
@@ -18685,7 +18683,7 @@
       <c r="V23" s="7" t="inlineStr"/>
       <c r="W23" s="8" t="inlineStr">
         <is>
-          <t>e4f6deef9389498e73820b4056b013ac2b6ff363</t>
+          <t>48f0639d9505de53304e65370c31dc2b91415006</t>
         </is>
       </c>
     </row>
@@ -18699,10 +18697,10 @@
         </is>
       </c>
       <c r="C24" s="17" t="n">
-        <v>1950</v>
+        <v>1050</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E24" s="8" t="n">
         <v>1</v>
@@ -18714,7 +18712,7 @@
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>Cheltenham House, 24A Clare Street, Bristol</t>
+          <t>Caslon Court, Somerset Street, Redcliffe, Bristol, BS1</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr">
@@ -18722,15 +18720,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I24" s="8" t="n">
-        <v>668</v>
-      </c>
+      <c r="I24" s="8" t="n"/>
       <c r="J24" s="8" t="n"/>
       <c r="K24" s="8" t="n"/>
       <c r="L24" s="8" t="n"/>
       <c r="M24" s="8" t="n"/>
       <c r="N24" s="8" t="n">
-        <v>21044</v>
+        <v>18424</v>
       </c>
       <c r="O24" s="8" t="n">
         <v>0</v>
@@ -18738,12 +18734,12 @@
       <c r="P24" s="8" t="n"/>
       <c r="Q24" s="8" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="R24" s="8" t="inlineStr">
         <is>
-          <t>Mariana Real Estate, London</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S24" s="9" t="inlineStr">
@@ -18764,7 +18760,7 @@
       <c r="V24" s="7" t="inlineStr"/>
       <c r="W24" s="8" t="inlineStr">
         <is>
-          <t>9bdc8fdc90a88180cfd80c66940dfb5055afd30b</t>
+          <t>7183e0bb70a3ff586aa635a21825e38757f1f13d</t>
         </is>
       </c>
     </row>
@@ -18778,10 +18774,10 @@
         </is>
       </c>
       <c r="C25" s="17" t="n">
-        <v>1500</v>
+        <v>1450</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E25" s="8" t="n">
         <v>1</v>
@@ -18793,7 +18789,7 @@
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>The Metropolitan, Redcliff Backs, BRISTOL, BS1</t>
+          <t>The Crescent, Bristol, BS1</t>
         </is>
       </c>
       <c r="H25" s="8" t="inlineStr">
@@ -18807,7 +18803,7 @@
       <c r="L25" s="8" t="n"/>
       <c r="M25" s="8" t="n"/>
       <c r="N25" s="8" t="n">
-        <v>20320</v>
+        <v>16792</v>
       </c>
       <c r="O25" s="8" t="n">
         <v>0</v>
@@ -18815,12 +18811,12 @@
       <c r="P25" s="8" t="n"/>
       <c r="Q25" s="8" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="R25" s="8" t="inlineStr">
         <is>
-          <t>Andrews Letting and Management, Clifton</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S25" s="9" t="inlineStr">
@@ -18841,7 +18837,7 @@
       <c r="V25" s="7" t="inlineStr"/>
       <c r="W25" s="8" t="inlineStr">
         <is>
-          <t>48f0639d9505de53304e65370c31dc2b91415006</t>
+          <t>d447d1158e90abd2c82eb7828f8a98e7f5fbe2bd</t>
         </is>
       </c>
     </row>
@@ -18855,13 +18851,13 @@
         </is>
       </c>
       <c r="C26" s="17" t="n">
-        <v>1050</v>
+        <v>1650</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
@@ -18870,7 +18866,7 @@
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>Caslon Court, Somerset Street, Redcliffe, Bristol, BS1</t>
+          <t>Harbourside, Purifier House, BS1 5AU</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">
@@ -18878,13 +18874,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I26" s="8" t="n"/>
+      <c r="I26" s="8" t="n">
+        <v>689</v>
+      </c>
       <c r="J26" s="8" t="n"/>
       <c r="K26" s="8" t="n"/>
       <c r="L26" s="8" t="n"/>
       <c r="M26" s="8" t="n"/>
       <c r="N26" s="8" t="n">
-        <v>18424</v>
+        <v>16240</v>
       </c>
       <c r="O26" s="8" t="n">
         <v>0</v>
@@ -18892,12 +18890,12 @@
       <c r="P26" s="8" t="n"/>
       <c r="Q26" s="8" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="R26" s="8" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>The Bristol Residential Letting Co, Clifton</t>
         </is>
       </c>
       <c r="S26" s="9" t="inlineStr">
@@ -18918,7 +18916,7 @@
       <c r="V26" s="7" t="inlineStr"/>
       <c r="W26" s="8" t="inlineStr">
         <is>
-          <t>7183e0bb70a3ff586aa635a21825e38757f1f13d</t>
+          <t>7ec8aa4d9388bb5e923c445c92ac24d6496094c5</t>
         </is>
       </c>
     </row>
@@ -18932,13 +18930,13 @@
         </is>
       </c>
       <c r="C27" s="17" t="n">
-        <v>1450</v>
+        <v>1900</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
@@ -18947,7 +18945,7 @@
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>The Crescent, Bristol, BS1</t>
+          <t>Wapping Wharf, Anchorage, BS1</t>
         </is>
       </c>
       <c r="H27" s="8" t="inlineStr">
@@ -18955,13 +18953,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I27" s="8" t="n"/>
+      <c r="I27" s="8" t="n">
+        <v>799</v>
+      </c>
       <c r="J27" s="8" t="n"/>
       <c r="K27" s="8" t="n"/>
       <c r="L27" s="8" t="n"/>
       <c r="M27" s="8" t="n"/>
       <c r="N27" s="8" t="n">
-        <v>16792</v>
+        <v>16416</v>
       </c>
       <c r="O27" s="8" t="n">
         <v>0</v>
@@ -18969,12 +18969,12 @@
       <c r="P27" s="8" t="n"/>
       <c r="Q27" s="8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="R27" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S27" s="9" t="inlineStr">
@@ -18995,7 +18995,7 @@
       <c r="V27" s="7" t="inlineStr"/>
       <c r="W27" s="8" t="inlineStr">
         <is>
-          <t>d447d1158e90abd2c82eb7828f8a98e7f5fbe2bd</t>
+          <t>6b74ba6dcca9cfc12cf5e5d10aaa942cfd63c0e6</t>
         </is>
       </c>
     </row>
@@ -19009,13 +19009,13 @@
         </is>
       </c>
       <c r="C28" s="17" t="n">
-        <v>1650</v>
+        <v>1225</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
@@ -19024,23 +19024,21 @@
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>Harbourside, Purifier House, BS1 5AU</t>
+          <t>New Walls, Totterdown, BS4</t>
         </is>
       </c>
       <c r="H28" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I28" s="8" t="n">
-        <v>689</v>
-      </c>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="n"/>
       <c r="J28" s="8" t="n"/>
       <c r="K28" s="8" t="n"/>
       <c r="L28" s="8" t="n"/>
       <c r="M28" s="8" t="n"/>
       <c r="N28" s="8" t="n">
-        <v>16240</v>
+        <v>8540</v>
       </c>
       <c r="O28" s="8" t="n">
         <v>0</v>
@@ -19053,7 +19051,7 @@
       </c>
       <c r="R28" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Clifton</t>
+          <t>Bristol Property Centre, Bristol</t>
         </is>
       </c>
       <c r="S28" s="9" t="inlineStr">
@@ -19074,7 +19072,7 @@
       <c r="V28" s="7" t="inlineStr"/>
       <c r="W28" s="8" t="inlineStr">
         <is>
-          <t>7ec8aa4d9388bb5e923c445c92ac24d6496094c5</t>
+          <t>ff7cade97c52dbe0ee822ce3951fd4f71c9b4146</t>
         </is>
       </c>
     </row>
@@ -19088,13 +19086,13 @@
         </is>
       </c>
       <c r="C29" s="17" t="n">
-        <v>1900</v>
+        <v>1680</v>
       </c>
       <c r="D29" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E29" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
@@ -19103,23 +19101,23 @@
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>Wapping Wharf, Anchorage, BS1</t>
+          <t>904 Dovetail, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H29" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I29" s="8" t="n">
-        <v>799</v>
+        <v>557</v>
       </c>
       <c r="J29" s="8" t="n"/>
       <c r="K29" s="8" t="n"/>
       <c r="L29" s="8" t="n"/>
       <c r="M29" s="8" t="n"/>
       <c r="N29" s="8" t="n">
-        <v>16416</v>
+        <v>20800</v>
       </c>
       <c r="O29" s="8" t="n">
         <v>0</v>
@@ -19132,7 +19130,7 @@
       </c>
       <c r="R29" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S29" s="9" t="inlineStr">
@@ -19153,7 +19151,7 @@
       <c r="V29" s="7" t="inlineStr"/>
       <c r="W29" s="8" t="inlineStr">
         <is>
-          <t>6b74ba6dcca9cfc12cf5e5d10aaa942cfd63c0e6</t>
+          <t>3d5fce4a62f2bd2b3bbd100f6bd7598155b266f2</t>
         </is>
       </c>
     </row>
@@ -19167,7 +19165,7 @@
         </is>
       </c>
       <c r="C30" s="17" t="n">
-        <v>1225</v>
+        <v>1733</v>
       </c>
       <c r="D30" s="8" t="n">
         <v>1</v>
@@ -19182,34 +19180,34 @@
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>New Walls, Totterdown, BS4</t>
+          <t>Cheltenham House, Clare Street, Bristol</t>
         </is>
       </c>
       <c r="H30" s="8" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I30" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="n">
+        <v>455</v>
+      </c>
       <c r="J30" s="8" t="n"/>
       <c r="K30" s="8" t="n"/>
       <c r="L30" s="8" t="n"/>
       <c r="M30" s="8" t="n"/>
-      <c r="N30" s="8" t="n">
-        <v>8540</v>
-      </c>
+      <c r="N30" s="8" t="n"/>
       <c r="O30" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P30" s="8" t="n"/>
       <c r="Q30" s="8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
-          <t>Bristol Property Centre, Bristol</t>
+          <t>Mariana Real Estate, London</t>
         </is>
       </c>
       <c r="S30" s="9" t="inlineStr">
@@ -19230,7 +19228,7 @@
       <c r="V30" s="7" t="inlineStr"/>
       <c r="W30" s="8" t="inlineStr">
         <is>
-          <t>ff7cade97c52dbe0ee822ce3951fd4f71c9b4146</t>
+          <t>10b717aabd38544480501915d97cf63dfbd0bcbd</t>
         </is>
       </c>
     </row>
@@ -19244,7 +19242,7 @@
         </is>
       </c>
       <c r="C31" s="17" t="n">
-        <v>1680</v>
+        <v>1715</v>
       </c>
       <c r="D31" s="8" t="n">
         <v>1</v>
@@ -19259,7 +19257,7 @@
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>904 Dovetail, New Kingsley Road, Bristol, BS2</t>
+          <t>1006 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H31" s="8" t="inlineStr">
@@ -19268,7 +19266,7 @@
         </is>
       </c>
       <c r="I31" s="8" t="n">
-        <v>557</v>
+        <v>547</v>
       </c>
       <c r="J31" s="8" t="n"/>
       <c r="K31" s="8" t="n"/>
@@ -19309,7 +19307,7 @@
       <c r="V31" s="7" t="inlineStr"/>
       <c r="W31" s="8" t="inlineStr">
         <is>
-          <t>3d5fce4a62f2bd2b3bbd100f6bd7598155b266f2</t>
+          <t>baed14f153217bbfa48df27148f4a5b45559a145</t>
         </is>
       </c>
     </row>
@@ -19323,14 +19321,12 @@
         </is>
       </c>
       <c r="C32" s="17" t="n">
-        <v>1733</v>
+        <v>1400</v>
       </c>
       <c r="D32" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="8" t="n">
-        <v>1</v>
-      </c>
+      <c r="E32" s="8" t="n"/>
       <c r="F32" s="8" t="inlineStr">
         <is>
           <t>flat</t>
@@ -19338,7 +19334,7 @@
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>Cheltenham House, Clare Street, Bristol</t>
+          <t>Millennium Promenade, Bristol, BS1</t>
         </is>
       </c>
       <c r="H32" s="8" t="inlineStr">
@@ -19346,26 +19342,26 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I32" s="8" t="n">
-        <v>455</v>
-      </c>
+      <c r="I32" s="8" t="n"/>
       <c r="J32" s="8" t="n"/>
       <c r="K32" s="8" t="n"/>
       <c r="L32" s="8" t="n"/>
       <c r="M32" s="8" t="n"/>
-      <c r="N32" s="8" t="n"/>
+      <c r="N32" s="8" t="n">
+        <v>16168</v>
+      </c>
       <c r="O32" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P32" s="8" t="n"/>
       <c r="Q32" s="8" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
-          <t>Mariana Real Estate, London</t>
+          <t>Phoenix Property Company, Bristol</t>
         </is>
       </c>
       <c r="S32" s="9" t="inlineStr">
@@ -19386,7 +19382,7 @@
       <c r="V32" s="7" t="inlineStr"/>
       <c r="W32" s="8" t="inlineStr">
         <is>
-          <t>10b717aabd38544480501915d97cf63dfbd0bcbd</t>
+          <t>5ec68f33756a2f8f7606ead5febd7f33ed18c280</t>
         </is>
       </c>
     </row>
@@ -19400,7 +19396,7 @@
         </is>
       </c>
       <c r="C33" s="17" t="n">
-        <v>1715</v>
+        <v>1655</v>
       </c>
       <c r="D33" s="8" t="n">
         <v>1</v>
@@ -19415,7 +19411,7 @@
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
-          <t>1006 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>712 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H33" s="8" t="inlineStr">
@@ -19439,7 +19435,7 @@
       <c r="P33" s="8" t="n"/>
       <c r="Q33" s="8" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="R33" s="8" t="inlineStr">
@@ -19465,7 +19461,7 @@
       <c r="V33" s="7" t="inlineStr"/>
       <c r="W33" s="8" t="inlineStr">
         <is>
-          <t>baed14f153217bbfa48df27148f4a5b45559a145</t>
+          <t>219bc0a98e52a6b4cd0d3939d181df307abb678d</t>
         </is>
       </c>
     </row>
@@ -19479,12 +19475,14 @@
         </is>
       </c>
       <c r="C34" s="17" t="n">
-        <v>1400</v>
+        <v>1665</v>
       </c>
       <c r="D34" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="E34" s="8" t="n"/>
+      <c r="E34" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
           <t>flat</t>
@@ -19492,21 +19490,23 @@
       </c>
       <c r="G34" s="9" t="inlineStr">
         <is>
-          <t>Millennium Promenade, Bristol, BS1</t>
+          <t>425 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H34" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I34" s="8" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="n">
+        <v>548</v>
+      </c>
       <c r="J34" s="8" t="n"/>
       <c r="K34" s="8" t="n"/>
       <c r="L34" s="8" t="n"/>
       <c r="M34" s="8" t="n"/>
       <c r="N34" s="8" t="n">
-        <v>16168</v>
+        <v>20800</v>
       </c>
       <c r="O34" s="8" t="n">
         <v>0</v>
@@ -19519,7 +19519,7 @@
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
-          <t>Phoenix Property Company, Bristol</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S34" s="9" t="inlineStr">
@@ -19540,7 +19540,7 @@
       <c r="V34" s="7" t="inlineStr"/>
       <c r="W34" s="8" t="inlineStr">
         <is>
-          <t>5ec68f33756a2f8f7606ead5febd7f33ed18c280</t>
+          <t>51bc0e8bb190437e4c5c4710bf40ee90758a79f0</t>
         </is>
       </c>
     </row>
@@ -19569,7 +19569,7 @@
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
-          <t>712 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>712 Rosewood New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H35" s="8" t="inlineStr">
@@ -19593,7 +19593,7 @@
       <c r="P35" s="8" t="n"/>
       <c r="Q35" s="8" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R35" s="8" t="inlineStr">
@@ -19619,7 +19619,7 @@
       <c r="V35" s="7" t="inlineStr"/>
       <c r="W35" s="8" t="inlineStr">
         <is>
-          <t>219bc0a98e52a6b4cd0d3939d181df307abb678d</t>
+          <t>1f8489d296d842011bdf7a2ca1f952e6b948c3d3</t>
         </is>
       </c>
     </row>
@@ -19672,7 +19672,7 @@
       <c r="P36" s="8" t="n"/>
       <c r="Q36" s="8" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="R36" s="8" t="inlineStr">
@@ -19698,7 +19698,7 @@
       <c r="V36" s="7" t="inlineStr"/>
       <c r="W36" s="8" t="inlineStr">
         <is>
-          <t>51bc0e8bb190437e4c5c4710bf40ee90758a79f0</t>
+          <t>c340a6dabc6dc987b590f784ea30b8d4f34f9e0c</t>
         </is>
       </c>
     </row>
@@ -24829,10 +24829,10 @@
         </is>
       </c>
       <c r="C104" s="17" t="n">
-        <v>1300</v>
+        <v>1675</v>
       </c>
       <c r="D104" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E104" s="8" t="n">
         <v>1</v>
@@ -24844,21 +24844,23 @@
       </c>
       <c r="G104" s="9" t="inlineStr">
         <is>
-          <t>Champion Court, City Centre, Bristol, BS2</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H104" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I104" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I104" s="8" t="n">
+        <v>486</v>
+      </c>
       <c r="J104" s="8" t="n"/>
       <c r="K104" s="8" t="n"/>
       <c r="L104" s="8" t="n"/>
       <c r="M104" s="8" t="n"/>
       <c r="N104" s="8" t="n">
-        <v>21484</v>
+        <v>21504</v>
       </c>
       <c r="O104" s="8" t="n">
         <v>0</v>
@@ -24866,12 +24868,12 @@
       <c r="P104" s="8" t="n"/>
       <c r="Q104" s="8" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="R104" s="8" t="inlineStr">
         <is>
-          <t>Taylors Lettings, Bedminster</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S104" s="9" t="inlineStr"/>
@@ -24888,7 +24890,7 @@
       <c r="V104" s="7" t="inlineStr"/>
       <c r="W104" s="8" t="inlineStr">
         <is>
-          <t>5864fa4083267aba7fb2c38a58e549510d3d67b7</t>
+          <t>e8a909f17ced8cb8f577e6a31c3521c3ba10f6df</t>
         </is>
       </c>
     </row>
@@ -24902,13 +24904,13 @@
         </is>
       </c>
       <c r="C105" s="17" t="n">
-        <v>1675</v>
+        <v>2100</v>
       </c>
       <c r="D105" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E105" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F105" s="8" t="inlineStr">
         <is>
@@ -24917,7 +24919,7 @@
       </c>
       <c r="G105" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H105" s="8" t="inlineStr">
@@ -24926,14 +24928,14 @@
         </is>
       </c>
       <c r="I105" s="8" t="n">
-        <v>486</v>
+        <v>685</v>
       </c>
       <c r="J105" s="8" t="n"/>
       <c r="K105" s="8" t="n"/>
       <c r="L105" s="8" t="n"/>
       <c r="M105" s="8" t="n"/>
       <c r="N105" s="8" t="n">
-        <v>21504</v>
+        <v>20856</v>
       </c>
       <c r="O105" s="8" t="n">
         <v>0</v>
@@ -24946,7 +24948,7 @@
       </c>
       <c r="R105" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S105" s="9" t="inlineStr"/>
@@ -24963,7 +24965,7 @@
       <c r="V105" s="7" t="inlineStr"/>
       <c r="W105" s="8" t="inlineStr">
         <is>
-          <t>e8a909f17ced8cb8f577e6a31c3521c3ba10f6df</t>
+          <t>ef7856e14dd97f4fc0c67b4d6b67b3700390662d</t>
         </is>
       </c>
     </row>
@@ -24977,13 +24979,13 @@
         </is>
       </c>
       <c r="C106" s="17" t="n">
-        <v>2100</v>
+        <v>1500</v>
       </c>
       <c r="D106" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E106" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F106" s="8" t="inlineStr">
         <is>
@@ -24992,7 +24994,7 @@
       </c>
       <c r="G106" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Flat 109, Invicta, Millennium Promenade, Bristol, Bristol, City of, BS1</t>
         </is>
       </c>
       <c r="H106" s="8" t="inlineStr">
@@ -25000,15 +25002,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I106" s="8" t="n">
-        <v>685</v>
-      </c>
+      <c r="I106" s="8" t="n"/>
       <c r="J106" s="8" t="n"/>
       <c r="K106" s="8" t="n"/>
       <c r="L106" s="8" t="n"/>
       <c r="M106" s="8" t="n"/>
       <c r="N106" s="8" t="n">
-        <v>20856</v>
+        <v>16168</v>
       </c>
       <c r="O106" s="8" t="n">
         <v>0</v>
@@ -25021,7 +25021,7 @@
       </c>
       <c r="R106" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>CJ Hole, Bishopston</t>
         </is>
       </c>
       <c r="S106" s="9" t="inlineStr"/>
@@ -25038,7 +25038,7 @@
       <c r="V106" s="7" t="inlineStr"/>
       <c r="W106" s="8" t="inlineStr">
         <is>
-          <t>ef7856e14dd97f4fc0c67b4d6b67b3700390662d</t>
+          <t>f987cb39e8da7d77742156cb9d1860ba1ec36a04</t>
         </is>
       </c>
     </row>
@@ -25052,7 +25052,7 @@
         </is>
       </c>
       <c r="C107" s="17" t="n">
-        <v>1500</v>
+        <v>1635</v>
       </c>
       <c r="D107" s="8" t="n">
         <v>1</v>
@@ -25067,7 +25067,7 @@
       </c>
       <c r="G107" s="9" t="inlineStr">
         <is>
-          <t>Flat 109, Invicta, Millennium Promenade, Bristol, Bristol, City of, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H107" s="8" t="inlineStr">
@@ -25075,13 +25075,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I107" s="8" t="n"/>
+      <c r="I107" s="8" t="n">
+        <v>494</v>
+      </c>
       <c r="J107" s="8" t="n"/>
       <c r="K107" s="8" t="n"/>
       <c r="L107" s="8" t="n"/>
       <c r="M107" s="8" t="n"/>
       <c r="N107" s="8" t="n">
-        <v>16168</v>
+        <v>20820</v>
       </c>
       <c r="O107" s="8" t="n">
         <v>0</v>
@@ -25094,7 +25096,7 @@
       </c>
       <c r="R107" s="8" t="inlineStr">
         <is>
-          <t>CJ Hole, Bishopston</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S107" s="9" t="inlineStr"/>
@@ -25111,7 +25113,7 @@
       <c r="V107" s="7" t="inlineStr"/>
       <c r="W107" s="8" t="inlineStr">
         <is>
-          <t>f987cb39e8da7d77742156cb9d1860ba1ec36a04</t>
+          <t>1707adbd47900a5a7010b3d0b6e3b1b5ba6ffb6d</t>
         </is>
       </c>
     </row>
@@ -25125,7 +25127,7 @@
         </is>
       </c>
       <c r="C108" s="17" t="n">
-        <v>1635</v>
+        <v>1650</v>
       </c>
       <c r="D108" s="8" t="n">
         <v>1</v>
@@ -25140,7 +25142,7 @@
       </c>
       <c r="G108" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H108" s="8" t="inlineStr">
@@ -25149,14 +25151,14 @@
         </is>
       </c>
       <c r="I108" s="8" t="n">
-        <v>494</v>
+        <v>486</v>
       </c>
       <c r="J108" s="8" t="n"/>
       <c r="K108" s="8" t="n"/>
       <c r="L108" s="8" t="n"/>
       <c r="M108" s="8" t="n"/>
       <c r="N108" s="8" t="n">
-        <v>20820</v>
+        <v>21504</v>
       </c>
       <c r="O108" s="8" t="n">
         <v>0</v>
@@ -25164,12 +25166,12 @@
       <c r="P108" s="8" t="n"/>
       <c r="Q108" s="8" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="R108" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S108" s="9" t="inlineStr"/>
@@ -25186,7 +25188,7 @@
       <c r="V108" s="7" t="inlineStr"/>
       <c r="W108" s="8" t="inlineStr">
         <is>
-          <t>1707adbd47900a5a7010b3d0b6e3b1b5ba6ffb6d</t>
+          <t>e26a5dedfb7c4bcd1308250a8955318f00994505</t>
         </is>
       </c>
     </row>
@@ -25200,13 +25202,13 @@
         </is>
       </c>
       <c r="C109" s="17" t="n">
-        <v>1650</v>
+        <v>2130</v>
       </c>
       <c r="D109" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E109" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F109" s="8" t="inlineStr">
         <is>
@@ -25215,7 +25217,7 @@
       </c>
       <c r="G109" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H109" s="8" t="inlineStr">
@@ -25224,14 +25226,14 @@
         </is>
       </c>
       <c r="I109" s="8" t="n">
-        <v>486</v>
+        <v>685</v>
       </c>
       <c r="J109" s="8" t="n"/>
       <c r="K109" s="8" t="n"/>
       <c r="L109" s="8" t="n"/>
       <c r="M109" s="8" t="n"/>
       <c r="N109" s="8" t="n">
-        <v>21504</v>
+        <v>20820</v>
       </c>
       <c r="O109" s="8" t="n">
         <v>0</v>
@@ -25244,7 +25246,7 @@
       </c>
       <c r="R109" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S109" s="9" t="inlineStr"/>
@@ -25261,7 +25263,7 @@
       <c r="V109" s="7" t="inlineStr"/>
       <c r="W109" s="8" t="inlineStr">
         <is>
-          <t>e26a5dedfb7c4bcd1308250a8955318f00994505</t>
+          <t>510968acc1d86247d0ff3178d6c87ca0cfe58973</t>
         </is>
       </c>
     </row>
@@ -25275,13 +25277,13 @@
         </is>
       </c>
       <c r="C110" s="17" t="n">
-        <v>2130</v>
+        <v>1645</v>
       </c>
       <c r="D110" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E110" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F110" s="8" t="inlineStr">
         <is>
@@ -25299,7 +25301,7 @@
         </is>
       </c>
       <c r="I110" s="8" t="n">
-        <v>685</v>
+        <v>488</v>
       </c>
       <c r="J110" s="8" t="n"/>
       <c r="K110" s="8" t="n"/>
@@ -25336,7 +25338,7 @@
       <c r="V110" s="7" t="inlineStr"/>
       <c r="W110" s="8" t="inlineStr">
         <is>
-          <t>510968acc1d86247d0ff3178d6c87ca0cfe58973</t>
+          <t>fe6eedf667721b56be5a770dfd447378831f3e52</t>
         </is>
       </c>
     </row>
@@ -25350,7 +25352,7 @@
         </is>
       </c>
       <c r="C111" s="17" t="n">
-        <v>1645</v>
+        <v>1250</v>
       </c>
       <c r="D111" s="8" t="n">
         <v>1</v>
@@ -25365,23 +25367,21 @@
       </c>
       <c r="G111" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hillgrove Street, Bristol, BS2</t>
         </is>
       </c>
       <c r="H111" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I111" s="8" t="n">
-        <v>488</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I111" s="8" t="n"/>
       <c r="J111" s="8" t="n"/>
       <c r="K111" s="8" t="n"/>
       <c r="L111" s="8" t="n"/>
       <c r="M111" s="8" t="n"/>
       <c r="N111" s="8" t="n">
-        <v>20820</v>
+        <v>21644</v>
       </c>
       <c r="O111" s="8" t="n">
         <v>0</v>
@@ -25394,7 +25394,7 @@
       </c>
       <c r="R111" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S111" s="9" t="inlineStr"/>
@@ -25411,7 +25411,7 @@
       <c r="V111" s="7" t="inlineStr"/>
       <c r="W111" s="8" t="inlineStr">
         <is>
-          <t>fe6eedf667721b56be5a770dfd447378831f3e52</t>
+          <t>0db27cfb877874271e6046a606b2268e3733f233</t>
         </is>
       </c>
     </row>
@@ -25425,27 +25425,27 @@
         </is>
       </c>
       <c r="C112" s="17" t="n">
-        <v>1250</v>
+        <v>2570</v>
       </c>
       <c r="D112" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E112" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F112" s="8" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G112" s="9" t="inlineStr">
         <is>
-          <t>Hillgrove Street, Bristol, BS2</t>
+          <t>Balmain Street, Totterdown, Bristol, BS4</t>
         </is>
       </c>
       <c r="H112" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS4</t>
         </is>
       </c>
       <c r="I112" s="8" t="n"/>
@@ -25454,7 +25454,7 @@
       <c r="L112" s="8" t="n"/>
       <c r="M112" s="8" t="n"/>
       <c r="N112" s="8" t="n">
-        <v>21644</v>
+        <v>5524</v>
       </c>
       <c r="O112" s="8" t="n">
         <v>0</v>
@@ -25467,7 +25467,7 @@
       </c>
       <c r="R112" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S112" s="9" t="inlineStr"/>
@@ -25484,7 +25484,7 @@
       <c r="V112" s="7" t="inlineStr"/>
       <c r="W112" s="8" t="inlineStr">
         <is>
-          <t>0db27cfb877874271e6046a606b2268e3733f233</t>
+          <t>dd411af39a083f886127138c0a969254da83858b</t>
         </is>
       </c>
     </row>
@@ -25498,27 +25498,27 @@
         </is>
       </c>
       <c r="C113" s="17" t="n">
-        <v>2570</v>
+        <v>2250</v>
       </c>
       <c r="D113" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E113" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F113" s="8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G113" s="9" t="inlineStr">
         <is>
-          <t>Balmain Street, Totterdown, Bristol, BS4</t>
+          <t>Eclipse, Bristol, BS1</t>
         </is>
       </c>
       <c r="H113" s="8" t="inlineStr">
         <is>
-          <t>BS4</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I113" s="8" t="n"/>
@@ -25527,7 +25527,7 @@
       <c r="L113" s="8" t="n"/>
       <c r="M113" s="8" t="n"/>
       <c r="N113" s="8" t="n">
-        <v>5524</v>
+        <v>22080</v>
       </c>
       <c r="O113" s="8" t="n">
         <v>0</v>
@@ -25540,7 +25540,7 @@
       </c>
       <c r="R113" s="8" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S113" s="9" t="inlineStr"/>
@@ -25557,7 +25557,7 @@
       <c r="V113" s="7" t="inlineStr"/>
       <c r="W113" s="8" t="inlineStr">
         <is>
-          <t>dd411af39a083f886127138c0a969254da83858b</t>
+          <t>dc210d0a40d826c0930a4e847048280bbe1d9b17</t>
         </is>
       </c>
     </row>
@@ -25571,7 +25571,7 @@
         </is>
       </c>
       <c r="C114" s="17" t="n">
-        <v>1600</v>
+        <v>1350</v>
       </c>
       <c r="D114" s="8" t="n">
         <v>1</v>
@@ -25586,12 +25586,12 @@
       </c>
       <c r="G114" s="9" t="inlineStr">
         <is>
-          <t>Hope Quay, Wapping Wharf, Bristol, BS1</t>
+          <t>Wilder House, Wilder Street, St Pauls, Bristol, BS2</t>
         </is>
       </c>
       <c r="H114" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I114" s="8" t="n"/>
@@ -25600,7 +25600,7 @@
       <c r="L114" s="8" t="n"/>
       <c r="M114" s="8" t="n"/>
       <c r="N114" s="8" t="n">
-        <v>17492</v>
+        <v>22116</v>
       </c>
       <c r="O114" s="8" t="n">
         <v>0</v>
@@ -25608,12 +25608,12 @@
       <c r="P114" s="8" t="n"/>
       <c r="Q114" s="8" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="R114" s="8" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>CJ Hole, Southville</t>
         </is>
       </c>
       <c r="S114" s="9" t="inlineStr"/>
@@ -25630,7 +25630,7 @@
       <c r="V114" s="7" t="inlineStr"/>
       <c r="W114" s="8" t="inlineStr">
         <is>
-          <t>0b4cabfdda5392a4334f6f62b950d7a645376650</t>
+          <t>1efa637d6b56be9e12499f93807a86c947ec8a11</t>
         </is>
       </c>
     </row>
@@ -25644,13 +25644,13 @@
         </is>
       </c>
       <c r="C115" s="17" t="n">
-        <v>2250</v>
+        <v>1400</v>
       </c>
       <c r="D115" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E115" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F115" s="8" t="inlineStr">
         <is>
@@ -25659,12 +25659,12 @@
       </c>
       <c r="G115" s="9" t="inlineStr">
         <is>
-          <t>Eclipse, Bristol, BS1</t>
+          <t>Glass Wharf, Bristol</t>
         </is>
       </c>
       <c r="H115" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I115" s="8" t="n"/>
@@ -25673,7 +25673,7 @@
       <c r="L115" s="8" t="n"/>
       <c r="M115" s="8" t="n"/>
       <c r="N115" s="8" t="n">
-        <v>22080</v>
+        <v>20972</v>
       </c>
       <c r="O115" s="8" t="n">
         <v>0</v>
@@ -25681,12 +25681,12 @@
       <c r="P115" s="8" t="n"/>
       <c r="Q115" s="8" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="R115" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S115" s="9" t="inlineStr"/>
@@ -25703,7 +25703,7 @@
       <c r="V115" s="7" t="inlineStr"/>
       <c r="W115" s="8" t="inlineStr">
         <is>
-          <t>dc210d0a40d826c0930a4e847048280bbe1d9b17</t>
+          <t>58386ab060e5ad520b5bcba6592f39f1e64abdfa</t>
         </is>
       </c>
     </row>
@@ -25717,13 +25717,13 @@
         </is>
       </c>
       <c r="C116" s="17" t="n">
-        <v>1350</v>
+        <v>2240</v>
       </c>
       <c r="D116" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E116" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F116" s="8" t="inlineStr">
         <is>
@@ -25732,21 +25732,23 @@
       </c>
       <c r="G116" s="9" t="inlineStr">
         <is>
-          <t>Wilder House, Wilder Street, St Pauls, Bristol, BS2</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H116" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I116" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I116" s="8" t="n">
+        <v>884</v>
+      </c>
       <c r="J116" s="8" t="n"/>
       <c r="K116" s="8" t="n"/>
       <c r="L116" s="8" t="n"/>
       <c r="M116" s="8" t="n"/>
       <c r="N116" s="8" t="n">
-        <v>22116</v>
+        <v>20856</v>
       </c>
       <c r="O116" s="8" t="n">
         <v>0</v>
@@ -25754,12 +25756,12 @@
       <c r="P116" s="8" t="n"/>
       <c r="Q116" s="8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="R116" s="8" t="inlineStr">
         <is>
-          <t>CJ Hole, Southville</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S116" s="9" t="inlineStr"/>
@@ -25776,7 +25778,7 @@
       <c r="V116" s="7" t="inlineStr"/>
       <c r="W116" s="8" t="inlineStr">
         <is>
-          <t>1efa637d6b56be9e12499f93807a86c947ec8a11</t>
+          <t>0b2cd6178fe0f6128804b82d5b9e39ea5967f124</t>
         </is>
       </c>
     </row>
@@ -25790,7 +25792,7 @@
         </is>
       </c>
       <c r="C117" s="17" t="n">
-        <v>1400</v>
+        <v>1650</v>
       </c>
       <c r="D117" s="8" t="n">
         <v>1</v>
@@ -25805,21 +25807,23 @@
       </c>
       <c r="G117" s="9" t="inlineStr">
         <is>
-          <t>Glass Wharf, Bristol</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H117" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I117" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I117" s="8" t="n">
+        <v>546</v>
+      </c>
       <c r="J117" s="8" t="n"/>
       <c r="K117" s="8" t="n"/>
       <c r="L117" s="8" t="n"/>
       <c r="M117" s="8" t="n"/>
       <c r="N117" s="8" t="n">
-        <v>20972</v>
+        <v>20820</v>
       </c>
       <c r="O117" s="8" t="n">
         <v>0</v>
@@ -25827,12 +25831,12 @@
       <c r="P117" s="8" t="n"/>
       <c r="Q117" s="8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="R117" s="8" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S117" s="9" t="inlineStr"/>
@@ -25849,7 +25853,7 @@
       <c r="V117" s="7" t="inlineStr"/>
       <c r="W117" s="8" t="inlineStr">
         <is>
-          <t>58386ab060e5ad520b5bcba6592f39f1e64abdfa</t>
+          <t>c81c605f4b9d5949dfaedebc49eb5f2643430f3f</t>
         </is>
       </c>
     </row>
@@ -25863,13 +25867,13 @@
         </is>
       </c>
       <c r="C118" s="17" t="n">
-        <v>2240</v>
+        <v>1585</v>
       </c>
       <c r="D118" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E118" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F118" s="8" t="inlineStr">
         <is>
@@ -25878,7 +25882,7 @@
       </c>
       <c r="G118" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H118" s="8" t="inlineStr">
@@ -25887,14 +25891,14 @@
         </is>
       </c>
       <c r="I118" s="8" t="n">
-        <v>884</v>
+        <v>505</v>
       </c>
       <c r="J118" s="8" t="n"/>
       <c r="K118" s="8" t="n"/>
       <c r="L118" s="8" t="n"/>
       <c r="M118" s="8" t="n"/>
       <c r="N118" s="8" t="n">
-        <v>20856</v>
+        <v>21680</v>
       </c>
       <c r="O118" s="8" t="n">
         <v>0</v>
@@ -25907,7 +25911,7 @@
       </c>
       <c r="R118" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S118" s="9" t="inlineStr"/>
@@ -25924,7 +25928,7 @@
       <c r="V118" s="7" t="inlineStr"/>
       <c r="W118" s="8" t="inlineStr">
         <is>
-          <t>0b2cd6178fe0f6128804b82d5b9e39ea5967f124</t>
+          <t>4fc7c891593aa7586ebede2a12c2a9af8edbe973</t>
         </is>
       </c>
     </row>
@@ -25938,13 +25942,13 @@
         </is>
       </c>
       <c r="C119" s="17" t="n">
-        <v>1650</v>
+        <v>2165</v>
       </c>
       <c r="D119" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E119" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F119" s="8" t="inlineStr">
         <is>
@@ -25953,7 +25957,7 @@
       </c>
       <c r="G119" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H119" s="8" t="inlineStr">
@@ -25962,14 +25966,14 @@
         </is>
       </c>
       <c r="I119" s="8" t="n">
-        <v>546</v>
+        <v>682</v>
       </c>
       <c r="J119" s="8" t="n"/>
       <c r="K119" s="8" t="n"/>
       <c r="L119" s="8" t="n"/>
       <c r="M119" s="8" t="n"/>
       <c r="N119" s="8" t="n">
-        <v>20820</v>
+        <v>21680</v>
       </c>
       <c r="O119" s="8" t="n">
         <v>0</v>
@@ -25982,7 +25986,7 @@
       </c>
       <c r="R119" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S119" s="9" t="inlineStr"/>
@@ -25999,7 +26003,7 @@
       <c r="V119" s="7" t="inlineStr"/>
       <c r="W119" s="8" t="inlineStr">
         <is>
-          <t>c81c605f4b9d5949dfaedebc49eb5f2643430f3f</t>
+          <t>961a17b763c937b1487659c1c7677c280a80afc6</t>
         </is>
       </c>
     </row>
@@ -26013,7 +26017,7 @@
         </is>
       </c>
       <c r="C120" s="17" t="n">
-        <v>1585</v>
+        <v>1195</v>
       </c>
       <c r="D120" s="8" t="n">
         <v>1</v>
@@ -26028,23 +26032,21 @@
       </c>
       <c r="G120" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Anvil St, Bristol, BS2</t>
         </is>
       </c>
       <c r="H120" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I120" s="8" t="n">
-        <v>505</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I120" s="8" t="n"/>
       <c r="J120" s="8" t="n"/>
       <c r="K120" s="8" t="n"/>
       <c r="L120" s="8" t="n"/>
       <c r="M120" s="8" t="n"/>
       <c r="N120" s="8" t="n">
-        <v>21680</v>
+        <v>19560</v>
       </c>
       <c r="O120" s="8" t="n">
         <v>0</v>
@@ -26057,7 +26059,7 @@
       </c>
       <c r="R120" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S120" s="9" t="inlineStr"/>
@@ -26074,7 +26076,7 @@
       <c r="V120" s="7" t="inlineStr"/>
       <c r="W120" s="8" t="inlineStr">
         <is>
-          <t>4fc7c891593aa7586ebede2a12c2a9af8edbe973</t>
+          <t>a608da1ef7a49c906f54f438e11d72a5205aa499</t>
         </is>
       </c>
     </row>
@@ -26088,13 +26090,13 @@
         </is>
       </c>
       <c r="C121" s="17" t="n">
-        <v>2165</v>
+        <v>1650</v>
       </c>
       <c r="D121" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E121" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F121" s="8" t="inlineStr">
         <is>
@@ -26103,7 +26105,7 @@
       </c>
       <c r="G121" s="9" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H121" s="8" t="inlineStr">
@@ -26112,14 +26114,14 @@
         </is>
       </c>
       <c r="I121" s="8" t="n">
-        <v>682</v>
+        <v>553</v>
       </c>
       <c r="J121" s="8" t="n"/>
       <c r="K121" s="8" t="n"/>
       <c r="L121" s="8" t="n"/>
       <c r="M121" s="8" t="n"/>
       <c r="N121" s="8" t="n">
-        <v>21680</v>
+        <v>20820</v>
       </c>
       <c r="O121" s="8" t="n">
         <v>0</v>
@@ -26127,12 +26129,12 @@
       <c r="P121" s="8" t="n"/>
       <c r="Q121" s="8" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="R121" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S121" s="9" t="inlineStr"/>
@@ -26149,7 +26151,7 @@
       <c r="V121" s="7" t="inlineStr"/>
       <c r="W121" s="8" t="inlineStr">
         <is>
-          <t>961a17b763c937b1487659c1c7677c280a80afc6</t>
+          <t>d6bb31b3e903e1ec64e3eea9a96c3b08bb9873e3</t>
         </is>
       </c>
     </row>
@@ -26163,10 +26165,10 @@
         </is>
       </c>
       <c r="C122" s="17" t="n">
-        <v>1195</v>
+        <v>1500</v>
       </c>
       <c r="D122" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E122" s="8" t="n">
         <v>1</v>
@@ -26178,7 +26180,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>Anvil St, Bristol, BS2</t>
+          <t>The Quadrant, Barleyfields, Bristol, BS2</t>
         </is>
       </c>
       <c r="H122" s="8" t="inlineStr">
@@ -26192,7 +26194,7 @@
       <c r="L122" s="8" t="n"/>
       <c r="M122" s="8" t="n"/>
       <c r="N122" s="8" t="n">
-        <v>19560</v>
+        <v>20056</v>
       </c>
       <c r="O122" s="8" t="n">
         <v>0</v>
@@ -26200,12 +26202,12 @@
       <c r="P122" s="8" t="n"/>
       <c r="Q122" s="8" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="R122" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S122" s="9" t="inlineStr"/>
@@ -26222,7 +26224,7 @@
       <c r="V122" s="7" t="inlineStr"/>
       <c r="W122" s="8" t="inlineStr">
         <is>
-          <t>a608da1ef7a49c906f54f438e11d72a5205aa499</t>
+          <t>c77814f9166c93a32f4a1ce46b46c87a68a6196a</t>
         </is>
       </c>
     </row>
@@ -26236,14 +26238,12 @@
         </is>
       </c>
       <c r="C123" s="17" t="n">
-        <v>1650</v>
+        <v>1450</v>
       </c>
       <c r="D123" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E123" s="8" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="E123" s="8" t="n"/>
       <c r="F123" s="8" t="inlineStr">
         <is>
           <t>flat</t>
@@ -26251,23 +26251,21 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Stapleton Road, Bristol, BS5</t>
         </is>
       </c>
       <c r="H123" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I123" s="8" t="n">
-        <v>553</v>
-      </c>
+          <t>BS5</t>
+        </is>
+      </c>
+      <c r="I123" s="8" t="n"/>
       <c r="J123" s="8" t="n"/>
       <c r="K123" s="8" t="n"/>
       <c r="L123" s="8" t="n"/>
       <c r="M123" s="8" t="n"/>
       <c r="N123" s="8" t="n">
-        <v>20820</v>
+        <v>19488</v>
       </c>
       <c r="O123" s="8" t="n">
         <v>0</v>
@@ -26280,7 +26278,7 @@
       </c>
       <c r="R123" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Phoenix Property Company, Bristol</t>
         </is>
       </c>
       <c r="S123" s="9" t="inlineStr"/>
@@ -26297,7 +26295,7 @@
       <c r="V123" s="7" t="inlineStr"/>
       <c r="W123" s="8" t="inlineStr">
         <is>
-          <t>d6bb31b3e903e1ec64e3eea9a96c3b08bb9873e3</t>
+          <t>9696d556a9ab494e09c67abf76046ac09e9d61cc</t>
         </is>
       </c>
     </row>
@@ -26311,10 +26309,10 @@
         </is>
       </c>
       <c r="C124" s="17" t="n">
-        <v>1500</v>
+        <v>1400</v>
       </c>
       <c r="D124" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E124" s="8" t="n">
         <v>1</v>
@@ -26326,7 +26324,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>The Quadrant, Barleyfields, Bristol, BS2</t>
+          <t>Redcross Village, Bristol, BS2</t>
         </is>
       </c>
       <c r="H124" s="8" t="inlineStr">
@@ -26340,7 +26338,7 @@
       <c r="L124" s="8" t="n"/>
       <c r="M124" s="8" t="n"/>
       <c r="N124" s="8" t="n">
-        <v>20056</v>
+        <v>21420</v>
       </c>
       <c r="O124" s="8" t="n">
         <v>0</v>
@@ -26370,7 +26368,7 @@
       <c r="V124" s="7" t="inlineStr"/>
       <c r="W124" s="8" t="inlineStr">
         <is>
-          <t>c77814f9166c93a32f4a1ce46b46c87a68a6196a</t>
+          <t>5397132583b1a56a54c39041a79ad2d6eb42879d</t>
         </is>
       </c>
     </row>
@@ -26384,12 +26382,14 @@
         </is>
       </c>
       <c r="C125" s="17" t="n">
-        <v>1450</v>
+        <v>1640</v>
       </c>
       <c r="D125" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E125" s="8" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="E125" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="F125" s="8" t="inlineStr">
         <is>
           <t>flat</t>
@@ -26397,21 +26397,23 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>Stapleton Road, Bristol, BS5</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H125" s="8" t="inlineStr">
         <is>
-          <t>BS5</t>
-        </is>
-      </c>
-      <c r="I125" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I125" s="8" t="n">
+        <v>485</v>
+      </c>
       <c r="J125" s="8" t="n"/>
       <c r="K125" s="8" t="n"/>
       <c r="L125" s="8" t="n"/>
       <c r="M125" s="8" t="n"/>
       <c r="N125" s="8" t="n">
-        <v>19488</v>
+        <v>21504</v>
       </c>
       <c r="O125" s="8" t="n">
         <v>0</v>
@@ -26424,7 +26426,7 @@
       </c>
       <c r="R125" s="8" t="inlineStr">
         <is>
-          <t>Phoenix Property Company, Bristol</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S125" s="9" t="inlineStr"/>
@@ -26441,7 +26443,7 @@
       <c r="V125" s="7" t="inlineStr"/>
       <c r="W125" s="8" t="inlineStr">
         <is>
-          <t>9696d556a9ab494e09c67abf76046ac09e9d61cc</t>
+          <t>47301f8a472393cf4550a7380ee71363e6337581</t>
         </is>
       </c>
     </row>
@@ -26455,7 +26457,7 @@
         </is>
       </c>
       <c r="C126" s="17" t="n">
-        <v>1400</v>
+        <v>1600</v>
       </c>
       <c r="D126" s="8" t="n">
         <v>1</v>
@@ -26470,12 +26472,12 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>Redcross Village, Bristol, BS2</t>
+          <t>Hope Quay, Wapping Wharf, Bristol, BS1</t>
         </is>
       </c>
       <c r="H126" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I126" s="8" t="n"/>
@@ -26483,9 +26485,7 @@
       <c r="K126" s="8" t="n"/>
       <c r="L126" s="8" t="n"/>
       <c r="M126" s="8" t="n"/>
-      <c r="N126" s="8" t="n">
-        <v>21420</v>
-      </c>
+      <c r="N126" s="8" t="n"/>
       <c r="O126" s="8" t="n">
         <v>0</v>
       </c>
@@ -26514,7 +26514,7 @@
       <c r="V126" s="7" t="inlineStr"/>
       <c r="W126" s="8" t="inlineStr">
         <is>
-          <t>5397132583b1a56a54c39041a79ad2d6eb42879d</t>
+          <t>782d0a253814b27fb94b8f2b1f467fac15db0b7e</t>
         </is>
       </c>
     </row>
@@ -26528,10 +26528,10 @@
         </is>
       </c>
       <c r="C127" s="17" t="n">
-        <v>1640</v>
+        <v>1300</v>
       </c>
       <c r="D127" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E127" s="8" t="n">
         <v>1</v>
@@ -26543,23 +26543,21 @@
       </c>
       <c r="G127" s="9" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Champion Court, City Centre, Bristol, BS2</t>
         </is>
       </c>
       <c r="H127" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I127" s="8" t="n">
-        <v>485</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I127" s="8" t="n"/>
       <c r="J127" s="8" t="n"/>
       <c r="K127" s="8" t="n"/>
       <c r="L127" s="8" t="n"/>
       <c r="M127" s="8" t="n"/>
       <c r="N127" s="8" t="n">
-        <v>21504</v>
+        <v>21484</v>
       </c>
       <c r="O127" s="8" t="n">
         <v>0</v>
@@ -26567,12 +26565,12 @@
       <c r="P127" s="8" t="n"/>
       <c r="Q127" s="8" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="R127" s="8" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Taylors Lettings, Bedminster</t>
         </is>
       </c>
       <c r="S127" s="9" t="inlineStr"/>
@@ -26589,7 +26587,7 @@
       <c r="V127" s="7" t="inlineStr"/>
       <c r="W127" s="8" t="inlineStr">
         <is>
-          <t>47301f8a472393cf4550a7380ee71363e6337581</t>
+          <t>5864fa4083267aba7fb2c38a58e549510d3d67b7</t>
         </is>
       </c>
     </row>
@@ -26631,14 +26629,16 @@
       <c r="K128" s="8" t="n"/>
       <c r="L128" s="8" t="n"/>
       <c r="M128" s="8" t="n"/>
-      <c r="N128" s="8" t="n"/>
+      <c r="N128" s="8" t="n">
+        <v>17492</v>
+      </c>
       <c r="O128" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P128" s="8" t="n"/>
       <c r="Q128" s="8" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="R128" s="8" t="inlineStr">
@@ -26660,7 +26660,7 @@
       <c r="V128" s="7" t="inlineStr"/>
       <c r="W128" s="8" t="inlineStr">
         <is>
-          <t>782d0a253814b27fb94b8f2b1f467fac15db0b7e</t>
+          <t>0b4cabfdda5392a4334f6f62b950d7a645376650</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
House search data from run 47
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -17759,7 +17759,7 @@
         </is>
       </c>
       <c r="C12" s="17" t="n">
-        <v>1650</v>
+        <v>2000</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>2</v>
@@ -17774,21 +17774,23 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>Sweetman Place, Bristol, BS2</t>
+          <t>Chatfield House, Marsh Street, Bristol</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I12" s="8" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>705</v>
+      </c>
       <c r="J12" s="8" t="n"/>
       <c r="K12" s="8" t="n"/>
       <c r="L12" s="8" t="n"/>
       <c r="M12" s="8" t="n"/>
       <c r="N12" s="8" t="n">
-        <v>20416</v>
+        <v>20932</v>
       </c>
       <c r="O12" s="8" t="n">
         <v>0</v>
@@ -17796,12 +17798,12 @@
       <c r="P12" s="8" t="n"/>
       <c r="Q12" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="R12" s="8" t="inlineStr">
         <is>
-          <t>Andrews Letting and Management, Clifton</t>
+          <t>Mariana Real Estate, London</t>
         </is>
       </c>
       <c r="S12" s="9" t="inlineStr">
@@ -17822,7 +17824,7 @@
       <c r="V12" s="7" t="inlineStr"/>
       <c r="W12" s="8" t="inlineStr">
         <is>
-          <t>54fa42ef8d0349a295f45392644c43dec3321c5b</t>
+          <t>be4fdd18faf2bcf44d894da42e9c874b7d868fbe</t>
         </is>
       </c>
     </row>
@@ -17836,13 +17838,13 @@
         </is>
       </c>
       <c r="C13" s="17" t="n">
-        <v>2000</v>
+        <v>1600</v>
       </c>
       <c r="D13" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
@@ -17851,7 +17853,7 @@
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>Chatfield House, Marsh Street, Bristol</t>
+          <t>St. Stephens Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H13" s="8" t="inlineStr">
@@ -17859,15 +17861,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I13" s="8" t="n">
-        <v>705</v>
-      </c>
+      <c r="I13" s="8" t="n"/>
       <c r="J13" s="8" t="n"/>
       <c r="K13" s="8" t="n"/>
       <c r="L13" s="8" t="n"/>
       <c r="M13" s="8" t="n"/>
       <c r="N13" s="8" t="n">
-        <v>20932</v>
+        <v>21428</v>
       </c>
       <c r="O13" s="8" t="n">
         <v>0</v>
@@ -17880,7 +17880,7 @@
       </c>
       <c r="R13" s="8" t="inlineStr">
         <is>
-          <t>Mariana Real Estate, London</t>
+          <t>Romans, Clifton</t>
         </is>
       </c>
       <c r="S13" s="9" t="inlineStr">
@@ -17901,7 +17901,7 @@
       <c r="V13" s="7" t="inlineStr"/>
       <c r="W13" s="8" t="inlineStr">
         <is>
-          <t>be4fdd18faf2bcf44d894da42e9c874b7d868fbe</t>
+          <t>cd770dd603af2e6f4f23a72c9685c7468c731a6d</t>
         </is>
       </c>
     </row>
@@ -17915,10 +17915,10 @@
         </is>
       </c>
       <c r="C14" s="17" t="n">
-        <v>1600</v>
+        <v>1200</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" s="8" t="n">
         <v>1</v>
@@ -17930,12 +17930,12 @@
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>St. Stephens Street, Bristol, BS1</t>
+          <t>Union Road, Bristol BS2 0FN</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I14" s="8" t="n"/>
@@ -17944,7 +17944,7 @@
       <c r="L14" s="8" t="n"/>
       <c r="M14" s="8" t="n"/>
       <c r="N14" s="8" t="n">
-        <v>21428</v>
+        <v>20144</v>
       </c>
       <c r="O14" s="8" t="n">
         <v>0</v>
@@ -17952,12 +17952,12 @@
       <c r="P14" s="8" t="n"/>
       <c r="Q14" s="8" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="R14" s="8" t="inlineStr">
         <is>
-          <t>Romans, Clifton</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S14" s="9" t="inlineStr">
@@ -17978,7 +17978,7 @@
       <c r="V14" s="7" t="inlineStr"/>
       <c r="W14" s="8" t="inlineStr">
         <is>
-          <t>cd770dd603af2e6f4f23a72c9685c7468c731a6d</t>
+          <t>2b2295e0c22bd50658835eb43d2eb433f6d1cd1b</t>
         </is>
       </c>
     </row>
@@ -17992,13 +17992,13 @@
         </is>
       </c>
       <c r="C15" s="17" t="n">
-        <v>1200</v>
+        <v>2850</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
@@ -18007,21 +18007,23 @@
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>Union Road, Bristol BS2 0FN</t>
+          <t>Capricorn Place, Hotwells, BS8</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I15" s="8" t="n"/>
+          <t>BS8</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="n">
+        <v>1615</v>
+      </c>
       <c r="J15" s="8" t="n"/>
       <c r="K15" s="8" t="n"/>
       <c r="L15" s="8" t="n"/>
       <c r="M15" s="8" t="n"/>
       <c r="N15" s="8" t="n">
-        <v>20144</v>
+        <v>15104</v>
       </c>
       <c r="O15" s="8" t="n">
         <v>0</v>
@@ -18034,7 +18036,7 @@
       </c>
       <c r="R15" s="8" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Sarah Kenny Residential Lettings, Bristol</t>
         </is>
       </c>
       <c r="S15" s="9" t="inlineStr">
@@ -18055,7 +18057,7 @@
       <c r="V15" s="7" t="inlineStr"/>
       <c r="W15" s="8" t="inlineStr">
         <is>
-          <t>2b2295e0c22bd50658835eb43d2eb433f6d1cd1b</t>
+          <t>11c93771b8963d430763c083c575b56042e71418</t>
         </is>
       </c>
     </row>
@@ -18069,7 +18071,7 @@
         </is>
       </c>
       <c r="C16" s="17" t="n">
-        <v>2850</v>
+        <v>2050</v>
       </c>
       <c r="D16" s="8" t="n">
         <v>2</v>
@@ -18084,23 +18086,23 @@
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>Capricorn Place, Hotwells, BS8</t>
+          <t>421 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>BS8</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I16" s="8" t="n">
-        <v>1615</v>
+        <v>802</v>
       </c>
       <c r="J16" s="8" t="n"/>
       <c r="K16" s="8" t="n"/>
       <c r="L16" s="8" t="n"/>
       <c r="M16" s="8" t="n"/>
       <c r="N16" s="8" t="n">
-        <v>15104</v>
+        <v>20800</v>
       </c>
       <c r="O16" s="8" t="n">
         <v>0</v>
@@ -18108,12 +18110,12 @@
       <c r="P16" s="8" t="n"/>
       <c r="Q16" s="8" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="R16" s="8" t="inlineStr">
         <is>
-          <t>Sarah Kenny Residential Lettings, Bristol</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S16" s="9" t="inlineStr">
@@ -18134,7 +18136,7 @@
       <c r="V16" s="7" t="inlineStr"/>
       <c r="W16" s="8" t="inlineStr">
         <is>
-          <t>11c93771b8963d430763c083c575b56042e71418</t>
+          <t>b7d86b41b199aaf040e0304048e519e961081fd2</t>
         </is>
       </c>
     </row>
@@ -18148,14 +18150,12 @@
         </is>
       </c>
       <c r="C17" s="17" t="n">
-        <v>2050</v>
+        <v>2100</v>
       </c>
       <c r="D17" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="E17" s="8" t="n">
-        <v>2</v>
-      </c>
+      <c r="E17" s="8" t="n"/>
       <c r="F17" s="8" t="inlineStr">
         <is>
           <t>flat</t>
@@ -18163,7 +18163,7 @@
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>421 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>526 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
@@ -18172,7 +18172,7 @@
         </is>
       </c>
       <c r="I17" s="8" t="n">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="J17" s="8" t="n"/>
       <c r="K17" s="8" t="n"/>
@@ -18213,7 +18213,7 @@
       <c r="V17" s="7" t="inlineStr"/>
       <c r="W17" s="8" t="inlineStr">
         <is>
-          <t>b7d86b41b199aaf040e0304048e519e961081fd2</t>
+          <t>74d41470c07849b906ad0a12b07a1745551d8e6f</t>
         </is>
       </c>
     </row>
@@ -18227,12 +18227,14 @@
         </is>
       </c>
       <c r="C18" s="17" t="n">
-        <v>2100</v>
+        <v>2120</v>
       </c>
       <c r="D18" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="E18" s="8" t="n"/>
+      <c r="E18" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
           <t>flat</t>
@@ -18240,7 +18242,7 @@
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>526 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>522 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
@@ -18249,7 +18251,7 @@
         </is>
       </c>
       <c r="I18" s="8" t="n">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="J18" s="8" t="n"/>
       <c r="K18" s="8" t="n"/>
@@ -18290,7 +18292,7 @@
       <c r="V18" s="7" t="inlineStr"/>
       <c r="W18" s="8" t="inlineStr">
         <is>
-          <t>74d41470c07849b906ad0a12b07a1745551d8e6f</t>
+          <t>4a3dbf2b76e61d3a02d3b62cb6a5a56affeadff0</t>
         </is>
       </c>
     </row>
@@ -18304,7 +18306,7 @@
         </is>
       </c>
       <c r="C19" s="17" t="n">
-        <v>2120</v>
+        <v>2150</v>
       </c>
       <c r="D19" s="8" t="n">
         <v>2</v>
@@ -18319,7 +18321,7 @@
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>522 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>802 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
@@ -18328,7 +18330,7 @@
         </is>
       </c>
       <c r="I19" s="8" t="n">
-        <v>799</v>
+        <v>809</v>
       </c>
       <c r="J19" s="8" t="n"/>
       <c r="K19" s="8" t="n"/>
@@ -18369,7 +18371,7 @@
       <c r="V19" s="7" t="inlineStr"/>
       <c r="W19" s="8" t="inlineStr">
         <is>
-          <t>4a3dbf2b76e61d3a02d3b62cb6a5a56affeadff0</t>
+          <t>fcdcdd1da915be6f6b065ad9cbeea66062d00301</t>
         </is>
       </c>
     </row>
@@ -18383,10 +18385,10 @@
         </is>
       </c>
       <c r="C20" s="17" t="n">
-        <v>2150</v>
+        <v>2830</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E20" s="8" t="n">
         <v>2</v>
@@ -18398,7 +18400,7 @@
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>802 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>315 Dovetail, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H20" s="8" t="inlineStr">
@@ -18407,7 +18409,7 @@
         </is>
       </c>
       <c r="I20" s="8" t="n">
-        <v>809</v>
+        <v>1120</v>
       </c>
       <c r="J20" s="8" t="n"/>
       <c r="K20" s="8" t="n"/>
@@ -18422,7 +18424,7 @@
       <c r="P20" s="8" t="n"/>
       <c r="Q20" s="8" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="R20" s="8" t="inlineStr">
@@ -18448,7 +18450,7 @@
       <c r="V20" s="7" t="inlineStr"/>
       <c r="W20" s="8" t="inlineStr">
         <is>
-          <t>fcdcdd1da915be6f6b065ad9cbeea66062d00301</t>
+          <t>e4f6deef9389498e73820b4056b013ac2b6ff363</t>
         </is>
       </c>
     </row>
@@ -18462,13 +18464,13 @@
         </is>
       </c>
       <c r="C21" s="17" t="n">
-        <v>2830</v>
+        <v>1950</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
@@ -18477,23 +18479,23 @@
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>315 Dovetail, New Kingsley Road, Bristol, BS2</t>
+          <t>Cheltenham House, 24A Clare Street, Bristol</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I21" s="8" t="n">
-        <v>1120</v>
+        <v>668</v>
       </c>
       <c r="J21" s="8" t="n"/>
       <c r="K21" s="8" t="n"/>
       <c r="L21" s="8" t="n"/>
       <c r="M21" s="8" t="n"/>
       <c r="N21" s="8" t="n">
-        <v>20800</v>
+        <v>21044</v>
       </c>
       <c r="O21" s="8" t="n">
         <v>0</v>
@@ -18501,12 +18503,12 @@
       <c r="P21" s="8" t="n"/>
       <c r="Q21" s="8" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="R21" s="8" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>Mariana Real Estate, London</t>
         </is>
       </c>
       <c r="S21" s="9" t="inlineStr">
@@ -18527,7 +18529,7 @@
       <c r="V21" s="7" t="inlineStr"/>
       <c r="W21" s="8" t="inlineStr">
         <is>
-          <t>e4f6deef9389498e73820b4056b013ac2b6ff363</t>
+          <t>9bdc8fdc90a88180cfd80c66940dfb5055afd30b</t>
         </is>
       </c>
     </row>
@@ -18541,7 +18543,7 @@
         </is>
       </c>
       <c r="C22" s="17" t="n">
-        <v>1950</v>
+        <v>1500</v>
       </c>
       <c r="D22" s="8" t="n">
         <v>2</v>
@@ -18556,7 +18558,7 @@
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>Cheltenham House, 24A Clare Street, Bristol</t>
+          <t>The Metropolitan, Redcliff Backs, BRISTOL, BS1</t>
         </is>
       </c>
       <c r="H22" s="8" t="inlineStr">
@@ -18564,15 +18566,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I22" s="8" t="n">
-        <v>668</v>
-      </c>
+      <c r="I22" s="8" t="n"/>
       <c r="J22" s="8" t="n"/>
       <c r="K22" s="8" t="n"/>
       <c r="L22" s="8" t="n"/>
       <c r="M22" s="8" t="n"/>
       <c r="N22" s="8" t="n">
-        <v>21044</v>
+        <v>20320</v>
       </c>
       <c r="O22" s="8" t="n">
         <v>0</v>
@@ -18585,7 +18585,7 @@
       </c>
       <c r="R22" s="8" t="inlineStr">
         <is>
-          <t>Mariana Real Estate, London</t>
+          <t>Andrews Letting and Management, Clifton</t>
         </is>
       </c>
       <c r="S22" s="9" t="inlineStr">
@@ -18606,7 +18606,7 @@
       <c r="V22" s="7" t="inlineStr"/>
       <c r="W22" s="8" t="inlineStr">
         <is>
-          <t>9bdc8fdc90a88180cfd80c66940dfb5055afd30b</t>
+          <t>48f0639d9505de53304e65370c31dc2b91415006</t>
         </is>
       </c>
     </row>
@@ -18620,10 +18620,10 @@
         </is>
       </c>
       <c r="C23" s="17" t="n">
-        <v>1500</v>
+        <v>1050</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23" s="8" t="n">
         <v>1</v>
@@ -18635,7 +18635,7 @@
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>The Metropolitan, Redcliff Backs, BRISTOL, BS1</t>
+          <t>Caslon Court, Somerset Street, Redcliffe, Bristol, BS1</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
@@ -18649,7 +18649,7 @@
       <c r="L23" s="8" t="n"/>
       <c r="M23" s="8" t="n"/>
       <c r="N23" s="8" t="n">
-        <v>20320</v>
+        <v>18424</v>
       </c>
       <c r="O23" s="8" t="n">
         <v>0</v>
@@ -18657,12 +18657,12 @@
       <c r="P23" s="8" t="n"/>
       <c r="Q23" s="8" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="R23" s="8" t="inlineStr">
         <is>
-          <t>Andrews Letting and Management, Clifton</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S23" s="9" t="inlineStr">
@@ -18683,7 +18683,7 @@
       <c r="V23" s="7" t="inlineStr"/>
       <c r="W23" s="8" t="inlineStr">
         <is>
-          <t>48f0639d9505de53304e65370c31dc2b91415006</t>
+          <t>7183e0bb70a3ff586aa635a21825e38757f1f13d</t>
         </is>
       </c>
     </row>
@@ -18697,7 +18697,7 @@
         </is>
       </c>
       <c r="C24" s="17" t="n">
-        <v>1050</v>
+        <v>1450</v>
       </c>
       <c r="D24" s="8" t="n">
         <v>1</v>
@@ -18712,7 +18712,7 @@
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>Caslon Court, Somerset Street, Redcliffe, Bristol, BS1</t>
+          <t>The Crescent, Bristol, BS1</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr">
@@ -18726,7 +18726,7 @@
       <c r="L24" s="8" t="n"/>
       <c r="M24" s="8" t="n"/>
       <c r="N24" s="8" t="n">
-        <v>18424</v>
+        <v>16792</v>
       </c>
       <c r="O24" s="8" t="n">
         <v>0</v>
@@ -18734,12 +18734,12 @@
       <c r="P24" s="8" t="n"/>
       <c r="Q24" s="8" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="R24" s="8" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S24" s="9" t="inlineStr">
@@ -18760,7 +18760,7 @@
       <c r="V24" s="7" t="inlineStr"/>
       <c r="W24" s="8" t="inlineStr">
         <is>
-          <t>7183e0bb70a3ff586aa635a21825e38757f1f13d</t>
+          <t>d447d1158e90abd2c82eb7828f8a98e7f5fbe2bd</t>
         </is>
       </c>
     </row>
@@ -18774,13 +18774,13 @@
         </is>
       </c>
       <c r="C25" s="17" t="n">
-        <v>1450</v>
+        <v>1650</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
@@ -18789,7 +18789,7 @@
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>The Crescent, Bristol, BS1</t>
+          <t>Harbourside, Purifier House, BS1 5AU</t>
         </is>
       </c>
       <c r="H25" s="8" t="inlineStr">
@@ -18797,13 +18797,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I25" s="8" t="n"/>
+      <c r="I25" s="8" t="n">
+        <v>689</v>
+      </c>
       <c r="J25" s="8" t="n"/>
       <c r="K25" s="8" t="n"/>
       <c r="L25" s="8" t="n"/>
       <c r="M25" s="8" t="n"/>
       <c r="N25" s="8" t="n">
-        <v>16792</v>
+        <v>16240</v>
       </c>
       <c r="O25" s="8" t="n">
         <v>0</v>
@@ -18816,7 +18818,7 @@
       </c>
       <c r="R25" s="8" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>The Bristol Residential Letting Co, Clifton</t>
         </is>
       </c>
       <c r="S25" s="9" t="inlineStr">
@@ -18837,7 +18839,7 @@
       <c r="V25" s="7" t="inlineStr"/>
       <c r="W25" s="8" t="inlineStr">
         <is>
-          <t>d447d1158e90abd2c82eb7828f8a98e7f5fbe2bd</t>
+          <t>7ec8aa4d9388bb5e923c445c92ac24d6496094c5</t>
         </is>
       </c>
     </row>
@@ -18851,7 +18853,7 @@
         </is>
       </c>
       <c r="C26" s="17" t="n">
-        <v>1650</v>
+        <v>1900</v>
       </c>
       <c r="D26" s="8" t="n">
         <v>2</v>
@@ -18866,7 +18868,7 @@
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>Harbourside, Purifier House, BS1 5AU</t>
+          <t>Wapping Wharf, Anchorage, BS1</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">
@@ -18875,14 +18877,14 @@
         </is>
       </c>
       <c r="I26" s="8" t="n">
-        <v>689</v>
+        <v>799</v>
       </c>
       <c r="J26" s="8" t="n"/>
       <c r="K26" s="8" t="n"/>
       <c r="L26" s="8" t="n"/>
       <c r="M26" s="8" t="n"/>
       <c r="N26" s="8" t="n">
-        <v>16240</v>
+        <v>16416</v>
       </c>
       <c r="O26" s="8" t="n">
         <v>0</v>
@@ -18890,12 +18892,12 @@
       <c r="P26" s="8" t="n"/>
       <c r="Q26" s="8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="R26" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Clifton</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S26" s="9" t="inlineStr">
@@ -18916,7 +18918,7 @@
       <c r="V26" s="7" t="inlineStr"/>
       <c r="W26" s="8" t="inlineStr">
         <is>
-          <t>7ec8aa4d9388bb5e923c445c92ac24d6496094c5</t>
+          <t>6b74ba6dcca9cfc12cf5e5d10aaa942cfd63c0e6</t>
         </is>
       </c>
     </row>
@@ -18930,13 +18932,13 @@
         </is>
       </c>
       <c r="C27" s="17" t="n">
-        <v>1900</v>
+        <v>1225</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
@@ -18945,23 +18947,21 @@
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>Wapping Wharf, Anchorage, BS1</t>
+          <t>New Walls, Totterdown, BS4</t>
         </is>
       </c>
       <c r="H27" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I27" s="8" t="n">
-        <v>799</v>
-      </c>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="n"/>
       <c r="J27" s="8" t="n"/>
       <c r="K27" s="8" t="n"/>
       <c r="L27" s="8" t="n"/>
       <c r="M27" s="8" t="n"/>
       <c r="N27" s="8" t="n">
-        <v>16416</v>
+        <v>8540</v>
       </c>
       <c r="O27" s="8" t="n">
         <v>0</v>
@@ -18969,12 +18969,12 @@
       <c r="P27" s="8" t="n"/>
       <c r="Q27" s="8" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="R27" s="8" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Bristol Property Centre, Bristol</t>
         </is>
       </c>
       <c r="S27" s="9" t="inlineStr">
@@ -18995,7 +18995,7 @@
       <c r="V27" s="7" t="inlineStr"/>
       <c r="W27" s="8" t="inlineStr">
         <is>
-          <t>6b74ba6dcca9cfc12cf5e5d10aaa942cfd63c0e6</t>
+          <t>ff7cade97c52dbe0ee822ce3951fd4f71c9b4146</t>
         </is>
       </c>
     </row>
@@ -19009,7 +19009,7 @@
         </is>
       </c>
       <c r="C28" s="17" t="n">
-        <v>1225</v>
+        <v>1680</v>
       </c>
       <c r="D28" s="8" t="n">
         <v>1</v>
@@ -19024,21 +19024,23 @@
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>New Walls, Totterdown, BS4</t>
+          <t>904 Dovetail, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H28" s="8" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I28" s="8" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="n">
+        <v>557</v>
+      </c>
       <c r="J28" s="8" t="n"/>
       <c r="K28" s="8" t="n"/>
       <c r="L28" s="8" t="n"/>
       <c r="M28" s="8" t="n"/>
       <c r="N28" s="8" t="n">
-        <v>8540</v>
+        <v>20800</v>
       </c>
       <c r="O28" s="8" t="n">
         <v>0</v>
@@ -19046,12 +19048,12 @@
       <c r="P28" s="8" t="n"/>
       <c r="Q28" s="8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="R28" s="8" t="inlineStr">
         <is>
-          <t>Bristol Property Centre, Bristol</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S28" s="9" t="inlineStr">
@@ -19072,7 +19074,7 @@
       <c r="V28" s="7" t="inlineStr"/>
       <c r="W28" s="8" t="inlineStr">
         <is>
-          <t>ff7cade97c52dbe0ee822ce3951fd4f71c9b4146</t>
+          <t>3d5fce4a62f2bd2b3bbd100f6bd7598155b266f2</t>
         </is>
       </c>
     </row>
@@ -19086,7 +19088,7 @@
         </is>
       </c>
       <c r="C29" s="17" t="n">
-        <v>1680</v>
+        <v>1733</v>
       </c>
       <c r="D29" s="8" t="n">
         <v>1</v>
@@ -19101,24 +19103,22 @@
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>904 Dovetail, New Kingsley Road, Bristol, BS2</t>
+          <t>Cheltenham House, Clare Street, Bristol</t>
         </is>
       </c>
       <c r="H29" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I29" s="8" t="n">
-        <v>557</v>
+        <v>455</v>
       </c>
       <c r="J29" s="8" t="n"/>
       <c r="K29" s="8" t="n"/>
       <c r="L29" s="8" t="n"/>
       <c r="M29" s="8" t="n"/>
-      <c r="N29" s="8" t="n">
-        <v>20800</v>
-      </c>
+      <c r="N29" s="8" t="n"/>
       <c r="O29" s="8" t="n">
         <v>0</v>
       </c>
@@ -19130,7 +19130,7 @@
       </c>
       <c r="R29" s="8" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>Mariana Real Estate, London</t>
         </is>
       </c>
       <c r="S29" s="9" t="inlineStr">
@@ -19151,7 +19151,7 @@
       <c r="V29" s="7" t="inlineStr"/>
       <c r="W29" s="8" t="inlineStr">
         <is>
-          <t>3d5fce4a62f2bd2b3bbd100f6bd7598155b266f2</t>
+          <t>10b717aabd38544480501915d97cf63dfbd0bcbd</t>
         </is>
       </c>
     </row>
@@ -19165,7 +19165,7 @@
         </is>
       </c>
       <c r="C30" s="17" t="n">
-        <v>1733</v>
+        <v>1715</v>
       </c>
       <c r="D30" s="8" t="n">
         <v>1</v>
@@ -19180,22 +19180,24 @@
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>Cheltenham House, Clare Street, Bristol</t>
+          <t>1006 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H30" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I30" s="8" t="n">
-        <v>455</v>
+        <v>547</v>
       </c>
       <c r="J30" s="8" t="n"/>
       <c r="K30" s="8" t="n"/>
       <c r="L30" s="8" t="n"/>
       <c r="M30" s="8" t="n"/>
-      <c r="N30" s="8" t="n"/>
+      <c r="N30" s="8" t="n">
+        <v>20800</v>
+      </c>
       <c r="O30" s="8" t="n">
         <v>0</v>
       </c>
@@ -19207,7 +19209,7 @@
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
-          <t>Mariana Real Estate, London</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S30" s="9" t="inlineStr">
@@ -19228,7 +19230,7 @@
       <c r="V30" s="7" t="inlineStr"/>
       <c r="W30" s="8" t="inlineStr">
         <is>
-          <t>10b717aabd38544480501915d97cf63dfbd0bcbd</t>
+          <t>baed14f153217bbfa48df27148f4a5b45559a145</t>
         </is>
       </c>
     </row>
@@ -19242,14 +19244,12 @@
         </is>
       </c>
       <c r="C31" s="17" t="n">
-        <v>1715</v>
+        <v>1400</v>
       </c>
       <c r="D31" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="E31" s="8" t="n">
-        <v>1</v>
-      </c>
+      <c r="E31" s="8" t="n"/>
       <c r="F31" s="8" t="inlineStr">
         <is>
           <t>flat</t>
@@ -19257,23 +19257,21 @@
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>1006 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>Millennium Promenade, Bristol, BS1</t>
         </is>
       </c>
       <c r="H31" s="8" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I31" s="8" t="n">
-        <v>547</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="n"/>
       <c r="J31" s="8" t="n"/>
       <c r="K31" s="8" t="n"/>
       <c r="L31" s="8" t="n"/>
       <c r="M31" s="8" t="n"/>
       <c r="N31" s="8" t="n">
-        <v>20800</v>
+        <v>16168</v>
       </c>
       <c r="O31" s="8" t="n">
         <v>0</v>
@@ -19281,12 +19279,12 @@
       <c r="P31" s="8" t="n"/>
       <c r="Q31" s="8" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>Phoenix Property Company, Bristol</t>
         </is>
       </c>
       <c r="S31" s="9" t="inlineStr">
@@ -19307,7 +19305,7 @@
       <c r="V31" s="7" t="inlineStr"/>
       <c r="W31" s="8" t="inlineStr">
         <is>
-          <t>baed14f153217bbfa48df27148f4a5b45559a145</t>
+          <t>5ec68f33756a2f8f7606ead5febd7f33ed18c280</t>
         </is>
       </c>
     </row>
@@ -19321,12 +19319,14 @@
         </is>
       </c>
       <c r="C32" s="17" t="n">
-        <v>1400</v>
+        <v>1655</v>
       </c>
       <c r="D32" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="8" t="n"/>
+      <c r="E32" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
           <t>flat</t>
@@ -19334,21 +19334,23 @@
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>Millennium Promenade, Bristol, BS1</t>
+          <t>712 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I32" s="8" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="n">
+        <v>547</v>
+      </c>
       <c r="J32" s="8" t="n"/>
       <c r="K32" s="8" t="n"/>
       <c r="L32" s="8" t="n"/>
       <c r="M32" s="8" t="n"/>
       <c r="N32" s="8" t="n">
-        <v>16168</v>
+        <v>20800</v>
       </c>
       <c r="O32" s="8" t="n">
         <v>0</v>
@@ -19361,7 +19363,7 @@
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
-          <t>Phoenix Property Company, Bristol</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S32" s="9" t="inlineStr">
@@ -19382,7 +19384,7 @@
       <c r="V32" s="7" t="inlineStr"/>
       <c r="W32" s="8" t="inlineStr">
         <is>
-          <t>5ec68f33756a2f8f7606ead5febd7f33ed18c280</t>
+          <t>219bc0a98e52a6b4cd0d3939d181df307abb678d</t>
         </is>
       </c>
     </row>
@@ -19396,7 +19398,7 @@
         </is>
       </c>
       <c r="C33" s="17" t="n">
-        <v>1655</v>
+        <v>1665</v>
       </c>
       <c r="D33" s="8" t="n">
         <v>1</v>
@@ -19411,7 +19413,7 @@
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
-          <t>712 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>425 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H33" s="8" t="inlineStr">
@@ -19420,7 +19422,7 @@
         </is>
       </c>
       <c r="I33" s="8" t="n">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="J33" s="8" t="n"/>
       <c r="K33" s="8" t="n"/>
@@ -19461,7 +19463,7 @@
       <c r="V33" s="7" t="inlineStr"/>
       <c r="W33" s="8" t="inlineStr">
         <is>
-          <t>219bc0a98e52a6b4cd0d3939d181df307abb678d</t>
+          <t>51bc0e8bb190437e4c5c4710bf40ee90758a79f0</t>
         </is>
       </c>
     </row>
@@ -19475,13 +19477,13 @@
         </is>
       </c>
       <c r="C34" s="17" t="n">
-        <v>1665</v>
+        <v>1650</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
@@ -19490,7 +19492,7 @@
       </c>
       <c r="G34" s="9" t="inlineStr">
         <is>
-          <t>425 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>Sweetman Place, Bristol, BS2</t>
         </is>
       </c>
       <c r="H34" s="8" t="inlineStr">
@@ -19498,15 +19500,13 @@
           <t>BS2</t>
         </is>
       </c>
-      <c r="I34" s="8" t="n">
-        <v>548</v>
-      </c>
+      <c r="I34" s="8" t="n"/>
       <c r="J34" s="8" t="n"/>
       <c r="K34" s="8" t="n"/>
       <c r="L34" s="8" t="n"/>
       <c r="M34" s="8" t="n"/>
       <c r="N34" s="8" t="n">
-        <v>20800</v>
+        <v>20416</v>
       </c>
       <c r="O34" s="8" t="n">
         <v>0</v>
@@ -19514,12 +19514,12 @@
       <c r="P34" s="8" t="n"/>
       <c r="Q34" s="8" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>Andrews Letting and Management, Clifton</t>
         </is>
       </c>
       <c r="S34" s="9" t="inlineStr">
@@ -19540,7 +19540,7 @@
       <c r="V34" s="7" t="inlineStr"/>
       <c r="W34" s="8" t="inlineStr">
         <is>
-          <t>51bc0e8bb190437e4c5c4710bf40ee90758a79f0</t>
+          <t>54fa42ef8d0349a295f45392644c43dec3321c5b</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
House search data from run 60
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -2280,7 +2280,9 @@
       <c r="K21" s="2" t="n"/>
       <c r="L21" s="2" t="n"/>
       <c r="M21" s="2" t="n"/>
-      <c r="N21" s="2" t="n"/>
+      <c r="N21" s="2" t="n">
+        <v>21392</v>
+      </c>
       <c r="O21" s="2" t="n">
         <v>0</v>
       </c>
@@ -6695,7 +6697,7 @@
         <v>21504</v>
       </c>
       <c r="O78" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P78" s="2" t="n"/>
       <c r="Q78" s="2" t="inlineStr">
@@ -9215,7 +9217,9 @@
       <c r="K112" s="2" t="n"/>
       <c r="L112" s="2" t="n"/>
       <c r="M112" s="2" t="n"/>
-      <c r="N112" s="2" t="n"/>
+      <c r="N112" s="2" t="n">
+        <v>21504</v>
+      </c>
       <c r="O112" s="2" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
House search data from run 63
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$204</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$197</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -600,7 +600,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199 U200 U201 U202 U203 U204" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -614,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W204"/>
+  <dimension ref="A1:W197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8816,7 +8816,7 @@
         </is>
       </c>
       <c r="C107" s="4" t="n">
-        <v>1250</v>
+        <v>1670</v>
       </c>
       <c r="D107" s="2" t="n">
         <v>1</v>
@@ -8831,21 +8831,23 @@
       </c>
       <c r="G107" s="3" t="inlineStr">
         <is>
-          <t>Southville, Bristol, BS3</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I107" s="2" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="n">
+        <v>553</v>
+      </c>
       <c r="J107" s="2" t="n"/>
       <c r="K107" s="2" t="n"/>
       <c r="L107" s="2" t="n"/>
       <c r="M107" s="2" t="n"/>
       <c r="N107" s="2" t="n">
-        <v>11576</v>
+        <v>20820</v>
       </c>
       <c r="O107" s="2" t="n">
         <v>0</v>
@@ -8858,7 +8860,7 @@
       </c>
       <c r="R107" s="2" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S107" s="3" t="inlineStr"/>
@@ -8875,7 +8877,7 @@
       <c r="V107" s="6" t="inlineStr"/>
       <c r="W107" s="2" t="inlineStr">
         <is>
-          <t>805d107aec4cff74fe0c62f5dbc8a4b4cfbadeec</t>
+          <t>356b325a4d0cab2ee5015a2e235f5fd99b2faa91</t>
         </is>
       </c>
     </row>
@@ -8889,7 +8891,7 @@
         </is>
       </c>
       <c r="C108" s="4" t="n">
-        <v>1670</v>
+        <v>1890</v>
       </c>
       <c r="D108" s="2" t="n">
         <v>1</v>
@@ -8913,7 +8915,7 @@
         </is>
       </c>
       <c r="I108" s="2" t="n">
-        <v>553</v>
+        <v>538</v>
       </c>
       <c r="J108" s="2" t="n"/>
       <c r="K108" s="2" t="n"/>
@@ -8950,7 +8952,7 @@
       <c r="V108" s="6" t="inlineStr"/>
       <c r="W108" s="2" t="inlineStr">
         <is>
-          <t>356b325a4d0cab2ee5015a2e235f5fd99b2faa91</t>
+          <t>f819b6d7cea8e4f9f3bc624d2737801ca68a6b49</t>
         </is>
       </c>
     </row>
@@ -8964,38 +8966,36 @@
         </is>
       </c>
       <c r="C109" s="4" t="n">
-        <v>1890</v>
+        <v>2050</v>
       </c>
       <c r="D109" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G109" s="3" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Webb Street, Bristol, BS5</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I109" s="2" t="n">
-        <v>538</v>
-      </c>
+          <t>BS5</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="n"/>
       <c r="J109" s="2" t="n"/>
       <c r="K109" s="2" t="n"/>
       <c r="L109" s="2" t="n"/>
       <c r="M109" s="2" t="n"/>
       <c r="N109" s="2" t="n">
-        <v>20820</v>
+        <v>19580</v>
       </c>
       <c r="O109" s="2" t="n">
         <v>0</v>
@@ -9008,7 +9008,7 @@
       </c>
       <c r="R109" s="2" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S109" s="3" t="inlineStr"/>
@@ -9025,7 +9025,7 @@
       <c r="V109" s="6" t="inlineStr"/>
       <c r="W109" s="2" t="inlineStr">
         <is>
-          <t>f819b6d7cea8e4f9f3bc624d2737801ca68a6b49</t>
+          <t>aef99c3165f6b6530e2b7bb4c35465760a386735</t>
         </is>
       </c>
     </row>
@@ -9039,36 +9039,38 @@
         </is>
       </c>
       <c r="C110" s="4" t="n">
-        <v>2050</v>
+        <v>1615</v>
       </c>
       <c r="D110" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E110" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G110" s="3" t="inlineStr">
         <is>
-          <t>Webb Street, Bristol, BS5</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>BS5</t>
-        </is>
-      </c>
-      <c r="I110" s="2" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="n">
+        <v>487</v>
+      </c>
       <c r="J110" s="2" t="n"/>
       <c r="K110" s="2" t="n"/>
       <c r="L110" s="2" t="n"/>
       <c r="M110" s="2" t="n"/>
       <c r="N110" s="2" t="n">
-        <v>19580</v>
+        <v>21504</v>
       </c>
       <c r="O110" s="2" t="n">
         <v>0</v>
@@ -9081,7 +9083,7 @@
       </c>
       <c r="R110" s="2" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S110" s="3" t="inlineStr"/>
@@ -9098,7 +9100,7 @@
       <c r="V110" s="6" t="inlineStr"/>
       <c r="W110" s="2" t="inlineStr">
         <is>
-          <t>aef99c3165f6b6530e2b7bb4c35465760a386735</t>
+          <t>9cff0990c507752682af58c22f5de8882d7b889a</t>
         </is>
       </c>
     </row>
@@ -9112,7 +9114,7 @@
         </is>
       </c>
       <c r="C111" s="4" t="n">
-        <v>1615</v>
+        <v>1500</v>
       </c>
       <c r="D111" s="2" t="n">
         <v>1</v>
@@ -9127,23 +9129,21 @@
       </c>
       <c r="G111" s="3" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Cutting Room, Bedminster</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I111" s="2" t="n">
-        <v>487</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="n"/>
       <c r="J111" s="2" t="n"/>
       <c r="K111" s="2" t="n"/>
       <c r="L111" s="2" t="n"/>
       <c r="M111" s="2" t="n"/>
       <c r="N111" s="2" t="n">
-        <v>21504</v>
+        <v>13796</v>
       </c>
       <c r="O111" s="2" t="n">
         <v>0</v>
@@ -9156,7 +9156,7 @@
       </c>
       <c r="R111" s="2" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Taylors Lettings, Bedminster</t>
         </is>
       </c>
       <c r="S111" s="3" t="inlineStr"/>
@@ -9173,7 +9173,7 @@
       <c r="V111" s="6" t="inlineStr"/>
       <c r="W111" s="2" t="inlineStr">
         <is>
-          <t>9cff0990c507752682af58c22f5de8882d7b889a</t>
+          <t>9c1c90149ff9e9ef3f44e220729613570307258e</t>
         </is>
       </c>
     </row>
@@ -9187,7 +9187,7 @@
         </is>
       </c>
       <c r="C112" s="4" t="n">
-        <v>1500</v>
+        <v>1250</v>
       </c>
       <c r="D112" s="2" t="n">
         <v>1</v>
@@ -9202,7 +9202,7 @@
       </c>
       <c r="G112" s="3" t="inlineStr">
         <is>
-          <t>Cutting Room, Bedminster</t>
+          <t>Southville, Bristol, BS3</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
@@ -9216,7 +9216,7 @@
       <c r="L112" s="2" t="n"/>
       <c r="M112" s="2" t="n"/>
       <c r="N112" s="2" t="n">
-        <v>13796</v>
+        <v>11576</v>
       </c>
       <c r="O112" s="2" t="n">
         <v>0</v>
@@ -9229,7 +9229,7 @@
       </c>
       <c r="R112" s="2" t="inlineStr">
         <is>
-          <t>Taylors Lettings, Bedminster</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S112" s="3" t="inlineStr"/>
@@ -9246,7 +9246,7 @@
       <c r="V112" s="6" t="inlineStr"/>
       <c r="W112" s="2" t="inlineStr">
         <is>
-          <t>9c1c90149ff9e9ef3f44e220729613570307258e</t>
+          <t>805d107aec4cff74fe0c62f5dbc8a4b4cfbadeec</t>
         </is>
       </c>
     </row>
@@ -15521,525 +15521,10 @@
         </is>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B198" s="3" t="inlineStr">
-        <is>
-          <t>Keyword match only (no API key configured for full scoring).</t>
-        </is>
-      </c>
-      <c r="C198" s="4" t="n">
-        <v>2085</v>
-      </c>
-      <c r="D198" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E198" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F198" s="2" t="inlineStr">
-        <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="G198" s="3" t="inlineStr">
-        <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
-        </is>
-      </c>
-      <c r="H198" s="2" t="inlineStr">
-        <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I198" s="2" t="n">
-        <v>722</v>
-      </c>
-      <c r="J198" s="2" t="n"/>
-      <c r="K198" s="2" t="n"/>
-      <c r="L198" s="2" t="n"/>
-      <c r="M198" s="2" t="n"/>
-      <c r="N198" s="2" t="n">
-        <v>21504</v>
-      </c>
-      <c r="O198" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P198" s="2" t="n"/>
-      <c r="Q198" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="R198" s="2" t="inlineStr">
-        <is>
-          <t>Grainger, Millwrights Place</t>
-        </is>
-      </c>
-      <c r="S198" s="3" t="inlineStr"/>
-      <c r="T198" s="5" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U198" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V198" s="6" t="inlineStr"/>
-      <c r="W198" s="2" t="inlineStr">
-        <is>
-          <t>12a5f2c4f1be2a8f1a9b2c6cbe66191abf1d7975</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B199" s="3" t="inlineStr">
-        <is>
-          <t>Keyword match only (no API key configured for full scoring).</t>
-        </is>
-      </c>
-      <c r="C199" s="4" t="n">
-        <v>1640</v>
-      </c>
-      <c r="D199" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E199" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F199" s="2" t="inlineStr">
-        <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="G199" s="3" t="inlineStr">
-        <is>
-          <t>Glasshouse Square Bristol BS1</t>
-        </is>
-      </c>
-      <c r="H199" s="2" t="inlineStr">
-        <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I199" s="2" t="n">
-        <v>570</v>
-      </c>
-      <c r="J199" s="2" t="n"/>
-      <c r="K199" s="2" t="n"/>
-      <c r="L199" s="2" t="n"/>
-      <c r="M199" s="2" t="n"/>
-      <c r="N199" s="2" t="n">
-        <v>20820</v>
-      </c>
-      <c r="O199" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P199" s="2" t="n"/>
-      <c r="Q199" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="R199" s="2" t="inlineStr">
-        <is>
-          <t>Grainger, Glasshouse Square</t>
-        </is>
-      </c>
-      <c r="S199" s="3" t="inlineStr"/>
-      <c r="T199" s="5" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U199" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V199" s="6" t="inlineStr"/>
-      <c r="W199" s="2" t="inlineStr">
-        <is>
-          <t>f7afd1bbb106a22d180a78614dde509c1dbfa8c1</t>
-        </is>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B200" s="3" t="inlineStr">
-        <is>
-          <t>Keyword match only (no API key configured for full scoring).</t>
-        </is>
-      </c>
-      <c r="C200" s="4" t="n">
-        <v>1595</v>
-      </c>
-      <c r="D200" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E200" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F200" s="2" t="inlineStr">
-        <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="G200" s="3" t="inlineStr">
-        <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
-        </is>
-      </c>
-      <c r="H200" s="2" t="inlineStr">
-        <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I200" s="2" t="n">
-        <v>499</v>
-      </c>
-      <c r="J200" s="2" t="n"/>
-      <c r="K200" s="2" t="n"/>
-      <c r="L200" s="2" t="n"/>
-      <c r="M200" s="2" t="n"/>
-      <c r="N200" s="2" t="n"/>
-      <c r="O200" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P200" s="2" t="n"/>
-      <c r="Q200" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
-        </is>
-      </c>
-      <c r="R200" s="2" t="inlineStr">
-        <is>
-          <t>Grainger, Hawkins &amp; George</t>
-        </is>
-      </c>
-      <c r="S200" s="3" t="inlineStr"/>
-      <c r="T200" s="5" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U200" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V200" s="6" t="inlineStr"/>
-      <c r="W200" s="2" t="inlineStr">
-        <is>
-          <t>f2f3afa9f34b35c1d7d84b8e8f6c80b9a91340b1</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B201" s="3" t="inlineStr">
-        <is>
-          <t>Keyword match only (no API key configured for full scoring).</t>
-        </is>
-      </c>
-      <c r="C201" s="4" t="n">
-        <v>1625</v>
-      </c>
-      <c r="D201" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E201" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F201" s="2" t="inlineStr">
-        <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="G201" s="3" t="inlineStr">
-        <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
-        </is>
-      </c>
-      <c r="H201" s="2" t="inlineStr">
-        <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I201" s="2" t="n">
-        <v>485</v>
-      </c>
-      <c r="J201" s="2" t="n"/>
-      <c r="K201" s="2" t="n"/>
-      <c r="L201" s="2" t="n"/>
-      <c r="M201" s="2" t="n"/>
-      <c r="N201" s="2" t="n"/>
-      <c r="O201" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P201" s="2" t="n"/>
-      <c r="Q201" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-16</t>
-        </is>
-      </c>
-      <c r="R201" s="2" t="inlineStr">
-        <is>
-          <t>Grainger, Millwrights Place</t>
-        </is>
-      </c>
-      <c r="S201" s="3" t="inlineStr"/>
-      <c r="T201" s="5" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U201" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V201" s="6" t="inlineStr"/>
-      <c r="W201" s="2" t="inlineStr">
-        <is>
-          <t>ea3758a9fd1b4190b4e5ae17519645f00d2e6a8f</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B202" s="3" t="inlineStr">
-        <is>
-          <t>Keyword match only (no API key configured for full scoring).</t>
-        </is>
-      </c>
-      <c r="C202" s="4" t="n">
-        <v>2175</v>
-      </c>
-      <c r="D202" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E202" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F202" s="2" t="inlineStr">
-        <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="G202" s="3" t="inlineStr">
-        <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
-        </is>
-      </c>
-      <c r="H202" s="2" t="inlineStr">
-        <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I202" s="2" t="n">
-        <v>722</v>
-      </c>
-      <c r="J202" s="2" t="n"/>
-      <c r="K202" s="2" t="n"/>
-      <c r="L202" s="2" t="n"/>
-      <c r="M202" s="2" t="n"/>
-      <c r="N202" s="2" t="n"/>
-      <c r="O202" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P202" s="2" t="n"/>
-      <c r="Q202" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="R202" s="2" t="inlineStr">
-        <is>
-          <t>Grainger, Millwrights Place</t>
-        </is>
-      </c>
-      <c r="S202" s="3" t="inlineStr"/>
-      <c r="T202" s="5" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U202" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V202" s="6" t="inlineStr"/>
-      <c r="W202" s="2" t="inlineStr">
-        <is>
-          <t>ab566c9b065047cd166a2ad3ae56e88704bc1358</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B203" s="3" t="inlineStr">
-        <is>
-          <t>Keyword match only (no API key configured for full scoring).</t>
-        </is>
-      </c>
-      <c r="C203" s="4" t="n">
-        <v>1900</v>
-      </c>
-      <c r="D203" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E203" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F203" s="2" t="inlineStr">
-        <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="G203" s="3" t="inlineStr">
-        <is>
-          <t>The Granary, Queen Charlotte Street, BRISTOL, BS1</t>
-        </is>
-      </c>
-      <c r="H203" s="2" t="inlineStr">
-        <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I203" s="2" t="n"/>
-      <c r="J203" s="2" t="n"/>
-      <c r="K203" s="2" t="n"/>
-      <c r="L203" s="2" t="n"/>
-      <c r="M203" s="2" t="n"/>
-      <c r="N203" s="2" t="n"/>
-      <c r="O203" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P203" s="2" t="n"/>
-      <c r="Q203" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="R203" s="2" t="inlineStr">
-        <is>
-          <t>Andrews Letting and Management, Clifton</t>
-        </is>
-      </c>
-      <c r="S203" s="3" t="inlineStr"/>
-      <c r="T203" s="5" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U203" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V203" s="6" t="inlineStr"/>
-      <c r="W203" s="2" t="inlineStr">
-        <is>
-          <t>b19bc62dddbc90526344a15be65fbc2e74a96d22</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B204" s="3" t="inlineStr">
-        <is>
-          <t>Keyword match only (no API key configured for full scoring).</t>
-        </is>
-      </c>
-      <c r="C204" s="4" t="n">
-        <v>2145</v>
-      </c>
-      <c r="D204" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E204" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F204" s="2" t="inlineStr">
-        <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="G204" s="3" t="inlineStr">
-        <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
-        </is>
-      </c>
-      <c r="H204" s="2" t="inlineStr">
-        <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I204" s="2" t="n">
-        <v>796</v>
-      </c>
-      <c r="J204" s="2" t="n"/>
-      <c r="K204" s="2" t="n"/>
-      <c r="L204" s="2" t="n"/>
-      <c r="M204" s="2" t="n"/>
-      <c r="N204" s="2" t="n">
-        <v>20820</v>
-      </c>
-      <c r="O204" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P204" s="2" t="n"/>
-      <c r="Q204" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="R204" s="2" t="inlineStr">
-        <is>
-          <t>Grainger, Glasshouse Square</t>
-        </is>
-      </c>
-      <c r="S204" s="3" t="inlineStr"/>
-      <c r="T204" s="5" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U204" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V204" s="6" t="inlineStr"/>
-      <c r="W204" s="2" t="inlineStr">
-        <is>
-          <t>898ba227d5b949e4e7f18b49536b3c908560d145</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:W204"/>
+  <autoFilter ref="A1:W197"/>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199 U200 U201 U202 U203 U204" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -16240,13 +15725,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T195" r:id="rId194"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T196" r:id="rId195"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T197" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T198" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T199" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T200" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T201" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T202" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T203" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T204" r:id="rId203"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
House search data from run 81
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$171</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$169</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -600,7 +600,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -614,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W171"/>
+  <dimension ref="A1:W169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1006,14 +1006,12 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1450</v>
+        <v>1400</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="E5" s="2" t="n"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>flat</t>
@@ -1021,7 +1019,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>The Crescent, Bristol, BS1</t>
+          <t>Millennium Promenade, Bristol, BS1</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1035,7 +1033,7 @@
       <c r="L5" s="2" t="n"/>
       <c r="M5" s="2" t="n"/>
       <c r="N5" s="2" t="n">
-        <v>16792</v>
+        <v>16168</v>
       </c>
       <c r="O5" s="2" t="n">
         <v>0</v>
@@ -1043,12 +1041,12 @@
       <c r="P5" s="2" t="n"/>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Phoenix Property Company, Bristol</t>
         </is>
       </c>
       <c r="S5" s="3" t="inlineStr">
@@ -1069,7 +1067,7 @@
       <c r="V5" s="6" t="inlineStr"/>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>d447d1158e90abd2c82eb7828f8a98e7f5fbe2bd</t>
+          <t>5ec68f33756a2f8f7606ead5febd7f33ed18c280</t>
         </is>
       </c>
     </row>
@@ -1083,12 +1081,14 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1400</v>
+        <v>4333</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="2" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>flat</t>
@@ -1096,21 +1096,23 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Millennium Promenade, Bristol, BS1</t>
+          <t>Portland Square 19, Bristol City, England</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1023</v>
+      </c>
       <c r="J6" s="2" t="n"/>
       <c r="K6" s="2" t="n"/>
       <c r="L6" s="2" t="n"/>
       <c r="M6" s="2" t="n"/>
       <c r="N6" s="2" t="n">
-        <v>16168</v>
+        <v>21392</v>
       </c>
       <c r="O6" s="2" t="n">
         <v>0</v>
@@ -1118,12 +1120,12 @@
       <c r="P6" s="2" t="n"/>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>Phoenix Property Company, Bristol</t>
+          <t>Upgraded Property Management, Bristol</t>
         </is>
       </c>
       <c r="S6" s="3" t="inlineStr">
@@ -1144,7 +1146,7 @@
       <c r="V6" s="6" t="inlineStr"/>
       <c r="W6" s="2" t="inlineStr">
         <is>
-          <t>5ec68f33756a2f8f7606ead5febd7f33ed18c280</t>
+          <t>36c6ae3217cb986edf670dca0e32cced89b1f8ef</t>
         </is>
       </c>
     </row>
@@ -1158,13 +1160,13 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>4333</v>
+        <v>1650</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -1173,23 +1175,21 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Portland Square 19, Bristol City, England</t>
+          <t>Deanery Road, Bristol, BS1</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="n">
-        <v>1023</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="n"/>
       <c r="J7" s="2" t="n"/>
       <c r="K7" s="2" t="n"/>
       <c r="L7" s="2" t="n"/>
       <c r="M7" s="2" t="n"/>
       <c r="N7" s="2" t="n">
-        <v>21392</v>
+        <v>11916</v>
       </c>
       <c r="O7" s="2" t="n">
         <v>0</v>
@@ -1197,12 +1197,12 @@
       <c r="P7" s="2" t="n"/>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>Upgraded Property Management, Bristol</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S7" s="3" t="inlineStr">
@@ -1223,7 +1223,7 @@
       <c r="V7" s="6" t="inlineStr"/>
       <c r="W7" s="2" t="inlineStr">
         <is>
-          <t>36c6ae3217cb986edf670dca0e32cced89b1f8ef</t>
+          <t>15ee559ffc7409539eee4e435f932975b92b010e</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Deanery Road, Bristol, BS1</t>
+          <t>Horizon, Broad Weir, BS1</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1266,7 +1266,7 @@
       <c r="L8" s="2" t="n"/>
       <c r="M8" s="2" t="n"/>
       <c r="N8" s="2" t="n">
-        <v>11916</v>
+        <v>21996</v>
       </c>
       <c r="O8" s="2" t="n">
         <v>0</v>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="S8" s="3" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T8" s="5" t="inlineStr">
@@ -1300,7 +1300,7 @@
       <c r="V8" s="6" t="inlineStr"/>
       <c r="W8" s="2" t="inlineStr">
         <is>
-          <t>15ee559ffc7409539eee4e435f932975b92b010e</t>
+          <t>48fa0ece469b09f31eb9d082a42a7c6ed00c6aac</t>
         </is>
       </c>
     </row>
@@ -1314,13 +1314,13 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>1650</v>
+        <v>1700</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -1329,12 +1329,12 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Horizon, Broad Weir, BS1</t>
+          <t>City Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I9" s="2" t="n"/>
@@ -1343,7 +1343,7 @@
       <c r="L9" s="2" t="n"/>
       <c r="M9" s="2" t="n"/>
       <c r="N9" s="2" t="n">
-        <v>21996</v>
+        <v>21256</v>
       </c>
       <c r="O9" s="2" t="n">
         <v>0</v>
@@ -1351,12 +1351,12 @@
       <c r="P9" s="2" t="n"/>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Howard, Bristol</t>
         </is>
       </c>
       <c r="S9" s="3" t="inlineStr">
@@ -1377,7 +1377,7 @@
       <c r="V9" s="6" t="inlineStr"/>
       <c r="W9" s="2" t="inlineStr">
         <is>
-          <t>48fa0ece469b09f31eb9d082a42a7c6ed00c6aac</t>
+          <t>bd0c4d092ffc5f51dc8a4f1bb0b8ba6bc8e71933</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>1700</v>
+        <v>1900</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>2</v>
@@ -1406,12 +1406,12 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>City Road, Bristol, BS2</t>
+          <t>Deanery Road, BRISTOL</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I10" s="2" t="n"/>
@@ -1420,7 +1420,7 @@
       <c r="L10" s="2" t="n"/>
       <c r="M10" s="2" t="n"/>
       <c r="N10" s="2" t="n">
-        <v>21256</v>
+        <v>11916</v>
       </c>
       <c r="O10" s="2" t="n">
         <v>0</v>
@@ -1428,17 +1428,17 @@
       <c r="P10" s="2" t="n"/>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>Howard, Bristol</t>
+          <t>Allen &amp; Harris, Clifton</t>
         </is>
       </c>
       <c r="S10" s="3" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T10" s="5" t="inlineStr">
@@ -1454,7 +1454,7 @@
       <c r="V10" s="6" t="inlineStr"/>
       <c r="W10" s="2" t="inlineStr">
         <is>
-          <t>bd0c4d092ffc5f51dc8a4f1bb0b8ba6bc8e71933</t>
+          <t>7de28a016a4c688c515861dbb81f78d510e563cb</t>
         </is>
       </c>
     </row>
@@ -1468,10 +1468,10 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1900</v>
+        <v>2830</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2</v>
@@ -1483,21 +1483,23 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Deanery Road, BRISTOL</t>
+          <t>315 Dovetail, New Kingsley Road, St Philips, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>1120</v>
+      </c>
       <c r="J11" s="2" t="n"/>
       <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="n"/>
       <c r="M11" s="2" t="n"/>
       <c r="N11" s="2" t="n">
-        <v>11916</v>
+        <v>21152</v>
       </c>
       <c r="O11" s="2" t="n">
         <v>0</v>
@@ -1505,12 +1507,12 @@
       <c r="P11" s="2" t="n"/>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>Allen &amp; Harris, Clifton</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S11" s="3" t="inlineStr">
@@ -1531,7 +1533,7 @@
       <c r="V11" s="6" t="inlineStr"/>
       <c r="W11" s="2" t="inlineStr">
         <is>
-          <t>7de28a016a4c688c515861dbb81f78d510e563cb</t>
+          <t>b70e24d9417674d7a16e52abd8d5a34b925d04ea</t>
         </is>
       </c>
     </row>
@@ -1545,13 +1547,13 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>2830</v>
+        <v>1550</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -1560,7 +1562,7 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>315 Dovetail, New Kingsley Road, St Philips, Bristol, Bristol City</t>
+          <t>City Road, St Pauls, Bristol, BS2</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1569,14 +1571,14 @@
         </is>
       </c>
       <c r="I12" s="2" t="n">
-        <v>1120</v>
+        <v>872</v>
       </c>
       <c r="J12" s="2" t="n"/>
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="n"/>
       <c r="M12" s="2" t="n"/>
       <c r="N12" s="2" t="n">
-        <v>21152</v>
+        <v>13004</v>
       </c>
       <c r="O12" s="2" t="n">
         <v>0</v>
@@ -1584,17 +1586,17 @@
       <c r="P12" s="2" t="n"/>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>CJ Hole, Bishopston</t>
         </is>
       </c>
       <c r="S12" s="3" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T12" s="5" t="inlineStr">
@@ -1610,7 +1612,7 @@
       <c r="V12" s="6" t="inlineStr"/>
       <c r="W12" s="2" t="inlineStr">
         <is>
-          <t>b70e24d9417674d7a16e52abd8d5a34b925d04ea</t>
+          <t>f0084682d29703f51fa0be542fd382e673d76549</t>
         </is>
       </c>
     </row>
@@ -1624,10 +1626,10 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1550</v>
+        <v>1450</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>1</v>
@@ -1639,7 +1641,7 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>City Road, St Pauls, Bristol, BS2</t>
+          <t>Norfolk House, Norfolk Avenue, St Paul's, BS2</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1647,15 +1649,13 @@
           <t>BS2</t>
         </is>
       </c>
-      <c r="I13" s="2" t="n">
-        <v>872</v>
-      </c>
+      <c r="I13" s="2" t="n"/>
       <c r="J13" s="2" t="n"/>
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="n"/>
       <c r="M13" s="2" t="n"/>
       <c r="N13" s="2" t="n">
-        <v>13004</v>
+        <v>14016</v>
       </c>
       <c r="O13" s="2" t="n">
         <v>0</v>
@@ -1663,17 +1663,17 @@
       <c r="P13" s="2" t="n"/>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>CJ Hole, Bishopston</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S13" s="3" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T13" s="5" t="inlineStr">
@@ -1689,7 +1689,7 @@
       <c r="V13" s="6" t="inlineStr"/>
       <c r="W13" s="2" t="inlineStr">
         <is>
-          <t>f0084682d29703f51fa0be542fd382e673d76549</t>
+          <t>a6e3aa5da01b2c2d03e0168a413f098ce4121aa0</t>
         </is>
       </c>
     </row>
@@ -1703,13 +1703,13 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1450</v>
+        <v>1850</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -1718,12 +1718,12 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Norfolk House, Norfolk Avenue, St Paul's, BS2</t>
+          <t>The Laureate, Charles Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I14" s="2" t="n"/>
@@ -1732,7 +1732,7 @@
       <c r="L14" s="2" t="n"/>
       <c r="M14" s="2" t="n"/>
       <c r="N14" s="2" t="n">
-        <v>14016</v>
+        <v>21912</v>
       </c>
       <c r="O14" s="2" t="n">
         <v>0</v>
@@ -1740,12 +1740,12 @@
       <c r="P14" s="2" t="n"/>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S14" s="3" t="inlineStr">
@@ -1766,7 +1766,7 @@
       <c r="V14" s="6" t="inlineStr"/>
       <c r="W14" s="2" t="inlineStr">
         <is>
-          <t>a6e3aa5da01b2c2d03e0168a413f098ce4121aa0</t>
+          <t>8d6d721187298dcfb94d30d9172f6f10952dc87d</t>
         </is>
       </c>
     </row>
@@ -1780,7 +1780,7 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1850</v>
+        <v>2000</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>2</v>
@@ -1795,7 +1795,7 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>The Laureate, Charles Street, Bristol, BS1</t>
+          <t>Anchorage, Gaol Ferry Steps, Bristol</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1809,7 +1809,7 @@
       <c r="L15" s="2" t="n"/>
       <c r="M15" s="2" t="n"/>
       <c r="N15" s="2" t="n">
-        <v>21912</v>
+        <v>16416</v>
       </c>
       <c r="O15" s="2" t="n">
         <v>0</v>
@@ -1822,7 +1822,7 @@
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Hopewell, Bristol</t>
         </is>
       </c>
       <c r="S15" s="3" t="inlineStr">
@@ -1843,7 +1843,7 @@
       <c r="V15" s="6" t="inlineStr"/>
       <c r="W15" s="2" t="inlineStr">
         <is>
-          <t>8d6d721187298dcfb94d30d9172f6f10952dc87d</t>
+          <t>1e517b09a4d3bd665354a55c719f877b837af199</t>
         </is>
       </c>
     </row>
@@ -1857,27 +1857,27 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>2000</v>
+        <v>2600</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Anchorage, Gaol Ferry Steps, Bristol</t>
+          <t>Norfolk Heights, BS2</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I16" s="2" t="n"/>
@@ -1886,7 +1886,7 @@
       <c r="L16" s="2" t="n"/>
       <c r="M16" s="2" t="n"/>
       <c r="N16" s="2" t="n">
-        <v>16416</v>
+        <v>21828</v>
       </c>
       <c r="O16" s="2" t="n">
         <v>0</v>
@@ -1899,7 +1899,7 @@
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>Hopewell, Bristol</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol</t>
         </is>
       </c>
       <c r="S16" s="3" t="inlineStr">
@@ -1920,7 +1920,7 @@
       <c r="V16" s="6" t="inlineStr"/>
       <c r="W16" s="2" t="inlineStr">
         <is>
-          <t>1e517b09a4d3bd665354a55c719f877b837af199</t>
+          <t>2c2a0756e18994fc5ddb57fd3f3b4e46f6b18829</t>
         </is>
       </c>
     </row>
@@ -1934,27 +1934,27 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>2600</v>
+        <v>1600</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Norfolk Heights, BS2</t>
+          <t>Magdalena Court, Redcliffe, Bristol City Centre</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I17" s="2" t="n"/>
@@ -1963,7 +1963,7 @@
       <c r="L17" s="2" t="n"/>
       <c r="M17" s="2" t="n"/>
       <c r="N17" s="2" t="n">
-        <v>21828</v>
+        <v>18672</v>
       </c>
       <c r="O17" s="2" t="n">
         <v>0</v>
@@ -1971,7 +1971,7 @@
       <c r="P17" s="2" t="n"/>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
@@ -1997,7 +1997,7 @@
       <c r="V17" s="6" t="inlineStr"/>
       <c r="W17" s="2" t="inlineStr">
         <is>
-          <t>2c2a0756e18994fc5ddb57fd3f3b4e46f6b18829</t>
+          <t>d1a94a3de68ac71225d3643c6e5ec331fbc7261e</t>
         </is>
       </c>
     </row>
@@ -2011,10 +2011,10 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>1600</v>
+        <v>1758</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>1</v>
@@ -2026,21 +2026,23 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Magdalena Court, Redcliffe, Bristol City Centre</t>
+          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="n"/>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>524</v>
+      </c>
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n"/>
       <c r="M18" s="2" t="n"/>
       <c r="N18" s="2" t="n">
-        <v>18672</v>
+        <v>11632</v>
       </c>
       <c r="O18" s="2" t="n">
         <v>0</v>
@@ -2053,7 +2055,7 @@
       </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol</t>
+          <t>CompassRock International, Stafford Yard</t>
         </is>
       </c>
       <c r="S18" s="3" t="inlineStr">
@@ -2074,7 +2076,7 @@
       <c r="V18" s="6" t="inlineStr"/>
       <c r="W18" s="2" t="inlineStr">
         <is>
-          <t>d1a94a3de68ac71225d3643c6e5ec331fbc7261e</t>
+          <t>2a07769bc6317adeb6dd550e1e056ddeac2ac129</t>
         </is>
       </c>
     </row>
@@ -2088,22 +2090,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1758</v>
+        <v>1800</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
+          <t>Osborne Road, Southville, Bristol, BS3</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -2111,15 +2113,13 @@
           <t>BS3</t>
         </is>
       </c>
-      <c r="I19" s="2" t="n">
-        <v>524</v>
-      </c>
+      <c r="I19" s="2" t="n"/>
       <c r="J19" s="2" t="n"/>
       <c r="K19" s="2" t="n"/>
       <c r="L19" s="2" t="n"/>
       <c r="M19" s="2" t="n"/>
       <c r="N19" s="2" t="n">
-        <v>11632</v>
+        <v>14028</v>
       </c>
       <c r="O19" s="2" t="n">
         <v>0</v>
@@ -2127,17 +2127,17 @@
       <c r="P19" s="2" t="n"/>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>CompassRock International, Stafford Yard</t>
+          <t>CJ Hole, Southville</t>
         </is>
       </c>
       <c r="S19" s="3" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T19" s="5" t="inlineStr">
@@ -2153,7 +2153,7 @@
       <c r="V19" s="6" t="inlineStr"/>
       <c r="W19" s="2" t="inlineStr">
         <is>
-          <t>2a07769bc6317adeb6dd550e1e056ddeac2ac129</t>
+          <t>69ee3b35f8d9109c2a36a94ae5b3d0b237a035bd</t>
         </is>
       </c>
     </row>
@@ -2173,21 +2173,21 @@
         <v>2</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Osborne Road, Southville, Bristol, BS3</t>
+          <t>The Panoramic, Park Row, BS1</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>BS3</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I20" s="2" t="n"/>
@@ -2196,7 +2196,7 @@
       <c r="L20" s="2" t="n"/>
       <c r="M20" s="2" t="n"/>
       <c r="N20" s="2" t="n">
-        <v>14028</v>
+        <v>20940</v>
       </c>
       <c r="O20" s="2" t="n">
         <v>0</v>
@@ -2209,12 +2209,12 @@
       </c>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>CJ Hole, Southville</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S20" s="3" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T20" s="5" t="inlineStr">
@@ -2230,7 +2230,7 @@
       <c r="V20" s="6" t="inlineStr"/>
       <c r="W20" s="2" t="inlineStr">
         <is>
-          <t>69ee3b35f8d9109c2a36a94ae5b3d0b237a035bd</t>
+          <t>454917a7536fb9944c891f2559e33e66404388a1</t>
         </is>
       </c>
     </row>
@@ -2244,13 +2244,13 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>1800</v>
+        <v>1250</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -2259,7 +2259,7 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>The Panoramic, Park Row, BS1</t>
+          <t>City Centre, Jessop Court, BS1</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -2267,13 +2267,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I21" s="2" t="n"/>
+      <c r="I21" s="2" t="n">
+        <v>538</v>
+      </c>
       <c r="J21" s="2" t="n"/>
       <c r="K21" s="2" t="n"/>
       <c r="L21" s="2" t="n"/>
       <c r="M21" s="2" t="n"/>
       <c r="N21" s="2" t="n">
-        <v>20940</v>
+        <v>20788</v>
       </c>
       <c r="O21" s="2" t="n">
         <v>0</v>
@@ -2281,12 +2283,12 @@
       <c r="P21" s="2" t="n"/>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S21" s="3" t="inlineStr">
@@ -2307,7 +2309,7 @@
       <c r="V21" s="6" t="inlineStr"/>
       <c r="W21" s="2" t="inlineStr">
         <is>
-          <t>454917a7536fb9944c891f2559e33e66404388a1</t>
+          <t>34093b6e05a2deb3da2e1a98a249e966d7af0cdf</t>
         </is>
       </c>
     </row>
@@ -2321,7 +2323,7 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>1758</v>
+        <v>1450</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>1</v>
@@ -2336,23 +2338,21 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
+          <t>The Crescent, Bristol, BS1</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="n">
-        <v>524</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="n"/>
       <c r="J22" s="2" t="n"/>
       <c r="K22" s="2" t="n"/>
       <c r="L22" s="2" t="n"/>
       <c r="M22" s="2" t="n"/>
       <c r="N22" s="2" t="n">
-        <v>11632</v>
+        <v>16792</v>
       </c>
       <c r="O22" s="2" t="n">
         <v>0</v>
@@ -2360,12 +2360,12 @@
       <c r="P22" s="2" t="n"/>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>CompassRock International, Stafford Yard</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S22" s="3" t="inlineStr">
@@ -2386,7 +2386,7 @@
       <c r="V22" s="6" t="inlineStr"/>
       <c r="W22" s="2" t="inlineStr">
         <is>
-          <t>cb7836e81328c8e3f4365c151c332c5f761e9d2b</t>
+          <t>d447d1158e90abd2c82eb7828f8a98e7f5fbe2bd</t>
         </is>
       </c>
     </row>
@@ -2400,7 +2400,7 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>1225</v>
+        <v>1758</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>1</v>
@@ -2415,21 +2415,23 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>New Walls, Totterdown, BS4</t>
+          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="n"/>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>524</v>
+      </c>
       <c r="J23" s="2" t="n"/>
       <c r="K23" s="2" t="n"/>
       <c r="L23" s="2" t="n"/>
       <c r="M23" s="2" t="n"/>
       <c r="N23" s="2" t="n">
-        <v>8540</v>
+        <v>11632</v>
       </c>
       <c r="O23" s="2" t="n">
         <v>0</v>
@@ -2437,12 +2439,12 @@
       <c r="P23" s="2" t="n"/>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>Bristol Property Centre, Bristol</t>
+          <t>CompassRock International, Stafford Yard</t>
         </is>
       </c>
       <c r="S23" s="3" t="inlineStr">
@@ -2463,7 +2465,7 @@
       <c r="V23" s="6" t="inlineStr"/>
       <c r="W23" s="2" t="inlineStr">
         <is>
-          <t>ff7cade97c52dbe0ee822ce3951fd4f71c9b4146</t>
+          <t>cb7836e81328c8e3f4365c151c332c5f761e9d2b</t>
         </is>
       </c>
     </row>
@@ -2477,13 +2479,13 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>2000</v>
+        <v>1225</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -2492,12 +2494,12 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>Caledonian Road, Bristol, BS1</t>
+          <t>New Walls, Totterdown, BS4</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS4</t>
         </is>
       </c>
       <c r="I24" s="2" t="n"/>
@@ -2506,7 +2508,7 @@
       <c r="L24" s="2" t="n"/>
       <c r="M24" s="2" t="n"/>
       <c r="N24" s="2" t="n">
-        <v>14632</v>
+        <v>8540</v>
       </c>
       <c r="O24" s="2" t="n">
         <v>0</v>
@@ -2514,12 +2516,12 @@
       <c r="P24" s="2" t="n"/>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="R24" s="2" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Bristol Property Centre, Bristol</t>
         </is>
       </c>
       <c r="S24" s="3" t="inlineStr">
@@ -2540,7 +2542,7 @@
       <c r="V24" s="6" t="inlineStr"/>
       <c r="W24" s="2" t="inlineStr">
         <is>
-          <t>9a270cf54e31627246aef21daa26a60bb5f977ad</t>
+          <t>ff7cade97c52dbe0ee822ce3951fd4f71c9b4146</t>
         </is>
       </c>
     </row>
@@ -2554,13 +2556,13 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>1400</v>
+        <v>2000</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -2569,7 +2571,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>The Crescent, Harbourside, BS1</t>
+          <t>Caledonian Road, Bristol, BS1</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -2583,7 +2585,7 @@
       <c r="L25" s="2" t="n"/>
       <c r="M25" s="2" t="n"/>
       <c r="N25" s="2" t="n">
-        <v>16368</v>
+        <v>14632</v>
       </c>
       <c r="O25" s="2" t="n">
         <v>0</v>
@@ -2591,12 +2593,12 @@
       <c r="P25" s="2" t="n"/>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R25" s="2" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S25" s="3" t="inlineStr">
@@ -2617,7 +2619,7 @@
       <c r="V25" s="6" t="inlineStr"/>
       <c r="W25" s="2" t="inlineStr">
         <is>
-          <t>59af10441dff618517a35c62d6a67a8485c2f2fa</t>
+          <t>9a270cf54e31627246aef21daa26a60bb5f977ad</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2633,7 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>1200</v>
+        <v>1400</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>1</v>
@@ -2646,12 +2648,12 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Union Road, Bristol BS2 0FN</t>
+          <t>The Crescent, Harbourside, BS1</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I26" s="2" t="n"/>
@@ -2660,7 +2662,7 @@
       <c r="L26" s="2" t="n"/>
       <c r="M26" s="2" t="n"/>
       <c r="N26" s="2" t="n">
-        <v>20144</v>
+        <v>16368</v>
       </c>
       <c r="O26" s="2" t="n">
         <v>0</v>
@@ -2668,12 +2670,12 @@
       <c r="P26" s="2" t="n"/>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R26" s="2" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S26" s="3" t="inlineStr">
@@ -2694,7 +2696,7 @@
       <c r="V26" s="6" t="inlineStr"/>
       <c r="W26" s="2" t="inlineStr">
         <is>
-          <t>2b2295e0c22bd50658835eb43d2eb433f6d1cd1b</t>
+          <t>59af10441dff618517a35c62d6a67a8485c2f2fa</t>
         </is>
       </c>
     </row>
@@ -2708,7 +2710,7 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>1758</v>
+        <v>1200</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>1</v>
@@ -2723,23 +2725,21 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
+          <t>Union Road, Bristol BS2 0FN</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="n">
-        <v>524</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="n"/>
       <c r="J27" s="2" t="n"/>
       <c r="K27" s="2" t="n"/>
       <c r="L27" s="2" t="n"/>
       <c r="M27" s="2" t="n"/>
       <c r="N27" s="2" t="n">
-        <v>11632</v>
+        <v>20144</v>
       </c>
       <c r="O27" s="2" t="n">
         <v>0</v>
@@ -2747,12 +2747,12 @@
       <c r="P27" s="2" t="n"/>
       <c r="Q27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="R27" s="2" t="inlineStr">
         <is>
-          <t>CompassRock International, Stafford Yard</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S27" s="3" t="inlineStr">
@@ -2773,7 +2773,7 @@
       <c r="V27" s="6" t="inlineStr"/>
       <c r="W27" s="2" t="inlineStr">
         <is>
-          <t>e01353518e32ee855b640499d951960a537bb160</t>
+          <t>2b2295e0c22bd50658835eb43d2eb433f6d1cd1b</t>
         </is>
       </c>
     </row>
@@ -2787,13 +2787,13 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>1900</v>
+        <v>1758</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -2802,21 +2802,23 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>51.02 - St James Barton</t>
+          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="n"/>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>524</v>
+      </c>
       <c r="J28" s="2" t="n"/>
       <c r="K28" s="2" t="n"/>
       <c r="L28" s="2" t="n"/>
       <c r="M28" s="2" t="n"/>
       <c r="N28" s="2" t="n">
-        <v>22132</v>
+        <v>11632</v>
       </c>
       <c r="O28" s="2" t="n">
         <v>0</v>
@@ -2824,12 +2826,12 @@
       <c r="P28" s="2" t="n"/>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R28" s="2" t="inlineStr">
         <is>
-          <t>Ocean, Clifton</t>
+          <t>CompassRock International, Stafford Yard</t>
         </is>
       </c>
       <c r="S28" s="3" t="inlineStr">
@@ -2850,7 +2852,7 @@
       <c r="V28" s="6" t="inlineStr"/>
       <c r="W28" s="2" t="inlineStr">
         <is>
-          <t>1d421f07eb2d142471d3e293f8cb751813656c56</t>
+          <t>e01353518e32ee855b640499d951960a537bb160</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2866,7 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1850</v>
+        <v>1900</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>2</v>
@@ -2879,7 +2881,7 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Horizon - City Centre</t>
+          <t>51.02 - St James Barton</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2893,7 +2895,7 @@
       <c r="L29" s="2" t="n"/>
       <c r="M29" s="2" t="n"/>
       <c r="N29" s="2" t="n">
-        <v>22020</v>
+        <v>22132</v>
       </c>
       <c r="O29" s="2" t="n">
         <v>0</v>
@@ -2901,7 +2903,7 @@
       <c r="P29" s="2" t="n"/>
       <c r="Q29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R29" s="2" t="inlineStr">
@@ -2911,7 +2913,7 @@
       </c>
       <c r="S29" s="3" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T29" s="5" t="inlineStr">
@@ -2927,7 +2929,7 @@
       <c r="V29" s="6" t="inlineStr"/>
       <c r="W29" s="2" t="inlineStr">
         <is>
-          <t>dcc16fa39cff678f7a157aec0c52e4b6b97a0fb3</t>
+          <t>1d421f07eb2d142471d3e293f8cb751813656c56</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2943,7 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>2300</v>
+        <v>1850</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>2</v>
@@ -2956,7 +2958,7 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Electricity House, Bristol, BS1</t>
+          <t>Horizon - City Centre</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2970,7 +2972,7 @@
       <c r="L30" s="2" t="n"/>
       <c r="M30" s="2" t="n"/>
       <c r="N30" s="2" t="n">
-        <v>21876</v>
+        <v>22020</v>
       </c>
       <c r="O30" s="2" t="n">
         <v>0</v>
@@ -2978,17 +2980,17 @@
       <c r="P30" s="2" t="n"/>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="R30" s="2" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Ocean, Clifton</t>
         </is>
       </c>
       <c r="S30" s="3" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T30" s="5" t="inlineStr">
@@ -3004,7 +3006,7 @@
       <c r="V30" s="6" t="inlineStr"/>
       <c r="W30" s="2" t="inlineStr">
         <is>
-          <t>35ca98fa51e87bf8bad5117293380e1cb3a5cc07</t>
+          <t>dcc16fa39cff678f7a157aec0c52e4b6b97a0fb3</t>
         </is>
       </c>
     </row>
@@ -3018,13 +3020,13 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>1500</v>
+        <v>2300</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -3033,7 +3035,7 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Horizon - City Centre</t>
+          <t>Electricity House, Bristol, BS1</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -3047,7 +3049,7 @@
       <c r="L31" s="2" t="n"/>
       <c r="M31" s="2" t="n"/>
       <c r="N31" s="2" t="n">
-        <v>22020</v>
+        <v>21876</v>
       </c>
       <c r="O31" s="2" t="n">
         <v>0</v>
@@ -3055,17 +3057,17 @@
       <c r="P31" s="2" t="n"/>
       <c r="Q31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="R31" s="2" t="inlineStr">
         <is>
-          <t>Ocean, Clifton</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S31" s="3" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T31" s="5" t="inlineStr">
@@ -3081,7 +3083,7 @@
       <c r="V31" s="6" t="inlineStr"/>
       <c r="W31" s="2" t="inlineStr">
         <is>
-          <t>25fbd71b098a83412bb2a614282b6fb33b9a3c90</t>
+          <t>35ca98fa51e87bf8bad5117293380e1cb3a5cc07</t>
         </is>
       </c>
     </row>
@@ -3095,10 +3097,10 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>1550</v>
+        <v>1500</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>1</v>
@@ -3110,12 +3112,12 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Beaufort Street, Stapleton, Bristol</t>
+          <t>Horizon - City Centre</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>BS5</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I32" s="2" t="n"/>
@@ -3124,7 +3126,7 @@
       <c r="L32" s="2" t="n"/>
       <c r="M32" s="2" t="n"/>
       <c r="N32" s="2" t="n">
-        <v>19400</v>
+        <v>22020</v>
       </c>
       <c r="O32" s="2" t="n">
         <v>0</v>
@@ -3132,17 +3134,17 @@
       <c r="P32" s="2" t="n"/>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="R32" s="2" t="inlineStr">
         <is>
-          <t>Taylors Lettings, Bradley Stoke</t>
+          <t>Ocean, Clifton</t>
         </is>
       </c>
       <c r="S32" s="3" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T32" s="5" t="inlineStr">
@@ -3158,7 +3160,7 @@
       <c r="V32" s="6" t="inlineStr"/>
       <c r="W32" s="2" t="inlineStr">
         <is>
-          <t>81712a02a3a8827c0a71232c3b582e0d2b990a2a</t>
+          <t>25fbd71b098a83412bb2a614282b6fb33b9a3c90</t>
         </is>
       </c>
     </row>
@@ -3172,12 +3174,14 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>2100</v>
+        <v>1550</v>
       </c>
       <c r="D33" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E33" s="2" t="n"/>
+      <c r="E33" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
           <t>flat</t>
@@ -3185,23 +3189,21 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>526 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>Beaufort Street, Stapleton, Bristol</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="n">
-        <v>800</v>
-      </c>
+          <t>BS5</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="n"/>
       <c r="J33" s="2" t="n"/>
       <c r="K33" s="2" t="n"/>
       <c r="L33" s="2" t="n"/>
       <c r="M33" s="2" t="n"/>
       <c r="N33" s="2" t="n">
-        <v>20800</v>
+        <v>19400</v>
       </c>
       <c r="O33" s="2" t="n">
         <v>0</v>
@@ -3209,12 +3211,12 @@
       <c r="P33" s="2" t="n"/>
       <c r="Q33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R33" s="2" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>Taylors Lettings, Bradley Stoke</t>
         </is>
       </c>
       <c r="S33" s="3" t="inlineStr">
@@ -3235,7 +3237,7 @@
       <c r="V33" s="6" t="inlineStr"/>
       <c r="W33" s="2" t="inlineStr">
         <is>
-          <t>74d41470c07849b906ad0a12b07a1745551d8e6f</t>
+          <t>81712a02a3a8827c0a71232c3b582e0d2b990a2a</t>
         </is>
       </c>
     </row>
@@ -3249,14 +3251,12 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>2120</v>
+        <v>2100</v>
       </c>
       <c r="D34" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E34" s="2" t="n">
-        <v>2</v>
-      </c>
+      <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
           <t>flat</t>
@@ -3264,7 +3264,7 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>522 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>526 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -3273,7 +3273,7 @@
         </is>
       </c>
       <c r="I34" s="2" t="n">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="J34" s="2" t="n"/>
       <c r="K34" s="2" t="n"/>
@@ -3314,7 +3314,7 @@
       <c r="V34" s="6" t="inlineStr"/>
       <c r="W34" s="2" t="inlineStr">
         <is>
-          <t>4a3dbf2b76e61d3a02d3b62cb6a5a56affeadff0</t>
+          <t>74d41470c07849b906ad0a12b07a1745551d8e6f</t>
         </is>
       </c>
     </row>
@@ -3328,7 +3328,7 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>2150</v>
+        <v>2120</v>
       </c>
       <c r="D35" s="2" t="n">
         <v>2</v>
@@ -3343,7 +3343,7 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>802 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>522 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -3352,7 +3352,7 @@
         </is>
       </c>
       <c r="I35" s="2" t="n">
-        <v>809</v>
+        <v>799</v>
       </c>
       <c r="J35" s="2" t="n"/>
       <c r="K35" s="2" t="n"/>
@@ -3393,7 +3393,7 @@
       <c r="V35" s="6" t="inlineStr"/>
       <c r="W35" s="2" t="inlineStr">
         <is>
-          <t>fcdcdd1da915be6f6b065ad9cbeea66062d00301</t>
+          <t>4a3dbf2b76e61d3a02d3b62cb6a5a56affeadff0</t>
         </is>
       </c>
     </row>
@@ -3407,10 +3407,10 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>2830</v>
+        <v>2150</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>2</v>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>315 Dovetail, New Kingsley Road, Bristol, BS2</t>
+          <t>802 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="I36" s="2" t="n">
-        <v>1120</v>
+        <v>809</v>
       </c>
       <c r="J36" s="2" t="n"/>
       <c r="K36" s="2" t="n"/>
@@ -3446,7 +3446,7 @@
       <c r="P36" s="2" t="n"/>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="R36" s="2" t="inlineStr">
@@ -3472,7 +3472,7 @@
       <c r="V36" s="6" t="inlineStr"/>
       <c r="W36" s="2" t="inlineStr">
         <is>
-          <t>e4f6deef9389498e73820b4056b013ac2b6ff363</t>
+          <t>fcdcdd1da915be6f6b065ad9cbeea66062d00301</t>
         </is>
       </c>
     </row>
@@ -3486,13 +3486,13 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>1680</v>
+        <v>2830</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>904 Dovetail, New Kingsley Road, Bristol, BS2</t>
+          <t>315 Dovetail, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -3510,7 +3510,7 @@
         </is>
       </c>
       <c r="I37" s="2" t="n">
-        <v>557</v>
+        <v>1120</v>
       </c>
       <c r="J37" s="2" t="n"/>
       <c r="K37" s="2" t="n"/>
@@ -3525,7 +3525,7 @@
       <c r="P37" s="2" t="n"/>
       <c r="Q37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="R37" s="2" t="inlineStr">
@@ -3551,7 +3551,7 @@
       <c r="V37" s="6" t="inlineStr"/>
       <c r="W37" s="2" t="inlineStr">
         <is>
-          <t>3d5fce4a62f2bd2b3bbd100f6bd7598155b266f2</t>
+          <t>e4f6deef9389498e73820b4056b013ac2b6ff363</t>
         </is>
       </c>
     </row>
@@ -3565,7 +3565,7 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>1715</v>
+        <v>1680</v>
       </c>
       <c r="D38" s="2" t="n">
         <v>1</v>
@@ -3580,7 +3580,7 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>1006 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>904 Dovetail, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -3589,7 +3589,7 @@
         </is>
       </c>
       <c r="I38" s="2" t="n">
-        <v>547</v>
+        <v>557</v>
       </c>
       <c r="J38" s="2" t="n"/>
       <c r="K38" s="2" t="n"/>
@@ -3630,7 +3630,7 @@
       <c r="V38" s="6" t="inlineStr"/>
       <c r="W38" s="2" t="inlineStr">
         <is>
-          <t>baed14f153217bbfa48df27148f4a5b45559a145</t>
+          <t>3d5fce4a62f2bd2b3bbd100f6bd7598155b266f2</t>
         </is>
       </c>
     </row>
@@ -3644,7 +3644,7 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>1655</v>
+        <v>1715</v>
       </c>
       <c r="D39" s="2" t="n">
         <v>1</v>
@@ -3659,7 +3659,7 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>712 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>1006 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -3683,7 +3683,7 @@
       <c r="P39" s="2" t="n"/>
       <c r="Q39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="R39" s="2" t="inlineStr">
@@ -3709,7 +3709,7 @@
       <c r="V39" s="6" t="inlineStr"/>
       <c r="W39" s="2" t="inlineStr">
         <is>
-          <t>219bc0a98e52a6b4cd0d3939d181df307abb678d</t>
+          <t>baed14f153217bbfa48df27148f4a5b45559a145</t>
         </is>
       </c>
     </row>
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>1665</v>
+        <v>1655</v>
       </c>
       <c r="D40" s="2" t="n">
         <v>1</v>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>425 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>712 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -3747,7 +3747,7 @@
         </is>
       </c>
       <c r="I40" s="2" t="n">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="J40" s="2" t="n"/>
       <c r="K40" s="2" t="n"/>
@@ -3788,7 +3788,7 @@
       <c r="V40" s="6" t="inlineStr"/>
       <c r="W40" s="2" t="inlineStr">
         <is>
-          <t>51bc0e8bb190437e4c5c4710bf40ee90758a79f0</t>
+          <t>219bc0a98e52a6b4cd0d3939d181df307abb678d</t>
         </is>
       </c>
     </row>
@@ -3802,13 +3802,13 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>2400</v>
+        <v>1665</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -3817,21 +3817,23 @@
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Gaol Ferry Steps, Bristol, BS1</t>
+          <t>425 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="n">
+        <v>548</v>
+      </c>
       <c r="J41" s="2" t="n"/>
       <c r="K41" s="2" t="n"/>
       <c r="L41" s="2" t="n"/>
       <c r="M41" s="2" t="n"/>
       <c r="N41" s="2" t="n">
-        <v>16416</v>
+        <v>20800</v>
       </c>
       <c r="O41" s="2" t="n">
         <v>0</v>
@@ -3839,12 +3841,12 @@
       <c r="P41" s="2" t="n"/>
       <c r="Q41" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="R41" s="2" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S41" s="3" t="inlineStr">
@@ -3865,7 +3867,7 @@
       <c r="V41" s="6" t="inlineStr"/>
       <c r="W41" s="2" t="inlineStr">
         <is>
-          <t>80580eaf8f14d71d98570c27e868e28d7528cf0d</t>
+          <t>51bc0e8bb190437e4c5c4710bf40ee90758a79f0</t>
         </is>
       </c>
     </row>
@@ -3879,7 +3881,7 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>1825</v>
+        <v>2400</v>
       </c>
       <c r="D42" s="2" t="n">
         <v>2</v>
@@ -3894,23 +3896,21 @@
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>Arnos Vale, Paintworks, BS4</t>
+          <t>Gaol Ferry Steps, Bristol, BS1</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="n">
-        <v>783</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="n"/>
       <c r="J42" s="2" t="n"/>
       <c r="K42" s="2" t="n"/>
       <c r="L42" s="2" t="n"/>
       <c r="M42" s="2" t="n"/>
       <c r="N42" s="2" t="n">
-        <v>4680</v>
+        <v>16416</v>
       </c>
       <c r="O42" s="2" t="n">
         <v>0</v>
@@ -3918,12 +3918,12 @@
       <c r="P42" s="2" t="n"/>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Acen Properties, Bristol</t>
         </is>
       </c>
       <c r="S42" s="3" t="inlineStr">
@@ -3944,7 +3944,7 @@
       <c r="V42" s="6" t="inlineStr"/>
       <c r="W42" s="2" t="inlineStr">
         <is>
-          <t>ec80bfb810dff72d9cbd21b8e12b70951ce557a7</t>
+          <t>80580eaf8f14d71d98570c27e868e28d7528cf0d</t>
         </is>
       </c>
     </row>
@@ -3958,7 +3958,7 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>1995</v>
+        <v>1825</v>
       </c>
       <c r="D43" s="2" t="n">
         <v>2</v>
@@ -3973,21 +3973,23 @@
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>Sugar House, French Yard, City Centre, Bristol, BS1</t>
+          <t>Arnos Vale, Paintworks, BS4</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="n"/>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="n">
+        <v>783</v>
+      </c>
       <c r="J43" s="2" t="n"/>
       <c r="K43" s="2" t="n"/>
       <c r="L43" s="2" t="n"/>
       <c r="M43" s="2" t="n"/>
       <c r="N43" s="2" t="n">
-        <v>18544</v>
+        <v>4680</v>
       </c>
       <c r="O43" s="2" t="n">
         <v>0</v>
@@ -3995,12 +3997,12 @@
       <c r="P43" s="2" t="n"/>
       <c r="Q43" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="R43" s="2" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S43" s="3" t="inlineStr">
@@ -4021,7 +4023,7 @@
       <c r="V43" s="6" t="inlineStr"/>
       <c r="W43" s="2" t="inlineStr">
         <is>
-          <t>f829bfa651ebc050b5c2fa24aea7bca4147d62c3</t>
+          <t>ec80bfb810dff72d9cbd21b8e12b70951ce557a7</t>
         </is>
       </c>
     </row>
@@ -4035,13 +4037,13 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>1600</v>
+        <v>1995</v>
       </c>
       <c r="D44" s="2" t="n">
         <v>2</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -4050,7 +4052,7 @@
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>St. Stephens Street, Bristol, BS1</t>
+          <t>Sugar House, French Yard, City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -4064,7 +4066,7 @@
       <c r="L44" s="2" t="n"/>
       <c r="M44" s="2" t="n"/>
       <c r="N44" s="2" t="n">
-        <v>21428</v>
+        <v>18544</v>
       </c>
       <c r="O44" s="2" t="n">
         <v>0</v>
@@ -4072,12 +4074,12 @@
       <c r="P44" s="2" t="n"/>
       <c r="Q44" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="R44" s="2" t="inlineStr">
         <is>
-          <t>Romans, Clifton</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S44" s="3" t="inlineStr">
@@ -4098,7 +4100,7 @@
       <c r="V44" s="6" t="inlineStr"/>
       <c r="W44" s="2" t="inlineStr">
         <is>
-          <t>cd770dd603af2e6f4f23a72c9685c7468c731a6d</t>
+          <t>f829bfa651ebc050b5c2fa24aea7bca4147d62c3</t>
         </is>
       </c>
     </row>
@@ -4112,13 +4114,13 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>1900</v>
+        <v>1600</v>
       </c>
       <c r="D45" s="2" t="n">
         <v>2</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -4127,7 +4129,7 @@
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>Wapping Wharf, Anchorage, BS1</t>
+          <t>St. Stephens Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -4135,15 +4137,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I45" s="2" t="n">
-        <v>799</v>
-      </c>
+      <c r="I45" s="2" t="n"/>
       <c r="J45" s="2" t="n"/>
       <c r="K45" s="2" t="n"/>
       <c r="L45" s="2" t="n"/>
       <c r="M45" s="2" t="n"/>
       <c r="N45" s="2" t="n">
-        <v>16416</v>
+        <v>21428</v>
       </c>
       <c r="O45" s="2" t="n">
         <v>0</v>
@@ -4151,12 +4151,12 @@
       <c r="P45" s="2" t="n"/>
       <c r="Q45" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="R45" s="2" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Romans, Clifton</t>
         </is>
       </c>
       <c r="S45" s="3" t="inlineStr">
@@ -4177,7 +4177,7 @@
       <c r="V45" s="6" t="inlineStr"/>
       <c r="W45" s="2" t="inlineStr">
         <is>
-          <t>6b74ba6dcca9cfc12cf5e5d10aaa942cfd63c0e6</t>
+          <t>cd770dd603af2e6f4f23a72c9685c7468c731a6d</t>
         </is>
       </c>
     </row>
@@ -4206,7 +4206,7 @@
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>City Centre, The Milliners, BS1 6WU</t>
+          <t>Wapping Wharf, Anchorage, BS1</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -4215,14 +4215,14 @@
         </is>
       </c>
       <c r="I46" s="2" t="n">
-        <v>818</v>
+        <v>799</v>
       </c>
       <c r="J46" s="2" t="n"/>
       <c r="K46" s="2" t="n"/>
       <c r="L46" s="2" t="n"/>
       <c r="M46" s="2" t="n"/>
       <c r="N46" s="2" t="n">
-        <v>21148</v>
+        <v>16416</v>
       </c>
       <c r="O46" s="2" t="n">
         <v>0</v>
@@ -4230,12 +4230,12 @@
       <c r="P46" s="2" t="n"/>
       <c r="Q46" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="R46" s="2" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S46" s="3" t="inlineStr">
@@ -4256,7 +4256,7 @@
       <c r="V46" s="6" t="inlineStr"/>
       <c r="W46" s="2" t="inlineStr">
         <is>
-          <t>d521fc0c870050f132722614c931ac6182bb2dbe</t>
+          <t>6b74ba6dcca9cfc12cf5e5d10aaa942cfd63c0e6</t>
         </is>
       </c>
     </row>
@@ -4270,7 +4270,7 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>2000</v>
+        <v>1900</v>
       </c>
       <c r="D47" s="2" t="n">
         <v>2</v>
@@ -4285,7 +4285,7 @@
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>Horizon - City Centre</t>
+          <t>City Centre, The Milliners, BS1 6WU</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -4293,13 +4293,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I47" s="2" t="n"/>
+      <c r="I47" s="2" t="n">
+        <v>818</v>
+      </c>
       <c r="J47" s="2" t="n"/>
       <c r="K47" s="2" t="n"/>
       <c r="L47" s="2" t="n"/>
       <c r="M47" s="2" t="n"/>
       <c r="N47" s="2" t="n">
-        <v>22020</v>
+        <v>21148</v>
       </c>
       <c r="O47" s="2" t="n">
         <v>0</v>
@@ -4307,17 +4309,17 @@
       <c r="P47" s="2" t="n"/>
       <c r="Q47" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="R47" s="2" t="inlineStr">
         <is>
-          <t>Ocean, Clifton</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S47" s="3" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T47" s="5" t="inlineStr">
@@ -4333,7 +4335,7 @@
       <c r="V47" s="6" t="inlineStr"/>
       <c r="W47" s="2" t="inlineStr">
         <is>
-          <t>8988913a4580793e64d3ae8351174e2d71317d16</t>
+          <t>d521fc0c870050f132722614c931ac6182bb2dbe</t>
         </is>
       </c>
     </row>
@@ -4347,13 +4349,13 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
       <c r="D48" s="2" t="n">
         <v>2</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -4362,7 +4364,7 @@
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>The Metropolitan, Redcliff Backs, BRISTOL, BS1</t>
+          <t>Horizon - City Centre</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -4376,7 +4378,7 @@
       <c r="L48" s="2" t="n"/>
       <c r="M48" s="2" t="n"/>
       <c r="N48" s="2" t="n">
-        <v>20320</v>
+        <v>22020</v>
       </c>
       <c r="O48" s="2" t="n">
         <v>0</v>
@@ -4384,17 +4386,17 @@
       <c r="P48" s="2" t="n"/>
       <c r="Q48" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R48" s="2" t="inlineStr">
         <is>
-          <t>Andrews Letting and Management, Clifton</t>
+          <t>Ocean, Clifton</t>
         </is>
       </c>
       <c r="S48" s="3" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T48" s="5" t="inlineStr">
@@ -4410,7 +4412,7 @@
       <c r="V48" s="6" t="inlineStr"/>
       <c r="W48" s="2" t="inlineStr">
         <is>
-          <t>48f0639d9505de53304e65370c31dc2b91415006</t>
+          <t>8988913a4580793e64d3ae8351174e2d71317d16</t>
         </is>
       </c>
     </row>
@@ -4424,10 +4426,10 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>1050</v>
+        <v>1500</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E49" s="2" t="n">
         <v>1</v>
@@ -4439,7 +4441,7 @@
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>Caslon Court, Somerset Street, Redcliffe, Bristol, BS1</t>
+          <t>The Metropolitan, Redcliff Backs, BRISTOL, BS1</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -4453,7 +4455,7 @@
       <c r="L49" s="2" t="n"/>
       <c r="M49" s="2" t="n"/>
       <c r="N49" s="2" t="n">
-        <v>18424</v>
+        <v>20320</v>
       </c>
       <c r="O49" s="2" t="n">
         <v>0</v>
@@ -4461,12 +4463,12 @@
       <c r="P49" s="2" t="n"/>
       <c r="Q49" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="R49" s="2" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>Andrews Letting and Management, Clifton</t>
         </is>
       </c>
       <c r="S49" s="3" t="inlineStr">
@@ -4487,7 +4489,7 @@
       <c r="V49" s="6" t="inlineStr"/>
       <c r="W49" s="2" t="inlineStr">
         <is>
-          <t>7183e0bb70a3ff586aa635a21825e38757f1f13d</t>
+          <t>48f0639d9505de53304e65370c31dc2b91415006</t>
         </is>
       </c>
     </row>
@@ -4501,13 +4503,13 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>1650</v>
+        <v>1050</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -4516,7 +4518,7 @@
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>Harbourside, Purifier House, BS1 5AU</t>
+          <t>Caslon Court, Somerset Street, Redcliffe, Bristol, BS1</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -4524,15 +4526,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I50" s="2" t="n">
-        <v>689</v>
-      </c>
+      <c r="I50" s="2" t="n"/>
       <c r="J50" s="2" t="n"/>
       <c r="K50" s="2" t="n"/>
       <c r="L50" s="2" t="n"/>
       <c r="M50" s="2" t="n"/>
       <c r="N50" s="2" t="n">
-        <v>16240</v>
+        <v>18424</v>
       </c>
       <c r="O50" s="2" t="n">
         <v>0</v>
@@ -4540,12 +4540,12 @@
       <c r="P50" s="2" t="n"/>
       <c r="Q50" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="R50" s="2" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Clifton</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S50" s="3" t="inlineStr">
@@ -4566,7 +4566,7 @@
       <c r="V50" s="6" t="inlineStr"/>
       <c r="W50" s="2" t="inlineStr">
         <is>
-          <t>7ec8aa4d9388bb5e923c445c92ac24d6496094c5</t>
+          <t>7183e0bb70a3ff586aa635a21825e38757f1f13d</t>
         </is>
       </c>
     </row>
@@ -4580,7 +4580,7 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>2500</v>
+        <v>1650</v>
       </c>
       <c r="D51" s="2" t="n">
         <v>2</v>
@@ -4595,7 +4595,7 @@
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>Electricity House, Colston Avenue, BS1</t>
+          <t>Harbourside, Purifier House, BS1 5AU</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -4603,13 +4603,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I51" s="2" t="n"/>
+      <c r="I51" s="2" t="n">
+        <v>689</v>
+      </c>
       <c r="J51" s="2" t="n"/>
       <c r="K51" s="2" t="n"/>
       <c r="L51" s="2" t="n"/>
       <c r="M51" s="2" t="n"/>
       <c r="N51" s="2" t="n">
-        <v>21876</v>
+        <v>16240</v>
       </c>
       <c r="O51" s="2" t="n">
         <v>0</v>
@@ -4617,12 +4619,12 @@
       <c r="P51" s="2" t="n"/>
       <c r="Q51" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="R51" s="2" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>The Bristol Residential Letting Co, Clifton</t>
         </is>
       </c>
       <c r="S51" s="3" t="inlineStr">
@@ -4643,7 +4645,7 @@
       <c r="V51" s="6" t="inlineStr"/>
       <c r="W51" s="2" t="inlineStr">
         <is>
-          <t>b2e83643f78121776465be4134c64aa64f0141c3</t>
+          <t>7ec8aa4d9388bb5e923c445c92ac24d6496094c5</t>
         </is>
       </c>
     </row>
@@ -4657,13 +4659,13 @@
         </is>
       </c>
       <c r="C52" s="4" t="n">
-        <v>1500</v>
+        <v>2500</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -4672,7 +4674,7 @@
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>The Crescent, Hannover Quay, BS1</t>
+          <t>Electricity House, Colston Avenue, BS1</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -4686,7 +4688,7 @@
       <c r="L52" s="2" t="n"/>
       <c r="M52" s="2" t="n"/>
       <c r="N52" s="2" t="n">
-        <v>16232</v>
+        <v>21876</v>
       </c>
       <c r="O52" s="2" t="n">
         <v>0</v>
@@ -4720,7 +4722,7 @@
       <c r="V52" s="6" t="inlineStr"/>
       <c r="W52" s="2" t="inlineStr">
         <is>
-          <t>6bb8673e1999d1e987f72fb4720f3d7b072fa45e</t>
+          <t>b2e83643f78121776465be4134c64aa64f0141c3</t>
         </is>
       </c>
     </row>
@@ -4734,10 +4736,10 @@
         </is>
       </c>
       <c r="C53" s="4" t="n">
-        <v>1950</v>
+        <v>1500</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>1</v>
@@ -4749,7 +4751,7 @@
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>Cheltenham House, 24A Clare Street, Bristol</t>
+          <t>The Crescent, Hannover Quay, BS1</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -4757,15 +4759,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I53" s="2" t="n">
-        <v>668</v>
-      </c>
+      <c r="I53" s="2" t="n"/>
       <c r="J53" s="2" t="n"/>
       <c r="K53" s="2" t="n"/>
       <c r="L53" s="2" t="n"/>
       <c r="M53" s="2" t="n"/>
       <c r="N53" s="2" t="n">
-        <v>21044</v>
+        <v>16232</v>
       </c>
       <c r="O53" s="2" t="n">
         <v>0</v>
@@ -4773,12 +4773,12 @@
       <c r="P53" s="2" t="n"/>
       <c r="Q53" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R53" s="2" t="inlineStr">
         <is>
-          <t>Mariana Real Estate, London</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S53" s="3" t="inlineStr">
@@ -4799,7 +4799,7 @@
       <c r="V53" s="6" t="inlineStr"/>
       <c r="W53" s="2" t="inlineStr">
         <is>
-          <t>9bdc8fdc90a88180cfd80c66940dfb5055afd30b</t>
+          <t>6bb8673e1999d1e987f72fb4720f3d7b072fa45e</t>
         </is>
       </c>
     </row>
@@ -4813,10 +4813,10 @@
         </is>
       </c>
       <c r="C54" s="4" t="n">
-        <v>1733</v>
+        <v>1950</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>1</v>
@@ -4828,7 +4828,7 @@
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>Cheltenham House, Clare Street, Bristol</t>
+          <t>Cheltenham House, 24A Clare Street, Bristol</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -4837,20 +4837,22 @@
         </is>
       </c>
       <c r="I54" s="2" t="n">
-        <v>455</v>
+        <v>668</v>
       </c>
       <c r="J54" s="2" t="n"/>
       <c r="K54" s="2" t="n"/>
       <c r="L54" s="2" t="n"/>
       <c r="M54" s="2" t="n"/>
-      <c r="N54" s="2" t="n"/>
+      <c r="N54" s="2" t="n">
+        <v>21044</v>
+      </c>
       <c r="O54" s="2" t="n">
         <v>0</v>
       </c>
       <c r="P54" s="2" t="n"/>
       <c r="Q54" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="R54" s="2" t="inlineStr">
@@ -4876,7 +4878,7 @@
       <c r="V54" s="6" t="inlineStr"/>
       <c r="W54" s="2" t="inlineStr">
         <is>
-          <t>10b717aabd38544480501915d97cf63dfbd0bcbd</t>
+          <t>9bdc8fdc90a88180cfd80c66940dfb5055afd30b</t>
         </is>
       </c>
     </row>
@@ -4890,13 +4892,13 @@
         </is>
       </c>
       <c r="C55" s="4" t="n">
-        <v>1650</v>
+        <v>1733</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -4905,34 +4907,34 @@
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>Sweetman Place, Bristol, BS2</t>
+          <t>Cheltenham House, Clare Street, Bristol</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I55" s="2" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="n">
+        <v>455</v>
+      </c>
       <c r="J55" s="2" t="n"/>
       <c r="K55" s="2" t="n"/>
       <c r="L55" s="2" t="n"/>
       <c r="M55" s="2" t="n"/>
-      <c r="N55" s="2" t="n">
-        <v>20416</v>
-      </c>
+      <c r="N55" s="2" t="n"/>
       <c r="O55" s="2" t="n">
         <v>0</v>
       </c>
       <c r="P55" s="2" t="n"/>
       <c r="Q55" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="R55" s="2" t="inlineStr">
         <is>
-          <t>Andrews Letting and Management, Clifton</t>
+          <t>Mariana Real Estate, London</t>
         </is>
       </c>
       <c r="S55" s="3" t="inlineStr">
@@ -4953,7 +4955,7 @@
       <c r="V55" s="6" t="inlineStr"/>
       <c r="W55" s="2" t="inlineStr">
         <is>
-          <t>54fa42ef8d0349a295f45392644c43dec3321c5b</t>
+          <t>10b717aabd38544480501915d97cf63dfbd0bcbd</t>
         </is>
       </c>
     </row>
@@ -4967,13 +4969,13 @@
         </is>
       </c>
       <c r="C56" s="4" t="n">
-        <v>1655</v>
+        <v>1650</v>
       </c>
       <c r="D56" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -4982,7 +4984,7 @@
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>712 Rosewood New Kingsley Road, Bristol, BS2</t>
+          <t>Sweetman Place, Bristol, BS2</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -4990,15 +4992,13 @@
           <t>BS2</t>
         </is>
       </c>
-      <c r="I56" s="2" t="n">
-        <v>547</v>
-      </c>
+      <c r="I56" s="2" t="n"/>
       <c r="J56" s="2" t="n"/>
       <c r="K56" s="2" t="n"/>
       <c r="L56" s="2" t="n"/>
       <c r="M56" s="2" t="n"/>
       <c r="N56" s="2" t="n">
-        <v>20800</v>
+        <v>20416</v>
       </c>
       <c r="O56" s="2" t="n">
         <v>0</v>
@@ -5006,12 +5006,12 @@
       <c r="P56" s="2" t="n"/>
       <c r="Q56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R56" s="2" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>Andrews Letting and Management, Clifton</t>
         </is>
       </c>
       <c r="S56" s="3" t="inlineStr">
@@ -5032,7 +5032,7 @@
       <c r="V56" s="6" t="inlineStr"/>
       <c r="W56" s="2" t="inlineStr">
         <is>
-          <t>1f8489d296d842011bdf7a2ca1f952e6b948c3d3</t>
+          <t>54fa42ef8d0349a295f45392644c43dec3321c5b</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
         </is>
       </c>
       <c r="C57" s="4" t="n">
-        <v>1665</v>
+        <v>1655</v>
       </c>
       <c r="D57" s="2" t="n">
         <v>1</v>
@@ -5061,7 +5061,7 @@
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>425 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>712 Rosewood New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -5070,7 +5070,7 @@
         </is>
       </c>
       <c r="I57" s="2" t="n">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="J57" s="2" t="n"/>
       <c r="K57" s="2" t="n"/>
@@ -5085,7 +5085,7 @@
       <c r="P57" s="2" t="n"/>
       <c r="Q57" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="R57" s="2" t="inlineStr">
@@ -5111,7 +5111,7 @@
       <c r="V57" s="6" t="inlineStr"/>
       <c r="W57" s="2" t="inlineStr">
         <is>
-          <t>c340a6dabc6dc987b590f784ea30b8d4f34f9e0c</t>
+          <t>1f8489d296d842011bdf7a2ca1f952e6b948c3d3</t>
         </is>
       </c>
     </row>
@@ -5125,13 +5125,13 @@
         </is>
       </c>
       <c r="C58" s="4" t="n">
-        <v>1700</v>
+        <v>1665</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -5140,21 +5140,23 @@
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>Steamship House, Gas Ferry Road, BS1</t>
+          <t>425 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I58" s="2" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="n">
+        <v>548</v>
+      </c>
       <c r="J58" s="2" t="n"/>
       <c r="K58" s="2" t="n"/>
       <c r="L58" s="2" t="n"/>
       <c r="M58" s="2" t="n"/>
       <c r="N58" s="2" t="n">
-        <v>14420</v>
+        <v>20800</v>
       </c>
       <c r="O58" s="2" t="n">
         <v>0</v>
@@ -5162,12 +5164,12 @@
       <c r="P58" s="2" t="n"/>
       <c r="Q58" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="R58" s="2" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S58" s="3" t="inlineStr">
@@ -5188,7 +5190,7 @@
       <c r="V58" s="6" t="inlineStr"/>
       <c r="W58" s="2" t="inlineStr">
         <is>
-          <t>f7b6312c22af08d7f7e765adf92d9a3fb0f82781</t>
+          <t>c340a6dabc6dc987b590f784ea30b8d4f34f9e0c</t>
         </is>
       </c>
     </row>
@@ -5202,13 +5204,13 @@
         </is>
       </c>
       <c r="C59" s="4" t="n">
-        <v>1200</v>
+        <v>1700</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -5217,7 +5219,7 @@
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>City Centre, Corinthian Court, BS1</t>
+          <t>Steamship House, Gas Ferry Road, BS1</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -5225,15 +5227,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I59" s="2" t="n">
-        <v>389</v>
-      </c>
+      <c r="I59" s="2" t="n"/>
       <c r="J59" s="2" t="n"/>
       <c r="K59" s="2" t="n"/>
       <c r="L59" s="2" t="n"/>
       <c r="M59" s="2" t="n"/>
       <c r="N59" s="2" t="n">
-        <v>18820</v>
+        <v>14420</v>
       </c>
       <c r="O59" s="2" t="n">
         <v>0</v>
@@ -5241,12 +5241,12 @@
       <c r="P59" s="2" t="n"/>
       <c r="Q59" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R59" s="2" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S59" s="3" t="inlineStr">
@@ -5267,7 +5267,7 @@
       <c r="V59" s="6" t="inlineStr"/>
       <c r="W59" s="2" t="inlineStr">
         <is>
-          <t>5aed40eba285a7fa0266bfe8eb49613bb2f96c97</t>
+          <t>f7b6312c22af08d7f7e765adf92d9a3fb0f82781</t>
         </is>
       </c>
     </row>
@@ -5281,13 +5281,13 @@
         </is>
       </c>
       <c r="C60" s="4" t="n">
-        <v>2750</v>
+        <v>1200</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -5296,23 +5296,23 @@
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>St. Johns Road, Southville, BS3</t>
+          <t>City Centre, Corinthian Court, BS1</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>BS3</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I60" s="2" t="n">
-        <v>872</v>
+        <v>389</v>
       </c>
       <c r="J60" s="2" t="n"/>
       <c r="K60" s="2" t="n"/>
       <c r="L60" s="2" t="n"/>
       <c r="M60" s="2" t="n"/>
       <c r="N60" s="2" t="n">
-        <v>13836</v>
+        <v>18820</v>
       </c>
       <c r="O60" s="2" t="n">
         <v>0</v>
@@ -5320,12 +5320,12 @@
       <c r="P60" s="2" t="n"/>
       <c r="Q60" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="R60" s="2" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S60" s="3" t="inlineStr">
@@ -5346,7 +5346,7 @@
       <c r="V60" s="6" t="inlineStr"/>
       <c r="W60" s="2" t="inlineStr">
         <is>
-          <t>1ef2a873cf32bf32a071baeaf2161ff3ecb818e3</t>
+          <t>5aed40eba285a7fa0266bfe8eb49613bb2f96c97</t>
         </is>
       </c>
     </row>
@@ -5360,13 +5360,13 @@
         </is>
       </c>
       <c r="C61" s="4" t="n">
-        <v>1150</v>
+        <v>2750</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -5375,21 +5375,23 @@
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>Stokes Croft, Stokes Croft, Bristol, BS1</t>
+          <t>St. Johns Road, Southville, BS3</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I61" s="2" t="n"/>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="n">
+        <v>872</v>
+      </c>
       <c r="J61" s="2" t="n"/>
       <c r="K61" s="2" t="n"/>
       <c r="L61" s="2" t="n"/>
       <c r="M61" s="2" t="n"/>
       <c r="N61" s="2" t="n">
-        <v>21780</v>
+        <v>13836</v>
       </c>
       <c r="O61" s="2" t="n">
         <v>0</v>
@@ -5397,12 +5399,12 @@
       <c r="P61" s="2" t="n"/>
       <c r="Q61" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="R61" s="2" t="inlineStr">
         <is>
-          <t>CJ Hole, Bishopston</t>
+          <t>Acen Properties, Bristol</t>
         </is>
       </c>
       <c r="S61" s="3" t="inlineStr">
@@ -5423,7 +5425,7 @@
       <c r="V61" s="6" t="inlineStr"/>
       <c r="W61" s="2" t="inlineStr">
         <is>
-          <t>b7b81b252c97079f6dd65df48976cfecbee9e434</t>
+          <t>1ef2a873cf32bf32a071baeaf2161ff3ecb818e3</t>
         </is>
       </c>
     </row>
@@ -5437,10 +5439,10 @@
         </is>
       </c>
       <c r="C62" s="4" t="n">
-        <v>1900</v>
+        <v>1150</v>
       </c>
       <c r="D62" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E62" s="2" t="n">
         <v>1</v>
@@ -5452,7 +5454,7 @@
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>Redcliff Street, Bristol, BS1</t>
+          <t>Stokes Croft, Stokes Croft, Bristol, BS1</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -5460,28 +5462,26 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I62" s="2" t="n">
-        <v>731</v>
-      </c>
+      <c r="I62" s="2" t="n"/>
       <c r="J62" s="2" t="n"/>
       <c r="K62" s="2" t="n"/>
       <c r="L62" s="2" t="n"/>
       <c r="M62" s="2" t="n"/>
       <c r="N62" s="2" t="n">
-        <v>20892</v>
+        <v>21780</v>
       </c>
       <c r="O62" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P62" s="2" t="n"/>
       <c r="Q62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="R62" s="2" t="inlineStr">
         <is>
-          <t>A2Dominion Group, A2Dominion Lettings</t>
+          <t>CJ Hole, Bishopston</t>
         </is>
       </c>
       <c r="S62" s="3" t="inlineStr">
@@ -5502,7 +5502,7 @@
       <c r="V62" s="6" t="inlineStr"/>
       <c r="W62" s="2" t="inlineStr">
         <is>
-          <t>c11b7a868ede7c3b0a3d524aa4d4e8f661494706</t>
+          <t>b7b81b252c97079f6dd65df48976cfecbee9e434</t>
         </is>
       </c>
     </row>
@@ -5516,10 +5516,10 @@
         </is>
       </c>
       <c r="C63" s="4" t="n">
-        <v>1400</v>
+        <v>1900</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>1</v>
@@ -5531,7 +5531,7 @@
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>St. James Barton, Bristol, Somerset, BS1</t>
+          <t>Redcliff Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -5539,26 +5539,28 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I63" s="2" t="n"/>
+      <c r="I63" s="2" t="n">
+        <v>731</v>
+      </c>
       <c r="J63" s="2" t="n"/>
       <c r="K63" s="2" t="n"/>
       <c r="L63" s="2" t="n"/>
       <c r="M63" s="2" t="n"/>
       <c r="N63" s="2" t="n">
-        <v>22132</v>
+        <v>20892</v>
       </c>
       <c r="O63" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P63" s="2" t="n"/>
       <c r="Q63" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="R63" s="2" t="inlineStr">
         <is>
-          <t>Balloon Letting Company, Bristol</t>
+          <t>A2Dominion Group, A2Dominion Lettings</t>
         </is>
       </c>
       <c r="S63" s="3" t="inlineStr">
@@ -5579,7 +5581,7 @@
       <c r="V63" s="6" t="inlineStr"/>
       <c r="W63" s="2" t="inlineStr">
         <is>
-          <t>f2c75a0f99c7c358be96a67019a6c639e60845fb</t>
+          <t>c11b7a868ede7c3b0a3d524aa4d4e8f661494706</t>
         </is>
       </c>
     </row>
@@ -5593,13 +5595,13 @@
         </is>
       </c>
       <c r="C64" s="4" t="n">
-        <v>2770</v>
+        <v>1400</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -5608,23 +5610,21 @@
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>223 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>St. James Barton, Bristol, Somerset, BS1</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I64" s="2" t="n">
-        <v>1047</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="n"/>
       <c r="J64" s="2" t="n"/>
       <c r="K64" s="2" t="n"/>
       <c r="L64" s="2" t="n"/>
       <c r="M64" s="2" t="n"/>
       <c r="N64" s="2" t="n">
-        <v>20800</v>
+        <v>22132</v>
       </c>
       <c r="O64" s="2" t="n">
         <v>0</v>
@@ -5632,12 +5632,12 @@
       <c r="P64" s="2" t="n"/>
       <c r="Q64" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="R64" s="2" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>Balloon Letting Company, Bristol</t>
         </is>
       </c>
       <c r="S64" s="3" t="inlineStr">
@@ -5658,7 +5658,7 @@
       <c r="V64" s="6" t="inlineStr"/>
       <c r="W64" s="2" t="inlineStr">
         <is>
-          <t>c100863cd4596aeb0516b88e90339b58d5383f81</t>
+          <t>f2c75a0f99c7c358be96a67019a6c639e60845fb</t>
         </is>
       </c>
     </row>
@@ -5672,13 +5672,13 @@
         </is>
       </c>
       <c r="C65" s="4" t="n">
-        <v>1195</v>
+        <v>2770</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -5687,21 +5687,23 @@
       </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
-          <t>St Johns Lane, Bedminster, Bristol, BS3</t>
+          <t>223 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I65" s="2" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="n">
+        <v>1047</v>
+      </c>
       <c r="J65" s="2" t="n"/>
       <c r="K65" s="2" t="n"/>
       <c r="L65" s="2" t="n"/>
       <c r="M65" s="2" t="n"/>
       <c r="N65" s="2" t="n">
-        <v>7052</v>
+        <v>20800</v>
       </c>
       <c r="O65" s="2" t="n">
         <v>0</v>
@@ -5709,12 +5711,12 @@
       <c r="P65" s="2" t="n"/>
       <c r="Q65" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="R65" s="2" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S65" s="3" t="inlineStr">
@@ -5735,7 +5737,7 @@
       <c r="V65" s="6" t="inlineStr"/>
       <c r="W65" s="2" t="inlineStr">
         <is>
-          <t>debefb53a4e113c2e87087647138ae147bbe2ce7</t>
+          <t>c100863cd4596aeb0516b88e90339b58d5383f81</t>
         </is>
       </c>
     </row>
@@ -5749,7 +5751,7 @@
         </is>
       </c>
       <c r="C66" s="4" t="n">
-        <v>1400</v>
+        <v>1195</v>
       </c>
       <c r="D66" s="2" t="n">
         <v>1</v>
@@ -5764,23 +5766,21 @@
       </c>
       <c r="G66" s="3" t="inlineStr">
         <is>
-          <t>Harbourside, The Crescent, BS1 5JP</t>
+          <t>St Johns Lane, Bedminster, Bristol, BS3</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I66" s="2" t="n">
-        <v>517</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="n"/>
       <c r="J66" s="2" t="n"/>
       <c r="K66" s="2" t="n"/>
       <c r="L66" s="2" t="n"/>
       <c r="M66" s="2" t="n"/>
       <c r="N66" s="2" t="n">
-        <v>16368</v>
+        <v>7052</v>
       </c>
       <c r="O66" s="2" t="n">
         <v>0</v>
@@ -5788,12 +5788,12 @@
       <c r="P66" s="2" t="n"/>
       <c r="Q66" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="R66" s="2" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Clifton</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S66" s="3" t="inlineStr">
@@ -5814,7 +5814,7 @@
       <c r="V66" s="6" t="inlineStr"/>
       <c r="W66" s="2" t="inlineStr">
         <is>
-          <t>bfcffcdb5bdab46e12aada59c56fe3f93ba997e3</t>
+          <t>debefb53a4e113c2e87087647138ae147bbe2ce7</t>
         </is>
       </c>
     </row>
@@ -5828,49 +5828,51 @@
         </is>
       </c>
       <c r="C67" s="4" t="n">
-        <v>2600</v>
+        <v>1400</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
         <is>
-          <t>Northfolk Heights, BS2</t>
+          <t>Harbourside, The Crescent, BS1 5JP</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I67" s="2" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="n">
+        <v>517</v>
+      </c>
       <c r="J67" s="2" t="n"/>
       <c r="K67" s="2" t="n"/>
       <c r="L67" s="2" t="n"/>
       <c r="M67" s="2" t="n"/>
       <c r="N67" s="2" t="n">
-        <v>21828</v>
+        <v>16368</v>
       </c>
       <c r="O67" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P67" s="2" t="n"/>
       <c r="Q67" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="R67" s="2" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol</t>
+          <t>The Bristol Residential Letting Co, Clifton</t>
         </is>
       </c>
       <c r="S67" s="3" t="inlineStr">
@@ -5891,7 +5893,7 @@
       <c r="V67" s="6" t="inlineStr"/>
       <c r="W67" s="2" t="inlineStr">
         <is>
-          <t>0298e5d4f5c982dcf613c87aeb4743c13a5f97e5</t>
+          <t>bfcffcdb5bdab46e12aada59c56fe3f93ba997e3</t>
         </is>
       </c>
     </row>
@@ -9181,7 +9183,9 @@
       <c r="K112" s="2" t="n"/>
       <c r="L112" s="2" t="n"/>
       <c r="M112" s="2" t="n"/>
-      <c r="N112" s="2" t="n"/>
+      <c r="N112" s="2" t="n">
+        <v>20592</v>
+      </c>
       <c r="O112" s="2" t="n">
         <v>0</v>
       </c>
@@ -13423,158 +13427,10 @@
         </is>
       </c>
     </row>
-    <row r="170">
-      <c r="A170" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B170" s="3" t="inlineStr">
-        <is>
-          <t>Keyword match only (no API key configured for full scoring).</t>
-        </is>
-      </c>
-      <c r="C170" s="4" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D170" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E170" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F170" s="2" t="inlineStr">
-        <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="G170" s="3" t="inlineStr">
-        <is>
-          <t>Baldwin Street, Bristol, BS1</t>
-        </is>
-      </c>
-      <c r="H170" s="2" t="inlineStr">
-        <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I170" s="2" t="n">
-        <v>413</v>
-      </c>
-      <c r="J170" s="2" t="n"/>
-      <c r="K170" s="2" t="n"/>
-      <c r="L170" s="2" t="n"/>
-      <c r="M170" s="2" t="n"/>
-      <c r="N170" s="2" t="n">
-        <v>21148</v>
-      </c>
-      <c r="O170" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="P170" s="2" t="n"/>
-      <c r="Q170" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="R170" s="2" t="inlineStr">
-        <is>
-          <t>Savills Lettings, Clifton</t>
-        </is>
-      </c>
-      <c r="S170" s="3" t="inlineStr"/>
-      <c r="T170" s="5" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U170" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V170" s="6" t="inlineStr"/>
-      <c r="W170" s="2" t="inlineStr">
-        <is>
-          <t>ca58d4891f705dc219b7ca74ef59637a2959afb0</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B171" s="3" t="inlineStr">
-        <is>
-          <t>Keyword match only (no API key configured for full scoring).</t>
-        </is>
-      </c>
-      <c r="C171" s="4" t="n">
-        <v>1850</v>
-      </c>
-      <c r="D171" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E171" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F171" s="2" t="inlineStr">
-        <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="G171" s="3" t="inlineStr">
-        <is>
-          <t>Waverley House, Cathedral Walk, Bristol, BS1</t>
-        </is>
-      </c>
-      <c r="H171" s="2" t="inlineStr">
-        <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I171" s="2" t="n"/>
-      <c r="J171" s="2" t="n"/>
-      <c r="K171" s="2" t="n"/>
-      <c r="L171" s="2" t="n"/>
-      <c r="M171" s="2" t="n"/>
-      <c r="N171" s="2" t="n">
-        <v>17744</v>
-      </c>
-      <c r="O171" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P171" s="2" t="n"/>
-      <c r="Q171" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="R171" s="2" t="inlineStr">
-        <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
-        </is>
-      </c>
-      <c r="S171" s="3" t="inlineStr"/>
-      <c r="T171" s="5" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U171" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V171" s="6" t="inlineStr"/>
-      <c r="W171" s="2" t="inlineStr">
-        <is>
-          <t>6cceb5caf1d4ecfbb28b35bd698eadc65e6909ed</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:W171"/>
+  <autoFilter ref="A1:W169"/>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -13747,8 +13603,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T167" r:id="rId166"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T168" r:id="rId167"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T169" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T170" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T171" r:id="rId170"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>